<commit_message>
Aprimora redações do mapa e da matriz pós-comentários
</commit_message>
<xml_diff>
--- a/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
+++ b/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
@@ -669,7 +669,7 @@
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>Procedimento para verificar a questão Q6: A organização adota controles mínimos na fase preparatória das contratações de TIC, com processo definido e análise técnica pela unidade competente?</t>
+          <t>Procedimento para verificar a questão Q6: A organização adota processo formal e padronizado para a fase preparatória das contratações de TIC, com responsabilidades definidas, análise técnica pela área de TIC e alinhamento aos instrumentos de planejamento?</t>
         </is>
       </c>
       <c r="C9" s="1" t="inlineStr">
@@ -1777,7 +1777,7 @@
       <c r="I19" s="1" t="n"/>
       <c r="J19" s="1" t="inlineStr">
         <is>
-          <t>Plano de TIC sem previsão orçamentária demonstrada.</t>
+          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
         </is>
       </c>
       <c r="K19" s="1" t="inlineStr">
@@ -1795,7 +1795,7 @@
       <c r="O19" s="1" t="n"/>
       <c r="P19" s="1" t="inlineStr">
         <is>
-          <t>inclua no plano de TIC a estimativa dos recursos orçamentários necessários à execução das iniciativas priorizadas, com memória ou referência que permita acompanhar sua viabilidade</t>
+          <t>integre o plano de TIC à elaboração da proposta orçamentária e do plano de contratações, de maneira proporcional ao porte, à estrutura e à capacidade de planejamento da organização</t>
         </is>
       </c>
     </row>
@@ -3750,7 +3750,7 @@
       <c r="I54" s="1" t="n"/>
       <c r="J54" s="1" t="inlineStr">
         <is>
-          <t>Plano de TIC sem previsão orçamentária demonstrada.</t>
+          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
         </is>
       </c>
       <c r="K54" s="1" t="inlineStr">
@@ -3768,7 +3768,7 @@
       <c r="O54" s="1" t="n"/>
       <c r="P54" s="1" t="inlineStr">
         <is>
-          <t>inclua no plano de TIC a estimativa dos recursos orçamentários necessários à execução das iniciativas priorizadas, com memória ou referência que permita acompanhar sua viabilidade</t>
+          <t>integre o plano de TIC à elaboração da proposta orçamentária e do plano de contratações, de maneira proporcional ao porte, à estrutura e à capacidade de planejamento da organização</t>
         </is>
       </c>
     </row>
@@ -6065,7 +6065,7 @@
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Plano de TIC sem previsão orçamentária demonstrada.</t>
+          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
         </is>
       </c>
       <c r="D28" s="9" t="n">
@@ -6103,7 +6103,7 @@
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Plano de TIC sem previsão orçamentária demonstrada.</t>
+          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
         </is>
       </c>
       <c r="D29" s="9" t="n">

</xml_diff>

<commit_message>
Revisa a Questão 1 da matriz e do mapa
</commit_message>
<xml_diff>
--- a/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
+++ b/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
@@ -557,7 +557,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>Estrutura de TIC insuficiente para coordenar, gerir e sustentar a tecnologia da informação.</t>
+          <t>Estrutura de TIC insuficientemente formalizada, definida ou posicionada para gerir a tecnologia da informação.</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>Procedimento para verificar a questão Q4: A organização dispõe de capacidade institucional mínima, em termos de força de trabalho, perfis profissionais, competências, funções e vínculos, para planejar, gerir, proteger, contratar, fiscalizar e sustentar a TIC e a segurança da informação de forma adequada às suas necessidades institucionais?</t>
+          <t>Procedimento para verificar a questão Q4: A organização dispõe de capacidade institucional mínima, em termos de força de trabalho, funções e vínculos, para planejar, gerir, proteger, contratar, fiscalizar e sustentar a TIC e a segurança da informação de forma adequada às suas necessidades institucionais?</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
@@ -907,10 +907,7 @@
       <c r="G4" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO01.04 - Definir e implementar as estruturas organizacionais: estabelecer estruturas organizacionais internas e externas necessárias para apoiar os objetivos de governança e gestão de TI.
-COBIT 2019, APO01.09 - Definição e comunicação de políticas e procedimentos: estabelecer e comunicar políticas e procedimentos de gestão de TI que orientem papéis, responsabilidades e controles.
-ABNT NBR ISO/IEC 38500:2025, item 5.6.1 - Governança efetiva de TI: responsabilização clara, estrutura adequada de tomada de decisão e direção organizacional compatível com o uso atual e futuro da tecnologia.
-Constituição Federal, art. 37, caput: princípios da legalidade e da eficiência.
-Lei nº 14.133/2021, art. 11, parágrafo único: dever da alta administração de implementar processos e estruturas de governança das contratações.</t>
+Constituição Federal, art. 37, caput - Princípio da eficiência.</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
@@ -933,13 +930,13 @@
       <c r="M4" s="1" t="n"/>
       <c r="N4" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O4" s="1" t="n"/>
       <c r="P4" s="1" t="inlineStr">
         <is>
-          <t>formalize a área, unidade, setor ou função de TIC em instrumento compatível com a organização, definindo vinculação e responsabilidades essenciais, admitida estrutura equivalente que assegure o resultado de governança exigido</t>
+          <t>formalize a área, unidade, setor ou função de TIC em instrumento compatível com a organização, definindo vinculação e responsabilidades essenciais de modo compatível com o porte, a complexidade e a dependência tecnológica da organização</t>
         </is>
       </c>
     </row>
@@ -965,10 +962,7 @@
       <c r="G5" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TI.
-COBIT 2019, APO01.09 - Definição e comunicação de políticas e procedimentos: estabelecer e comunicar políticas e procedimentos de gestão de TI que orientem papéis, responsabilidades e controles.
-ABNT NBR ISO/IEC 38500:2025, item 5.6.1 - Governança efetiva de TI: responsabilização clara, estrutura adequada de tomada de decisão e direção organizacional compatível com o uso atual e futuro da tecnologia.
-Constituição Federal, art. 37, caput: princípios da legalidade e da eficiência.
-Lei nº 14.133/2021, art. 11, parágrafo único: dever da alta administração de implementar processos e estruturas de governança das contratações.</t>
+Constituição Federal, art. 37, caput - Princípio da eficiência.</t>
         </is>
       </c>
       <c r="H5" s="1" t="inlineStr">
@@ -979,7 +973,7 @@
       <c r="I5" s="1" t="n"/>
       <c r="J5" s="1" t="inlineStr">
         <is>
-          <t>Área de TIC sem atribuições formalmente definidas ou sem atribuições formais de governança, planejamento ou gestão de TIC.</t>
+          <t>Área de TIC sem atribuições formalmente definidas ou sem atribuições formais de gestão de TIC.</t>
         </is>
       </c>
       <c r="K5" s="1" t="inlineStr">
@@ -991,13 +985,13 @@
       <c r="M5" s="1" t="n"/>
       <c r="N5" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O5" s="1" t="n"/>
       <c r="P5" s="1" t="inlineStr">
         <is>
-          <t>defina formalmente as atribuições da área de TIC, incluindo, no mínimo, responsabilidades de governança, planejamento e gestão de TIC, em instrumento compatível com a estrutura da organização</t>
+          <t>defina formalmente as atribuições da área de TIC, atentando-se, minimamente, em abranger as atividades de planejamento, coordenação, gestão e controle da TIC</t>
         </is>
       </c>
     </row>
@@ -1023,10 +1017,7 @@
       <c r="G6" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TI.
-COBIT 2019, APO01.09 - Definição e comunicação de políticas e procedimentos: estabelecer e comunicar políticas e procedimentos de gestão de TI que orientem papéis, responsabilidades e controles.
-ABNT NBR ISO/IEC 38500:2025, item 5.6.1 - Governança efetiva de TI: responsabilização clara, estrutura adequada de tomada de decisão e direção organizacional compatível com o uso atual e futuro da tecnologia.
-Constituição Federal, art. 37, caput: princípios da legalidade e da eficiência.
-Lei nº 14.133/2021, art. 11, parágrafo único: dever da alta administração de implementar processos e estruturas de governança das contratações.</t>
+Constituição Federal, art. 37, caput - Princípio da eficiência.</t>
         </is>
       </c>
       <c r="H6" s="1" t="inlineStr">
@@ -1037,7 +1028,7 @@
       <c r="I6" s="1" t="n"/>
       <c r="J6" s="1" t="inlineStr">
         <is>
-          <t>Área de TIC sem atribuições formalmente definidas ou sem atribuições formais de governança, planejamento ou gestão de TIC.</t>
+          <t>Área de TIC sem atribuições formalmente definidas ou sem atribuições formais de gestão de TIC.</t>
         </is>
       </c>
       <c r="K6" s="1" t="inlineStr">
@@ -1049,13 +1040,13 @@
       <c r="M6" s="1" t="n"/>
       <c r="N6" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O6" s="1" t="n"/>
       <c r="P6" s="1" t="inlineStr">
         <is>
-          <t>defina formalmente as atribuições da área de TIC, incluindo, no mínimo, responsabilidades de governança, planejamento e gestão de TIC, em instrumento compatível com a estrutura da organização</t>
+          <t>defina formalmente as atribuições da área de TIC, atentando-se, minimamente, em abranger as atividades de planejamento, coordenação, gestão e controle da TIC</t>
         </is>
       </c>
     </row>
@@ -1081,10 +1072,7 @@
       <c r="G7" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TI.
-COBIT 2019, APO01.09 - Definição e comunicação de políticas e procedimentos: estabelecer e comunicar políticas e procedimentos de gestão de TI que orientem papéis, responsabilidades e controles.
-ABNT NBR ISO/IEC 38500:2025, item 5.6.1 - Governança efetiva de TI: responsabilização clara, estrutura adequada de tomada de decisão e direção organizacional compatível com o uso atual e futuro da tecnologia.
-Constituição Federal, art. 37, caput: princípios da legalidade e da eficiência.
-Lei nº 14.133/2021, art. 11, parágrafo único: dever da alta administração de implementar processos e estruturas de governança das contratações.</t>
+Constituição Federal, art. 37, caput - Princípio da eficiência.</t>
         </is>
       </c>
       <c r="H7" s="1" t="inlineStr">
@@ -1095,7 +1083,7 @@
       <c r="I7" s="1" t="n"/>
       <c r="J7" s="1" t="inlineStr">
         <is>
-          <t>Área de TIC sem atribuições formalmente definidas ou sem atribuições formais de governança, planejamento ou gestão de TIC.</t>
+          <t>Área de TIC sem atribuições formalmente definidas ou sem atribuições formais de gestão de TIC.</t>
         </is>
       </c>
       <c r="K7" s="1" t="inlineStr">
@@ -1107,13 +1095,13 @@
       <c r="M7" s="1" t="n"/>
       <c r="N7" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O7" s="1" t="n"/>
       <c r="P7" s="1" t="inlineStr">
         <is>
-          <t>defina formalmente as atribuições da área de TIC, incluindo, no mínimo, responsabilidades de governança, planejamento e gestão de TIC, em instrumento compatível com a estrutura da organização</t>
+          <t>defina formalmente as atribuições da área de TIC, atentando-se, minimamente, em abranger as atividades de planejamento, coordenação, gestão e controle da TIC</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1127,6 @@
       <c r="G8" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO01.06 - Aprimorar o posicionamento da função de TI: posicionar a função de tecnologia de modo compatível com sua relevância estratégica, responsabilidades e necessidade de interação com a alta administração.
-ABNT NBR ISO/IEC 38500:2025, item 5.6.1 - Governança efetiva de TI: responsabilização clara, estrutura adequada de tomada de decisão e direção organizacional compatível com o uso atual e futuro da tecnologia.
 Portaria SGD/ME nº 778/2019, art. 4º, § 1º - Referência de posicionamento organizacional: para a obtenção de melhores resultados, a área de TIC de cada órgão ou entidade deve, preferencialmente, estar vinculada à alta administração, com o intuito de apoiá-la na tomada de decisões e no alcance dos objetivos estratégicos.</t>
         </is>
       </c>
@@ -1169,7 +1156,7 @@
       <c r="O8" s="1" t="n"/>
       <c r="P8" s="1" t="inlineStr">
         <is>
-          <t>avalie e ajuste o posicionamento organizacional da área de TIC, atentando-se, minimamente, em assegurar interlocução adequada com a alta administração e participação nas decisões estratégicas, orçamentárias, contratuais e de gestão de riscos relacionadas à tecnologia da informação</t>
+          <t>avalie o posicionamento organizacional da área de TIC e adote, quando necessário, medidas para assegurar interlocução adequada com a alta administração e participação nas decisões estratégicas, orçamentárias, contratuais e de gestão de riscos relacionadas à tecnologia da informação.</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1182,6 @@
       <c r="G9" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO01.06 - Aprimorar o posicionamento da função de TI: posicionar a função de tecnologia de modo compatível com sua relevância estratégica, responsabilidades e necessidade de interação com a alta administração.
-ABNT NBR ISO/IEC 38500:2025, item 5.6.1 - Governança efetiva de TI: responsabilização clara, estrutura adequada de tomada de decisão e direção organizacional compatível com o uso atual e futuro da tecnologia.
 Portaria SGD/ME nº 778/2019, art. 4º, § 1º - Referência de posicionamento organizacional: para a obtenção de melhores resultados, a área de TIC de cada órgão ou entidade deve, preferencialmente, estar vinculada à alta administração, com o intuito de apoiá-la na tomada de decisões e no alcance dos objetivos estratégicos.</t>
         </is>
       </c>
@@ -1225,7 +1211,7 @@
       <c r="O9" s="1" t="n"/>
       <c r="P9" s="1" t="inlineStr">
         <is>
-          <t>avalie e ajuste o posicionamento organizacional da área de TIC, atentando-se, minimamente, em assegurar interlocução adequada com a alta administração e participação nas decisões estratégicas, orçamentárias, contratuais e de gestão de riscos relacionadas à tecnologia da informação</t>
+          <t>avalie o posicionamento organizacional da área de TIC e adote, quando necessário, medidas para assegurar interlocução adequada com a alta administração e participação nas decisões estratégicas, orçamentárias, contratuais e de gestão de riscos relacionadas à tecnologia da informação.</t>
         </is>
       </c>
     </row>
@@ -1250,8 +1236,7 @@
       </c>
       <c r="G10" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, EDM01.02 - Dirigir o sistema de governança: orientar estruturas, princípios, processos e práticas de governança para assegurar que a TI apoie os objetivos organizacionais.
-COBIT 2019, MEA01.04 - Avaliar o desempenho: monitorar e avaliar periodicamente o desempenho e a conformidade da TI em relação a objetivos, indicadores, metas e expectativas das partes interessadas.
+          <t>COBIT 2019, MEA01.04 - Avaliar o desempenho: monitorar e avaliar periodicamente o desempenho e a conformidade da TI em relação a objetivos, indicadores, metas e expectativas das partes interessadas.
 Acórdão TCE-RJ 44.490/2024-PLEN, item II.1: necessidade de estrutura de governança de TI, especialmente Comitê de Tecnologia da Informação ou instância equivalente, com participação de áreas relevantes, responsabilidade de alinhar as ações de TI aos objetivos institucionais, priorizar investimentos e monitorar o desempenho da TI com base em indicadores e metas.</t>
         </is>
       </c>
@@ -1275,13 +1260,13 @@
       <c r="M10" s="1" t="n"/>
       <c r="N10" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O10" s="1" t="n"/>
       <c r="P10" s="1" t="inlineStr">
         <is>
-          <t>estabeleça objetivos, indicadores e metas para a gestão de TIC, aprovados ou formalmente definidos pela alta administração, e mantenha-os vinculados aos resultados institucionais pretendidos</t>
+          <t>estabeleça modelo básico de governança e gestão de TIC definindo objetivos, indicadores, metas e forma de acompanhamento periódico do desempenho da TIC pela alta administração</t>
         </is>
       </c>
     </row>
@@ -1306,9 +1291,7 @@
       </c>
       <c r="G11" s="1" t="inlineStr">
         <is>
-          <t>Decreto nº 12.198/2024, art. 5º - Instituição do CGD, colegiado responsável por definir diretrizes e estratégias sobre uso de recursos digitais nos órgãos e entidades da administração pública federal direta, autárquica e fundacional.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.1: necessidade de estrutura de governança de TI, especialmente Comitê de Tecnologia da Informação ou instância equivalente, com participação de áreas relevantes, responsabilidade de alinhar as ações de TI aos objetivos institucionais, priorizar investimentos e monitorar o desempenho da TI com base em indicadores e metas.
-COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TI.
+          <t>Acórdão TCE-RJ 44.490/2024-PLEN, item II.1: necessidade de estrutura de governança de TI, especialmente Comitê de Tecnologia da Informação ou instância equivalente, com participação de áreas relevantes, responsabilidade de alinhar as ações de TI aos objetivos institucionais, priorizar investimentos e monitorar o desempenho da TI com base em indicadores e metas.
 Lei nº 14.133/2021, art. 11, parágrafo único: dever da alta administração de implementar estruturas de governança das contratações.
 Acórdão TCU nº 1.411/2014-Plenário, item 9.1.2: precedente sobre funcionamento permanente e composição relevante do Comitê de TIC.</t>
         </is>
@@ -1339,7 +1322,7 @@
       <c r="O11" s="1" t="n"/>
       <c r="P11" s="1" t="inlineStr">
         <is>
-          <t>institua formalmente Comitê de TIC ou instância colegiada equivalente, compatível com o porte e a estrutura decisória da organização, com composição, competências, periodicidade e forma de registro definidas</t>
+          <t>institua formalmente Comitê de TIC ou instância colegiada equivalente, compatível com o porte e a estrutura decisória da organização, atentando-se, minimamente, em definir sua composição, competências, periodicidade de reuniões, forma de registro das deliberações e acompanhamento dos encaminhamentos</t>
         </is>
       </c>
     </row>
@@ -1365,10 +1348,7 @@
       <c r="G12" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, MEA01.04 - Avaliar o desempenho: monitorar e avaliar periodicamente o desempenho e a conformidade da TI em relação a objetivos, indicadores, metas e expectativas das partes interessadas.
-Decreto nº 12.198/2024, art. 5º - Instituição do CGD, colegiado responsável por definir diretrizes e estratégias sobre uso de recursos digitais nos órgãos e entidades da administração pública federal direta, autárquica e fundacional.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.1: necessidade de estrutura de governança de TI, especialmente Comitê de Tecnologia da Informação ou instância equivalente, com participação de áreas relevantes, responsabilidade de alinhar as ações de TI aos objetivos institucionais, priorizar investimentos e monitorar o desempenho da TI com base em indicadores e metas.
-Constituição Federal, art. 37, caput: princípio da eficiência.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, item II.1: precedente de determinação para Comitê de TIC com responsabilidades de alinhamento, priorização e monitoramento.</t>
+Acórdão TCE-RJ 44.490/2024-PLEN, item II.1: necessidade de estrutura de governança de TI, especialmente Comitê de Tecnologia da Informação ou instância equivalente, com participação de áreas relevantes, responsabilidade de alinhar as ações de TI aos objetivos institucionais, priorizar investimentos e monitorar o desempenho da TI com base em indicadores e metas.</t>
         </is>
       </c>
       <c r="H12" s="1" t="inlineStr">
@@ -1397,7 +1377,7 @@
       <c r="O12" s="1" t="n"/>
       <c r="P12" s="1" t="inlineStr">
         <is>
-          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância equivalente, realizando reuniões, registrando deliberações e acompanhando os encaminhamentos relevantes</t>
+          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância colegiada equivalente, compatível com o porte e a estrutura decisória da organização, atentando-se, minimamente, em realizar reuniões periódicas, registrar deliberações e acompanhar decisões sobre prioridades, projetos, riscos, serviços, orçamento e contratações de TIC</t>
         </is>
       </c>
     </row>
@@ -1423,10 +1403,7 @@
       <c r="G13" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, MEA01.04 - Avaliar o desempenho: monitorar e avaliar periodicamente o desempenho e a conformidade da TI em relação a objetivos, indicadores, metas e expectativas das partes interessadas.
-Decreto nº 12.198/2024, art. 5º - Instituição do CGD, colegiado responsável por definir diretrizes e estratégias sobre uso de recursos digitais nos órgãos e entidades da administração pública federal direta, autárquica e fundacional.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.1: necessidade de estrutura de governança de TI, especialmente Comitê de Tecnologia da Informação ou instância equivalente, com participação de áreas relevantes, responsabilidade de alinhar as ações de TI aos objetivos institucionais, priorizar investimentos e monitorar o desempenho da TI com base em indicadores e metas.
-Constituição Federal, art. 37, caput: princípio da eficiência.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, item II.1: precedente de determinação para Comitê de TIC com responsabilidades de alinhamento, priorização e monitoramento.</t>
+Acórdão TCE-RJ 44.490/2024-PLEN, item II.1: necessidade de estrutura de governança de TI, especialmente Comitê de Tecnologia da Informação ou instância equivalente, com participação de áreas relevantes, responsabilidade de alinhar as ações de TI aos objetivos institucionais, priorizar investimentos e monitorar o desempenho da TI com base em indicadores e metas.</t>
         </is>
       </c>
       <c r="H13" s="1" t="inlineStr">
@@ -1455,7 +1432,7 @@
       <c r="O13" s="1" t="n"/>
       <c r="P13" s="1" t="inlineStr">
         <is>
-          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância equivalente, realizando reuniões, registrando deliberações e acompanhando os encaminhamentos relevantes</t>
+          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância colegiada equivalente, compatível com o porte e a estrutura decisória da organização, atentando-se, minimamente, em realizar reuniões periódicas, registrar deliberações e acompanhar decisões sobre prioridades, projetos, riscos, serviços, orçamento e contratações de TIC</t>
         </is>
       </c>
     </row>
@@ -1482,8 +1459,7 @@
         <is>
           <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
 Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.
-Lei nº 14.133/2021, arts. 11, parágrafo único, e 18, caput: governança e planejamento da fase preparatória das contratações.</t>
+Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
         </is>
       </c>
       <c r="H14" s="1" t="inlineStr">
@@ -1512,7 +1488,7 @@
       <c r="O14" s="1" t="n"/>
       <c r="P14" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, com participação das áreas demandantes, critérios de priorização, etapas e responsabilidades definidos</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
@@ -1539,8 +1515,7 @@
         <is>
           <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
 Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.
-Lei nº 14.133/2021, arts. 11, parágrafo único, e 18, caput: governança e planejamento da fase preparatória das contratações.</t>
+Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
         </is>
       </c>
       <c r="H15" s="1" t="inlineStr">
@@ -1569,7 +1544,7 @@
       <c r="O15" s="1" t="n"/>
       <c r="P15" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, com participação das áreas demandantes, critérios de priorização, etapas e responsabilidades definidos</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
@@ -1596,8 +1571,7 @@
         <is>
           <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
 Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.
-Lei nº 14.133/2021, arts. 11, parágrafo único, e 18, caput: governança e planejamento da fase preparatória das contratações.</t>
+Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
         </is>
       </c>
       <c r="H16" s="1" t="inlineStr">
@@ -1626,7 +1600,7 @@
       <c r="O16" s="1" t="n"/>
       <c r="P16" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, com participação das áreas demandantes, critérios de priorização, etapas e responsabilidades definidos</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
@@ -1651,10 +1625,8 @@
       </c>
       <c r="G17" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.
-Lei nº 14.133/2021, arts. 11, parágrafo único, e 18, caput: governança e planejamento da fase preparatória das contratações.</t>
+          <t>Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
         </is>
       </c>
       <c r="H17" s="1" t="inlineStr">
@@ -1683,7 +1655,7 @@
       <c r="O17" s="1" t="n"/>
       <c r="P17" s="1" t="inlineStr">
         <is>
-          <t>submeta o plano de TIC à aprovação formal do dirigente máximo ou de instância competente da alta administração, mantendo registro do ato de aprovação</t>
+          <t>submeta o plano de TIC à aprovação formal do dirigente máximo ou de instância competente da alta administração, mantendo registro do respectivo ato de aprovação</t>
         </is>
       </c>
     </row>
@@ -1733,7 +1705,7 @@
       <c r="M18" s="1" t="n"/>
       <c r="N18" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O18" s="1" t="n"/>
@@ -1765,8 +1737,8 @@
       <c r="G19" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO06.03 - Criar e manter orçamentos: elaborar e manter orçamento de TIC alinhado ao portfólio, ao planejamento e às prioridades aprovadas.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
+Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.
+Lei nº 14.133/2021, art. 12, inciso VII e § 1º - Planejamento das contratações: o Plano de Contratações Anual, quando elaborado, deve alinhar-se ao planejamento estratégico, subsidiar a elaboração das leis orçamentárias e ser observado nas licitações e na execução contratual.</t>
         </is>
       </c>
       <c r="H19" s="1" t="inlineStr">
@@ -1789,7 +1761,7 @@
       <c r="M19" s="1" t="n"/>
       <c r="N19" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O19" s="1" t="n"/>
@@ -1820,11 +1792,7 @@
       </c>
       <c r="G20" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.
-Constituição Federal, art. 37, caput: princípio da eficiência.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, item II.3.5: precedente de determinação para divulgação e monitoramento do PDTI após aprovação.</t>
+          <t>Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
         </is>
       </c>
       <c r="H20" s="1" t="inlineStr">
@@ -1879,8 +1847,7 @@
       <c r="G21" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.
-COBIT 2019, APO07.05 - Planejar e monitorar o uso de recursos humanos de TI e de negócio: planejar, alocar e acompanhar capacidade de pessoal para iniciativas, operações e serviços de TIC.
-ABNT NBR ISO/IEC 27001:2022, cláusulas 5.3 e 7.2: definir responsabilidades e autoridades para segurança da informação e assegurar competências necessárias às funções atribuídas.</t>
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.7 - A organização deve adotar providências para dotar o setor de TI de quantitativo adequado às necessidades de trabalho em TI, consideradas as necessidades das demais áreas.</t>
         </is>
       </c>
       <c r="H21" s="1" t="inlineStr">
@@ -1909,7 +1876,7 @@
       <c r="O21" s="1" t="n"/>
       <c r="P21" s="1" t="inlineStr">
         <is>
-          <t>avalie a força de trabalho dedicada à TIC e adote medidas proporcionais para assegurar capacidade mínima de planejamento, gestão, contratação, fiscalização e sustentação dos serviços e ativos de TIC</t>
+          <t>avalie a força de trabalho dedicada à TIC e adote medidas proporcionais para assegurar capacidade mínima de planejamento, gestão, proteção, contratação, fiscalização e sustentação dos serviços e ativos de TIC</t>
         </is>
       </c>
     </row>
@@ -1935,8 +1902,7 @@
       <c r="G22" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.
-COBIT 2019, APO07.05 - Planejar e monitorar o uso de recursos humanos de TI e de negócio: planejar, alocar e acompanhar capacidade de pessoal para iniciativas, operações e serviços de TIC.
-ABNT NBR ISO/IEC 27001:2022, cláusulas 5.3 e 7.2: definir responsabilidades e autoridades para segurança da informação e assegurar competências necessárias às funções atribuídas.</t>
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.7 - A organização deve adotar providências para dotar o setor de TI de quantitativo adequado às necessidades de trabalho em TI, consideradas as necessidades das demais áreas.</t>
         </is>
       </c>
       <c r="H22" s="1" t="inlineStr">
@@ -1965,7 +1931,7 @@
       <c r="O22" s="1" t="n"/>
       <c r="P22" s="1" t="inlineStr">
         <is>
-          <t>avalie a força de trabalho dedicada à TIC e adote medidas proporcionais para assegurar capacidade mínima de planejamento, gestão, contratação, fiscalização e sustentação dos serviços e ativos de TIC</t>
+          <t>avalie a força de trabalho dedicada à TIC e adote medidas proporcionais para assegurar capacidade mínima de planejamento, gestão, proteção, contratação, fiscalização e sustentação dos serviços e ativos de TIC</t>
         </is>
       </c>
     </row>
@@ -1990,9 +1956,8 @@
       </c>
       <c r="G23" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.
-COBIT 2019, APO07.05 - Planejar e monitorar o uso de recursos humanos de TI e de negócio: planejar, alocar e acompanhar capacidade de pessoal para iniciativas, operações e serviços de TIC.
-ABNT NBR ISO/IEC 27001:2022, cláusulas 5.3 e 7.2: definir responsabilidades e autoridades para segurança da informação e assegurar competências necessárias às funções atribuídas.</t>
+          <t>COBIT 2019, APO07.05 - Planejar e monitorar o uso de recursos humanos de TI e de negócio: planejar, alocar e acompanhar capacidade de pessoal para iniciativas, operações e serviços de TIC.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6.5 - O PDTI deve contemplar o quantitativo necessário ou ideal para a força de trabalho em TI.</t>
         </is>
       </c>
       <c r="H23" s="1" t="inlineStr">
@@ -2047,8 +2012,7 @@
       <c r="G24" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
-COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.
-COBIT 2019, APO07.02 - Identificar pessoal-chave de TI: identificar funções e pessoas críticas para reduzir dependência individual, perda de conhecimento e descontinuidade.</t>
+COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
         </is>
       </c>
       <c r="H24" s="1" t="inlineStr">
@@ -2059,7 +2023,7 @@
       <c r="I24" s="1" t="n"/>
       <c r="J24" s="1" t="inlineStr">
         <is>
-          <t>Ausência de cargos, funções, perfis ou ocupações específicas de TIC e segurança da informação.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="K24" s="1" t="inlineStr">
@@ -2077,7 +2041,7 @@
       <c r="O24" s="1" t="n"/>
       <c r="P24" s="1" t="inlineStr">
         <is>
-          <t>avalie a necessidade de instituir cargos, funções, gratificações, perfis ou ocupações específicas de TIC e segurança da informação e adote a solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
+          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
         </is>
       </c>
     </row>
@@ -2103,8 +2067,7 @@
       <c r="G25" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
-COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.
-COBIT 2019, APO07.02 - Identificar pessoal-chave de TI: identificar funções e pessoas críticas para reduzir dependência individual, perda de conhecimento e descontinuidade.</t>
+COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
         </is>
       </c>
       <c r="H25" s="1" t="inlineStr">
@@ -2115,7 +2078,7 @@
       <c r="I25" s="1" t="n"/>
       <c r="J25" s="1" t="inlineStr">
         <is>
-          <t>Ausência de cargos, funções, perfis ou ocupações específicas de TIC e segurança da informação.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="K25" s="1" t="inlineStr">
@@ -2133,7 +2096,7 @@
       <c r="O25" s="1" t="n"/>
       <c r="P25" s="1" t="inlineStr">
         <is>
-          <t>avalie a necessidade de instituir cargos, funções, gratificações, perfis ou ocupações específicas de TIC e segurança da informação e adote a solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
+          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
         </is>
       </c>
     </row>
@@ -2159,8 +2122,6 @@
       <c r="G26" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO07.06 - Gerenciar pessoal contratado: controlar o uso de pessoal terceirizado ou externo, preservando responsabilização, supervisão e retenção de conhecimento.
-COBIT 2019, APO10.04 - Gerenciar risco de fornecedores: identificar e tratar riscos decorrentes de fornecedores, contratos e dependências externas relevantes para TIC.
-COBIT 2019, DSS01.02 - Gerenciar serviços de TI terceirizados: assegurar que serviços terceirizados sejam supervisionados, medidos e integrados aos controles da organização.
 Lei nº 14.133/2021, art. 117: dever de acompanhamento e fiscalização da execução contratual por representantes da Administração especialmente designados.</t>
         </is>
       </c>
@@ -2190,7 +2151,7 @@
       <c r="O26" s="1" t="n"/>
       <c r="P26" s="1" t="inlineStr">
         <is>
-          <t>assegure capacidade interna suficiente para coordenar, aprovar tecnicamente e fiscalizar as atividades e os contratos de TIC executados predominantemente por terceiros, preservando responsabilização e retenção de conhecimento</t>
+          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente para coordenar, aprovar tecnicamente e fiscalizar as atividades e os contratos de TIC executados predominantemente por terceiros, preservando responsabilização e retenção de conhecimento</t>
         </is>
       </c>
     </row>
@@ -2216,8 +2177,6 @@
       <c r="G27" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO07.06 - Gerenciar pessoal contratado: controlar o uso de pessoal terceirizado ou externo, preservando responsabilização, supervisão e retenção de conhecimento.
-COBIT 2019, APO10.04 - Gerenciar risco de fornecedores: identificar e tratar riscos decorrentes de fornecedores, contratos e dependências externas relevantes para TIC.
-COBIT 2019, DSS01.02 - Gerenciar serviços de TI terceirizados: assegurar que serviços terceirizados sejam supervisionados, medidos e integrados aos controles da organização.
 Lei nº 14.133/2021, art. 117: dever de acompanhamento e fiscalização da execução contratual por representantes da Administração especialmente designados.</t>
         </is>
       </c>
@@ -2247,7 +2206,7 @@
       <c r="O27" s="1" t="n"/>
       <c r="P27" s="1" t="inlineStr">
         <is>
-          <t>assegure capacidade interna suficiente para coordenar, aprovar tecnicamente e fiscalizar as atividades e os contratos de TIC executados predominantemente por terceiros, preservando responsabilização e retenção de conhecimento</t>
+          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente para coordenar, aprovar tecnicamente e fiscalizar as atividades e os contratos de TIC executados predominantemente por terceiros, preservando responsabilização e retenção de conhecimento</t>
         </is>
       </c>
     </row>
@@ -2302,7 +2261,7 @@
       <c r="O28" s="1" t="n"/>
       <c r="P28" s="1" t="inlineStr">
         <is>
-          <t>defina, pactue e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, incluindo metas no catálogo, indicadores, responsáveis e periodicidade de medição</t>
+          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2426,7 @@
       <c r="O31" s="1" t="n"/>
       <c r="P31" s="1" t="inlineStr">
         <is>
-          <t>defina, pactue e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, incluindo metas no catálogo, indicadores, responsáveis e periodicidade de medição</t>
+          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2481,7 @@
       <c r="O32" s="1" t="n"/>
       <c r="P32" s="1" t="inlineStr">
         <is>
-          <t>defina, pactue e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, incluindo metas no catálogo, indicadores, responsáveis e periodicidade de medição</t>
+          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
         </is>
       </c>
     </row>
@@ -2548,7 +2507,6 @@
       <c r="G33" s="1" t="inlineStr">
         <is>
           <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-ITIL 4, prática de gerenciamento de configuração de serviço: assegurar informações precisas e confiáveis sobre itens de configuração e seus relacionamentos com serviços, sistemas e infraestrutura.
 Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
         </is>
       </c>
@@ -2578,7 +2536,7 @@
       <c r="O33" s="1" t="n"/>
       <c r="P33" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, com informações suficientes sobre equipamentos, sistemas, softwares, licenças, serviços em nuvem, responsáveis e ciclo de vida</t>
+          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
         </is>
       </c>
     </row>
@@ -2604,7 +2562,6 @@
       <c r="G34" s="1" t="inlineStr">
         <is>
           <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-ITIL 4, prática de gerenciamento de configuração de serviço: assegurar informações precisas e confiáveis sobre itens de configuração e seus relacionamentos com serviços, sistemas e infraestrutura.
 Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
         </is>
       </c>
@@ -2634,7 +2591,7 @@
       <c r="O34" s="1" t="n"/>
       <c r="P34" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, com informações suficientes sobre equipamentos, sistemas, softwares, licenças, serviços em nuvem, responsáveis e ciclo de vida</t>
+          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2617,6 @@
       <c r="G35" s="1" t="inlineStr">
         <is>
           <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-ITIL 4, prática de gerenciamento de configuração de serviço: assegurar informações precisas e confiáveis sobre itens de configuração e seus relacionamentos com serviços, sistemas e infraestrutura.
 Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
         </is>
       </c>
@@ -2690,7 +2646,7 @@
       <c r="O35" s="1" t="n"/>
       <c r="P35" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, com informações suficientes sobre equipamentos, sistemas, softwares, licenças, serviços em nuvem, responsáveis e ciclo de vida</t>
+          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
         </is>
       </c>
     </row>
@@ -2745,7 +2701,7 @@
       <c r="O36" s="1" t="n"/>
       <c r="P36" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de configuração, mantendo base, ferramenta ou registro equivalente com os itens relevantes e seus relacionamentos, responsabilidades e rotina de atualização</t>
+          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
         </is>
       </c>
     </row>
@@ -2770,10 +2726,8 @@
       </c>
       <c r="G37" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de incidentes: minimizar o impacto negativo dos incidentes por meio da restauração tempestiva da operação normal dos serviços e do registro rastreável do tratamento realizado.
-COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.
-Acórdão TCE-RJ nº 44.490/2024-PLEN: precedente de controle sobre governança e gestão de TIC.</t>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
         </is>
       </c>
       <c r="H37" s="1" t="inlineStr">
@@ -2796,13 +2750,13 @@
       <c r="M37" s="1" t="n"/>
       <c r="N37" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O37" s="1" t="n"/>
       <c r="P37" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, com papéis, priorização, escalamento, tratamento, registro rastreável e comunicação dos incidentes de segurança sujeitos à LGPD</t>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
     </row>
@@ -2827,10 +2781,8 @@
       </c>
       <c r="G38" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de incidentes: minimizar o impacto negativo dos incidentes por meio da restauração tempestiva da operação normal dos serviços e do registro rastreável do tratamento realizado.
-COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.
-Acórdão TCE-RJ nº 44.490/2024-PLEN: precedente de controle sobre governança e gestão de TIC.</t>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
         </is>
       </c>
       <c r="H38" s="1" t="inlineStr">
@@ -2853,13 +2805,13 @@
       <c r="M38" s="1" t="n"/>
       <c r="N38" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O38" s="1" t="n"/>
       <c r="P38" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, com papéis, priorização, escalamento, tratamento, registro rastreável e comunicação dos incidentes de segurança sujeitos à LGPD</t>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
     </row>
@@ -2884,10 +2836,8 @@
       </c>
       <c r="G39" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de incidentes: minimizar o impacto negativo dos incidentes por meio da restauração tempestiva da operação normal dos serviços e do registro rastreável do tratamento realizado.
-COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.
-Acórdão TCE-RJ nº 44.490/2024-PLEN: precedente de controle sobre governança e gestão de TIC.</t>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
         </is>
       </c>
       <c r="H39" s="1" t="inlineStr">
@@ -2910,13 +2860,13 @@
       <c r="M39" s="1" t="n"/>
       <c r="N39" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O39" s="1" t="n"/>
       <c r="P39" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, com papéis, priorização, escalamento, tratamento, registro rastreável e comunicação dos incidentes de segurança sujeitos à LGPD</t>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
     </row>
@@ -2942,9 +2892,7 @@
       <c r="G40" s="1" t="inlineStr">
         <is>
           <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.
-COBIT 2019, APO01.09 - Definir e comunicar políticas e procedimentos: manter políticas, procedimentos e orientações para direcionar processos de gestão de TIC.
-Lei nº 14.133/2021, arts. 11, parágrafo único, e 19, IV: governança das contratações e instituição de modelos padronizados.</t>
+Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
         </is>
       </c>
       <c r="H40" s="1" t="inlineStr">
@@ -3000,7 +2948,6 @@
         <is>
           <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
 COBIT 2019, BAI02.04 - Obter aprovação dos requisitos da solução: obter aprovação formal dos requisitos funcionais, técnicos, de segurança e de conformidade antes de prosseguir com a solução.
-COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir e comunicar papéis e responsabilidades relacionados à informação e à tecnologia.
 Instrução Normativa SGD/ME nº 94, de 23 de dezembro de 2022, art. 1º, § 1º: como referência de boa prática, a aplicação de ritos formais de contratação de TIC pode ser facultada para contratações diretas por dispensa em razão do valor (inciso II do art. 75 da Lei nº 14.133/2021), indicando a possibilidade de fluxos simplificados para aquisições de baixa complexidade ou valor.</t>
         </is>
       </c>
@@ -3030,7 +2977,7 @@
       <c r="O41" s="1" t="n"/>
       <c r="P41" s="1" t="inlineStr">
         <is>
-          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, com avaliação técnica mínima compatível com a complexidade e o risco da solução</t>
+          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo fluxos simplificados para contratações de baixa complexidade ou baixo valor, desde que preservada análise técnica mínima compatível com o risco da contratação</t>
         </is>
       </c>
     </row>
@@ -3056,8 +3003,7 @@
       <c r="G42" s="1" t="inlineStr">
         <is>
           <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 18, caput e §1º, incisos I, IV, V, VIII, IX, X e XIII, da Lei 14.133/2021: fase preparatória caracterizada pelo planejamento, compatibilização com o plano de contratações anual e elementos mínimos do estudo técnico preliminar.
-Lei nº 14.133/2021, arts. 12, VII, e 18, caput: plano de contratações anual e compatibilização da fase preparatória com o PCA, sempre que elaborado, e com as leis orçamentárias.</t>
+Art. 18, caput e §1º, incisos I, IV, V, VIII, IX, X e XIII, da Lei 14.133/2021: fase preparatória caracterizada pelo planejamento, compatibilização com o plano de contratações anual e elementos mínimos do estudo técnico preliminar.</t>
         </is>
       </c>
       <c r="H42" s="1" t="inlineStr">
@@ -3086,7 +3032,7 @@
       <c r="O42" s="1" t="n"/>
       <c r="P42" s="1" t="inlineStr">
         <is>
-          <t>compatibilize as contratações de TIC com os instrumentos de planejamento da organização e com o Plano de Contratações Anual, quando elaborado, justificando as situações excepcionais</t>
+          <t>integre as contratações de TIC com os instrumentos de planejamento da organização e com o Plano de Contratações Anual, quando elaborado, justificando as situações excepcionais</t>
         </is>
       </c>
     </row>
@@ -3112,8 +3058,7 @@
       <c r="G43" s="1" t="inlineStr">
         <is>
           <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 18, caput e §1º, incisos I, IV, V, VIII, IX, X e XIII, da Lei 14.133/2021: fase preparatória caracterizada pelo planejamento, compatibilização com o plano de contratações anual e elementos mínimos do estudo técnico preliminar.
-Lei nº 14.133/2021, arts. 12, VII, e 18, caput: plano de contratações anual e compatibilização da fase preparatória com o PCA, sempre que elaborado, e com as leis orçamentárias.</t>
+Art. 18, caput e §1º, incisos I, IV, V, VIII, IX, X e XIII, da Lei 14.133/2021: fase preparatória caracterizada pelo planejamento, compatibilização com o plano de contratações anual e elementos mínimos do estudo técnico preliminar.</t>
         </is>
       </c>
       <c r="H43" s="1" t="inlineStr">
@@ -3142,7 +3087,7 @@
       <c r="O43" s="1" t="n"/>
       <c r="P43" s="1" t="inlineStr">
         <is>
-          <t>compatibilize as contratações de TIC com os instrumentos de planejamento da organização e com o Plano de Contratações Anual, quando elaborado, justificando as situações excepcionais</t>
+          <t>integre as contratações de TIC com os instrumentos de planejamento da organização e com o Plano de Contratações Anual, quando elaborado, justificando as situações excepcionais</t>
         </is>
       </c>
     </row>
@@ -3168,8 +3113,7 @@
       <c r="G44" s="1" t="inlineStr">
         <is>
           <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 7º, caput, incisos I a III e §1º, da Lei 14.133/2021: designação de agentes públicos para funções essenciais, observados atribuições, formação, segregação de funções e inexistência de vínculos que comprometam a atuação.
-COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir e comunicar papéis e responsabilidades relacionados à informação e à tecnologia.</t>
+Art. 7º, caput, incisos I a III e §1º, da Lei 14.133/2021: designação de agentes públicos para funções essenciais, observados atribuições, formação, segregação de funções e inexistência de vínculos que comprometam a atuação.</t>
         </is>
       </c>
       <c r="H44" s="1" t="inlineStr">
@@ -3180,7 +3124,7 @@
       <c r="I44" s="1" t="n"/>
       <c r="J44" s="1" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem designação de Equipe de Planejamento com integrante técnico da área de TIC.</t>
+          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
         </is>
       </c>
       <c r="K44" s="1" t="inlineStr">
@@ -3198,7 +3142,7 @@
       <c r="O44" s="1" t="n"/>
       <c r="P44" s="1" t="inlineStr">
         <is>
-          <t>designe formalmente Equipe de Planejamento para as contratações de TIC, assegurando integrante técnico da área de TIC e definição das responsabilidades dos participantes</t>
+          <t>designe formalmente equipe de planejamento para as contratações de TIC, atentando-se, minimamente, em assegurar a participação de integrante da área requisitante e da área técnica de TIC, com definição das responsabilidades de seus integrantes</t>
         </is>
       </c>
     </row>
@@ -3224,10 +3168,7 @@
       <c r="G45" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TI.
-COBIT 2019, APO01.09 - Definição e comunicação de políticas e procedimentos: estabelecer e comunicar políticas e procedimentos de gestão de TI que orientem papéis, responsabilidades e controles.
-ABNT NBR ISO/IEC 38500:2025, item 5.6.1 - Governança efetiva de TI: responsabilização clara, estrutura adequada de tomada de decisão e direção organizacional compatível com o uso atual e futuro da tecnologia.
-Constituição Federal, art. 37, caput: princípios da legalidade e da eficiência.
-Lei nº 14.133/2021, art. 11, parágrafo único: dever da alta administração de implementar processos e estruturas de governança das contratações.</t>
+Constituição Federal, art. 37, caput - Princípio da eficiência.</t>
         </is>
       </c>
       <c r="H45" s="1" t="inlineStr">
@@ -3238,7 +3179,7 @@
       <c r="I45" s="1" t="n"/>
       <c r="J45" s="1" t="inlineStr">
         <is>
-          <t>Área de TIC sem atribuições formalmente definidas ou sem atribuições formais de governança, planejamento ou gestão de TIC.</t>
+          <t>Área de TIC sem atribuições formalmente definidas ou sem atribuições formais de gestão de TIC.</t>
         </is>
       </c>
       <c r="K45" s="1" t="inlineStr">
@@ -3250,13 +3191,13 @@
       <c r="M45" s="1" t="n"/>
       <c r="N45" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O45" s="1" t="n"/>
       <c r="P45" s="1" t="inlineStr">
         <is>
-          <t>defina formalmente as atribuições da área de TIC, incluindo, no mínimo, responsabilidades de governança, planejamento e gestão de TIC, em instrumento compatível com a estrutura da organização</t>
+          <t>defina formalmente as atribuições da área de TIC, atentando-se, minimamente, em abranger as atividades de planejamento, coordenação, gestão e controle da TIC</t>
         </is>
       </c>
     </row>
@@ -3281,8 +3222,7 @@
       </c>
       <c r="G46" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, EDM01.02 - Dirigir o sistema de governança: orientar estruturas, princípios, processos e práticas de governança para assegurar que a TI apoie os objetivos organizacionais.
-COBIT 2019, MEA01.04 - Avaliar o desempenho: monitorar e avaliar periodicamente o desempenho e a conformidade da TI em relação a objetivos, indicadores, metas e expectativas das partes interessadas.
+          <t>COBIT 2019, MEA01.04 - Avaliar o desempenho: monitorar e avaliar periodicamente o desempenho e a conformidade da TI em relação a objetivos, indicadores, metas e expectativas das partes interessadas.
 Acórdão TCE-RJ 44.490/2024-PLEN, item II.1: necessidade de estrutura de governança de TI, especialmente Comitê de Tecnologia da Informação ou instância equivalente, com participação de áreas relevantes, responsabilidade de alinhar as ações de TI aos objetivos institucionais, priorizar investimentos e monitorar o desempenho da TI com base em indicadores e metas.</t>
         </is>
       </c>
@@ -3306,13 +3246,13 @@
       <c r="M46" s="1" t="n"/>
       <c r="N46" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O46" s="1" t="n"/>
       <c r="P46" s="1" t="inlineStr">
         <is>
-          <t>estabeleça objetivos, indicadores e metas para a gestão de TIC, aprovados ou formalmente definidos pela alta administração, e mantenha-os vinculados aos resultados institucionais pretendidos</t>
+          <t>estabeleça modelo básico de governança e gestão de TIC definindo objetivos, indicadores, metas e forma de acompanhamento periódico do desempenho da TIC pela alta administração</t>
         </is>
       </c>
     </row>
@@ -3337,9 +3277,7 @@
       </c>
       <c r="G47" s="1" t="inlineStr">
         <is>
-          <t>Decreto nº 12.198/2024, art. 5º - Instituição do CGD, colegiado responsável por definir diretrizes e estratégias sobre uso de recursos digitais nos órgãos e entidades da administração pública federal direta, autárquica e fundacional.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.1: necessidade de estrutura de governança de TI, especialmente Comitê de Tecnologia da Informação ou instância equivalente, com participação de áreas relevantes, responsabilidade de alinhar as ações de TI aos objetivos institucionais, priorizar investimentos e monitorar o desempenho da TI com base em indicadores e metas.
-COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TI.
+          <t>Acórdão TCE-RJ 44.490/2024-PLEN, item II.1: necessidade de estrutura de governança de TI, especialmente Comitê de Tecnologia da Informação ou instância equivalente, com participação de áreas relevantes, responsabilidade de alinhar as ações de TI aos objetivos institucionais, priorizar investimentos e monitorar o desempenho da TI com base em indicadores e metas.
 Lei nº 14.133/2021, art. 11, parágrafo único: dever da alta administração de implementar estruturas de governança das contratações.
 Acórdão TCU nº 1.411/2014-Plenário, item 9.1.2: precedente sobre funcionamento permanente e composição relevante do Comitê de TIC.</t>
         </is>
@@ -3370,7 +3308,7 @@
       <c r="O47" s="1" t="n"/>
       <c r="P47" s="1" t="inlineStr">
         <is>
-          <t>institua formalmente Comitê de TIC ou instância colegiada equivalente, compatível com o porte e a estrutura decisória da organização, com composição, competências, periodicidade e forma de registro definidas</t>
+          <t>institua formalmente Comitê de TIC ou instância colegiada equivalente, compatível com o porte e a estrutura decisória da organização, atentando-se, minimamente, em definir sua composição, competências, periodicidade de reuniões, forma de registro das deliberações e acompanhamento dos encaminhamentos</t>
         </is>
       </c>
     </row>
@@ -3396,10 +3334,7 @@
       <c r="G48" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, MEA01.04 - Avaliar o desempenho: monitorar e avaliar periodicamente o desempenho e a conformidade da TI em relação a objetivos, indicadores, metas e expectativas das partes interessadas.
-Decreto nº 12.198/2024, art. 5º - Instituição do CGD, colegiado responsável por definir diretrizes e estratégias sobre uso de recursos digitais nos órgãos e entidades da administração pública federal direta, autárquica e fundacional.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.1: necessidade de estrutura de governança de TI, especialmente Comitê de Tecnologia da Informação ou instância equivalente, com participação de áreas relevantes, responsabilidade de alinhar as ações de TI aos objetivos institucionais, priorizar investimentos e monitorar o desempenho da TI com base em indicadores e metas.
-Constituição Federal, art. 37, caput: princípio da eficiência.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, item II.1: precedente de determinação para Comitê de TIC com responsabilidades de alinhamento, priorização e monitoramento.</t>
+Acórdão TCE-RJ 44.490/2024-PLEN, item II.1: necessidade de estrutura de governança de TI, especialmente Comitê de Tecnologia da Informação ou instância equivalente, com participação de áreas relevantes, responsabilidade de alinhar as ações de TI aos objetivos institucionais, priorizar investimentos e monitorar o desempenho da TI com base em indicadores e metas.</t>
         </is>
       </c>
       <c r="H48" s="1" t="inlineStr">
@@ -3428,7 +3363,7 @@
       <c r="O48" s="1" t="n"/>
       <c r="P48" s="1" t="inlineStr">
         <is>
-          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância equivalente, realizando reuniões, registrando deliberações e acompanhando os encaminhamentos relevantes</t>
+          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância colegiada equivalente, compatível com o porte e a estrutura decisória da organização, atentando-se, minimamente, em realizar reuniões periódicas, registrar deliberações e acompanhar decisões sobre prioridades, projetos, riscos, serviços, orçamento e contratações de TIC</t>
         </is>
       </c>
     </row>
@@ -3455,8 +3390,7 @@
         <is>
           <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
 Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.
-Lei nº 14.133/2021, arts. 11, parágrafo único, e 18, caput: governança e planejamento da fase preparatória das contratações.</t>
+Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
         </is>
       </c>
       <c r="H49" s="1" t="inlineStr">
@@ -3485,7 +3419,7 @@
       <c r="O49" s="1" t="n"/>
       <c r="P49" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, com participação das áreas demandantes, critérios de priorização, etapas e responsabilidades definidos</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
@@ -3512,8 +3446,7 @@
         <is>
           <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
 Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.
-Lei nº 14.133/2021, arts. 11, parágrafo único, e 18, caput: governança e planejamento da fase preparatória das contratações.</t>
+Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
         </is>
       </c>
       <c r="H50" s="1" t="inlineStr">
@@ -3542,7 +3475,7 @@
       <c r="O50" s="1" t="n"/>
       <c r="P50" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, com participação das áreas demandantes, critérios de priorização, etapas e responsabilidades definidos</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
@@ -3569,8 +3502,7 @@
         <is>
           <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
 Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.
-Lei nº 14.133/2021, arts. 11, parágrafo único, e 18, caput: governança e planejamento da fase preparatória das contratações.</t>
+Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
         </is>
       </c>
       <c r="H51" s="1" t="inlineStr">
@@ -3599,7 +3531,7 @@
       <c r="O51" s="1" t="n"/>
       <c r="P51" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, com participação das áreas demandantes, critérios de priorização, etapas e responsabilidades definidos</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
@@ -3624,10 +3556,8 @@
       </c>
       <c r="G52" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.
-Lei nº 14.133/2021, arts. 11, parágrafo único, e 18, caput: governança e planejamento da fase preparatória das contratações.</t>
+          <t>Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
         </is>
       </c>
       <c r="H52" s="1" t="inlineStr">
@@ -3656,7 +3586,7 @@
       <c r="O52" s="1" t="n"/>
       <c r="P52" s="1" t="inlineStr">
         <is>
-          <t>submeta o plano de TIC à aprovação formal do dirigente máximo ou de instância competente da alta administração, mantendo registro do ato de aprovação</t>
+          <t>submeta o plano de TIC à aprovação formal do dirigente máximo ou de instância competente da alta administração, mantendo registro do respectivo ato de aprovação</t>
         </is>
       </c>
     </row>
@@ -3706,7 +3636,7 @@
       <c r="M53" s="1" t="n"/>
       <c r="N53" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O53" s="1" t="n"/>
@@ -3738,8 +3668,8 @@
       <c r="G54" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO06.03 - Criar e manter orçamentos: elaborar e manter orçamento de TIC alinhado ao portfólio, ao planejamento e às prioridades aprovadas.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
+Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.
+Lei nº 14.133/2021, art. 12, inciso VII e § 1º - Planejamento das contratações: o Plano de Contratações Anual, quando elaborado, deve alinhar-se ao planejamento estratégico, subsidiar a elaboração das leis orçamentárias e ser observado nas licitações e na execução contratual.</t>
         </is>
       </c>
       <c r="H54" s="1" t="inlineStr">
@@ -3762,7 +3692,7 @@
       <c r="M54" s="1" t="n"/>
       <c r="N54" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O54" s="1" t="n"/>
@@ -3793,11 +3723,7 @@
       </c>
       <c r="G55" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.
-Constituição Federal, art. 37, caput: princípio da eficiência.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, item II.3.5: precedente de determinação para divulgação e monitoramento do PDTI após aprovação.</t>
+          <t>Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
         </is>
       </c>
       <c r="H55" s="1" t="inlineStr">
@@ -3851,9 +3777,8 @@
       </c>
       <c r="G56" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.
-COBIT 2019, APO07.05 - Planejar e monitorar o uso de recursos humanos de TI e de negócio: planejar, alocar e acompanhar capacidade de pessoal para iniciativas, operações e serviços de TIC.
-ABNT NBR ISO/IEC 27001:2022, cláusulas 5.3 e 7.2: definir responsabilidades e autoridades para segurança da informação e assegurar competências necessárias às funções atribuídas.</t>
+          <t>COBIT 2019, APO07.05 - Planejar e monitorar o uso de recursos humanos de TI e de negócio: planejar, alocar e acompanhar capacidade de pessoal para iniciativas, operações e serviços de TIC.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6.5 - O PDTI deve contemplar o quantitativo necessário ou ideal para a força de trabalho em TI.</t>
         </is>
       </c>
       <c r="H56" s="1" t="inlineStr">
@@ -3908,8 +3833,7 @@
       <c r="G57" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
-COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.
-COBIT 2019, APO07.02 - Identificar pessoal-chave de TI: identificar funções e pessoas críticas para reduzir dependência individual, perda de conhecimento e descontinuidade.</t>
+COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
         </is>
       </c>
       <c r="H57" s="1" t="inlineStr">
@@ -3920,7 +3844,7 @@
       <c r="I57" s="1" t="n"/>
       <c r="J57" s="1" t="inlineStr">
         <is>
-          <t>Ausência de cargos, funções, perfis ou ocupações específicas de TIC e segurança da informação.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="K57" s="1" t="inlineStr">
@@ -3938,7 +3862,7 @@
       <c r="O57" s="1" t="n"/>
       <c r="P57" s="1" t="inlineStr">
         <is>
-          <t>avalie a necessidade de instituir cargos, funções, gratificações, perfis ou ocupações específicas de TIC e segurança da informação e adote a solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
+          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
         </is>
       </c>
     </row>
@@ -3964,8 +3888,7 @@
       <c r="G58" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
-COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.
-COBIT 2019, APO07.02 - Identificar pessoal-chave de TI: identificar funções e pessoas críticas para reduzir dependência individual, perda de conhecimento e descontinuidade.</t>
+COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
         </is>
       </c>
       <c r="H58" s="1" t="inlineStr">
@@ -3976,7 +3899,7 @@
       <c r="I58" s="1" t="n"/>
       <c r="J58" s="1" t="inlineStr">
         <is>
-          <t>Ausência de cargos, funções, perfis ou ocupações específicas de TIC e segurança da informação.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="K58" s="1" t="inlineStr">
@@ -3994,7 +3917,7 @@
       <c r="O58" s="1" t="n"/>
       <c r="P58" s="1" t="inlineStr">
         <is>
-          <t>avalie a necessidade de instituir cargos, funções, gratificações, perfis ou ocupações específicas de TIC e segurança da informação e adote a solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
+          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
         </is>
       </c>
     </row>
@@ -4049,7 +3972,7 @@
       <c r="O59" s="1" t="n"/>
       <c r="P59" s="1" t="inlineStr">
         <is>
-          <t>defina, pactue e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, incluindo metas no catálogo, indicadores, responsáveis e periodicidade de medição</t>
+          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
         </is>
       </c>
     </row>
@@ -4214,7 +4137,7 @@
       <c r="O62" s="1" t="n"/>
       <c r="P62" s="1" t="inlineStr">
         <is>
-          <t>defina, pactue e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, incluindo metas no catálogo, indicadores, responsáveis e periodicidade de medição</t>
+          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
         </is>
       </c>
     </row>
@@ -4269,7 +4192,7 @@
       <c r="O63" s="1" t="n"/>
       <c r="P63" s="1" t="inlineStr">
         <is>
-          <t>defina, pactue e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, incluindo metas no catálogo, indicadores, responsáveis e periodicidade de medição</t>
+          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
         </is>
       </c>
     </row>
@@ -4295,7 +4218,6 @@
       <c r="G64" s="1" t="inlineStr">
         <is>
           <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-ITIL 4, prática de gerenciamento de configuração de serviço: assegurar informações precisas e confiáveis sobre itens de configuração e seus relacionamentos com serviços, sistemas e infraestrutura.
 Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
         </is>
       </c>
@@ -4325,7 +4247,7 @@
       <c r="O64" s="1" t="n"/>
       <c r="P64" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, com informações suficientes sobre equipamentos, sistemas, softwares, licenças, serviços em nuvem, responsáveis e ciclo de vida</t>
+          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
         </is>
       </c>
     </row>
@@ -4351,7 +4273,6 @@
       <c r="G65" s="1" t="inlineStr">
         <is>
           <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-ITIL 4, prática de gerenciamento de configuração de serviço: assegurar informações precisas e confiáveis sobre itens de configuração e seus relacionamentos com serviços, sistemas e infraestrutura.
 Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
         </is>
       </c>
@@ -4381,7 +4302,7 @@
       <c r="O65" s="1" t="n"/>
       <c r="P65" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, com informações suficientes sobre equipamentos, sistemas, softwares, licenças, serviços em nuvem, responsáveis e ciclo de vida</t>
+          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4328,6 @@
       <c r="G66" s="1" t="inlineStr">
         <is>
           <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-ITIL 4, prática de gerenciamento de configuração de serviço: assegurar informações precisas e confiáveis sobre itens de configuração e seus relacionamentos com serviços, sistemas e infraestrutura.
 Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
         </is>
       </c>
@@ -4437,7 +4357,7 @@
       <c r="O66" s="1" t="n"/>
       <c r="P66" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, com informações suficientes sobre equipamentos, sistemas, softwares, licenças, serviços em nuvem, responsáveis e ciclo de vida</t>
+          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
         </is>
       </c>
     </row>
@@ -4492,7 +4412,7 @@
       <c r="O67" s="1" t="n"/>
       <c r="P67" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de configuração, mantendo base, ferramenta ou registro equivalente com os itens relevantes e seus relacionamentos, responsabilidades e rotina de atualização</t>
+          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
         </is>
       </c>
     </row>
@@ -4517,10 +4437,8 @@
       </c>
       <c r="G68" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de incidentes: minimizar o impacto negativo dos incidentes por meio da restauração tempestiva da operação normal dos serviços e do registro rastreável do tratamento realizado.
-COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.
-Acórdão TCE-RJ nº 44.490/2024-PLEN: precedente de controle sobre governança e gestão de TIC.</t>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
         </is>
       </c>
       <c r="H68" s="1" t="inlineStr">
@@ -4543,13 +4461,13 @@
       <c r="M68" s="1" t="n"/>
       <c r="N68" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O68" s="1" t="n"/>
       <c r="P68" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, com papéis, priorização, escalamento, tratamento, registro rastreável e comunicação dos incidentes de segurança sujeitos à LGPD</t>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
     </row>
@@ -4574,10 +4492,8 @@
       </c>
       <c r="G69" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de incidentes: minimizar o impacto negativo dos incidentes por meio da restauração tempestiva da operação normal dos serviços e do registro rastreável do tratamento realizado.
-COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.
-Acórdão TCE-RJ nº 44.490/2024-PLEN: precedente de controle sobre governança e gestão de TIC.</t>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
         </is>
       </c>
       <c r="H69" s="1" t="inlineStr">
@@ -4600,13 +4516,13 @@
       <c r="M69" s="1" t="n"/>
       <c r="N69" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O69" s="1" t="n"/>
       <c r="P69" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, com papéis, priorização, escalamento, tratamento, registro rastreável e comunicação dos incidentes de segurança sujeitos à LGPD</t>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
     </row>
@@ -4631,10 +4547,8 @@
       </c>
       <c r="G70" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de incidentes: minimizar o impacto negativo dos incidentes por meio da restauração tempestiva da operação normal dos serviços e do registro rastreável do tratamento realizado.
-COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.
-Acórdão TCE-RJ nº 44.490/2024-PLEN: precedente de controle sobre governança e gestão de TIC.</t>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
         </is>
       </c>
       <c r="H70" s="1" t="inlineStr">
@@ -4657,13 +4571,13 @@
       <c r="M70" s="1" t="n"/>
       <c r="N70" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O70" s="1" t="n"/>
       <c r="P70" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, com papéis, priorização, escalamento, tratamento, registro rastreável e comunicação dos incidentes de segurança sujeitos à LGPD</t>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
     </row>
@@ -4689,9 +4603,7 @@
       <c r="G71" s="1" t="inlineStr">
         <is>
           <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.
-COBIT 2019, APO01.09 - Definir e comunicar políticas e procedimentos: manter políticas, procedimentos e orientações para direcionar processos de gestão de TIC.
-Lei nº 14.133/2021, arts. 11, parágrafo único, e 19, IV: governança das contratações e instituição de modelos padronizados.</t>
+Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
         </is>
       </c>
       <c r="H71" s="1" t="inlineStr">
@@ -4747,7 +4659,6 @@
         <is>
           <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
 COBIT 2019, BAI02.04 - Obter aprovação dos requisitos da solução: obter aprovação formal dos requisitos funcionais, técnicos, de segurança e de conformidade antes de prosseguir com a solução.
-COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir e comunicar papéis e responsabilidades relacionados à informação e à tecnologia.
 Instrução Normativa SGD/ME nº 94, de 23 de dezembro de 2022, art. 1º, § 1º: como referência de boa prática, a aplicação de ritos formais de contratação de TIC pode ser facultada para contratações diretas por dispensa em razão do valor (inciso II do art. 75 da Lei nº 14.133/2021), indicando a possibilidade de fluxos simplificados para aquisições de baixa complexidade ou valor.</t>
         </is>
       </c>
@@ -4777,7 +4688,7 @@
       <c r="O72" s="1" t="n"/>
       <c r="P72" s="1" t="inlineStr">
         <is>
-          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, com avaliação técnica mínima compatível com a complexidade e o risco da solução</t>
+          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo fluxos simplificados para contratações de baixa complexidade ou baixo valor, desde que preservada análise técnica mínima compatível com o risco da contratação</t>
         </is>
       </c>
     </row>
@@ -4803,8 +4714,7 @@
       <c r="G73" s="1" t="inlineStr">
         <is>
           <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 18, caput e §1º, incisos I, IV, V, VIII, IX, X e XIII, da Lei 14.133/2021: fase preparatória caracterizada pelo planejamento, compatibilização com o plano de contratações anual e elementos mínimos do estudo técnico preliminar.
-Lei nº 14.133/2021, arts. 12, VII, e 18, caput: plano de contratações anual e compatibilização da fase preparatória com o PCA, sempre que elaborado, e com as leis orçamentárias.</t>
+Art. 18, caput e §1º, incisos I, IV, V, VIII, IX, X e XIII, da Lei 14.133/2021: fase preparatória caracterizada pelo planejamento, compatibilização com o plano de contratações anual e elementos mínimos do estudo técnico preliminar.</t>
         </is>
       </c>
       <c r="H73" s="1" t="inlineStr">
@@ -4833,7 +4743,7 @@
       <c r="O73" s="1" t="n"/>
       <c r="P73" s="1" t="inlineStr">
         <is>
-          <t>compatibilize as contratações de TIC com os instrumentos de planejamento da organização e com o Plano de Contratações Anual, quando elaborado, justificando as situações excepcionais</t>
+          <t>integre as contratações de TIC com os instrumentos de planejamento da organização e com o Plano de Contratações Anual, quando elaborado, justificando as situações excepcionais</t>
         </is>
       </c>
     </row>
@@ -4859,9 +4769,7 @@
       <c r="G74" s="1" t="inlineStr">
         <is>
           <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.
-COBIT 2019, APO01.09 - Definir e comunicar políticas e procedimentos: manter políticas, procedimentos e orientações para direcionar processos de gestão de TIC.
-Lei nº 14.133/2021, arts. 11, parágrafo único, e 19, IV: governança das contratações e instituição de modelos padronizados.</t>
+Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
         </is>
       </c>
       <c r="H74" s="1" t="inlineStr">
@@ -4916,9 +4824,7 @@
       <c r="G75" s="1" t="inlineStr">
         <is>
           <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.
-COBIT 2019, APO01.09 - Definir e comunicar políticas e procedimentos: manter políticas, procedimentos e orientações para direcionar processos de gestão de TIC.
-Lei nº 14.133/2021, arts. 11, parágrafo único, e 19, IV: governança das contratações e instituição de modelos padronizados.</t>
+Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
         </is>
       </c>
       <c r="H75" s="1" t="inlineStr">
@@ -5191,7 +5097,7 @@
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Área de TIC sem atribuições formalmente definidas ou sem atribuições formais de governança, planejamento ou gestão de TIC.</t>
+          <t>Área de TIC sem atribuições formalmente definidas ou sem atribuições formais de gestão de TIC.</t>
         </is>
       </c>
       <c r="D5" s="9" t="n">
@@ -5229,7 +5135,7 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Área de TIC sem atribuições formalmente definidas ou sem atribuições formais de governança, planejamento ou gestão de TIC.</t>
+          <t>Área de TIC sem atribuições formalmente definidas ou sem atribuições formais de gestão de TIC.</t>
         </is>
       </c>
       <c r="D6" s="9" t="n">
@@ -5267,7 +5173,7 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>Área de TIC sem atribuições formalmente definidas ou sem atribuições formais de governança, planejamento ou gestão de TIC.</t>
+          <t>Área de TIC sem atribuições formalmente definidas ou sem atribuições formais de gestão de TIC.</t>
         </is>
       </c>
       <c r="D7" s="9" t="n">
@@ -5305,7 +5211,7 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Área de TIC sem atribuições formalmente definidas ou sem atribuições formais de governança, planejamento ou gestão de TIC.</t>
+          <t>Área de TIC sem atribuições formalmente definidas ou sem atribuições formais de gestão de TIC.</t>
         </is>
       </c>
       <c r="D8" s="9" t="n">
@@ -6331,7 +6237,7 @@
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>Ausência de cargos, funções, perfis ou ocupações específicas de TIC e segurança da informação.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="D35" s="9" t="n">
@@ -6369,7 +6275,7 @@
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>Ausência de cargos, funções, perfis ou ocupações específicas de TIC e segurança da informação.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="D36" s="9" t="n">
@@ -6407,7 +6313,7 @@
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>Ausência de cargos, funções, perfis ou ocupações específicas de TIC e segurança da informação.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="D37" s="9" t="n">
@@ -6445,7 +6351,7 @@
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>Ausência de cargos, funções, perfis ou ocupações específicas de TIC e segurança da informação.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="D38" s="9" t="n">
@@ -6501,7 +6407,7 @@
       </c>
       <c r="G39" s="9" t="inlineStr">
         <is>
-          <t>A organização informou modelo de operação de TIC com execução predominantemente terceirizada ou prestada por estrutura central externa, o que levou à análise de sua capacidade interna de coordenação e fiscalização</t>
+          <t>A organização informou modelo de operação de TIC com execução predominantemente terceirizada, o que levou à análise de sua capacidade interna de coordenação e fiscalização</t>
         </is>
       </c>
       <c r="H39" s="9" t="b">
@@ -6539,7 +6445,7 @@
       </c>
       <c r="G40" s="9" t="inlineStr">
         <is>
-          <t>Não foi identificado quantitativo de profissionais internos de TIC suficiente para coordenar e fiscalizar a execução das atividades de tecnologia da informação</t>
+          <t>Não foram identificados profissionais internos de TIC para coordenar e fiscalizar a execução das atividades de tecnologia da informação</t>
         </is>
       </c>
       <c r="H40" s="9" t="b">
@@ -7737,7 +7643,7 @@
       </c>
       <c r="C72" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem designação de Equipe de Planejamento com integrante técnico da área de TIC.</t>
+          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
         </is>
       </c>
       <c r="D72" s="9" t="n">
@@ -7793,7 +7699,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>Item 2801b: a organização informou que não disponibiliza artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+          <t>No subitem b) do item 2801, não houve declaração afirmativa quanto à prática avaliada: são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
         </is>
       </c>
       <c r="H73" s="9" t="b">
@@ -7831,7 +7737,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>Item 2801b: a organização declarou disponibilizar artefatos padronizados para o planejamento das contratações de TIC, mas a evidência foi insuficiente para comprovar a prática</t>
+          <t>No subitem b) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
         </is>
       </c>
       <c r="H74" s="9" t="b">

</xml_diff>

<commit_message>
Revisa a Questão 2 da matriz e do mapa
</commit_message>
<xml_diff>
--- a/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
+++ b/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
@@ -15,8 +15,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Fontes de Informação'!$A$3:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Procedimentos de Auditoria'!$A$3:$E$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ações de Verificação'!$A$3:$P$75</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Motivos do Relatório'!$A$3:$H$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ações de Verificação'!$A$3:$P$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Motivos do Relatório'!$A$3:$H$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Variáveis Temporárias'!$A$3:$E$5</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -569,12 +569,12 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>Procedimento para verificar a questão Q2: A organização possui mecanismos básicos de governança de TIC estabelecidos pela alta administração, incluindo modelo de governança e gestão, objetivos, indicadores, metas e Comitê de TIC ou instância equivalente formalmente instituída e atuante?</t>
+          <t>Procedimento para verificar a questão Q2: A organização possui mecanismos básicos de governança de TIC, incluindo objetivos, indicadores e metas, bem como Comitê de TIC ou instância equivalente formalmente instituída e atuante?</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>((AV08 | AV86) | (AV11 | AV89) | (AV12 &amp; (AV13 | AV91)))</t>
+          <t>(AV08 | AV11 | (AV12 &amp; AV13))</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
@@ -699,7 +699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P75"/>
+  <dimension ref="A1:P72"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1236,8 +1236,7 @@
       </c>
       <c r="G10" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, MEA01.04 - Avaliar o desempenho: monitorar e avaliar periodicamente o desempenho e a conformidade da TI em relação a objetivos, indicadores, metas e expectativas das partes interessadas.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.1: necessidade de estrutura de governança de TI, especialmente Comitê de Tecnologia da Informação ou instância equivalente, com participação de áreas relevantes, responsabilidade de alinhar as ações de TI aos objetivos institucionais, priorizar investimentos e monitorar o desempenho da TI com base em indicadores e metas.</t>
+          <t>COBIT 2019, MEA01.04 - Avaliar o desempenho: monitorar e avaliar periodicamente o desempenho e a conformidade da TI em relação a objetivos, indicadores, metas e expectativas das partes interessadas.</t>
         </is>
       </c>
       <c r="H10" s="1" t="inlineStr">
@@ -1260,13 +1259,13 @@
       <c r="M10" s="1" t="n"/>
       <c r="N10" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O10" s="1" t="n"/>
       <c r="P10" s="1" t="inlineStr">
         <is>
-          <t>estabeleça modelo básico de governança e gestão de TIC definindo objetivos, indicadores, metas e forma de acompanhamento periódico do desempenho da TIC pela alta administração</t>
+          <t>estabeleça objetivos, indicadores e metas para a gestão de TIC, de modo a possibilitar o acompanhamento periódico do desempenho da TIC pela alta administração</t>
         </is>
       </c>
     </row>
@@ -1291,9 +1290,9 @@
       </c>
       <c r="G11" s="1" t="inlineStr">
         <is>
-          <t>Acórdão TCE-RJ 44.490/2024-PLEN, item II.1: necessidade de estrutura de governança de TI, especialmente Comitê de Tecnologia da Informação ou instância equivalente, com participação de áreas relevantes, responsabilidade de alinhar as ações de TI aos objetivos institucionais, priorizar investimentos e monitorar o desempenho da TI com base em indicadores e metas.
-Lei nº 14.133/2021, art. 11, parágrafo único: dever da alta administração de implementar estruturas de governança das contratações.
-Acórdão TCU nº 1.411/2014-Plenário, item 9.1.2: precedente sobre funcionamento permanente e composição relevante do Comitê de TIC.</t>
+          <t>COBIT 2019, EDM01.02 - Dirigir o sistema de governança: orientar estruturas, princípios, processos e práticas de governança para assegurar que a TI apoie os objetivos organizacionais.
+Decreto nº 12.198/2024, arts. 5º e 6º, § 2º – Referência de governança digital: instituição, no âmbito da Administração Pública federal direta, autárquica e fundacional, de Comitê de Governança Digital ou colegiado equivalente com função deliberativa sobre ações de governo digital e uso de recursos de TIC, incluindo a aprovação dos instrumentos de planejamento previstos no Decreto.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.1, III.1 e V.1 – Precedente pela instituição e atuação efetiva de instância colegiada de governança de TIC, com responsabilidade pelo alinhamento das ações de TIC aos objetivos institucionais, priorização dos investimentos e monitoramento do desempenho da TIC.</t>
         </is>
       </c>
       <c r="H11" s="1" t="inlineStr">
@@ -1304,7 +1303,7 @@
       <c r="I11" s="1" t="n"/>
       <c r="J11" s="1" t="inlineStr">
         <is>
-          <t>Comitê de TIC ou instância equivalente não instituído formalmente.</t>
+          <t>Comitê de TIC ou instância equivalente não instituído formalmente ou sem representação de áreas relevantes da organização.</t>
         </is>
       </c>
       <c r="K11" s="1" t="inlineStr">
@@ -1322,7 +1321,7 @@
       <c r="O11" s="1" t="n"/>
       <c r="P11" s="1" t="inlineStr">
         <is>
-          <t>institua formalmente Comitê de TIC ou instância colegiada equivalente, compatível com o porte e a estrutura decisória da organização, atentando-se, minimamente, em definir sua composição, competências, periodicidade de reuniões, forma de registro das deliberações e acompanhamento dos encaminhamentos</t>
+          <t>institua formalmente Comitê de TIC ou instância colegiada equivalente, compatível com o porte e a estrutura decisória da organização, definindo em seu ato constitutivo, minimamente, a participação de representantes de áreas relevantes da organização, suas competências, a periodicidade de reuniões, a forma de registro das deliberações e os mecanismos de acompanhamento dos encaminhamentos</t>
         </is>
       </c>
     </row>
@@ -1347,8 +1346,9 @@
       </c>
       <c r="G12" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, MEA01.04 - Avaliar o desempenho: monitorar e avaliar periodicamente o desempenho e a conformidade da TI em relação a objetivos, indicadores, metas e expectativas das partes interessadas.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.1: necessidade de estrutura de governança de TI, especialmente Comitê de Tecnologia da Informação ou instância equivalente, com participação de áreas relevantes, responsabilidade de alinhar as ações de TI aos objetivos institucionais, priorizar investimentos e monitorar o desempenho da TI com base em indicadores e metas.</t>
+          <t>COBIT 2019, EDM01.02 - Dirigir o sistema de governança: orientar estruturas, princípios, processos e práticas de governança para assegurar que a TI apoie os objetivos organizacionais.
+Decreto nº 12.198/2024, arts. 5º e 6º, § 2º – Referência de governança digital: instituição, no âmbito da Administração Pública federal direta, autárquica e fundacional, de Comitê de Governança Digital ou colegiado equivalente com função deliberativa sobre ações de governo digital e uso de recursos de TIC, incluindo a aprovação dos instrumentos de planejamento previstos no Decreto.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.1, III.1 e V.1 – Precedente pela instituição e atuação efetiva de instância colegiada de governança de TIC, com responsabilidade pelo alinhamento das ações de TIC aos objetivos institucionais, priorização dos investimentos e monitoramento do desempenho da TIC.</t>
         </is>
       </c>
       <c r="H12" s="1" t="inlineStr">
@@ -1377,7 +1377,7 @@
       <c r="O12" s="1" t="n"/>
       <c r="P12" s="1" t="inlineStr">
         <is>
-          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância colegiada equivalente, compatível com o porte e a estrutura decisória da organização, atentando-se, minimamente, em realizar reuniões periódicas, registrar deliberações e acompanhar decisões sobre prioridades, projetos, riscos, serviços, orçamento e contratações de TIC</t>
+          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância colegiada equivalente, mediante o exercício das competências previstas em seu ato constitutivo, com registro das deliberações e acompanhamento dos respectivos encaminhamentos</t>
         </is>
       </c>
     </row>
@@ -1402,8 +1402,9 @@
       </c>
       <c r="G13" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, MEA01.04 - Avaliar o desempenho: monitorar e avaliar periodicamente o desempenho e a conformidade da TI em relação a objetivos, indicadores, metas e expectativas das partes interessadas.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.1: necessidade de estrutura de governança de TI, especialmente Comitê de Tecnologia da Informação ou instância equivalente, com participação de áreas relevantes, responsabilidade de alinhar as ações de TI aos objetivos institucionais, priorizar investimentos e monitorar o desempenho da TI com base em indicadores e metas.</t>
+          <t>COBIT 2019, EDM01.02 - Dirigir o sistema de governança: orientar estruturas, princípios, processos e práticas de governança para assegurar que a TI apoie os objetivos organizacionais.
+Decreto nº 12.198/2024, arts. 5º e 6º, § 2º – Referência de governança digital: instituição, no âmbito da Administração Pública federal direta, autárquica e fundacional, de Comitê de Governança Digital ou colegiado equivalente com função deliberativa sobre ações de governo digital e uso de recursos de TIC, incluindo a aprovação dos instrumentos de planejamento previstos no Decreto.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.1, III.1 e V.1 – Precedente pela instituição e atuação efetiva de instância colegiada de governança de TIC, com responsabilidade pelo alinhamento das ações de TIC aos objetivos institucionais, priorização dos investimentos e monitoramento do desempenho da TIC.</t>
         </is>
       </c>
       <c r="H13" s="1" t="inlineStr">
@@ -1432,7 +1433,7 @@
       <c r="O13" s="1" t="n"/>
       <c r="P13" s="1" t="inlineStr">
         <is>
-          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância colegiada equivalente, compatível com o porte e a estrutura decisória da organização, atentando-se, minimamente, em realizar reuniões periódicas, registrar deliberações e acompanhar decisões sobre prioridades, projetos, riscos, serviços, orçamento e contratações de TIC</t>
+          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância colegiada equivalente, mediante o exercício das competências previstas em seu ato constitutivo, com registro das deliberações e acompanhamento dos respectivos encaminhamentos</t>
         </is>
       </c>
     </row>
@@ -3204,7 +3205,7 @@
     <row r="46" ht="113.45" customHeight="1">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>AV86</t>
+          <t>AV92</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -3217,13 +3218,14 @@
       <c r="E46" s="1" t="n"/>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>q1001ext[H]</t>
+          <t>q2101ext[A]</t>
         </is>
       </c>
       <c r="G46" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, MEA01.04 - Avaliar o desempenho: monitorar e avaliar periodicamente o desempenho e a conformidade da TI em relação a objetivos, indicadores, metas e expectativas das partes interessadas.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.1: necessidade de estrutura de governança de TI, especialmente Comitê de Tecnologia da Informação ou instância equivalente, com participação de áreas relevantes, responsabilidade de alinhar as ações de TI aos objetivos institucionais, priorizar investimentos e monitorar o desempenho da TI com base em indicadores e metas.</t>
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
         </is>
       </c>
       <c r="H46" s="1" t="inlineStr">
@@ -3234,7 +3236,7 @@
       <c r="I46" s="1" t="n"/>
       <c r="J46" s="1" t="inlineStr">
         <is>
-          <t>Ausência de objetivos, indicadores ou metas para a gestão de TIC.</t>
+          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
         </is>
       </c>
       <c r="K46" s="1" t="inlineStr">
@@ -3252,14 +3254,14 @@
       <c r="O46" s="1" t="n"/>
       <c r="P46" s="1" t="inlineStr">
         <is>
-          <t>estabeleça modelo básico de governança e gestão de TIC definindo objetivos, indicadores, metas e forma de acompanhamento periódico do desempenho da TIC pela alta administração</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
     <row r="47" ht="113.45" customHeight="1">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>AV89</t>
+          <t>AV93</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -3272,14 +3274,14 @@
       <c r="E47" s="1" t="n"/>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>q1001ext[E]</t>
+          <t>q2101ext[B]</t>
         </is>
       </c>
       <c r="G47" s="1" t="inlineStr">
         <is>
-          <t>Acórdão TCE-RJ 44.490/2024-PLEN, item II.1: necessidade de estrutura de governança de TI, especialmente Comitê de Tecnologia da Informação ou instância equivalente, com participação de áreas relevantes, responsabilidade de alinhar as ações de TI aos objetivos institucionais, priorizar investimentos e monitorar o desempenho da TI com base em indicadores e metas.
-Lei nº 14.133/2021, art. 11, parágrafo único: dever da alta administração de implementar estruturas de governança das contratações.
-Acórdão TCU nº 1.411/2014-Plenário, item 9.1.2: precedente sobre funcionamento permanente e composição relevante do Comitê de TIC.</t>
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
         </is>
       </c>
       <c r="H47" s="1" t="inlineStr">
@@ -3290,7 +3292,7 @@
       <c r="I47" s="1" t="n"/>
       <c r="J47" s="1" t="inlineStr">
         <is>
-          <t>Comitê de TIC ou instância equivalente não instituído formalmente.</t>
+          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
         </is>
       </c>
       <c r="K47" s="1" t="inlineStr">
@@ -3308,14 +3310,14 @@
       <c r="O47" s="1" t="n"/>
       <c r="P47" s="1" t="inlineStr">
         <is>
-          <t>institua formalmente Comitê de TIC ou instância colegiada equivalente, compatível com o porte e a estrutura decisória da organização, atentando-se, minimamente, em definir sua composição, competências, periodicidade de reuniões, forma de registro das deliberações e acompanhamento dos encaminhamentos</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
     <row r="48" ht="113.45" customHeight="1">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>AV91</t>
+          <t>AV95</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -3328,13 +3330,14 @@
       <c r="E48" s="1" t="n"/>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>q1001ext[F]</t>
+          <t>q2101ext[D]</t>
         </is>
       </c>
       <c r="G48" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, MEA01.04 - Avaliar o desempenho: monitorar e avaliar periodicamente o desempenho e a conformidade da TI em relação a objetivos, indicadores, metas e expectativas das partes interessadas.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.1: necessidade de estrutura de governança de TI, especialmente Comitê de Tecnologia da Informação ou instância equivalente, com participação de áreas relevantes, responsabilidade de alinhar as ações de TI aos objetivos institucionais, priorizar investimentos e monitorar o desempenho da TI com base em indicadores e metas.</t>
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
         </is>
       </c>
       <c r="H48" s="1" t="inlineStr">
@@ -3345,7 +3348,7 @@
       <c r="I48" s="1" t="n"/>
       <c r="J48" s="1" t="inlineStr">
         <is>
-          <t>Comitê de TIC ou instância equivalente sem atuação efetiva comprovada.</t>
+          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
         </is>
       </c>
       <c r="K48" s="1" t="inlineStr">
@@ -3363,14 +3366,14 @@
       <c r="O48" s="1" t="n"/>
       <c r="P48" s="1" t="inlineStr">
         <is>
-          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância colegiada equivalente, compatível com o porte e a estrutura decisória da organização, atentando-se, minimamente, em realizar reuniões periódicas, registrar deliberações e acompanhar decisões sobre prioridades, projetos, riscos, serviços, orçamento e contratações de TIC</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
     <row r="49" ht="113.45" customHeight="1">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>AV92</t>
+          <t>AV96</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -3383,13 +3386,12 @@
       <c r="E49" s="1" t="n"/>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>q2101ext[A]</t>
+          <t>q2102ext[A]</t>
         </is>
       </c>
       <c r="G49" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+          <t>Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
 Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
         </is>
       </c>
@@ -3401,7 +3403,7 @@
       <c r="I49" s="1" t="n"/>
       <c r="J49" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
+          <t>Ausência de aprovação formal do plano de TIC.</t>
         </is>
       </c>
       <c r="K49" s="1" t="inlineStr">
@@ -3419,14 +3421,14 @@
       <c r="O49" s="1" t="n"/>
       <c r="P49" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>submeta o plano de TIC à aprovação formal do dirigente máximo ou de instância competente da alta administração, mantendo registro do respectivo ato de aprovação</t>
         </is>
       </c>
     </row>
     <row r="50" ht="113.45" customHeight="1">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>AV93</t>
+          <t>AV97</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -3439,7 +3441,7 @@
       <c r="E50" s="1" t="n"/>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>q2101ext[B]</t>
+          <t>q2102ext[D]</t>
         </is>
       </c>
       <c r="G50" s="1" t="inlineStr">
@@ -3457,7 +3459,7 @@
       <c r="I50" s="1" t="n"/>
       <c r="J50" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
+          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
         </is>
       </c>
       <c r="K50" s="1" t="inlineStr">
@@ -3475,14 +3477,14 @@
       <c r="O50" s="1" t="n"/>
       <c r="P50" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>revise o plano de TIC para explicitar seu alinhamento ao planejamento institucional, às diretrizes superiores e às necessidades das áreas finalísticas e administrativas, relacionando objetivos, iniciativas, indicadores e metas de TIC aos resultados institucionais pretendidos</t>
         </is>
       </c>
     </row>
     <row r="51" ht="113.45" customHeight="1">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>AV95</t>
+          <t>AV98</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -3495,14 +3497,14 @@
       <c r="E51" s="1" t="n"/>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>q2101ext[D]</t>
+          <t>q2102ext[C]</t>
         </is>
       </c>
       <c r="G51" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
+          <t>COBIT 2019, APO06.03 - Criar e manter orçamentos: elaborar e manter orçamento de TIC alinhado ao portfólio, ao planejamento e às prioridades aprovadas.
+Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.
+Lei nº 14.133/2021, art. 12, inciso VII e § 1º - Planejamento das contratações: o Plano de Contratações Anual, quando elaborado, deve alinhar-se ao planejamento estratégico, subsidiar a elaboração das leis orçamentárias e ser observado nas licitações e na execução contratual.</t>
         </is>
       </c>
       <c r="H51" s="1" t="inlineStr">
@@ -3513,7 +3515,7 @@
       <c r="I51" s="1" t="n"/>
       <c r="J51" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
+          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
         </is>
       </c>
       <c r="K51" s="1" t="inlineStr">
@@ -3531,14 +3533,14 @@
       <c r="O51" s="1" t="n"/>
       <c r="P51" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>integre o plano de TIC à elaboração da proposta orçamentária e do plano de contratações, de maneira proporcional ao porte, à estrutura e à capacidade de planejamento da organização</t>
         </is>
       </c>
     </row>
     <row r="52" ht="113.45" customHeight="1">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>AV96</t>
+          <t>AV101</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -3551,13 +3553,12 @@
       <c r="E52" s="1" t="n"/>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>q2102ext[A]</t>
+          <t>q2102ext[E]</t>
         </is>
       </c>
       <c r="G52" s="1" t="inlineStr">
         <is>
-          <t>Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
+          <t>Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
         </is>
       </c>
       <c r="H52" s="1" t="inlineStr">
@@ -3568,7 +3569,7 @@
       <c r="I52" s="1" t="n"/>
       <c r="J52" s="1" t="inlineStr">
         <is>
-          <t>Ausência de aprovação formal do plano de TIC.</t>
+          <t>Ausência de acompanhamento, revisão ou atualização periódica do plano de TIC.</t>
         </is>
       </c>
       <c r="K52" s="1" t="inlineStr">
@@ -3586,14 +3587,14 @@
       <c r="O52" s="1" t="n"/>
       <c r="P52" s="1" t="inlineStr">
         <is>
-          <t>submeta o plano de TIC à aprovação formal do dirigente máximo ou de instância competente da alta administração, mantendo registro do respectivo ato de aprovação</t>
+          <t>estabeleça e execute rotina periódica de acompanhamento, revisão e atualização do plano de TIC, registrando execução, pendências, reprogramações e deliberações</t>
         </is>
       </c>
     </row>
     <row r="53" ht="113.45" customHeight="1">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>AV97</t>
+          <t>AV103</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -3606,14 +3607,13 @@
       <c r="E53" s="1" t="n"/>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>q2102ext[D]</t>
+          <t>q2703ext[C]</t>
         </is>
       </c>
       <c r="G53" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
+          <t>COBIT 2019, APO07.05 - Planejar e monitorar o uso de recursos humanos de TI e de negócio: planejar, alocar e acompanhar capacidade de pessoal para iniciativas, operações e serviços de TIC.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6.5 - O PDTI deve contemplar o quantitativo necessário ou ideal para a força de trabalho em TI.</t>
         </is>
       </c>
       <c r="H53" s="1" t="inlineStr">
@@ -3624,7 +3624,7 @@
       <c r="I53" s="1" t="n"/>
       <c r="J53" s="1" t="inlineStr">
         <is>
-          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
+          <t>A organização não definiu o quantitativo necessário de pessoal de TIC e segurança da informação.</t>
         </is>
       </c>
       <c r="K53" s="1" t="inlineStr">
@@ -3636,20 +3636,20 @@
       <c r="M53" s="1" t="n"/>
       <c r="N53" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O53" s="1" t="n"/>
       <c r="P53" s="1" t="inlineStr">
         <is>
-          <t>revise o plano de TIC para explicitar seu alinhamento ao planejamento institucional, às diretrizes superiores e às necessidades das áreas finalísticas e administrativas, relacionando objetivos, iniciativas, indicadores e metas de TIC aos resultados institucionais pretendidos</t>
+          <t>estime e mantenha atualizado o quantitativo necessário de pessoal de TIC e segurança da informação, considerando o porte e a complexidade da organização, os serviços críticos, os sistemas mantidos, as contratações vigentes e os riscos relevantes</t>
         </is>
       </c>
     </row>
     <row r="54" ht="113.45" customHeight="1">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>AV98</t>
+          <t>AV105</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -3662,14 +3662,13 @@
       <c r="E54" s="1" t="n"/>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>q2102ext[C]</t>
+          <t>q2708[B]</t>
         </is>
       </c>
       <c r="G54" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO06.03 - Criar e manter orçamentos: elaborar e manter orçamento de TIC alinhado ao portfólio, ao planejamento e às prioridades aprovadas.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.
-Lei nº 14.133/2021, art. 12, inciso VII e § 1º - Planejamento das contratações: o Plano de Contratações Anual, quando elaborado, deve alinhar-se ao planejamento estratégico, subsidiar a elaboração das leis orçamentárias e ser observado nas licitações e na execução contratual.</t>
+          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
+COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
         </is>
       </c>
       <c r="H54" s="1" t="inlineStr">
@@ -3680,7 +3679,7 @@
       <c r="I54" s="1" t="n"/>
       <c r="J54" s="1" t="inlineStr">
         <is>
-          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="K54" s="1" t="inlineStr">
@@ -3692,20 +3691,20 @@
       <c r="M54" s="1" t="n"/>
       <c r="N54" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O54" s="1" t="n"/>
       <c r="P54" s="1" t="inlineStr">
         <is>
-          <t>integre o plano de TIC à elaboração da proposta orçamentária e do plano de contratações, de maneira proporcional ao porte, à estrutura e à capacidade de planejamento da organização</t>
+          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
         </is>
       </c>
     </row>
     <row r="55" ht="113.45" customHeight="1">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>AV101</t>
+          <t>AV107</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -3718,12 +3717,13 @@
       <c r="E55" s="1" t="n"/>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>q2102ext[E]</t>
+          <t>q2708[D]</t>
         </is>
       </c>
       <c r="G55" s="1" t="inlineStr">
         <is>
-          <t>Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
+          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
+COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
         </is>
       </c>
       <c r="H55" s="1" t="inlineStr">
@@ -3734,7 +3734,7 @@
       <c r="I55" s="1" t="n"/>
       <c r="J55" s="1" t="inlineStr">
         <is>
-          <t>Ausência de acompanhamento, revisão ou atualização periódica do plano de TIC.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="K55" s="1" t="inlineStr">
@@ -3746,20 +3746,20 @@
       <c r="M55" s="1" t="n"/>
       <c r="N55" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O55" s="1" t="n"/>
       <c r="P55" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e execute rotina periódica de acompanhamento, revisão e atualização do plano de TIC, registrando execução, pendências, reprogramações e deliberações</t>
+          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
         </is>
       </c>
     </row>
     <row r="56" ht="113.45" customHeight="1">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>AV103</t>
+          <t>AV124</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -3772,13 +3772,13 @@
       <c r="E56" s="1" t="n"/>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>q2703ext[C]</t>
+          <t>q2201ext[A]</t>
         </is>
       </c>
       <c r="G56" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO07.05 - Planejar e monitorar o uso de recursos humanos de TI e de negócio: planejar, alocar e acompanhar capacidade de pessoal para iniciativas, operações e serviços de TIC.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6.5 - O PDTI deve contemplar o quantitativo necessário ou ideal para a força de trabalho em TI.</t>
+          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
+ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.</t>
         </is>
       </c>
       <c r="H56" s="1" t="inlineStr">
@@ -3789,7 +3789,7 @@
       <c r="I56" s="1" t="n"/>
       <c r="J56" s="1" t="inlineStr">
         <is>
-          <t>A organização não definiu o quantitativo necessário de pessoal de TIC e segurança da informação.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="K56" s="1" t="inlineStr">
@@ -3807,14 +3807,14 @@
       <c r="O56" s="1" t="n"/>
       <c r="P56" s="1" t="inlineStr">
         <is>
-          <t>estime e mantenha atualizado o quantitativo necessário de pessoal de TIC e segurança da informação, considerando o porte e a complexidade da organização, os serviços críticos, os sistemas mantidos, as contratações vigentes e os riscos relevantes</t>
+          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
         </is>
       </c>
     </row>
     <row r="57" ht="90.95" customHeight="1">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>AV105</t>
+          <t>AV125</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -3827,13 +3827,13 @@
       <c r="E57" s="1" t="n"/>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>q2708[B]</t>
+          <t>q2201ext[B]</t>
         </is>
       </c>
       <c r="G57" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
-COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
+          <t>ITIL 4, prática de gerenciamento do catálogo de serviços: manter fonte única de informações consistentes sobre serviços e ofertas de serviço, disponível para usuários e equipes de suporte.
+COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.</t>
         </is>
       </c>
       <c r="H57" s="1" t="inlineStr">
@@ -3844,7 +3844,7 @@
       <c r="I57" s="1" t="n"/>
       <c r="J57" s="1" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="K57" s="1" t="inlineStr">
@@ -3862,14 +3862,14 @@
       <c r="O57" s="1" t="n"/>
       <c r="P57" s="1" t="inlineStr">
         <is>
-          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
+          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
         </is>
       </c>
     </row>
     <row r="58" ht="90.95" customHeight="1">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>AV107</t>
+          <t>AV126</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -3882,13 +3882,13 @@
       <c r="E58" s="1" t="n"/>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>q2708[D]</t>
+          <t>q2201ext[C]</t>
         </is>
       </c>
       <c r="G58" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
-COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
+          <t>ITIL 4, prática de gerenciamento do catálogo de serviços: manter fonte única de informações consistentes sobre serviços e ofertas de serviço, disponível para usuários e equipes de suporte.
+COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.</t>
         </is>
       </c>
       <c r="H58" s="1" t="inlineStr">
@@ -3899,7 +3899,7 @@
       <c r="I58" s="1" t="n"/>
       <c r="J58" s="1" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="K58" s="1" t="inlineStr">
@@ -3917,14 +3917,14 @@
       <c r="O58" s="1" t="n"/>
       <c r="P58" s="1" t="inlineStr">
         <is>
-          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
+          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
         </is>
       </c>
     </row>
     <row r="59" ht="90.95" customHeight="1">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>AV124</t>
+          <t>AV127</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -3937,7 +3937,7 @@
       <c r="E59" s="1" t="n"/>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[A]</t>
+          <t>q2201ext[D]</t>
         </is>
       </c>
       <c r="G59" s="1" t="inlineStr">
@@ -3979,7 +3979,7 @@
     <row r="60" ht="79.90000000000001" customHeight="1">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>AV125</t>
+          <t>AV128</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -3992,13 +3992,13 @@
       <c r="E60" s="1" t="n"/>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[B]</t>
+          <t>q2201ext[E]</t>
         </is>
       </c>
       <c r="G60" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento do catálogo de serviços: manter fonte única de informações consistentes sobre serviços e ofertas de serviço, disponível para usuários e equipes de suporte.
-COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.</t>
+          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
+ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.</t>
         </is>
       </c>
       <c r="H60" s="1" t="inlineStr">
@@ -4009,7 +4009,7 @@
       <c r="I60" s="1" t="n"/>
       <c r="J60" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="K60" s="1" t="inlineStr">
@@ -4027,14 +4027,14 @@
       <c r="O60" s="1" t="n"/>
       <c r="P60" s="1" t="inlineStr">
         <is>
-          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
+          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
         </is>
       </c>
     </row>
     <row r="61" ht="79.90000000000001" customHeight="1">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>AV126</t>
+          <t>AV129</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -4047,13 +4047,13 @@
       <c r="E61" s="1" t="n"/>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[C]</t>
+          <t>q2203ext[A]</t>
         </is>
       </c>
       <c r="G61" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento do catálogo de serviços: manter fonte única de informações consistentes sobre serviços e ofertas de serviço, disponível para usuários e equipes de suporte.
-COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.</t>
+          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
+Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
         </is>
       </c>
       <c r="H61" s="1" t="inlineStr">
@@ -4064,7 +4064,7 @@
       <c r="I61" s="1" t="n"/>
       <c r="J61" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="K61" s="1" t="inlineStr">
@@ -4076,20 +4076,20 @@
       <c r="M61" s="1" t="n"/>
       <c r="N61" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O61" s="1" t="n"/>
       <c r="P61" s="1" t="inlineStr">
         <is>
-          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
+          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
         </is>
       </c>
     </row>
     <row r="62" ht="90.95" customHeight="1">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>AV127</t>
+          <t>AV132</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -4102,13 +4102,13 @@
       <c r="E62" s="1" t="n"/>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[D]</t>
+          <t>q2504ext[A]</t>
         </is>
       </c>
       <c r="G62" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
-ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.</t>
+          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
+Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
         </is>
       </c>
       <c r="H62" s="1" t="inlineStr">
@@ -4119,7 +4119,7 @@
       <c r="I62" s="1" t="n"/>
       <c r="J62" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="K62" s="1" t="inlineStr">
@@ -4131,20 +4131,20 @@
       <c r="M62" s="1" t="n"/>
       <c r="N62" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O62" s="1" t="n"/>
       <c r="P62" s="1" t="inlineStr">
         <is>
-          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
+          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
         </is>
       </c>
     </row>
     <row r="63" ht="90.95" customHeight="1">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>AV128</t>
+          <t>AV133</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -4157,13 +4157,13 @@
       <c r="E63" s="1" t="n"/>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[E]</t>
+          <t>q2504ext[B]</t>
         </is>
       </c>
       <c r="G63" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
-ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.</t>
+          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
+Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
         </is>
       </c>
       <c r="H63" s="1" t="inlineStr">
@@ -4174,7 +4174,7 @@
       <c r="I63" s="1" t="n"/>
       <c r="J63" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="K63" s="1" t="inlineStr">
@@ -4186,20 +4186,20 @@
       <c r="M63" s="1" t="n"/>
       <c r="N63" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O63" s="1" t="n"/>
       <c r="P63" s="1" t="inlineStr">
         <is>
-          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
+          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
         </is>
       </c>
     </row>
     <row r="64" ht="90.95" customHeight="1">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>AV129</t>
+          <t>AV136</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -4212,13 +4212,13 @@
       <c r="E64" s="1" t="n"/>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>q2203ext[A]</t>
+          <t>q2203ext[C]</t>
         </is>
       </c>
       <c r="G64" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
+          <t>ITIL 4, prática de gerenciamento de configuração de serviço: assegurar informações precisas e confiáveis sobre itens de configuração e seus relacionamentos com serviços, sistemas e infraestrutura.
+COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.</t>
         </is>
       </c>
       <c r="H64" s="1" t="inlineStr">
@@ -4229,7 +4229,7 @@
       <c r="I64" s="1" t="n"/>
       <c r="J64" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="K64" s="1" t="inlineStr">
@@ -4241,20 +4241,20 @@
       <c r="M64" s="1" t="n"/>
       <c r="N64" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O64" s="1" t="n"/>
       <c r="P64" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
+          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
         </is>
       </c>
     </row>
     <row r="65" ht="90.95" customHeight="1">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>AV132</t>
+          <t>AV137</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -4267,13 +4267,13 @@
       <c r="E65" s="1" t="n"/>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>q2504ext[A]</t>
+          <t>q2204ext[A]</t>
         </is>
       </c>
       <c r="G65" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
         </is>
       </c>
       <c r="H65" s="1" t="inlineStr">
@@ -4284,7 +4284,7 @@
       <c r="I65" s="1" t="n"/>
       <c r="J65" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="K65" s="1" t="inlineStr">
@@ -4296,20 +4296,20 @@
       <c r="M65" s="1" t="n"/>
       <c r="N65" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O65" s="1" t="n"/>
       <c r="P65" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
     </row>
     <row r="66" ht="90.95" customHeight="1">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>AV133</t>
+          <t>AV140</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -4322,13 +4322,13 @@
       <c r="E66" s="1" t="n"/>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>q2504ext[B]</t>
+          <t>q2204ext[D]</t>
         </is>
       </c>
       <c r="G66" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
         </is>
       </c>
       <c r="H66" s="1" t="inlineStr">
@@ -4339,7 +4339,7 @@
       <c r="I66" s="1" t="n"/>
       <c r="J66" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="K66" s="1" t="inlineStr">
@@ -4351,20 +4351,20 @@
       <c r="M66" s="1" t="n"/>
       <c r="N66" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O66" s="1" t="n"/>
       <c r="P66" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
     </row>
     <row r="67" ht="79.90000000000001" customHeight="1">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>AV136</t>
+          <t>AV141</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -4377,13 +4377,13 @@
       <c r="E67" s="1" t="n"/>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>q2203ext[C]</t>
+          <t>q2204ext[E]</t>
         </is>
       </c>
       <c r="G67" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de configuração de serviço: assegurar informações precisas e confiáveis sobre itens de configuração e seus relacionamentos com serviços, sistemas e infraestrutura.
-COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.</t>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
         </is>
       </c>
       <c r="H67" s="1" t="inlineStr">
@@ -4394,7 +4394,7 @@
       <c r="I67" s="1" t="n"/>
       <c r="J67" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="K67" s="1" t="inlineStr">
@@ -4412,14 +4412,14 @@
       <c r="O67" s="1" t="n"/>
       <c r="P67" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
     </row>
     <row r="68" ht="79.90000000000001" customHeight="1">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>AV137</t>
+          <t>AV143</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -4432,13 +4432,13 @@
       <c r="E68" s="1" t="n"/>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>q2204ext[A]</t>
+          <t>q2801ext[A]</t>
         </is>
       </c>
       <c r="G68" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
+          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
         </is>
       </c>
       <c r="H68" s="1" t="inlineStr">
@@ -4449,7 +4449,7 @@
       <c r="I68" s="1" t="n"/>
       <c r="J68" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="K68" s="1" t="inlineStr">
@@ -4461,20 +4461,20 @@
       <c r="M68" s="1" t="n"/>
       <c r="N68" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O68" s="1" t="n"/>
       <c r="P68" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
+          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
         </is>
       </c>
     </row>
     <row r="69" ht="79.90000000000001" customHeight="1">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>AV140</t>
+          <t>AV148</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -4487,13 +4487,14 @@
       <c r="E69" s="1" t="n"/>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>q2204ext[D]</t>
+          <t>q2804[A]</t>
         </is>
       </c>
       <c r="G69" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
+          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+COBIT 2019, BAI02.04 - Obter aprovação dos requisitos da solução: obter aprovação formal dos requisitos funcionais, técnicos, de segurança e de conformidade antes de prosseguir com a solução.
+Instrução Normativa SGD/ME nº 94, de 23 de dezembro de 2022, art. 1º, § 1º: como referência de boa prática, a aplicação de ritos formais de contratação de TIC pode ser facultada para contratações diretas por dispensa em razão do valor (inciso II do art. 75 da Lei nº 14.133/2021), indicando a possibilidade de fluxos simplificados para aquisições de baixa complexidade ou valor.</t>
         </is>
       </c>
       <c r="H69" s="1" t="inlineStr">
@@ -4504,7 +4505,7 @@
       <c r="I69" s="1" t="n"/>
       <c r="J69" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
         </is>
       </c>
       <c r="K69" s="1" t="inlineStr">
@@ -4522,14 +4523,14 @@
       <c r="O69" s="1" t="n"/>
       <c r="P69" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
+          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo fluxos simplificados para contratações de baixa complexidade ou baixo valor, desde que preservada análise técnica mínima compatível com o risco da contratação</t>
         </is>
       </c>
     </row>
     <row r="70" ht="90.95" customHeight="1">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>AV141</t>
+          <t>AV150</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -4542,13 +4543,13 @@
       <c r="E70" s="1" t="n"/>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>q2204ext[E]</t>
+          <t>q2802ext[C]</t>
         </is>
       </c>
       <c r="G70" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
+          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Art. 18, caput e §1º, incisos I, IV, V, VIII, IX, X e XIII, da Lei 14.133/2021: fase preparatória caracterizada pelo planejamento, compatibilização com o plano de contratações anual e elementos mínimos do estudo técnico preliminar.</t>
         </is>
       </c>
       <c r="H70" s="1" t="inlineStr">
@@ -4559,7 +4560,7 @@
       <c r="I70" s="1" t="n"/>
       <c r="J70" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
         </is>
       </c>
       <c r="K70" s="1" t="inlineStr">
@@ -4571,25 +4572,25 @@
       <c r="M70" s="1" t="n"/>
       <c r="N70" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O70" s="1" t="n"/>
       <c r="P70" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
+          <t>integre as contratações de TIC com os instrumentos de planejamento da organização e com o Plano de Contratações Anual, quando elaborado, justificando as situações excepcionais</t>
         </is>
       </c>
     </row>
     <row r="71" ht="90.95" customHeight="1">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>AV143</t>
+          <t>AV152</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
-          <t>avaliacao_evidencias_ajustes</t>
+          <t>questionario</t>
         </is>
       </c>
       <c r="C71" s="1" t="n"/>
@@ -4597,7 +4598,7 @@
       <c r="E71" s="1" t="n"/>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>q2801ext[A]</t>
+          <t>q2801ext[B]</t>
         </is>
       </c>
       <c r="G71" s="1" t="inlineStr">
@@ -4608,7 +4609,7 @@
       </c>
       <c r="H71" s="1" t="inlineStr">
         <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+          <t>Resposta negativa ao detalhamento b) do item 2801 do Questionário, para verificar se são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
         </is>
       </c>
       <c r="I71" s="1" t="n"/>
@@ -4619,7 +4620,7 @@
       </c>
       <c r="K71" s="1" t="inlineStr">
         <is>
-          <t>Não conforme</t>
+          <t>(Não | N/A)</t>
         </is>
       </c>
       <c r="L71" s="1" t="n"/>
@@ -4639,7 +4640,7 @@
     <row r="72" ht="90.95" customHeight="1">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>AV148</t>
+          <t>AV153</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -4652,14 +4653,13 @@
       <c r="E72" s="1" t="n"/>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>q2804[A]</t>
+          <t>q2801ext[B]</t>
         </is>
       </c>
       <c r="G72" s="1" t="inlineStr">
         <is>
           <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-COBIT 2019, BAI02.04 - Obter aprovação dos requisitos da solução: obter aprovação formal dos requisitos funcionais, técnicos, de segurança e de conformidade antes de prosseguir com a solução.
-Instrução Normativa SGD/ME nº 94, de 23 de dezembro de 2022, art. 1º, § 1º: como referência de boa prática, a aplicação de ritos formais de contratação de TIC pode ser facultada para contratações diretas por dispensa em razão do valor (inciso II do art. 75 da Lei nº 14.133/2021), indicando a possibilidade de fluxos simplificados para aquisições de baixa complexidade ou valor.</t>
+Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
         </is>
       </c>
       <c r="H72" s="1" t="inlineStr">
@@ -4670,7 +4670,7 @@
       <c r="I72" s="1" t="n"/>
       <c r="J72" s="1" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="K72" s="1" t="inlineStr">
@@ -4682,181 +4682,19 @@
       <c r="M72" s="1" t="n"/>
       <c r="N72" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O72" s="1" t="n"/>
       <c r="P72" s="1" t="inlineStr">
         <is>
-          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo fluxos simplificados para contratações de baixa complexidade ou baixo valor, desde que preservada análise técnica mínima compatível com o risco da contratação</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="90.95" customHeight="1">
-      <c r="A73" s="1" t="inlineStr">
-        <is>
-          <t>AV150</t>
-        </is>
-      </c>
-      <c r="B73" s="1" t="inlineStr">
-        <is>
-          <t>avaliacao_evidencias_ajustes</t>
-        </is>
-      </c>
-      <c r="C73" s="1" t="n"/>
-      <c r="D73" s="1" t="n"/>
-      <c r="E73" s="1" t="n"/>
-      <c r="F73" s="1" t="inlineStr">
-        <is>
-          <t>q2802ext[C]</t>
-        </is>
-      </c>
-      <c r="G73" s="1" t="inlineStr">
-        <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 18, caput e §1º, incisos I, IV, V, VIII, IX, X e XIII, da Lei 14.133/2021: fase preparatória caracterizada pelo planejamento, compatibilização com o plano de contratações anual e elementos mínimos do estudo técnico preliminar.</t>
-        </is>
-      </c>
-      <c r="H73" s="1" t="inlineStr">
-        <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
-        </is>
-      </c>
-      <c r="I73" s="1" t="n"/>
-      <c r="J73" s="1" t="inlineStr">
-        <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
-        </is>
-      </c>
-      <c r="K73" s="1" t="inlineStr">
-        <is>
-          <t>Não conforme</t>
-        </is>
-      </c>
-      <c r="L73" s="1" t="n"/>
-      <c r="M73" s="1" t="n"/>
-      <c r="N73" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O73" s="1" t="n"/>
-      <c r="P73" s="1" t="inlineStr">
-        <is>
-          <t>integre as contratações de TIC com os instrumentos de planejamento da organização e com o Plano de Contratações Anual, quando elaborado, justificando as situações excepcionais</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="90.95" customHeight="1">
-      <c r="A74" s="1" t="inlineStr">
-        <is>
-          <t>AV152</t>
-        </is>
-      </c>
-      <c r="B74" s="1" t="inlineStr">
-        <is>
-          <t>questionario</t>
-        </is>
-      </c>
-      <c r="C74" s="1" t="n"/>
-      <c r="D74" s="1" t="n"/>
-      <c r="E74" s="1" t="n"/>
-      <c r="F74" s="1" t="inlineStr">
-        <is>
-          <t>q2801ext[B]</t>
-        </is>
-      </c>
-      <c r="G74" s="1" t="inlineStr">
-        <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
-        </is>
-      </c>
-      <c r="H74" s="1" t="inlineStr">
-        <is>
-          <t>Resposta negativa ao detalhamento b) do item 2801 do Questionário, para verificar se são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
-        </is>
-      </c>
-      <c r="I74" s="1" t="n"/>
-      <c r="J74" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="K74" s="1" t="inlineStr">
-        <is>
-          <t>(Não | N/A)</t>
-        </is>
-      </c>
-      <c r="L74" s="1" t="n"/>
-      <c r="M74" s="1" t="n"/>
-      <c r="N74" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O74" s="1" t="n"/>
-      <c r="P74" s="1" t="inlineStr">
-        <is>
           <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="90.95" customHeight="1">
-      <c r="A75" s="1" t="inlineStr">
-        <is>
-          <t>AV153</t>
-        </is>
-      </c>
-      <c r="B75" s="1" t="inlineStr">
-        <is>
-          <t>avaliacao_evidencias_ajustes</t>
-        </is>
-      </c>
-      <c r="C75" s="1" t="n"/>
-      <c r="D75" s="1" t="n"/>
-      <c r="E75" s="1" t="n"/>
-      <c r="F75" s="1" t="inlineStr">
-        <is>
-          <t>q2801ext[B]</t>
-        </is>
-      </c>
-      <c r="G75" s="1" t="inlineStr">
-        <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
-        </is>
-      </c>
-      <c r="H75" s="1" t="inlineStr">
-        <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
-        </is>
-      </c>
-      <c r="I75" s="1" t="n"/>
-      <c r="J75" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="K75" s="1" t="inlineStr">
-        <is>
-          <t>Não conforme</t>
-        </is>
-      </c>
-      <c r="L75" s="1" t="n"/>
-      <c r="M75" s="1" t="n"/>
-      <c r="N75" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O75" s="1" t="n"/>
-      <c r="P75" s="1" t="inlineStr">
-        <is>
-          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
-        </is>
-      </c>
-    </row>
+    <row r="73" ht="90.95" customHeight="1"/>
+    <row r="74" ht="90.95" customHeight="1"/>
+    <row r="75" ht="90.95" customHeight="1"/>
     <row r="76" ht="102.2" customHeight="1"/>
     <row r="77" ht="102.2" customHeight="1"/>
     <row r="78" ht="102.2" customHeight="1"/>
@@ -4937,7 +4775,7 @@
     <row r="153" ht="23.85" customHeight="1"/>
     <row r="154" ht="23.85" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A3:P75"/>
+  <autoFilter ref="A3:P72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -4949,7 +4787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H74"/>
+  <dimension ref="A2:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5333,7 +5171,7 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>AV08 &amp; ~AV86</t>
+          <t>AV08</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
@@ -5353,7 +5191,7 @@
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>MR011</t>
+          <t>MR016</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
@@ -5363,25 +5201,25 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Ausência de objetivos, indicadores ou metas para a gestão de TIC.</t>
+          <t>Comitê de TIC ou instância equivalente não instituído formalmente ou sem representação de áreas relevantes da organização.</t>
         </is>
       </c>
       <c r="D12" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>AV86</t>
+          <t>AV11</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>AV86</t>
+          <t>AV11</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>No subitem h) do item 1001, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que estabeleceu objetivos, indicadores e metas para a gestão de tecnologia da informação</t>
+          <t>No subitem e) do item 1001, não houve declaração afirmativa quanto à prática avaliada: dispõe de comitê de tecnologia da informação composto por representantes de áreas relevantes da organização</t>
         </is>
       </c>
       <c r="H12" s="9" t="b">
@@ -5391,7 +5229,7 @@
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>MR016</t>
+          <t>MR018</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
@@ -5401,7 +5239,7 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>Comitê de TIC ou instância equivalente não instituído formalmente.</t>
+          <t>Comitê de TIC ou instância equivalente sem atuação efetiva comprovada.</t>
         </is>
       </c>
       <c r="D13" s="9" t="n">
@@ -5409,17 +5247,17 @@
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>AV11 &amp; ~AV89</t>
+          <t>AV12 &amp; AV13</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>AV11</t>
+          <t>AV12</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 1001, não houve declaração afirmativa quanto à prática avaliada: dispõe de comitê de tecnologia da informação composto por representantes de áreas relevantes da organização</t>
+          <t>No subitem e) do item 1001, a organização declarou dispor de comitê de tecnologia da informação composto por representantes de áreas relevantes, o que levou à análise de sua atuação efetiva</t>
         </is>
       </c>
       <c r="H13" s="9" t="b">
@@ -5429,7 +5267,7 @@
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>MR017</t>
+          <t>MR020</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
@@ -5439,7 +5277,7 @@
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Comitê de TIC ou instância equivalente não instituído formalmente.</t>
+          <t>Comitê de TIC ou instância equivalente sem atuação efetiva comprovada.</t>
         </is>
       </c>
       <c r="D14" s="9" t="n">
@@ -5447,17 +5285,17 @@
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>AV89</t>
+          <t>AV12 &amp; AV13</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>AV89</t>
+          <t>AV13</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 1001, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que dispõe de comitê de tecnologia da informação composto por representantes de áreas relevantes da organização</t>
+          <t>No subitem f) do item 1001, não houve declaração afirmativa quanto à atuação do comitê de tecnologia da informação nas atividades previstas em ato constitutivo</t>
         </is>
       </c>
       <c r="H14" s="9" t="b">
@@ -5467,17 +5305,17 @@
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>MR018</t>
+          <t>MR022</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>PA02</t>
+          <t>PA03</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Comitê de TIC ou instância equivalente sem atuação efetiva comprovada.</t>
+          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
         </is>
       </c>
       <c r="D15" s="9" t="n">
@@ -5485,17 +5323,17 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>AV12 &amp; (AV13 | AV91)</t>
+          <t>AV14 &amp; ~AV92</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>AV12</t>
+          <t>AV14</t>
         </is>
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 1001, a organização declarou dispor de comitê de tecnologia da informação composto por representantes de áreas relevantes, o que levou à análise de sua atuação efetiva</t>
+          <t>No subitem a) do item 2101, não houve declaração afirmativa quanto à prática avaliada: as áreas demandantes de soluções de TI participam do processo de planejamento de tecnologia da informação</t>
         </is>
       </c>
       <c r="H15" s="9" t="b">
@@ -5505,17 +5343,17 @@
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>MR020</t>
+          <t>MR023</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>PA02</t>
+          <t>PA03</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Comitê de TIC ou instância equivalente sem atuação efetiva comprovada.</t>
+          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
         </is>
       </c>
       <c r="D16" s="9" t="n">
@@ -5523,17 +5361,17 @@
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>AV12 &amp; AV13 &amp; ~AV91</t>
+          <t>AV92</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>AV13</t>
+          <t>AV92</t>
         </is>
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>No subitem f) do item 1001, não houve declaração afirmativa quanto à atuação do comitê de tecnologia da informação nas atividades previstas em ato constitutivo</t>
+          <t>No subitem a) do item 2101, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as áreas demandantes de soluções de TI participam do processo de planejamento de tecnologia da informação</t>
         </is>
       </c>
       <c r="H16" s="9" t="b">
@@ -5543,17 +5381,17 @@
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>MR021</t>
+          <t>MR024</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>PA02</t>
+          <t>PA03</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Comitê de TIC ou instância equivalente sem atuação efetiva comprovada.</t>
+          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
         </is>
       </c>
       <c r="D17" s="9" t="n">
@@ -5561,17 +5399,17 @@
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>AV12 &amp; AV91</t>
+          <t>AV15 &amp; ~AV93</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>AV91</t>
+          <t>AV15</t>
         </is>
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>No subitem f) do item 1001, a organização declarou atuação do comitê de tecnologia da informação, mas a evidência foi insuficiente para comprovar a prática declarada</t>
+          <t>No subitem b) do item 2101, não houve declaração afirmativa quanto à prática avaliada: estabeleceu critérios para orientar a seleção e a priorização das iniciativas de TI (projetos e ações) e os mantêm atualizados</t>
         </is>
       </c>
       <c r="H17" s="9" t="b">
@@ -5581,7 +5419,7 @@
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>MR022</t>
+          <t>MR025</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
@@ -5595,21 +5433,21 @@
         </is>
       </c>
       <c r="D18" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>AV14 &amp; ~AV92</t>
+          <t>AV93</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>AV14</t>
+          <t>AV93</t>
         </is>
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2101, não houve declaração afirmativa quanto à prática avaliada: as áreas demandantes de soluções de TI participam do processo de planejamento de tecnologia da informação</t>
+          <t>No subitem b) do item 2101, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que estabeleceu critérios para orientar a seleção e a priorização das iniciativas de TI (projetos e ações) e os mantêm atualizados</t>
         </is>
       </c>
       <c r="H18" s="9" t="b">
@@ -5619,7 +5457,7 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>MR023</t>
+          <t>MR028</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
@@ -5633,21 +5471,21 @@
         </is>
       </c>
       <c r="D19" s="9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>AV92</t>
+          <t>AV17 &amp; ~AV95</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>AV92</t>
+          <t>AV17</t>
         </is>
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2101, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as áreas demandantes de soluções de TI participam do processo de planejamento de tecnologia da informação</t>
+          <t>No subitem d) do item 2101, não houve declaração afirmativa quanto à prática avaliada: o processo de planejamento de TI está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H19" s="9" t="b">
@@ -5657,7 +5495,7 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>MR024</t>
+          <t>MR029</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
@@ -5671,21 +5509,21 @@
         </is>
       </c>
       <c r="D20" s="9" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>AV15 &amp; ~AV93</t>
+          <t>AV95</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>AV15</t>
+          <t>AV95</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2101, não houve declaração afirmativa quanto à prática avaliada: estabeleceu critérios para orientar a seleção e a priorização das iniciativas de TI (projetos e ações) e os mantêm atualizados</t>
+          <t>No subitem d) do item 2101, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de planejamento de TI está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H20" s="9" t="b">
@@ -5695,7 +5533,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>MR025</t>
+          <t>MR030</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
@@ -5705,25 +5543,25 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
+          <t>Ausência de aprovação formal do plano de TIC.</t>
         </is>
       </c>
       <c r="D21" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>AV93</t>
+          <t>AV18 &amp; ~AV96</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>AV93</t>
+          <t>AV18</t>
         </is>
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2101, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que estabeleceu critérios para orientar a seleção e a priorização das iniciativas de TI (projetos e ações) e os mantêm atualizados</t>
+          <t>No subitem a) do item 2102, não houve declaração afirmativa quanto à prática avaliada: o plano de tecnologia da informação (plano de TI) é aprovado pelo dirigente máximo da organização ou por dirigente ou colegiado que integra a alta administração</t>
         </is>
       </c>
       <c r="H21" s="9" t="b">
@@ -5733,7 +5571,7 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>MR028</t>
+          <t>MR031</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
@@ -5743,25 +5581,25 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
+          <t>Ausência de aprovação formal do plano de TIC.</t>
         </is>
       </c>
       <c r="D22" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>AV17 &amp; ~AV95</t>
+          <t>AV96</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>AV17</t>
+          <t>AV96</t>
         </is>
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2101, não houve declaração afirmativa quanto à prática avaliada: o processo de planejamento de TI está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem a) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o plano de tecnologia da informação (plano de TI) é aprovado pelo dirigente máximo da organização ou por dirigente ou colegiado que integra a alta administração</t>
         </is>
       </c>
       <c r="H22" s="9" t="b">
@@ -5771,7 +5609,7 @@
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>MR029</t>
+          <t>MR032</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
@@ -5781,25 +5619,25 @@
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
+          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
         </is>
       </c>
       <c r="D23" s="9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>AV95</t>
+          <t>AV19 &amp; ~AV97</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>AV95</t>
+          <t>AV19</t>
         </is>
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2101, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de planejamento de TI está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem d) do item 2102, não houve declaração afirmativa quanto à prática avaliada: as iniciativas de TI (projetos e ações) constantes do plano de TI alinham-se aos objetivos e iniciativas definidos no planejamento institucional (como PPA, planos estratégicos, planos setoriais e plano de governo, no caso de municípios), bem como, quando aplicável, às estratégias e diretrizes estabelecidas por instâncias superiores de governança (como a Estratégia Nacional de Tecnologia da Informação e Comunicação do Poder Judiciário - ENTIC-JUD, normas e orientações do SETIC/PRODERJ (para órgãos estaduais) ou instâncias de governança equivalentes no âmbito municipal)</t>
         </is>
       </c>
       <c r="H23" s="9" t="b">
@@ -5809,7 +5647,7 @@
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>MR030</t>
+          <t>MR033</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
@@ -5819,25 +5657,25 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Ausência de aprovação formal do plano de TIC.</t>
+          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
         </is>
       </c>
       <c r="D24" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>AV18 &amp; ~AV96</t>
+          <t>AV97</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>AV18</t>
+          <t>AV97</t>
         </is>
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2102, não houve declaração afirmativa quanto à prática avaliada: o plano de tecnologia da informação (plano de TI) é aprovado pelo dirigente máximo da organização ou por dirigente ou colegiado que integra a alta administração</t>
+          <t>No subitem d) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as iniciativas de TI (projetos e ações) constantes do plano de TI alinham-se aos objetivos e iniciativas definidos no planejamento institucional (como PPA, planos estratégicos, planos setoriais e plano de governo, no caso de municípios), bem como, quando aplicável, às estratégias e diretrizes estabelecidas por instâncias superiores de governança (como a Estratégia Nacional de Tecnologia da Informação e Comunicação do Poder Judiciário - ENTIC-JUD, normas e orientações do SETIC/PRODERJ (para órgãos estaduais) ou instâncias de governança equivalentes no âmbito municipal)</t>
         </is>
       </c>
       <c r="H24" s="9" t="b">
@@ -5847,7 +5685,7 @@
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>MR031</t>
+          <t>MR034</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
@@ -5857,25 +5695,25 @@
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>Ausência de aprovação formal do plano de TIC.</t>
+          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
         </is>
       </c>
       <c r="D25" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>AV96</t>
+          <t>AV20 &amp; ~AV98</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>AV96</t>
+          <t>AV20</t>
         </is>
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o plano de tecnologia da informação (plano de TI) é aprovado pelo dirigente máximo da organização ou por dirigente ou colegiado que integra a alta administração</t>
+          <t>No subitem c) do item 2102, não houve declaração afirmativa quanto à prática avaliada: o plano de TI fundamenta a proposta orçamentária da área de TI e o plano de contratações</t>
         </is>
       </c>
       <c r="H25" s="9" t="b">
@@ -5885,7 +5723,7 @@
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>MR032</t>
+          <t>MR035</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
@@ -5895,25 +5733,25 @@
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
+          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
         </is>
       </c>
       <c r="D26" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>AV19 &amp; ~AV97</t>
+          <t>AV98</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>AV19</t>
+          <t>AV98</t>
         </is>
       </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2102, não houve declaração afirmativa quanto à prática avaliada: as iniciativas de TI (projetos e ações) constantes do plano de TI alinham-se aos objetivos e iniciativas definidos no planejamento institucional (como PPA, planos estratégicos, planos setoriais e plano de governo, no caso de municípios), bem como, quando aplicável, às estratégias e diretrizes estabelecidas por instâncias superiores de governança (como a Estratégia Nacional de Tecnologia da Informação e Comunicação do Poder Judiciário - ENTIC-JUD, normas e orientações do SETIC/PRODERJ (para órgãos estaduais) ou instâncias de governança equivalentes no âmbito municipal)</t>
+          <t>No subitem c) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o plano de TI fundamenta a proposta orçamentária da área de TI e o plano de contratações</t>
         </is>
       </c>
       <c r="H26" s="9" t="b">
@@ -5923,7 +5761,7 @@
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>MR033</t>
+          <t>MR041</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
@@ -5933,25 +5771,25 @@
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
+          <t>Ausência de acompanhamento, revisão ou atualização periódica do plano de TIC.</t>
         </is>
       </c>
       <c r="D27" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>AV97</t>
+          <t>AV24 &amp; ~AV101</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>AV97</t>
+          <t>AV24</t>
         </is>
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as iniciativas de TI (projetos e ações) constantes do plano de TI alinham-se aos objetivos e iniciativas definidos no planejamento institucional (como PPA, planos estratégicos, planos setoriais e plano de governo, no caso de municípios), bem como, quando aplicável, às estratégias e diretrizes estabelecidas por instâncias superiores de governança (como a Estratégia Nacional de Tecnologia da Informação e Comunicação do Poder Judiciário - ENTIC-JUD, normas e orientações do SETIC/PRODERJ (para órgãos estaduais) ou instâncias de governança equivalentes no âmbito municipal)</t>
+          <t>No subitem e) do item 2102, não houve declaração afirmativa quanto à prática avaliada: é feito acompanhamento concomitante à execução do plano de TI, com vistas a assegurar sua observância e possibilitar a realização de ajustes que se fizerem necessário</t>
         </is>
       </c>
       <c r="H27" s="9" t="b">
@@ -5961,7 +5799,7 @@
     <row r="28" ht="45" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>MR034</t>
+          <t>MR042</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
@@ -5971,25 +5809,25 @@
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
+          <t>Ausência de acompanhamento, revisão ou atualização periódica do plano de TIC.</t>
         </is>
       </c>
       <c r="D28" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>AV20 &amp; ~AV98</t>
+          <t>AV101</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>AV20</t>
+          <t>AV101</t>
         </is>
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2102, não houve declaração afirmativa quanto à prática avaliada: o plano de TI fundamenta a proposta orçamentária da área de TI e o plano de contratações</t>
+          <t>No subitem e) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que é feito acompanhamento concomitante à execução do plano de TI, com vistas a assegurar sua observância e possibilitar a realização de ajustes que se fizerem necessário</t>
         </is>
       </c>
       <c r="H28" s="9" t="b">
@@ -5999,35 +5837,35 @@
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>MR035</t>
+          <t>MR043</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>PA03</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
+          <t>Ausência de força de trabalho dedicada à TIC.</t>
         </is>
       </c>
       <c r="D29" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>AV98</t>
+          <t>AV26 &amp; AV25</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>AV98</t>
+          <t>AV25</t>
         </is>
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o plano de TI fundamenta a proposta orçamentária da área de TI e o plano de contratações</t>
+          <t>Item 0105: embora a organização tenha declarado estrutura formal de TIC no item 0101, informou não possuir profissionais atuando regularmente em tecnologia da informação</t>
         </is>
       </c>
       <c r="H29" s="9" t="b">
@@ -6037,17 +5875,17 @@
     <row r="30" ht="45" customHeight="1">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>MR041</t>
+          <t>MR045</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>PA03</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>Ausência de acompanhamento, revisão ou atualização periódica do plano de TIC.</t>
+          <t>A organização não definiu o quantitativo necessário de pessoal de TIC e segurança da informação.</t>
         </is>
       </c>
       <c r="D30" s="9" t="n">
@@ -6055,17 +5893,17 @@
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>AV24 &amp; ~AV101</t>
+          <t>AV29 &amp; ~AV103</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>AV24</t>
+          <t>AV29</t>
         </is>
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2102, não houve declaração afirmativa quanto à prática avaliada: é feito acompanhamento concomitante à execução do plano de TI, com vistas a assegurar sua observância e possibilitar a realização de ajustes que se fizerem necessário</t>
+          <t>No subitem c) do item 2703, não houve declaração afirmativa quanto à prática avaliada: definiu-se, de maneira documentada, um quantitativo necessário de pessoal da área de tecnologia da informação e segurança da informação</t>
         </is>
       </c>
       <c r="H30" s="9" t="b">
@@ -6075,17 +5913,17 @@
     <row r="31" ht="45" customHeight="1">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>MR042</t>
+          <t>MR046</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>PA03</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>Ausência de acompanhamento, revisão ou atualização periódica do plano de TIC.</t>
+          <t>A organização não definiu o quantitativo necessário de pessoal de TIC e segurança da informação.</t>
         </is>
       </c>
       <c r="D31" s="9" t="n">
@@ -6093,17 +5931,17 @@
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>AV101</t>
+          <t>AV103</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>AV101</t>
+          <t>AV103</t>
         </is>
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que é feito acompanhamento concomitante à execução do plano de TI, com vistas a assegurar sua observância e possibilitar a realização de ajustes que se fizerem necessário</t>
+          <t>No subitem c) do item 2703, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu-se, de maneira documentada, um quantitativo necessário de pessoal da área de tecnologia da informação e segurança da informação</t>
         </is>
       </c>
       <c r="H31" s="9" t="b">
@@ -6113,7 +5951,7 @@
     <row r="32" ht="45" customHeight="1">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>MR043</t>
+          <t>MR047</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
@@ -6123,7 +5961,7 @@
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Ausência de força de trabalho dedicada à TIC.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="D32" s="9" t="n">
@@ -6131,17 +5969,17 @@
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>AV26 &amp; AV25</t>
+          <t>AV31 &amp; ~AV105</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>AV25</t>
+          <t>AV31</t>
         </is>
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t>Item 0105: embora a organização tenha declarado estrutura formal de TIC no item 0101, informou não possuir profissionais atuando regularmente em tecnologia da informação</t>
+          <t>No subitem b) do item 2708, não houve declaração afirmativa quanto à prática avaliada: possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
         </is>
       </c>
       <c r="H32" s="9" t="b">
@@ -6151,7 +5989,7 @@
     <row r="33" ht="45" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>MR045</t>
+          <t>MR048</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
@@ -6161,25 +5999,25 @@
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>A organização não definiu o quantitativo necessário de pessoal de TIC e segurança da informação.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="D33" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>AV29 &amp; ~AV103</t>
+          <t>AV105</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>AV29</t>
+          <t>AV105</t>
         </is>
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2703, não houve declaração afirmativa quanto à prática avaliada: definiu-se, de maneira documentada, um quantitativo necessário de pessoal da área de tecnologia da informação e segurança da informação</t>
+          <t>No subitem b) do item 2708, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
         </is>
       </c>
       <c r="H33" s="9" t="b">
@@ -6189,7 +6027,7 @@
     <row r="34" ht="45" customHeight="1">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>MR046</t>
+          <t>MR049</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
@@ -6199,25 +6037,25 @@
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>A organização não definiu o quantitativo necessário de pessoal de TIC e segurança da informação.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="D34" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>AV103</t>
+          <t>AV33 &amp; ~AV107</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>AV103</t>
+          <t>AV33</t>
         </is>
       </c>
       <c r="G34" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2703, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu-se, de maneira documentada, um quantitativo necessário de pessoal da área de tecnologia da informação e segurança da informação</t>
+          <t>No subitem d) do item 2708, não houve declaração afirmativa quanto à prática avaliada: possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
         </is>
       </c>
       <c r="H34" s="9" t="b">
@@ -6227,7 +6065,7 @@
     <row r="35" ht="90" customHeight="1">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>MR047</t>
+          <t>MR050</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
@@ -6241,21 +6079,21 @@
         </is>
       </c>
       <c r="D35" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>AV31 &amp; ~AV105</t>
+          <t>AV107</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>AV31</t>
+          <t>AV107</t>
         </is>
       </c>
       <c r="G35" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2708, não houve declaração afirmativa quanto à prática avaliada: possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
+          <t>No subitem d) do item 2708, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
         </is>
       </c>
       <c r="H35" s="9" t="b">
@@ -6265,7 +6103,7 @@
     <row r="36" ht="105" customHeight="1">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>MR048</t>
+          <t>MR062</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
@@ -6275,25 +6113,25 @@
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Dependência externa relevante sem capacidade interna suficiente para coordenar e fiscalizar a TIC.</t>
         </is>
       </c>
       <c r="D36" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>AV105</t>
+          <t>AV45 &amp; AV46</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>AV105</t>
+          <t>AV45</t>
         </is>
       </c>
       <c r="G36" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2708, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
+          <t>A organização informou modelo de operação de TIC com execução predominantemente terceirizada, o que levou à análise de sua capacidade interna de coordenação e fiscalização</t>
         </is>
       </c>
       <c r="H36" s="9" t="b">
@@ -6303,7 +6141,7 @@
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>MR049</t>
+          <t>MR063</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
@@ -6313,25 +6151,25 @@
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Dependência externa relevante sem capacidade interna suficiente para coordenar e fiscalizar a TIC.</t>
         </is>
       </c>
       <c r="D37" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>AV33 &amp; ~AV107</t>
+          <t>AV45 &amp; AV46</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>AV33</t>
+          <t>AV46</t>
         </is>
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2708, não houve declaração afirmativa quanto à prática avaliada: possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
+          <t>Não foram identificados profissionais internos de TIC para coordenar e fiscalizar a execução das atividades de tecnologia da informação</t>
         </is>
       </c>
       <c r="H37" s="9" t="b">
@@ -6341,35 +6179,35 @@
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>MR050</t>
+          <t>MR065</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA05</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D38" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>AV107</t>
+          <t>AV54 &amp; ~AV124</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>AV107</t>
+          <t>AV54</t>
         </is>
       </c>
       <c r="G38" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2708, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
+          <t>No subitem a) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
         </is>
       </c>
       <c r="H38" s="9" t="b">
@@ -6379,35 +6217,35 @@
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>MR062</t>
+          <t>MR066</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA05</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>Dependência externa relevante sem capacidade interna suficiente para coordenar e fiscalizar a TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D39" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>AV45 &amp; AV46</t>
+          <t>AV124</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>AV45</t>
+          <t>AV124</t>
         </is>
       </c>
       <c r="G39" s="9" t="inlineStr">
         <is>
-          <t>A organização informou modelo de operação de TIC com execução predominantemente terceirizada, o que levou à análise de sua capacidade interna de coordenação e fiscalização</t>
+          <t>No subitem a) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
         </is>
       </c>
       <c r="H39" s="9" t="b">
@@ -6417,35 +6255,35 @@
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>MR063</t>
+          <t>MR067</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA05</t>
         </is>
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>Dependência externa relevante sem capacidade interna suficiente para coordenar e fiscalizar a TIC.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="D40" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>AV45 &amp; AV46</t>
+          <t>AV55 &amp; ~AV125</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>AV46</t>
+          <t>AV55</t>
         </is>
       </c>
       <c r="G40" s="9" t="inlineStr">
         <is>
-          <t>Não foram identificados profissionais internos de TIC para coordenar e fiscalizar a execução das atividades de tecnologia da informação</t>
+          <t>No subitem b) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
         </is>
       </c>
       <c r="H40" s="9" t="b">
@@ -6455,7 +6293,7 @@
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>MR065</t>
+          <t>MR068</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
@@ -6465,25 +6303,25 @@
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="D41" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>AV54 &amp; ~AV124</t>
+          <t>AV125</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>AV54</t>
+          <t>AV125</t>
         </is>
       </c>
       <c r="G41" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
+          <t>No subitem b) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
         </is>
       </c>
       <c r="H41" s="9" t="b">
@@ -6493,7 +6331,7 @@
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>MR066</t>
+          <t>MR069</t>
         </is>
       </c>
       <c r="B42" s="9" t="inlineStr">
@@ -6503,7 +6341,7 @@
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="D42" s="9" t="n">
@@ -6511,17 +6349,17 @@
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>AV124</t>
+          <t>AV56 &amp; ~AV126</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>AV124</t>
+          <t>AV56</t>
         </is>
       </c>
       <c r="G42" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
+          <t>No subitem c) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
         </is>
       </c>
       <c r="H42" s="9" t="b">
@@ -6531,7 +6369,7 @@
     <row r="43" ht="45" customHeight="1">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>MR067</t>
+          <t>MR070</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
@@ -6545,21 +6383,21 @@
         </is>
       </c>
       <c r="D43" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>AV55 &amp; ~AV125</t>
+          <t>AV126</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>AV55</t>
+          <t>AV126</t>
         </is>
       </c>
       <c r="G43" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
+          <t>No subitem c) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
         </is>
       </c>
       <c r="H43" s="9" t="b">
@@ -6569,7 +6407,7 @@
     <row r="44" ht="45" customHeight="1">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>MR068</t>
+          <t>MR071</t>
         </is>
       </c>
       <c r="B44" s="9" t="inlineStr">
@@ -6579,7 +6417,7 @@
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D44" s="9" t="n">
@@ -6587,17 +6425,17 @@
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>AV125</t>
+          <t>AV57 &amp; ~AV127</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>AV125</t>
+          <t>AV57</t>
         </is>
       </c>
       <c r="G44" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
+          <t>No subitem d) do item 2201, não houve declaração afirmativa quanto à prática avaliada: são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
         </is>
       </c>
       <c r="H44" s="9" t="b">
@@ -6607,7 +6445,7 @@
     <row r="45" ht="45" customHeight="1">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>MR069</t>
+          <t>MR072</t>
         </is>
       </c>
       <c r="B45" s="9" t="inlineStr">
@@ -6617,25 +6455,25 @@
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D45" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>AV56 &amp; ~AV126</t>
+          <t>AV127</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>AV56</t>
+          <t>AV127</t>
         </is>
       </c>
       <c r="G45" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
+          <t>No subitem d) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
         </is>
       </c>
       <c r="H45" s="9" t="b">
@@ -6645,7 +6483,7 @@
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>MR070</t>
+          <t>MR073</t>
         </is>
       </c>
       <c r="B46" s="9" t="inlineStr">
@@ -6655,25 +6493,25 @@
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D46" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>AV126</t>
+          <t>AV58 &amp; ~AV128</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>AV126</t>
+          <t>AV58</t>
         </is>
       </c>
       <c r="G46" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
+          <t>No subitem e) do item 2201, não houve declaração afirmativa quanto à prática avaliada: a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
         </is>
       </c>
       <c r="H46" s="9" t="b">
@@ -6683,7 +6521,7 @@
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>MR071</t>
+          <t>MR074</t>
         </is>
       </c>
       <c r="B47" s="9" t="inlineStr">
@@ -6697,21 +6535,21 @@
         </is>
       </c>
       <c r="D47" s="9" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>AV57 &amp; ~AV127</t>
+          <t>AV128</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>AV57</t>
+          <t>AV128</t>
         </is>
       </c>
       <c r="G47" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2201, não houve declaração afirmativa quanto à prática avaliada: são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
+          <t>No subitem e) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
         </is>
       </c>
       <c r="H47" s="9" t="b">
@@ -6721,7 +6559,7 @@
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>MR072</t>
+          <t>MR075</t>
         </is>
       </c>
       <c r="B48" s="9" t="inlineStr">
@@ -6731,25 +6569,25 @@
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="D48" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>AV127</t>
+          <t>AV59 &amp; ~AV129</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>AV127</t>
+          <t>AV59</t>
         </is>
       </c>
       <c r="G48" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
+          <t>No subitem a) do item 2203, não houve declaração afirmativa quanto à prática avaliada: mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
         </is>
       </c>
       <c r="H48" s="9" t="b">
@@ -6759,7 +6597,7 @@
     <row r="49" ht="45" customHeight="1">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>MR073</t>
+          <t>MR076</t>
         </is>
       </c>
       <c r="B49" s="9" t="inlineStr">
@@ -6769,25 +6607,25 @@
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="D49" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>AV58 &amp; ~AV128</t>
+          <t>AV129</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>AV58</t>
+          <t>AV129</t>
         </is>
       </c>
       <c r="G49" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2201, não houve declaração afirmativa quanto à prática avaliada: a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
+          <t>No subitem a) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
         </is>
       </c>
       <c r="H49" s="9" t="b">
@@ -6797,7 +6635,7 @@
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>MR074</t>
+          <t>MR077</t>
         </is>
       </c>
       <c r="B50" s="9" t="inlineStr">
@@ -6807,25 +6645,25 @@
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="D50" s="9" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>AV128</t>
+          <t>AV62 &amp; ~AV132</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>AV128</t>
+          <t>AV62</t>
         </is>
       </c>
       <c r="G50" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
+          <t>No subitem a) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H50" s="9" t="b">
@@ -6835,7 +6673,7 @@
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>MR075</t>
+          <t>MR078</t>
         </is>
       </c>
       <c r="B51" s="9" t="inlineStr">
@@ -6849,21 +6687,21 @@
         </is>
       </c>
       <c r="D51" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>AV59 &amp; ~AV129</t>
+          <t>AV132</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>AV59</t>
+          <t>AV132</t>
         </is>
       </c>
       <c r="G51" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2203, não houve declaração afirmativa quanto à prática avaliada: mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
+          <t>No subitem a) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H51" s="9" t="b">
@@ -6873,7 +6711,7 @@
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="9" t="inlineStr">
         <is>
-          <t>MR076</t>
+          <t>MR079</t>
         </is>
       </c>
       <c r="B52" s="9" t="inlineStr">
@@ -6887,21 +6725,21 @@
         </is>
       </c>
       <c r="D52" s="9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>AV129</t>
+          <t>AV63 &amp; ~AV133</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>AV129</t>
+          <t>AV63</t>
         </is>
       </c>
       <c r="G52" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
+          <t>No subitem b) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H52" s="9" t="b">
@@ -6911,7 +6749,7 @@
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>MR077</t>
+          <t>MR080</t>
         </is>
       </c>
       <c r="B53" s="9" t="inlineStr">
@@ -6925,21 +6763,21 @@
         </is>
       </c>
       <c r="D53" s="9" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>AV62 &amp; ~AV132</t>
+          <t>AV133</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>AV62</t>
+          <t>AV133</t>
         </is>
       </c>
       <c r="G53" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
+          <t>No subitem b) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H53" s="9" t="b">
@@ -6949,7 +6787,7 @@
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t>MR078</t>
+          <t>MR083</t>
         </is>
       </c>
       <c r="B54" s="9" t="inlineStr">
@@ -6959,25 +6797,25 @@
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="D54" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>AV132</t>
+          <t>AV66 &amp; ~AV136</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>AV132</t>
+          <t>AV66</t>
         </is>
       </c>
       <c r="G54" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
+          <t>No subitem c) do item 2203, não houve declaração afirmativa quanto à prática avaliada: o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H54" s="9" t="b">
@@ -6987,7 +6825,7 @@
     <row r="55" ht="45" customHeight="1">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>MR079</t>
+          <t>MR084</t>
         </is>
       </c>
       <c r="B55" s="9" t="inlineStr">
@@ -6997,25 +6835,25 @@
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="D55" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>AV63 &amp; ~AV133</t>
+          <t>AV136</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>AV63</t>
+          <t>AV136</t>
         </is>
       </c>
       <c r="G55" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
+          <t>No subitem c) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H55" s="9" t="b">
@@ -7025,7 +6863,7 @@
     <row r="56" ht="45" customHeight="1">
       <c r="A56" s="9" t="inlineStr">
         <is>
-          <t>MR080</t>
+          <t>MR085</t>
         </is>
       </c>
       <c r="B56" s="9" t="inlineStr">
@@ -7035,25 +6873,25 @@
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="D56" s="9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>AV133</t>
+          <t>AV67 &amp; ~AV137</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>AV133</t>
+          <t>AV67</t>
         </is>
       </c>
       <c r="G56" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
+          <t>No subitem a) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu regras para a priorização e o escalamento de incidentes</t>
         </is>
       </c>
       <c r="H56" s="9" t="b">
@@ -7063,7 +6901,7 @@
     <row r="57" ht="45" customHeight="1">
       <c r="A57" s="9" t="inlineStr">
         <is>
-          <t>MR083</t>
+          <t>MR086</t>
         </is>
       </c>
       <c r="B57" s="9" t="inlineStr">
@@ -7073,25 +6911,25 @@
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="D57" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>AV66 &amp; ~AV136</t>
+          <t>AV137</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>AV66</t>
+          <t>AV137</t>
         </is>
       </c>
       <c r="G57" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2203, não houve declaração afirmativa quanto à prática avaliada: o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem a) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu regras para a priorização e o escalamento de incidentes</t>
         </is>
       </c>
       <c r="H57" s="9" t="b">
@@ -7101,7 +6939,7 @@
     <row r="58" ht="45" customHeight="1">
       <c r="A58" s="9" t="inlineStr">
         <is>
-          <t>MR084</t>
+          <t>MR087</t>
         </is>
       </c>
       <c r="B58" s="9" t="inlineStr">
@@ -7111,25 +6949,25 @@
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="D58" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>AV136</t>
+          <t>AV70 &amp; ~AV140</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>AV136</t>
+          <t>AV70</t>
         </is>
       </c>
       <c r="G58" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem d) do item 2204, não houve declaração afirmativa quanto à prática avaliada: o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H58" s="9" t="b">
@@ -7139,7 +6977,7 @@
     <row r="59" ht="45" customHeight="1">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>MR085</t>
+          <t>MR088</t>
         </is>
       </c>
       <c r="B59" s="9" t="inlineStr">
@@ -7153,21 +6991,21 @@
         </is>
       </c>
       <c r="D59" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>AV67 &amp; ~AV137</t>
+          <t>AV140</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>AV67</t>
+          <t>AV140</t>
         </is>
       </c>
       <c r="G59" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu regras para a priorização e o escalamento de incidentes</t>
+          <t>No subitem d) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H59" s="9" t="b">
@@ -7177,7 +7015,7 @@
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="9" t="inlineStr">
         <is>
-          <t>MR086</t>
+          <t>MR089</t>
         </is>
       </c>
       <c r="B60" s="9" t="inlineStr">
@@ -7191,21 +7029,21 @@
         </is>
       </c>
       <c r="D60" s="9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>AV137</t>
+          <t>AV71 &amp; ~AV141</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>AV137</t>
+          <t>AV71</t>
         </is>
       </c>
       <c r="G60" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu regras para a priorização e o escalamento de incidentes</t>
+          <t>No subitem e) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
         </is>
       </c>
       <c r="H60" s="9" t="b">
@@ -7215,7 +7053,7 @@
     <row r="61" ht="45" customHeight="1">
       <c r="A61" s="9" t="inlineStr">
         <is>
-          <t>MR087</t>
+          <t>MR090</t>
         </is>
       </c>
       <c r="B61" s="9" t="inlineStr">
@@ -7229,21 +7067,21 @@
         </is>
       </c>
       <c r="D61" s="9" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>AV70 &amp; ~AV140</t>
+          <t>AV141</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>AV70</t>
+          <t>AV141</t>
         </is>
       </c>
       <c r="G61" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2204, não houve declaração afirmativa quanto à prática avaliada: o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem e) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
         </is>
       </c>
       <c r="H61" s="9" t="b">
@@ -7253,35 +7091,35 @@
     <row r="62" ht="45" customHeight="1">
       <c r="A62" s="9" t="inlineStr">
         <is>
-          <t>MR088</t>
+          <t>MR091</t>
         </is>
       </c>
       <c r="B62" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C62" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D62" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>AV140</t>
+          <t>AV73 &amp; ~AV143</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>AV140</t>
+          <t>AV73</t>
         </is>
       </c>
       <c r="G62" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem a) do item 2801, não houve declaração afirmativa quanto à prática avaliada: o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
         </is>
       </c>
       <c r="H62" s="9" t="b">
@@ -7291,35 +7129,35 @@
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>MR089</t>
+          <t>MR092</t>
         </is>
       </c>
       <c r="B63" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C63" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D63" s="9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>AV71 &amp; ~AV141</t>
+          <t>AV143</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>AV71</t>
+          <t>AV143</t>
         </is>
       </c>
       <c r="G63" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
+          <t>No subitem a) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
         </is>
       </c>
       <c r="H63" s="9" t="b">
@@ -7329,35 +7167,35 @@
     <row r="64" ht="45" customHeight="1">
       <c r="A64" s="9" t="inlineStr">
         <is>
-          <t>MR090</t>
+          <t>MR101</t>
         </is>
       </c>
       <c r="B64" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
         </is>
       </c>
       <c r="D64" s="9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>AV141</t>
+          <t>AV78 &amp; ~AV148</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>AV141</t>
+          <t>AV78</t>
         </is>
       </c>
       <c r="G64" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
+          <t>No subitem a) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
         </is>
       </c>
       <c r="H64" s="9" t="b">
@@ -7367,7 +7205,7 @@
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="9" t="inlineStr">
         <is>
-          <t>MR091</t>
+          <t>MR102</t>
         </is>
       </c>
       <c r="B65" s="9" t="inlineStr">
@@ -7377,25 +7215,25 @@
       </c>
       <c r="C65" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
         </is>
       </c>
       <c r="D65" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>AV73 &amp; ~AV143</t>
+          <t>AV148</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>AV73</t>
+          <t>AV148</t>
         </is>
       </c>
       <c r="G65" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2801, não houve declaração afirmativa quanto à prática avaliada: o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
+          <t>No subitem a) do item 2804, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
         </is>
       </c>
       <c r="H65" s="9" t="b">
@@ -7405,7 +7243,7 @@
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="9" t="inlineStr">
         <is>
-          <t>MR092</t>
+          <t>MR105</t>
         </is>
       </c>
       <c r="B66" s="9" t="inlineStr">
@@ -7415,25 +7253,25 @@
       </c>
       <c r="C66" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
         </is>
       </c>
       <c r="D66" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>AV143</t>
+          <t>AV80 &amp; ~AV150</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>AV143</t>
+          <t>AV80</t>
         </is>
       </c>
       <c r="G66" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
+          <t>No subitem c) do item 2802, não houve declaração afirmativa quanto à prática avaliada: na elaboração do PCA são considerados os demais instrumentos de planejamento da organização</t>
         </is>
       </c>
       <c r="H66" s="9" t="b">
@@ -7443,7 +7281,7 @@
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="9" t="inlineStr">
         <is>
-          <t>MR101</t>
+          <t>MR106</t>
         </is>
       </c>
       <c r="B67" s="9" t="inlineStr">
@@ -7453,25 +7291,25 @@
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
         </is>
       </c>
       <c r="D67" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>AV78 &amp; ~AV148</t>
+          <t>AV150</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>AV78</t>
+          <t>AV150</t>
         </is>
       </c>
       <c r="G67" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
+          <t>No subitem c) do item 2802, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que na elaboração do PCA são considerados os demais instrumentos de planejamento da organização</t>
         </is>
       </c>
       <c r="H67" s="9" t="b">
@@ -7481,7 +7319,7 @@
     <row r="68" ht="45" customHeight="1">
       <c r="A68" s="9" t="inlineStr">
         <is>
-          <t>MR102</t>
+          <t>MR109</t>
         </is>
       </c>
       <c r="B68" s="9" t="inlineStr">
@@ -7491,25 +7329,25 @@
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
         </is>
       </c>
       <c r="D68" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>AV148</t>
+          <t>AV82</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>AV148</t>
+          <t>AV82</t>
         </is>
       </c>
       <c r="G68" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2804, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
+          <t>No subitem b) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de TI executadas no exercício encontram-se previamente estabelecidas nos instrumentos de planejamento vigentes (PDTI/PEDTIC e PCA)</t>
         </is>
       </c>
       <c r="H68" s="9" t="b">
@@ -7519,7 +7357,7 @@
     <row r="69" ht="60" customHeight="1">
       <c r="A69" s="9" t="inlineStr">
         <is>
-          <t>MR105</t>
+          <t>MR110</t>
         </is>
       </c>
       <c r="B69" s="9" t="inlineStr">
@@ -7529,7 +7367,7 @@
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
+          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
         </is>
       </c>
       <c r="D69" s="9" t="n">
@@ -7537,17 +7375,17 @@
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>AV80 &amp; ~AV150</t>
+          <t>AV83</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>AV80</t>
+          <t>AV83</t>
         </is>
       </c>
       <c r="G69" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2802, não houve declaração afirmativa quanto à prática avaliada: na elaboração do PCA são considerados os demais instrumentos de planejamento da organização</t>
+          <t>No subitem c) do item 2804, não houve declaração afirmativa quanto à prática avaliada: a fase de planejamento de cada contratação de TI é conduzida por uma Equipe de Planejamento da Contratação formalmente designada (composta, minimamente, por integrante requisitante e integrante técnico da área de TI)</t>
         </is>
       </c>
       <c r="H69" s="9" t="b">
@@ -7557,7 +7395,7 @@
     <row r="70" ht="45" customHeight="1">
       <c r="A70" s="9" t="inlineStr">
         <is>
-          <t>MR106</t>
+          <t>MR111</t>
         </is>
       </c>
       <c r="B70" s="9" t="inlineStr">
@@ -7567,7 +7405,7 @@
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D70" s="9" t="n">
@@ -7575,17 +7413,17 @@
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>AV150</t>
+          <t>AV152 &amp; ~AV153</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>AV150</t>
+          <t>AV152</t>
         </is>
       </c>
       <c r="G70" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2802, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que na elaboração do PCA são considerados os demais instrumentos de planejamento da organização</t>
+          <t>No subitem b) do item 2801, não houve declaração afirmativa quanto à prática avaliada: são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
         </is>
       </c>
       <c r="H70" s="9" t="b">
@@ -7595,7 +7433,7 @@
     <row r="71" ht="45" customHeight="1">
       <c r="A71" s="9" t="inlineStr">
         <is>
-          <t>MR109</t>
+          <t>MR112</t>
         </is>
       </c>
       <c r="B71" s="9" t="inlineStr">
@@ -7605,145 +7443,34 @@
       </c>
       <c r="C71" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D71" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>AV82</t>
+          <t>AV153</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>AV82</t>
+          <t>AV153</t>
         </is>
       </c>
       <c r="G71" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de TI executadas no exercício encontram-se previamente estabelecidas nos instrumentos de planejamento vigentes (PDTI/PEDTIC e PCA)</t>
+          <t>No subitem b) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
         </is>
       </c>
       <c r="H71" s="9" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="72" ht="30" customHeight="1">
-      <c r="A72" s="9" t="inlineStr">
-        <is>
-          <t>MR110</t>
-        </is>
-      </c>
-      <c r="B72" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C72" s="9" t="inlineStr">
-        <is>
-          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
-        </is>
-      </c>
-      <c r="D72" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E72" s="9" t="inlineStr">
-        <is>
-          <t>AV83</t>
-        </is>
-      </c>
-      <c r="F72" s="9" t="inlineStr">
-        <is>
-          <t>AV83</t>
-        </is>
-      </c>
-      <c r="G72" s="9" t="inlineStr">
-        <is>
-          <t>No subitem c) do item 2804, não houve declaração afirmativa quanto à prática avaliada: a fase de planejamento de cada contratação de TI é conduzida por uma Equipe de Planejamento da Contratação formalmente designada (composta, minimamente, por integrante requisitante e integrante técnico da área de TI)</t>
-        </is>
-      </c>
-      <c r="H72" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="73" ht="30" customHeight="1">
-      <c r="A73" s="9" t="inlineStr">
-        <is>
-          <t>MR111</t>
-        </is>
-      </c>
-      <c r="B73" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C73" s="9" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="D73" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E73" s="9" t="inlineStr">
-        <is>
-          <t>AV152 &amp; ~AV153</t>
-        </is>
-      </c>
-      <c r="F73" s="9" t="inlineStr">
-        <is>
-          <t>AV152</t>
-        </is>
-      </c>
-      <c r="G73" s="9" t="inlineStr">
-        <is>
-          <t>No subitem b) do item 2801, não houve declaração afirmativa quanto à prática avaliada: são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
-        </is>
-      </c>
-      <c r="H73" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="74" ht="30" customHeight="1">
-      <c r="A74" s="9" t="inlineStr">
-        <is>
-          <t>MR112</t>
-        </is>
-      </c>
-      <c r="B74" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C74" s="9" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="D74" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="E74" s="9" t="inlineStr">
-        <is>
-          <t>AV153</t>
-        </is>
-      </c>
-      <c r="F74" s="9" t="inlineStr">
-        <is>
-          <t>AV153</t>
-        </is>
-      </c>
-      <c r="G74" s="9" t="inlineStr">
-        <is>
-          <t>No subitem b) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
-        </is>
-      </c>
-      <c r="H74" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
+    <row r="72" ht="30" customHeight="1"/>
+    <row r="73" ht="30" customHeight="1"/>
+    <row r="74" ht="30" customHeight="1"/>
     <row r="75" ht="45" customHeight="1"/>
     <row r="76" ht="30" customHeight="1"/>
     <row r="77" ht="45" customHeight="1"/>
@@ -7784,7 +7511,7 @@
     <row r="112" ht="45" customHeight="1"/>
     <row r="113" ht="45" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A3:H74"/>
+  <autoFilter ref="A3:H71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Revisa a Questão 3 da matriz e do mapa
</commit_message>
<xml_diff>
--- a/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
+++ b/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
@@ -15,9 +15,9 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Fontes de Informação'!$A$3:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Procedimentos de Auditoria'!$A$3:$E$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ações de Verificação'!$A$3:$P$72</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Motivos do Relatório'!$A$3:$H$71</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Variáveis Temporárias'!$A$3:$E$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ações de Verificação'!$A$3:$P$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Motivos do Relatório'!$A$3:$H$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Variáveis Temporárias'!$A$3:$E$6</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
@@ -599,7 +599,7 @@
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>(((AV17 | AV95) | ((AV14 | AV92) | (AV15 | AV93))) | (AV18 | AV96) | (AV19 | AV97) | (AV20 | AV98) | (AV24 | AV101))</t>
+          <t>((AV14 | AV15 | AV17 | AV154) | (AV155 &amp; (AV18 | AV19 | AV20 | AV24)))</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
@@ -699,7 +699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P72"/>
+  <dimension ref="A1:P67"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1460,7 +1460,7 @@
         <is>
           <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
 Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H14" s="1" t="inlineStr">
@@ -1471,7 +1471,7 @@
       <c r="I14" s="1" t="n"/>
       <c r="J14" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="K14" s="1" t="inlineStr">
@@ -1489,7 +1489,7 @@
       <c r="O14" s="1" t="n"/>
       <c r="P14" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1516,7 @@
         <is>
           <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
 Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H15" s="1" t="inlineStr">
@@ -1527,7 +1527,7 @@
       <c r="I15" s="1" t="n"/>
       <c r="J15" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="K15" s="1" t="inlineStr">
@@ -1545,7 +1545,7 @@
       <c r="O15" s="1" t="n"/>
       <c r="P15" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
@@ -1572,7 +1572,7 @@
         <is>
           <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
 Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H16" s="1" t="inlineStr">
@@ -1583,7 +1583,7 @@
       <c r="I16" s="1" t="n"/>
       <c r="J16" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="K16" s="1" t="inlineStr">
@@ -1601,7 +1601,7 @@
       <c r="O16" s="1" t="n"/>
       <c r="P16" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
@@ -1627,7 +1627,7 @@
       <c r="G17" s="1" t="inlineStr">
         <is>
           <t>Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H17" s="1" t="inlineStr">
@@ -1683,7 +1683,7 @@
         <is>
           <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
 Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H18" s="1" t="inlineStr">
@@ -1738,8 +1738,7 @@
       <c r="G19" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO06.03 - Criar e manter orçamentos: elaborar e manter orçamento de TIC alinhado ao portfólio, ao planejamento e às prioridades aprovadas.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.
-Lei nº 14.133/2021, art. 12, inciso VII e § 1º - Planejamento das contratações: o Plano de Contratações Anual, quando elaborado, deve alinhar-se ao planejamento estratégico, subsidiar a elaboração das leis orçamentárias e ser observado nas licitações e na execução contratual.</t>
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H19" s="1" t="inlineStr">
@@ -1793,7 +1792,7 @@
       </c>
       <c r="G20" s="1" t="inlineStr">
         <is>
-          <t>Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
+          <t>Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H20" s="1" t="inlineStr">
@@ -1804,7 +1803,7 @@
       <c r="I20" s="1" t="n"/>
       <c r="J20" s="1" t="inlineStr">
         <is>
-          <t>Ausência de acompanhamento, revisão ou atualização periódica do plano de TIC.</t>
+          <t>Ausência de acompanhamento da execução do plano de TIC.</t>
         </is>
       </c>
       <c r="K20" s="1" t="inlineStr">
@@ -1822,7 +1821,7 @@
       <c r="O20" s="1" t="n"/>
       <c r="P20" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e execute rotina periódica de acompanhamento, revisão e atualização do plano de TIC, registrando execução, pendências, reprogramações e deliberações</t>
+          <t>estabeleça e execute rotina periódica de acompanhamento da execução do plano de TIC, promovendo sua revisão periódica e os ajustes ou atualizações necessários, com registro das principais decisões e reprogramações</t>
         </is>
       </c>
     </row>
@@ -3205,7 +3204,7 @@
     <row r="46" ht="113.45" customHeight="1">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>AV92</t>
+          <t>AV103</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -3218,14 +3217,13 @@
       <c r="E46" s="1" t="n"/>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>q2101ext[A]</t>
+          <t>q2703ext[C]</t>
         </is>
       </c>
       <c r="G46" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
+          <t>COBIT 2019, APO07.05 - Planejar e monitorar o uso de recursos humanos de TI e de negócio: planejar, alocar e acompanhar capacidade de pessoal para iniciativas, operações e serviços de TIC.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6.5 - O PDTI deve contemplar o quantitativo necessário ou ideal para a força de trabalho em TI.</t>
         </is>
       </c>
       <c r="H46" s="1" t="inlineStr">
@@ -3236,7 +3234,7 @@
       <c r="I46" s="1" t="n"/>
       <c r="J46" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
+          <t>A organização não definiu o quantitativo necessário de pessoal de TIC e segurança da informação.</t>
         </is>
       </c>
       <c r="K46" s="1" t="inlineStr">
@@ -3248,20 +3246,20 @@
       <c r="M46" s="1" t="n"/>
       <c r="N46" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O46" s="1" t="n"/>
       <c r="P46" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>estime e mantenha atualizado o quantitativo necessário de pessoal de TIC e segurança da informação, considerando o porte e a complexidade da organização, os serviços críticos, os sistemas mantidos, as contratações vigentes e os riscos relevantes</t>
         </is>
       </c>
     </row>
     <row r="47" ht="113.45" customHeight="1">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>AV93</t>
+          <t>AV105</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -3274,14 +3272,13 @@
       <c r="E47" s="1" t="n"/>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>q2101ext[B]</t>
+          <t>q2708[B]</t>
         </is>
       </c>
       <c r="G47" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
+          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
+COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
         </is>
       </c>
       <c r="H47" s="1" t="inlineStr">
@@ -3292,7 +3289,7 @@
       <c r="I47" s="1" t="n"/>
       <c r="J47" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="K47" s="1" t="inlineStr">
@@ -3304,20 +3301,20 @@
       <c r="M47" s="1" t="n"/>
       <c r="N47" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O47" s="1" t="n"/>
       <c r="P47" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
         </is>
       </c>
     </row>
     <row r="48" ht="113.45" customHeight="1">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>AV95</t>
+          <t>AV107</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -3330,14 +3327,13 @@
       <c r="E48" s="1" t="n"/>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>q2101ext[D]</t>
+          <t>q2708[D]</t>
         </is>
       </c>
       <c r="G48" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
+          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
+COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
         </is>
       </c>
       <c r="H48" s="1" t="inlineStr">
@@ -3348,7 +3344,7 @@
       <c r="I48" s="1" t="n"/>
       <c r="J48" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="K48" s="1" t="inlineStr">
@@ -3360,20 +3356,20 @@
       <c r="M48" s="1" t="n"/>
       <c r="N48" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O48" s="1" t="n"/>
       <c r="P48" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a maturidade da organização, atentando-se, minimamente, em definir etapas, responsáveis, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
         </is>
       </c>
     </row>
     <row r="49" ht="113.45" customHeight="1">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>AV96</t>
+          <t>AV124</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -3386,13 +3382,13 @@
       <c r="E49" s="1" t="n"/>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>q2102ext[A]</t>
+          <t>q2201ext[A]</t>
         </is>
       </c>
       <c r="G49" s="1" t="inlineStr">
         <is>
-          <t>Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
+          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
+ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.</t>
         </is>
       </c>
       <c r="H49" s="1" t="inlineStr">
@@ -3403,7 +3399,7 @@
       <c r="I49" s="1" t="n"/>
       <c r="J49" s="1" t="inlineStr">
         <is>
-          <t>Ausência de aprovação formal do plano de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="K49" s="1" t="inlineStr">
@@ -3415,20 +3411,20 @@
       <c r="M49" s="1" t="n"/>
       <c r="N49" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O49" s="1" t="n"/>
       <c r="P49" s="1" t="inlineStr">
         <is>
-          <t>submeta o plano de TIC à aprovação formal do dirigente máximo ou de instância competente da alta administração, mantendo registro do respectivo ato de aprovação</t>
+          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
         </is>
       </c>
     </row>
     <row r="50" ht="113.45" customHeight="1">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>AV97</t>
+          <t>AV125</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -3441,14 +3437,13 @@
       <c r="E50" s="1" t="n"/>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>q2102ext[D]</t>
+          <t>q2201ext[B]</t>
         </is>
       </c>
       <c r="G50" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
+          <t>ITIL 4, prática de gerenciamento do catálogo de serviços: manter fonte única de informações consistentes sobre serviços e ofertas de serviço, disponível para usuários e equipes de suporte.
+COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.</t>
         </is>
       </c>
       <c r="H50" s="1" t="inlineStr">
@@ -3459,7 +3454,7 @@
       <c r="I50" s="1" t="n"/>
       <c r="J50" s="1" t="inlineStr">
         <is>
-          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="K50" s="1" t="inlineStr">
@@ -3471,20 +3466,20 @@
       <c r="M50" s="1" t="n"/>
       <c r="N50" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O50" s="1" t="n"/>
       <c r="P50" s="1" t="inlineStr">
         <is>
-          <t>revise o plano de TIC para explicitar seu alinhamento ao planejamento institucional, às diretrizes superiores e às necessidades das áreas finalísticas e administrativas, relacionando objetivos, iniciativas, indicadores e metas de TIC aos resultados institucionais pretendidos</t>
+          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
         </is>
       </c>
     </row>
     <row r="51" ht="113.45" customHeight="1">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>AV98</t>
+          <t>AV126</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -3497,14 +3492,13 @@
       <c r="E51" s="1" t="n"/>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>q2102ext[C]</t>
+          <t>q2201ext[C]</t>
         </is>
       </c>
       <c r="G51" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO06.03 - Criar e manter orçamentos: elaborar e manter orçamento de TIC alinhado ao portfólio, ao planejamento e às prioridades aprovadas.
-Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.
-Lei nº 14.133/2021, art. 12, inciso VII e § 1º - Planejamento das contratações: o Plano de Contratações Anual, quando elaborado, deve alinhar-se ao planejamento estratégico, subsidiar a elaboração das leis orçamentárias e ser observado nas licitações e na execução contratual.</t>
+          <t>ITIL 4, prática de gerenciamento do catálogo de serviços: manter fonte única de informações consistentes sobre serviços e ofertas de serviço, disponível para usuários e equipes de suporte.
+COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.</t>
         </is>
       </c>
       <c r="H51" s="1" t="inlineStr">
@@ -3515,7 +3509,7 @@
       <c r="I51" s="1" t="n"/>
       <c r="J51" s="1" t="inlineStr">
         <is>
-          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="K51" s="1" t="inlineStr">
@@ -3527,20 +3521,20 @@
       <c r="M51" s="1" t="n"/>
       <c r="N51" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O51" s="1" t="n"/>
       <c r="P51" s="1" t="inlineStr">
         <is>
-          <t>integre o plano de TIC à elaboração da proposta orçamentária e do plano de contratações, de maneira proporcional ao porte, à estrutura e à capacidade de planejamento da organização</t>
+          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
         </is>
       </c>
     </row>
     <row r="52" ht="113.45" customHeight="1">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>AV101</t>
+          <t>AV127</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -3553,12 +3547,13 @@
       <c r="E52" s="1" t="n"/>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>q2102ext[E]</t>
+          <t>q2201ext[D]</t>
         </is>
       </c>
       <c r="G52" s="1" t="inlineStr">
         <is>
-          <t>Acórdão TCE-RJ 44.490/2024-PLEN, item II.3 e subitens II.3.1 a II.3.5: necessidade de estabelecer processo estruturado, com participação de representantes das principais secretarias, para elaborar, manter e revisar periodicamente o PDTI, contemplando objetivos, indicadores e metas de TI alinhados aos objetivos de negócio, riscos que possam impactar objetivos e metas, projetos, aquisições e ações necessárias, alocação de recursos e ações de divulgação e monitoramento do PDTI após aprovação pela autoridade máxima.</t>
+          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
+ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.</t>
         </is>
       </c>
       <c r="H52" s="1" t="inlineStr">
@@ -3569,7 +3564,7 @@
       <c r="I52" s="1" t="n"/>
       <c r="J52" s="1" t="inlineStr">
         <is>
-          <t>Ausência de acompanhamento, revisão ou atualização periódica do plano de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="K52" s="1" t="inlineStr">
@@ -3581,20 +3576,20 @@
       <c r="M52" s="1" t="n"/>
       <c r="N52" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O52" s="1" t="n"/>
       <c r="P52" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e execute rotina periódica de acompanhamento, revisão e atualização do plano de TIC, registrando execução, pendências, reprogramações e deliberações</t>
+          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
         </is>
       </c>
     </row>
     <row r="53" ht="113.45" customHeight="1">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>AV103</t>
+          <t>AV128</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -3607,13 +3602,13 @@
       <c r="E53" s="1" t="n"/>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>q2703ext[C]</t>
+          <t>q2201ext[E]</t>
         </is>
       </c>
       <c r="G53" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO07.05 - Planejar e monitorar o uso de recursos humanos de TI e de negócio: planejar, alocar e acompanhar capacidade de pessoal para iniciativas, operações e serviços de TIC.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6.5 - O PDTI deve contemplar o quantitativo necessário ou ideal para a força de trabalho em TI.</t>
+          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
+ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.</t>
         </is>
       </c>
       <c r="H53" s="1" t="inlineStr">
@@ -3624,7 +3619,7 @@
       <c r="I53" s="1" t="n"/>
       <c r="J53" s="1" t="inlineStr">
         <is>
-          <t>A organização não definiu o quantitativo necessário de pessoal de TIC e segurança da informação.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="K53" s="1" t="inlineStr">
@@ -3642,14 +3637,14 @@
       <c r="O53" s="1" t="n"/>
       <c r="P53" s="1" t="inlineStr">
         <is>
-          <t>estime e mantenha atualizado o quantitativo necessário de pessoal de TIC e segurança da informação, considerando o porte e a complexidade da organização, os serviços críticos, os sistemas mantidos, as contratações vigentes e os riscos relevantes</t>
+          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
         </is>
       </c>
     </row>
     <row r="54" ht="113.45" customHeight="1">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>AV105</t>
+          <t>AV129</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -3662,13 +3657,13 @@
       <c r="E54" s="1" t="n"/>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>q2708[B]</t>
+          <t>q2203ext[A]</t>
         </is>
       </c>
       <c r="G54" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
-COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
+          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
+Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
         </is>
       </c>
       <c r="H54" s="1" t="inlineStr">
@@ -3679,7 +3674,7 @@
       <c r="I54" s="1" t="n"/>
       <c r="J54" s="1" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="K54" s="1" t="inlineStr">
@@ -3691,20 +3686,20 @@
       <c r="M54" s="1" t="n"/>
       <c r="N54" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O54" s="1" t="n"/>
       <c r="P54" s="1" t="inlineStr">
         <is>
-          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
+          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
         </is>
       </c>
     </row>
     <row r="55" ht="113.45" customHeight="1">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>AV107</t>
+          <t>AV132</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -3717,13 +3712,13 @@
       <c r="E55" s="1" t="n"/>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>q2708[D]</t>
+          <t>q2504ext[A]</t>
         </is>
       </c>
       <c r="G55" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
-COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
+          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
+Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
         </is>
       </c>
       <c r="H55" s="1" t="inlineStr">
@@ -3734,7 +3729,7 @@
       <c r="I55" s="1" t="n"/>
       <c r="J55" s="1" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="K55" s="1" t="inlineStr">
@@ -3746,20 +3741,20 @@
       <c r="M55" s="1" t="n"/>
       <c r="N55" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O55" s="1" t="n"/>
       <c r="P55" s="1" t="inlineStr">
         <is>
-          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
+          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
         </is>
       </c>
     </row>
     <row r="56" ht="113.45" customHeight="1">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>AV124</t>
+          <t>AV133</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -3772,13 +3767,13 @@
       <c r="E56" s="1" t="n"/>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[A]</t>
+          <t>q2504ext[B]</t>
         </is>
       </c>
       <c r="G56" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
-ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.</t>
+          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
+Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
         </is>
       </c>
       <c r="H56" s="1" t="inlineStr">
@@ -3789,7 +3784,7 @@
       <c r="I56" s="1" t="n"/>
       <c r="J56" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="K56" s="1" t="inlineStr">
@@ -3801,20 +3796,20 @@
       <c r="M56" s="1" t="n"/>
       <c r="N56" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O56" s="1" t="n"/>
       <c r="P56" s="1" t="inlineStr">
         <is>
-          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
+          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
         </is>
       </c>
     </row>
     <row r="57" ht="90.95" customHeight="1">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>AV125</t>
+          <t>AV136</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -3827,13 +3822,13 @@
       <c r="E57" s="1" t="n"/>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[B]</t>
+          <t>q2203ext[C]</t>
         </is>
       </c>
       <c r="G57" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento do catálogo de serviços: manter fonte única de informações consistentes sobre serviços e ofertas de serviço, disponível para usuários e equipes de suporte.
-COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.</t>
+          <t>ITIL 4, prática de gerenciamento de configuração de serviço: assegurar informações precisas e confiáveis sobre itens de configuração e seus relacionamentos com serviços, sistemas e infraestrutura.
+COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.</t>
         </is>
       </c>
       <c r="H57" s="1" t="inlineStr">
@@ -3844,7 +3839,7 @@
       <c r="I57" s="1" t="n"/>
       <c r="J57" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="K57" s="1" t="inlineStr">
@@ -3862,14 +3857,14 @@
       <c r="O57" s="1" t="n"/>
       <c r="P57" s="1" t="inlineStr">
         <is>
-          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
+          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
         </is>
       </c>
     </row>
     <row r="58" ht="90.95" customHeight="1">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>AV126</t>
+          <t>AV137</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -3882,13 +3877,13 @@
       <c r="E58" s="1" t="n"/>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[C]</t>
+          <t>q2204ext[A]</t>
         </is>
       </c>
       <c r="G58" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento do catálogo de serviços: manter fonte única de informações consistentes sobre serviços e ofertas de serviço, disponível para usuários e equipes de suporte.
-COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.</t>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
         </is>
       </c>
       <c r="H58" s="1" t="inlineStr">
@@ -3899,7 +3894,7 @@
       <c r="I58" s="1" t="n"/>
       <c r="J58" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="K58" s="1" t="inlineStr">
@@ -3917,14 +3912,14 @@
       <c r="O58" s="1" t="n"/>
       <c r="P58" s="1" t="inlineStr">
         <is>
-          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
     </row>
     <row r="59" ht="90.95" customHeight="1">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>AV127</t>
+          <t>AV140</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -3937,13 +3932,13 @@
       <c r="E59" s="1" t="n"/>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[D]</t>
+          <t>q2204ext[D]</t>
         </is>
       </c>
       <c r="G59" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
-ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.</t>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
         </is>
       </c>
       <c r="H59" s="1" t="inlineStr">
@@ -3954,7 +3949,7 @@
       <c r="I59" s="1" t="n"/>
       <c r="J59" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="K59" s="1" t="inlineStr">
@@ -3972,14 +3967,14 @@
       <c r="O59" s="1" t="n"/>
       <c r="P59" s="1" t="inlineStr">
         <is>
-          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
     </row>
     <row r="60" ht="79.90000000000001" customHeight="1">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>AV128</t>
+          <t>AV141</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -3992,13 +3987,13 @@
       <c r="E60" s="1" t="n"/>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[E]</t>
+          <t>q2204ext[E]</t>
         </is>
       </c>
       <c r="G60" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
-ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.</t>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
         </is>
       </c>
       <c r="H60" s="1" t="inlineStr">
@@ -4009,7 +4004,7 @@
       <c r="I60" s="1" t="n"/>
       <c r="J60" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="K60" s="1" t="inlineStr">
@@ -4027,14 +4022,14 @@
       <c r="O60" s="1" t="n"/>
       <c r="P60" s="1" t="inlineStr">
         <is>
-          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
     </row>
     <row r="61" ht="79.90000000000001" customHeight="1">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>AV129</t>
+          <t>AV143</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -4047,13 +4042,13 @@
       <c r="E61" s="1" t="n"/>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>q2203ext[A]</t>
+          <t>q2801ext[A]</t>
         </is>
       </c>
       <c r="G61" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
+          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
         </is>
       </c>
       <c r="H61" s="1" t="inlineStr">
@@ -4064,7 +4059,7 @@
       <c r="I61" s="1" t="n"/>
       <c r="J61" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="K61" s="1" t="inlineStr">
@@ -4082,14 +4077,14 @@
       <c r="O61" s="1" t="n"/>
       <c r="P61" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
+          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
         </is>
       </c>
     </row>
     <row r="62" ht="90.95" customHeight="1">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>AV132</t>
+          <t>AV148</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -4102,13 +4097,14 @@
       <c r="E62" s="1" t="n"/>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>q2504ext[A]</t>
+          <t>q2804[A]</t>
         </is>
       </c>
       <c r="G62" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
+          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+COBIT 2019, BAI02.04 - Obter aprovação dos requisitos da solução: obter aprovação formal dos requisitos funcionais, técnicos, de segurança e de conformidade antes de prosseguir com a solução.
+Instrução Normativa SGD/ME nº 94, de 23 de dezembro de 2022, art. 1º, § 1º: como referência de boa prática, a aplicação de ritos formais de contratação de TIC pode ser facultada para contratações diretas por dispensa em razão do valor (inciso II do art. 75 da Lei nº 14.133/2021), indicando a possibilidade de fluxos simplificados para aquisições de baixa complexidade ou valor.</t>
         </is>
       </c>
       <c r="H62" s="1" t="inlineStr">
@@ -4119,7 +4115,7 @@
       <c r="I62" s="1" t="n"/>
       <c r="J62" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
         </is>
       </c>
       <c r="K62" s="1" t="inlineStr">
@@ -4131,20 +4127,20 @@
       <c r="M62" s="1" t="n"/>
       <c r="N62" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O62" s="1" t="n"/>
       <c r="P62" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
+          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo fluxos simplificados para contratações de baixa complexidade ou baixo valor, desde que preservada análise técnica mínima compatível com o risco da contratação</t>
         </is>
       </c>
     </row>
     <row r="63" ht="90.95" customHeight="1">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>AV133</t>
+          <t>AV150</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -4157,13 +4153,13 @@
       <c r="E63" s="1" t="n"/>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>q2504ext[B]</t>
+          <t>q2802ext[C]</t>
         </is>
       </c>
       <c r="G63" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
+          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Art. 18, caput e §1º, incisos I, IV, V, VIII, IX, X e XIII, da Lei 14.133/2021: fase preparatória caracterizada pelo planejamento, compatibilização com o plano de contratações anual e elementos mínimos do estudo técnico preliminar.</t>
         </is>
       </c>
       <c r="H63" s="1" t="inlineStr">
@@ -4174,7 +4170,7 @@
       <c r="I63" s="1" t="n"/>
       <c r="J63" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
         </is>
       </c>
       <c r="K63" s="1" t="inlineStr">
@@ -4192,19 +4188,19 @@
       <c r="O63" s="1" t="n"/>
       <c r="P63" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
+          <t>integre as contratações de TIC com os instrumentos de planejamento da organização e com o Plano de Contratações Anual, quando elaborado, justificando as situações excepcionais</t>
         </is>
       </c>
     </row>
     <row r="64" ht="90.95" customHeight="1">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>AV136</t>
+          <t>AV152</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
-          <t>avaliacao_evidencias_ajustes</t>
+          <t>questionario</t>
         </is>
       </c>
       <c r="C64" s="1" t="n"/>
@@ -4212,49 +4208,49 @@
       <c r="E64" s="1" t="n"/>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>q2203ext[C]</t>
+          <t>q2801ext[B]</t>
         </is>
       </c>
       <c r="G64" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de configuração de serviço: assegurar informações precisas e confiáveis sobre itens de configuração e seus relacionamentos com serviços, sistemas e infraestrutura.
-COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.</t>
+          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
         </is>
       </c>
       <c r="H64" s="1" t="inlineStr">
         <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+          <t>Resposta negativa ao detalhamento b) do item 2801 do Questionário, para verificar se são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
         </is>
       </c>
       <c r="I64" s="1" t="n"/>
       <c r="J64" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="K64" s="1" t="inlineStr">
         <is>
-          <t>Não conforme</t>
+          <t>(Não | N/A)</t>
         </is>
       </c>
       <c r="L64" s="1" t="n"/>
       <c r="M64" s="1" t="n"/>
       <c r="N64" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O64" s="1" t="n"/>
       <c r="P64" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
+          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
         </is>
       </c>
     </row>
     <row r="65" ht="90.95" customHeight="1">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>AV137</t>
+          <t>AV153</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -4267,13 +4263,13 @@
       <c r="E65" s="1" t="n"/>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>q2204ext[A]</t>
+          <t>q2801ext[B]</t>
         </is>
       </c>
       <c r="G65" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
+          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
         </is>
       </c>
       <c r="H65" s="1" t="inlineStr">
@@ -4284,7 +4280,7 @@
       <c r="I65" s="1" t="n"/>
       <c r="J65" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="K65" s="1" t="inlineStr">
@@ -4296,25 +4292,25 @@
       <c r="M65" s="1" t="n"/>
       <c r="N65" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O65" s="1" t="n"/>
       <c r="P65" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
+          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
         </is>
       </c>
     </row>
     <row r="66" ht="90.95" customHeight="1">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>AV140</t>
+          <t>AV154</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
-          <t>avaliacao_evidencias_ajustes</t>
+          <t>questionario</t>
         </is>
       </c>
       <c r="C66" s="1" t="n"/>
@@ -4322,54 +4318,55 @@
       <c r="E66" s="1" t="n"/>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>q2204ext[D]</t>
+          <t>existe_plano_ti</t>
         </is>
       </c>
       <c r="G66" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H66" s="1" t="inlineStr">
         <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+          <t>Resposta ao item 2102 que não caracteriza a existência de plano de TIC vigente, ainda que parcialmente adotado</t>
         </is>
       </c>
       <c r="I66" s="1" t="n"/>
       <c r="J66" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="K66" s="1" t="inlineStr">
         <is>
-          <t>Não conforme</t>
+          <t>False</t>
         </is>
       </c>
       <c r="L66" s="1" t="n"/>
       <c r="M66" s="1" t="n"/>
       <c r="N66" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O66" s="1" t="n"/>
       <c r="P66" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
     <row r="67" ht="79.90000000000001" customHeight="1">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>AV141</t>
+          <t>AV155</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
-          <t>avaliacao_evidencias_ajustes</t>
+          <t>questionario</t>
         </is>
       </c>
       <c r="C67" s="1" t="n"/>
@@ -4377,321 +4374,47 @@
       <c r="E67" s="1" t="n"/>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>q2204ext[E]</t>
+          <t>existe_plano_ti</t>
         </is>
       </c>
       <c r="G67" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H67" s="1" t="inlineStr">
         <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+          <t>Plano de TIC vigente declarado no item 2102, ao menos parcialmente adotado</t>
         </is>
       </c>
       <c r="I67" s="1" t="n"/>
-      <c r="J67" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
-        </is>
-      </c>
+      <c r="J67" s="1" t="n"/>
       <c r="K67" s="1" t="inlineStr">
         <is>
-          <t>Não conforme</t>
+          <t>True</t>
         </is>
       </c>
       <c r="L67" s="1" t="n"/>
       <c r="M67" s="1" t="n"/>
       <c r="N67" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O67" s="1" t="n"/>
       <c r="P67" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="79.90000000000001" customHeight="1">
-      <c r="A68" s="1" t="inlineStr">
-        <is>
-          <t>AV143</t>
-        </is>
-      </c>
-      <c r="B68" s="1" t="inlineStr">
-        <is>
-          <t>avaliacao_evidencias_ajustes</t>
-        </is>
-      </c>
-      <c r="C68" s="1" t="n"/>
-      <c r="D68" s="1" t="n"/>
-      <c r="E68" s="1" t="n"/>
-      <c r="F68" s="1" t="inlineStr">
-        <is>
-          <t>q2801ext[A]</t>
-        </is>
-      </c>
-      <c r="G68" s="1" t="inlineStr">
-        <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
-        </is>
-      </c>
-      <c r="H68" s="1" t="inlineStr">
-        <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
-        </is>
-      </c>
-      <c r="I68" s="1" t="n"/>
-      <c r="J68" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="K68" s="1" t="inlineStr">
-        <is>
-          <t>Não conforme</t>
-        </is>
-      </c>
-      <c r="L68" s="1" t="n"/>
-      <c r="M68" s="1" t="n"/>
-      <c r="N68" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O68" s="1" t="n"/>
-      <c r="P68" s="1" t="inlineStr">
-        <is>
-          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="79.90000000000001" customHeight="1">
-      <c r="A69" s="1" t="inlineStr">
-        <is>
-          <t>AV148</t>
-        </is>
-      </c>
-      <c r="B69" s="1" t="inlineStr">
-        <is>
-          <t>avaliacao_evidencias_ajustes</t>
-        </is>
-      </c>
-      <c r="C69" s="1" t="n"/>
-      <c r="D69" s="1" t="n"/>
-      <c r="E69" s="1" t="n"/>
-      <c r="F69" s="1" t="inlineStr">
-        <is>
-          <t>q2804[A]</t>
-        </is>
-      </c>
-      <c r="G69" s="1" t="inlineStr">
-        <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-COBIT 2019, BAI02.04 - Obter aprovação dos requisitos da solução: obter aprovação formal dos requisitos funcionais, técnicos, de segurança e de conformidade antes de prosseguir com a solução.
-Instrução Normativa SGD/ME nº 94, de 23 de dezembro de 2022, art. 1º, § 1º: como referência de boa prática, a aplicação de ritos formais de contratação de TIC pode ser facultada para contratações diretas por dispensa em razão do valor (inciso II do art. 75 da Lei nº 14.133/2021), indicando a possibilidade de fluxos simplificados para aquisições de baixa complexidade ou valor.</t>
-        </is>
-      </c>
-      <c r="H69" s="1" t="inlineStr">
-        <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
-        </is>
-      </c>
-      <c r="I69" s="1" t="n"/>
-      <c r="J69" s="1" t="inlineStr">
-        <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
-        </is>
-      </c>
-      <c r="K69" s="1" t="inlineStr">
-        <is>
-          <t>Não conforme</t>
-        </is>
-      </c>
-      <c r="L69" s="1" t="n"/>
-      <c r="M69" s="1" t="n"/>
-      <c r="N69" s="1" t="inlineStr">
-        <is>
-          <t>Recomendação</t>
-        </is>
-      </c>
-      <c r="O69" s="1" t="n"/>
-      <c r="P69" s="1" t="inlineStr">
-        <is>
-          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo fluxos simplificados para contratações de baixa complexidade ou baixo valor, desde que preservada análise técnica mínima compatível com o risco da contratação</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="90.95" customHeight="1">
-      <c r="A70" s="1" t="inlineStr">
-        <is>
-          <t>AV150</t>
-        </is>
-      </c>
-      <c r="B70" s="1" t="inlineStr">
-        <is>
-          <t>avaliacao_evidencias_ajustes</t>
-        </is>
-      </c>
-      <c r="C70" s="1" t="n"/>
-      <c r="D70" s="1" t="n"/>
-      <c r="E70" s="1" t="n"/>
-      <c r="F70" s="1" t="inlineStr">
-        <is>
-          <t>q2802ext[C]</t>
-        </is>
-      </c>
-      <c r="G70" s="1" t="inlineStr">
-        <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 18, caput e §1º, incisos I, IV, V, VIII, IX, X e XIII, da Lei 14.133/2021: fase preparatória caracterizada pelo planejamento, compatibilização com o plano de contratações anual e elementos mínimos do estudo técnico preliminar.</t>
-        </is>
-      </c>
-      <c r="H70" s="1" t="inlineStr">
-        <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
-        </is>
-      </c>
-      <c r="I70" s="1" t="n"/>
-      <c r="J70" s="1" t="inlineStr">
-        <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
-        </is>
-      </c>
-      <c r="K70" s="1" t="inlineStr">
-        <is>
-          <t>Não conforme</t>
-        </is>
-      </c>
-      <c r="L70" s="1" t="n"/>
-      <c r="M70" s="1" t="n"/>
-      <c r="N70" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O70" s="1" t="n"/>
-      <c r="P70" s="1" t="inlineStr">
-        <is>
-          <t>integre as contratações de TIC com os instrumentos de planejamento da organização e com o Plano de Contratações Anual, quando elaborado, justificando as situações excepcionais</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="90.95" customHeight="1">
-      <c r="A71" s="1" t="inlineStr">
-        <is>
-          <t>AV152</t>
-        </is>
-      </c>
-      <c r="B71" s="1" t="inlineStr">
-        <is>
-          <t>questionario</t>
-        </is>
-      </c>
-      <c r="C71" s="1" t="n"/>
-      <c r="D71" s="1" t="n"/>
-      <c r="E71" s="1" t="n"/>
-      <c r="F71" s="1" t="inlineStr">
-        <is>
-          <t>q2801ext[B]</t>
-        </is>
-      </c>
-      <c r="G71" s="1" t="inlineStr">
-        <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
-        </is>
-      </c>
-      <c r="H71" s="1" t="inlineStr">
-        <is>
-          <t>Resposta negativa ao detalhamento b) do item 2801 do Questionário, para verificar se são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
-        </is>
-      </c>
-      <c r="I71" s="1" t="n"/>
-      <c r="J71" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="K71" s="1" t="inlineStr">
-        <is>
-          <t>(Não | N/A)</t>
-        </is>
-      </c>
-      <c r="L71" s="1" t="n"/>
-      <c r="M71" s="1" t="n"/>
-      <c r="N71" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O71" s="1" t="n"/>
-      <c r="P71" s="1" t="inlineStr">
-        <is>
-          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="90.95" customHeight="1">
-      <c r="A72" s="1" t="inlineStr">
-        <is>
-          <t>AV153</t>
-        </is>
-      </c>
-      <c r="B72" s="1" t="inlineStr">
-        <is>
-          <t>avaliacao_evidencias_ajustes</t>
-        </is>
-      </c>
-      <c r="C72" s="1" t="n"/>
-      <c r="D72" s="1" t="n"/>
-      <c r="E72" s="1" t="n"/>
-      <c r="F72" s="1" t="inlineStr">
-        <is>
-          <t>q2801ext[B]</t>
-        </is>
-      </c>
-      <c r="G72" s="1" t="inlineStr">
-        <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
-        </is>
-      </c>
-      <c r="H72" s="1" t="inlineStr">
-        <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
-        </is>
-      </c>
-      <c r="I72" s="1" t="n"/>
-      <c r="J72" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="K72" s="1" t="inlineStr">
-        <is>
-          <t>Não conforme</t>
-        </is>
-      </c>
-      <c r="L72" s="1" t="n"/>
-      <c r="M72" s="1" t="n"/>
-      <c r="N72" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O72" s="1" t="n"/>
-      <c r="P72" s="1" t="inlineStr">
-        <is>
-          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
-        </is>
-      </c>
-    </row>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="79.90000000000001" customHeight="1"/>
+    <row r="69" ht="79.90000000000001" customHeight="1"/>
+    <row r="70" ht="90.95" customHeight="1"/>
+    <row r="71" ht="90.95" customHeight="1"/>
+    <row r="72" ht="90.95" customHeight="1"/>
     <row r="73" ht="90.95" customHeight="1"/>
     <row r="74" ht="90.95" customHeight="1"/>
     <row r="75" ht="90.95" customHeight="1"/>
@@ -4775,7 +4498,7 @@
     <row r="153" ht="23.85" customHeight="1"/>
     <row r="154" ht="23.85" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A3:P72"/>
+  <autoFilter ref="A3:P67"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -4787,7 +4510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H71"/>
+  <dimension ref="A2:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5315,7 +5038,7 @@
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="D15" s="9" t="n">
@@ -5323,7 +5046,7 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>AV14 &amp; ~AV92</t>
+          <t>AV14</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
@@ -5343,7 +5066,7 @@
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>MR023</t>
+          <t>MR024</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
@@ -5353,25 +5076,25 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="D16" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>AV92</t>
+          <t>AV15</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>AV92</t>
+          <t>AV15</t>
         </is>
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2101, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as áreas demandantes de soluções de TI participam do processo de planejamento de tecnologia da informação</t>
+          <t>No subitem b) do item 2101, não houve declaração afirmativa quanto à prática avaliada: estabeleceu critérios para orientar a seleção e a priorização das iniciativas de TI (projetos e ações) e os mantêm atualizados</t>
         </is>
       </c>
       <c r="H16" s="9" t="b">
@@ -5381,7 +5104,7 @@
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>MR024</t>
+          <t>MR028</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
@@ -5391,25 +5114,25 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="D17" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>AV15 &amp; ~AV93</t>
+          <t>AV17</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>AV15</t>
+          <t>AV17</t>
         </is>
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2101, não houve declaração afirmativa quanto à prática avaliada: estabeleceu critérios para orientar a seleção e a priorização das iniciativas de TI (projetos e ações) e os mantêm atualizados</t>
+          <t>No subitem d) do item 2101, não houve declaração afirmativa quanto à prática avaliada: o processo de planejamento de TI está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H17" s="9" t="b">
@@ -5419,7 +5142,7 @@
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>MR025</t>
+          <t>MR030</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
@@ -5429,25 +5152,25 @@
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
+          <t>Ausência de aprovação formal do plano de TIC.</t>
         </is>
       </c>
       <c r="D18" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>AV93</t>
+          <t>AV155 &amp; AV18</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>AV93</t>
+          <t>AV18</t>
         </is>
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2101, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que estabeleceu critérios para orientar a seleção e a priorização das iniciativas de TI (projetos e ações) e os mantêm atualizados</t>
+          <t>No subitem a) do item 2102, não houve declaração afirmativa quanto à prática avaliada: o plano de tecnologia da informação (plano de TI) é aprovado pelo dirigente máximo da organização ou por dirigente ou colegiado que integra a alta administração</t>
         </is>
       </c>
       <c r="H18" s="9" t="b">
@@ -5457,7 +5180,7 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>MR028</t>
+          <t>MR032</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
@@ -5467,25 +5190,25 @@
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
+          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
         </is>
       </c>
       <c r="D19" s="9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>AV17 &amp; ~AV95</t>
+          <t>AV155 &amp; AV19</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>AV17</t>
+          <t>AV19</t>
         </is>
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2101, não houve declaração afirmativa quanto à prática avaliada: o processo de planejamento de TI está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem d) do item 2102, não houve declaração afirmativa quanto à prática avaliada: as iniciativas de TI (projetos e ações) constantes do plano de TI alinham-se aos objetivos e iniciativas definidos no planejamento institucional (como PPA, planos estratégicos, planos setoriais e plano de governo, no caso de municípios), bem como, quando aplicável, às estratégias e diretrizes estabelecidas por instâncias superiores de governança (como a Estratégia Nacional de Tecnologia da Informação e Comunicação do Poder Judiciário - ENTIC-JUD, normas e orientações do SETIC/PRODERJ (para órgãos estaduais) ou instâncias de governança equivalentes no âmbito municipal)</t>
         </is>
       </c>
       <c r="H19" s="9" t="b">
@@ -5495,7 +5218,7 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>MR029</t>
+          <t>MR034</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
@@ -5505,25 +5228,25 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo formal de planejamento de TIC.</t>
+          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
         </is>
       </c>
       <c r="D20" s="9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>AV95</t>
+          <t>AV155 &amp; AV20</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>AV95</t>
+          <t>AV20</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2101, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de planejamento de TI está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem c) do item 2102, não houve declaração afirmativa quanto à prática avaliada: o plano de TI fundamenta a proposta orçamentária da área de TI e o plano de contratações</t>
         </is>
       </c>
       <c r="H20" s="9" t="b">
@@ -5533,7 +5256,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>MR030</t>
+          <t>MR041</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
@@ -5543,7 +5266,7 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Ausência de aprovação formal do plano de TIC.</t>
+          <t>Ausência de acompanhamento da execução do plano de TIC.</t>
         </is>
       </c>
       <c r="D21" s="9" t="n">
@@ -5551,17 +5274,17 @@
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>AV18 &amp; ~AV96</t>
+          <t>AV155 &amp; AV24</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>AV18</t>
+          <t>AV24</t>
         </is>
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2102, não houve declaração afirmativa quanto à prática avaliada: o plano de tecnologia da informação (plano de TI) é aprovado pelo dirigente máximo da organização ou por dirigente ou colegiado que integra a alta administração</t>
+          <t>No subitem e) do item 2102, não houve declaração afirmativa quanto à prática avaliada: é feito acompanhamento concomitante à execução do plano de TI, com vistas a assegurar sua observância e possibilitar a realização de ajustes que se fizerem necessário</t>
         </is>
       </c>
       <c r="H21" s="9" t="b">
@@ -5571,35 +5294,35 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>MR031</t>
+          <t>MR043</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>PA03</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Ausência de aprovação formal do plano de TIC.</t>
+          <t>Ausência de força de trabalho dedicada à TIC.</t>
         </is>
       </c>
       <c r="D22" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>AV96</t>
+          <t>AV26 &amp; AV25</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>AV96</t>
+          <t>AV25</t>
         </is>
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o plano de tecnologia da informação (plano de TI) é aprovado pelo dirigente máximo da organização ou por dirigente ou colegiado que integra a alta administração</t>
+          <t>Item 0105: embora a organização tenha declarado estrutura formal de TIC no item 0101, informou não possuir profissionais atuando regularmente em tecnologia da informação</t>
         </is>
       </c>
       <c r="H22" s="9" t="b">
@@ -5609,17 +5332,17 @@
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>MR032</t>
+          <t>MR045</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>PA03</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
+          <t>A organização não definiu o quantitativo necessário de pessoal de TIC e segurança da informação.</t>
         </is>
       </c>
       <c r="D23" s="9" t="n">
@@ -5627,17 +5350,17 @@
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>AV19 &amp; ~AV97</t>
+          <t>AV29 &amp; ~AV103</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>AV19</t>
+          <t>AV29</t>
         </is>
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2102, não houve declaração afirmativa quanto à prática avaliada: as iniciativas de TI (projetos e ações) constantes do plano de TI alinham-se aos objetivos e iniciativas definidos no planejamento institucional (como PPA, planos estratégicos, planos setoriais e plano de governo, no caso de municípios), bem como, quando aplicável, às estratégias e diretrizes estabelecidas por instâncias superiores de governança (como a Estratégia Nacional de Tecnologia da Informação e Comunicação do Poder Judiciário - ENTIC-JUD, normas e orientações do SETIC/PRODERJ (para órgãos estaduais) ou instâncias de governança equivalentes no âmbito municipal)</t>
+          <t>No subitem c) do item 2703, não houve declaração afirmativa quanto à prática avaliada: definiu-se, de maneira documentada, um quantitativo necessário de pessoal da área de tecnologia da informação e segurança da informação</t>
         </is>
       </c>
       <c r="H23" s="9" t="b">
@@ -5647,17 +5370,17 @@
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>MR033</t>
+          <t>MR046</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>PA03</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
+          <t>A organização não definiu o quantitativo necessário de pessoal de TIC e segurança da informação.</t>
         </is>
       </c>
       <c r="D24" s="9" t="n">
@@ -5665,17 +5388,17 @@
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>AV97</t>
+          <t>AV103</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>AV97</t>
+          <t>AV103</t>
         </is>
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as iniciativas de TI (projetos e ações) constantes do plano de TI alinham-se aos objetivos e iniciativas definidos no planejamento institucional (como PPA, planos estratégicos, planos setoriais e plano de governo, no caso de municípios), bem como, quando aplicável, às estratégias e diretrizes estabelecidas por instâncias superiores de governança (como a Estratégia Nacional de Tecnologia da Informação e Comunicação do Poder Judiciário - ENTIC-JUD, normas e orientações do SETIC/PRODERJ (para órgãos estaduais) ou instâncias de governança equivalentes no âmbito municipal)</t>
+          <t>No subitem c) do item 2703, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu-se, de maneira documentada, um quantitativo necessário de pessoal da área de tecnologia da informação e segurança da informação</t>
         </is>
       </c>
       <c r="H24" s="9" t="b">
@@ -5685,17 +5408,17 @@
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>MR034</t>
+          <t>MR047</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>PA03</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="D25" s="9" t="n">
@@ -5703,17 +5426,17 @@
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>AV20 &amp; ~AV98</t>
+          <t>AV31 &amp; ~AV105</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>AV20</t>
+          <t>AV31</t>
         </is>
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2102, não houve declaração afirmativa quanto à prática avaliada: o plano de TI fundamenta a proposta orçamentária da área de TI e o plano de contratações</t>
+          <t>No subitem b) do item 2708, não houve declaração afirmativa quanto à prática avaliada: possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
         </is>
       </c>
       <c r="H25" s="9" t="b">
@@ -5723,17 +5446,17 @@
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>MR035</t>
+          <t>MR048</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>PA03</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="D26" s="9" t="n">
@@ -5741,17 +5464,17 @@
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>AV98</t>
+          <t>AV105</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>AV98</t>
+          <t>AV105</t>
         </is>
       </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o plano de TI fundamenta a proposta orçamentária da área de TI e o plano de contratações</t>
+          <t>No subitem b) do item 2708, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
         </is>
       </c>
       <c r="H26" s="9" t="b">
@@ -5761,35 +5484,35 @@
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>MR041</t>
+          <t>MR049</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>PA03</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>Ausência de acompanhamento, revisão ou atualização periódica do plano de TIC.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="D27" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>AV24 &amp; ~AV101</t>
+          <t>AV33 &amp; ~AV107</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>AV24</t>
+          <t>AV33</t>
         </is>
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2102, não houve declaração afirmativa quanto à prática avaliada: é feito acompanhamento concomitante à execução do plano de TI, com vistas a assegurar sua observância e possibilitar a realização de ajustes que se fizerem necessário</t>
+          <t>No subitem d) do item 2708, não houve declaração afirmativa quanto à prática avaliada: possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
         </is>
       </c>
       <c r="H27" s="9" t="b">
@@ -5799,35 +5522,35 @@
     <row r="28" ht="45" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>MR042</t>
+          <t>MR050</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>PA03</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Ausência de acompanhamento, revisão ou atualização periódica do plano de TIC.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="D28" s="9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>AV101</t>
+          <t>AV107</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>AV101</t>
+          <t>AV107</t>
         </is>
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que é feito acompanhamento concomitante à execução do plano de TI, com vistas a assegurar sua observância e possibilitar a realização de ajustes que se fizerem necessário</t>
+          <t>No subitem d) do item 2708, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
         </is>
       </c>
       <c r="H28" s="9" t="b">
@@ -5837,7 +5560,7 @@
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>MR043</t>
+          <t>MR062</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
@@ -5847,7 +5570,7 @@
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Ausência de força de trabalho dedicada à TIC.</t>
+          <t>Dependência externa relevante sem capacidade interna suficiente para coordenar e fiscalizar a TIC.</t>
         </is>
       </c>
       <c r="D29" s="9" t="n">
@@ -5855,17 +5578,17 @@
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>AV26 &amp; AV25</t>
+          <t>AV45 &amp; AV46</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>AV25</t>
+          <t>AV45</t>
         </is>
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>Item 0105: embora a organização tenha declarado estrutura formal de TIC no item 0101, informou não possuir profissionais atuando regularmente em tecnologia da informação</t>
+          <t>A organização informou modelo de operação de TIC com execução predominantemente terceirizada, o que levou à análise de sua capacidade interna de coordenação e fiscalização</t>
         </is>
       </c>
       <c r="H29" s="9" t="b">
@@ -5875,7 +5598,7 @@
     <row r="30" ht="45" customHeight="1">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>MR045</t>
+          <t>MR063</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
@@ -5885,25 +5608,25 @@
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>A organização não definiu o quantitativo necessário de pessoal de TIC e segurança da informação.</t>
+          <t>Dependência externa relevante sem capacidade interna suficiente para coordenar e fiscalizar a TIC.</t>
         </is>
       </c>
       <c r="D30" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>AV29 &amp; ~AV103</t>
+          <t>AV45 &amp; AV46</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>AV29</t>
+          <t>AV46</t>
         </is>
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2703, não houve declaração afirmativa quanto à prática avaliada: definiu-se, de maneira documentada, um quantitativo necessário de pessoal da área de tecnologia da informação e segurança da informação</t>
+          <t>Não foram identificados profissionais internos de TIC para coordenar e fiscalizar a execução das atividades de tecnologia da informação</t>
         </is>
       </c>
       <c r="H30" s="9" t="b">
@@ -5913,35 +5636,35 @@
     <row r="31" ht="45" customHeight="1">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>MR046</t>
+          <t>MR065</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA05</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>A organização não definiu o quantitativo necessário de pessoal de TIC e segurança da informação.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D31" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>AV103</t>
+          <t>AV54 &amp; ~AV124</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>AV103</t>
+          <t>AV54</t>
         </is>
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2703, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu-se, de maneira documentada, um quantitativo necessário de pessoal da área de tecnologia da informação e segurança da informação</t>
+          <t>No subitem a) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
         </is>
       </c>
       <c r="H31" s="9" t="b">
@@ -5951,35 +5674,35 @@
     <row r="32" ht="45" customHeight="1">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>MR047</t>
+          <t>MR066</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA05</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D32" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>AV31 &amp; ~AV105</t>
+          <t>AV124</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>AV31</t>
+          <t>AV124</t>
         </is>
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2708, não houve declaração afirmativa quanto à prática avaliada: possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
+          <t>No subitem a) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
         </is>
       </c>
       <c r="H32" s="9" t="b">
@@ -5989,35 +5712,35 @@
     <row r="33" ht="45" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>MR048</t>
+          <t>MR067</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA05</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="D33" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>AV105</t>
+          <t>AV55 &amp; ~AV125</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>AV105</t>
+          <t>AV55</t>
         </is>
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2708, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
+          <t>No subitem b) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
         </is>
       </c>
       <c r="H33" s="9" t="b">
@@ -6027,35 +5750,35 @@
     <row r="34" ht="45" customHeight="1">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>MR049</t>
+          <t>MR068</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA05</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="D34" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>AV33 &amp; ~AV107</t>
+          <t>AV125</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>AV33</t>
+          <t>AV125</t>
         </is>
       </c>
       <c r="G34" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2708, não houve declaração afirmativa quanto à prática avaliada: possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
+          <t>No subitem b) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
         </is>
       </c>
       <c r="H34" s="9" t="b">
@@ -6065,35 +5788,35 @@
     <row r="35" ht="90" customHeight="1">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>MR050</t>
+          <t>MR069</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA05</t>
         </is>
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="D35" s="9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>AV107</t>
+          <t>AV56 &amp; ~AV126</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>AV107</t>
+          <t>AV56</t>
         </is>
       </c>
       <c r="G35" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2708, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
+          <t>No subitem c) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
         </is>
       </c>
       <c r="H35" s="9" t="b">
@@ -6103,35 +5826,35 @@
     <row r="36" ht="105" customHeight="1">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>MR062</t>
+          <t>MR070</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA05</t>
         </is>
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>Dependência externa relevante sem capacidade interna suficiente para coordenar e fiscalizar a TIC.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="D36" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>AV45 &amp; AV46</t>
+          <t>AV126</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>AV45</t>
+          <t>AV126</t>
         </is>
       </c>
       <c r="G36" s="9" t="inlineStr">
         <is>
-          <t>A organização informou modelo de operação de TIC com execução predominantemente terceirizada, o que levou à análise de sua capacidade interna de coordenação e fiscalização</t>
+          <t>No subitem c) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
         </is>
       </c>
       <c r="H36" s="9" t="b">
@@ -6141,17 +5864,17 @@
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>MR063</t>
+          <t>MR071</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA05</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>Dependência externa relevante sem capacidade interna suficiente para coordenar e fiscalizar a TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D37" s="9" t="n">
@@ -6159,17 +5882,17 @@
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>AV45 &amp; AV46</t>
+          <t>AV57 &amp; ~AV127</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>AV46</t>
+          <t>AV57</t>
         </is>
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>Não foram identificados profissionais internos de TIC para coordenar e fiscalizar a execução das atividades de tecnologia da informação</t>
+          <t>No subitem d) do item 2201, não houve declaração afirmativa quanto à prática avaliada: são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
         </is>
       </c>
       <c r="H37" s="9" t="b">
@@ -6179,7 +5902,7 @@
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>MR065</t>
+          <t>MR072</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
@@ -6193,21 +5916,21 @@
         </is>
       </c>
       <c r="D38" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>AV54 &amp; ~AV124</t>
+          <t>AV127</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>AV54</t>
+          <t>AV127</t>
         </is>
       </c>
       <c r="G38" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
+          <t>No subitem d) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
         </is>
       </c>
       <c r="H38" s="9" t="b">
@@ -6217,7 +5940,7 @@
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>MR066</t>
+          <t>MR073</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
@@ -6231,21 +5954,21 @@
         </is>
       </c>
       <c r="D39" s="9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>AV124</t>
+          <t>AV58 &amp; ~AV128</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>AV124</t>
+          <t>AV58</t>
         </is>
       </c>
       <c r="G39" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
+          <t>No subitem e) do item 2201, não houve declaração afirmativa quanto à prática avaliada: a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
         </is>
       </c>
       <c r="H39" s="9" t="b">
@@ -6255,7 +5978,7 @@
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>MR067</t>
+          <t>MR074</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
@@ -6265,25 +5988,25 @@
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D40" s="9" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>AV55 &amp; ~AV125</t>
+          <t>AV128</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>AV55</t>
+          <t>AV128</t>
         </is>
       </c>
       <c r="G40" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
+          <t>No subitem e) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
         </is>
       </c>
       <c r="H40" s="9" t="b">
@@ -6293,7 +6016,7 @@
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>MR068</t>
+          <t>MR075</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
@@ -6303,25 +6026,25 @@
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="D41" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>AV125</t>
+          <t>AV59 &amp; ~AV129</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>AV125</t>
+          <t>AV59</t>
         </is>
       </c>
       <c r="G41" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
+          <t>No subitem a) do item 2203, não houve declaração afirmativa quanto à prática avaliada: mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
         </is>
       </c>
       <c r="H41" s="9" t="b">
@@ -6331,7 +6054,7 @@
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>MR069</t>
+          <t>MR076</t>
         </is>
       </c>
       <c r="B42" s="9" t="inlineStr">
@@ -6341,25 +6064,25 @@
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="D42" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>AV56 &amp; ~AV126</t>
+          <t>AV129</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>AV56</t>
+          <t>AV129</t>
         </is>
       </c>
       <c r="G42" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
+          <t>No subitem a) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
         </is>
       </c>
       <c r="H42" s="9" t="b">
@@ -6369,7 +6092,7 @@
     <row r="43" ht="45" customHeight="1">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>MR070</t>
+          <t>MR077</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
@@ -6379,25 +6102,25 @@
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="D43" s="9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>AV126</t>
+          <t>AV62 &amp; ~AV132</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>AV126</t>
+          <t>AV62</t>
         </is>
       </c>
       <c r="G43" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
+          <t>No subitem a) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H43" s="9" t="b">
@@ -6407,7 +6130,7 @@
     <row r="44" ht="45" customHeight="1">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>MR071</t>
+          <t>MR078</t>
         </is>
       </c>
       <c r="B44" s="9" t="inlineStr">
@@ -6417,25 +6140,25 @@
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="D44" s="9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>AV57 &amp; ~AV127</t>
+          <t>AV132</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>AV57</t>
+          <t>AV132</t>
         </is>
       </c>
       <c r="G44" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2201, não houve declaração afirmativa quanto à prática avaliada: são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
+          <t>No subitem a) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H44" s="9" t="b">
@@ -6445,7 +6168,7 @@
     <row r="45" ht="45" customHeight="1">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>MR072</t>
+          <t>MR079</t>
         </is>
       </c>
       <c r="B45" s="9" t="inlineStr">
@@ -6455,25 +6178,25 @@
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="D45" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>AV127</t>
+          <t>AV63 &amp; ~AV133</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>AV127</t>
+          <t>AV63</t>
         </is>
       </c>
       <c r="G45" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
+          <t>No subitem b) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H45" s="9" t="b">
@@ -6483,7 +6206,7 @@
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>MR073</t>
+          <t>MR080</t>
         </is>
       </c>
       <c r="B46" s="9" t="inlineStr">
@@ -6493,25 +6216,25 @@
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="D46" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>AV58 &amp; ~AV128</t>
+          <t>AV133</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>AV58</t>
+          <t>AV133</t>
         </is>
       </c>
       <c r="G46" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2201, não houve declaração afirmativa quanto à prática avaliada: a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
+          <t>No subitem b) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H46" s="9" t="b">
@@ -6521,7 +6244,7 @@
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>MR074</t>
+          <t>MR083</t>
         </is>
       </c>
       <c r="B47" s="9" t="inlineStr">
@@ -6531,25 +6254,25 @@
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="D47" s="9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>AV128</t>
+          <t>AV66 &amp; ~AV136</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>AV128</t>
+          <t>AV66</t>
         </is>
       </c>
       <c r="G47" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
+          <t>No subitem c) do item 2203, não houve declaração afirmativa quanto à prática avaliada: o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H47" s="9" t="b">
@@ -6559,7 +6282,7 @@
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>MR075</t>
+          <t>MR084</t>
         </is>
       </c>
       <c r="B48" s="9" t="inlineStr">
@@ -6569,25 +6292,25 @@
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="D48" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>AV59 &amp; ~AV129</t>
+          <t>AV136</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>AV59</t>
+          <t>AV136</t>
         </is>
       </c>
       <c r="G48" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2203, não houve declaração afirmativa quanto à prática avaliada: mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
+          <t>No subitem c) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H48" s="9" t="b">
@@ -6597,7 +6320,7 @@
     <row r="49" ht="45" customHeight="1">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>MR076</t>
+          <t>MR085</t>
         </is>
       </c>
       <c r="B49" s="9" t="inlineStr">
@@ -6607,25 +6330,25 @@
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="D49" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>AV129</t>
+          <t>AV67 &amp; ~AV137</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>AV129</t>
+          <t>AV67</t>
         </is>
       </c>
       <c r="G49" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
+          <t>No subitem a) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu regras para a priorização e o escalamento de incidentes</t>
         </is>
       </c>
       <c r="H49" s="9" t="b">
@@ -6635,7 +6358,7 @@
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>MR077</t>
+          <t>MR086</t>
         </is>
       </c>
       <c r="B50" s="9" t="inlineStr">
@@ -6645,25 +6368,25 @@
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="D50" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>AV62 &amp; ~AV132</t>
+          <t>AV137</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>AV62</t>
+          <t>AV137</t>
         </is>
       </c>
       <c r="G50" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
+          <t>No subitem a) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu regras para a priorização e o escalamento de incidentes</t>
         </is>
       </c>
       <c r="H50" s="9" t="b">
@@ -6673,7 +6396,7 @@
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>MR078</t>
+          <t>MR087</t>
         </is>
       </c>
       <c r="B51" s="9" t="inlineStr">
@@ -6683,25 +6406,25 @@
       </c>
       <c r="C51" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="D51" s="9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>AV132</t>
+          <t>AV70 &amp; ~AV140</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>AV132</t>
+          <t>AV70</t>
         </is>
       </c>
       <c r="G51" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
+          <t>No subitem d) do item 2204, não houve declaração afirmativa quanto à prática avaliada: o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H51" s="9" t="b">
@@ -6711,7 +6434,7 @@
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="9" t="inlineStr">
         <is>
-          <t>MR079</t>
+          <t>MR088</t>
         </is>
       </c>
       <c r="B52" s="9" t="inlineStr">
@@ -6721,25 +6444,25 @@
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="D52" s="9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>AV63 &amp; ~AV133</t>
+          <t>AV140</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>AV63</t>
+          <t>AV140</t>
         </is>
       </c>
       <c r="G52" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
+          <t>No subitem d) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H52" s="9" t="b">
@@ -6749,7 +6472,7 @@
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>MR080</t>
+          <t>MR089</t>
         </is>
       </c>
       <c r="B53" s="9" t="inlineStr">
@@ -6759,25 +6482,25 @@
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="D53" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>AV133</t>
+          <t>AV71 &amp; ~AV141</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>AV133</t>
+          <t>AV71</t>
         </is>
       </c>
       <c r="G53" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
+          <t>No subitem e) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
         </is>
       </c>
       <c r="H53" s="9" t="b">
@@ -6787,7 +6510,7 @@
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t>MR083</t>
+          <t>MR090</t>
         </is>
       </c>
       <c r="B54" s="9" t="inlineStr">
@@ -6797,25 +6520,25 @@
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="D54" s="9" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>AV66 &amp; ~AV136</t>
+          <t>AV141</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>AV66</t>
+          <t>AV141</t>
         </is>
       </c>
       <c r="G54" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2203, não houve declaração afirmativa quanto à prática avaliada: o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem e) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
         </is>
       </c>
       <c r="H54" s="9" t="b">
@@ -6825,35 +6548,35 @@
     <row r="55" ht="45" customHeight="1">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>MR084</t>
+          <t>MR091</t>
         </is>
       </c>
       <c r="B55" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D55" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>AV136</t>
+          <t>AV73 &amp; ~AV143</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>AV136</t>
+          <t>AV73</t>
         </is>
       </c>
       <c r="G55" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem a) do item 2801, não houve declaração afirmativa quanto à prática avaliada: o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
         </is>
       </c>
       <c r="H55" s="9" t="b">
@@ -6863,35 +6586,35 @@
     <row r="56" ht="45" customHeight="1">
       <c r="A56" s="9" t="inlineStr">
         <is>
-          <t>MR085</t>
+          <t>MR092</t>
         </is>
       </c>
       <c r="B56" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D56" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>AV67 &amp; ~AV137</t>
+          <t>AV143</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>AV67</t>
+          <t>AV143</t>
         </is>
       </c>
       <c r="G56" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu regras para a priorização e o escalamento de incidentes</t>
+          <t>No subitem a) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
         </is>
       </c>
       <c r="H56" s="9" t="b">
@@ -6901,35 +6624,35 @@
     <row r="57" ht="45" customHeight="1">
       <c r="A57" s="9" t="inlineStr">
         <is>
-          <t>MR086</t>
+          <t>MR101</t>
         </is>
       </c>
       <c r="B57" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
         </is>
       </c>
       <c r="D57" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>AV137</t>
+          <t>AV78 &amp; ~AV148</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>AV137</t>
+          <t>AV78</t>
         </is>
       </c>
       <c r="G57" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu regras para a priorização e o escalamento de incidentes</t>
+          <t>No subitem a) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
         </is>
       </c>
       <c r="H57" s="9" t="b">
@@ -6939,35 +6662,35 @@
     <row r="58" ht="45" customHeight="1">
       <c r="A58" s="9" t="inlineStr">
         <is>
-          <t>MR087</t>
+          <t>MR102</t>
         </is>
       </c>
       <c r="B58" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
         </is>
       </c>
       <c r="D58" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>AV70 &amp; ~AV140</t>
+          <t>AV148</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>AV70</t>
+          <t>AV148</t>
         </is>
       </c>
       <c r="G58" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2204, não houve declaração afirmativa quanto à prática avaliada: o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem a) do item 2804, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
         </is>
       </c>
       <c r="H58" s="9" t="b">
@@ -6977,35 +6700,35 @@
     <row r="59" ht="45" customHeight="1">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>MR088</t>
+          <t>MR105</t>
         </is>
       </c>
       <c r="B59" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
         </is>
       </c>
       <c r="D59" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>AV140</t>
+          <t>AV80 &amp; ~AV150</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>AV140</t>
+          <t>AV80</t>
         </is>
       </c>
       <c r="G59" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem c) do item 2802, não houve declaração afirmativa quanto à prática avaliada: na elaboração do PCA são considerados os demais instrumentos de planejamento da organização</t>
         </is>
       </c>
       <c r="H59" s="9" t="b">
@@ -7015,35 +6738,35 @@
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="9" t="inlineStr">
         <is>
-          <t>MR089</t>
+          <t>MR106</t>
         </is>
       </c>
       <c r="B60" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C60" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
         </is>
       </c>
       <c r="D60" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>AV71 &amp; ~AV141</t>
+          <t>AV150</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>AV71</t>
+          <t>AV150</t>
         </is>
       </c>
       <c r="G60" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
+          <t>No subitem c) do item 2802, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que na elaboração do PCA são considerados os demais instrumentos de planejamento da organização</t>
         </is>
       </c>
       <c r="H60" s="9" t="b">
@@ -7053,35 +6776,35 @@
     <row r="61" ht="45" customHeight="1">
       <c r="A61" s="9" t="inlineStr">
         <is>
-          <t>MR090</t>
+          <t>MR109</t>
         </is>
       </c>
       <c r="B61" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C61" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
         </is>
       </c>
       <c r="D61" s="9" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>AV141</t>
+          <t>AV82</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>AV141</t>
+          <t>AV82</t>
         </is>
       </c>
       <c r="G61" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
+          <t>No subitem b) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de TI executadas no exercício encontram-se previamente estabelecidas nos instrumentos de planejamento vigentes (PDTI/PEDTIC e PCA)</t>
         </is>
       </c>
       <c r="H61" s="9" t="b">
@@ -7091,7 +6814,7 @@
     <row r="62" ht="45" customHeight="1">
       <c r="A62" s="9" t="inlineStr">
         <is>
-          <t>MR091</t>
+          <t>MR110</t>
         </is>
       </c>
       <c r="B62" s="9" t="inlineStr">
@@ -7101,7 +6824,7 @@
       </c>
       <c r="C62" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
         </is>
       </c>
       <c r="D62" s="9" t="n">
@@ -7109,17 +6832,17 @@
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>AV73 &amp; ~AV143</t>
+          <t>AV83</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>AV73</t>
+          <t>AV83</t>
         </is>
       </c>
       <c r="G62" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2801, não houve declaração afirmativa quanto à prática avaliada: o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
+          <t>No subitem c) do item 2804, não houve declaração afirmativa quanto à prática avaliada: a fase de planejamento de cada contratação de TI é conduzida por uma Equipe de Planejamento da Contratação formalmente designada (composta, minimamente, por integrante requisitante e integrante técnico da área de TI)</t>
         </is>
       </c>
       <c r="H62" s="9" t="b">
@@ -7129,7 +6852,7 @@
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>MR092</t>
+          <t>MR111</t>
         </is>
       </c>
       <c r="B63" s="9" t="inlineStr">
@@ -7143,21 +6866,21 @@
         </is>
       </c>
       <c r="D63" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>AV143</t>
+          <t>AV152 &amp; ~AV153</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>AV143</t>
+          <t>AV152</t>
         </is>
       </c>
       <c r="G63" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
+          <t>No subitem b) do item 2801, não houve declaração afirmativa quanto à prática avaliada: são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
         </is>
       </c>
       <c r="H63" s="9" t="b">
@@ -7167,7 +6890,7 @@
     <row r="64" ht="45" customHeight="1">
       <c r="A64" s="9" t="inlineStr">
         <is>
-          <t>MR101</t>
+          <t>MR112</t>
         </is>
       </c>
       <c r="B64" s="9" t="inlineStr">
@@ -7177,25 +6900,25 @@
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D64" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>AV78 &amp; ~AV148</t>
+          <t>AV153</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>AV78</t>
+          <t>AV153</t>
         </is>
       </c>
       <c r="G64" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
+          <t>No subitem b) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
         </is>
       </c>
       <c r="H64" s="9" t="b">
@@ -7205,17 +6928,17 @@
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="9" t="inlineStr">
         <is>
-          <t>MR102</t>
+          <t>MR113</t>
         </is>
       </c>
       <c r="B65" s="9" t="inlineStr">
         <is>
-          <t>PA06</t>
+          <t>PA03</t>
         </is>
       </c>
       <c r="C65" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="D65" s="9" t="n">
@@ -7223,251 +6946,29 @@
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>AV148</t>
+          <t>AV154</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>AV148</t>
+          <t>AV154</t>
         </is>
       </c>
       <c r="G65" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2804, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
+          <t>No item 2102, a organização não declarou possuir plano de tecnologia da informação vigente, ainda que parcialmente adotado</t>
         </is>
       </c>
       <c r="H65" s="9" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="66" ht="30" customHeight="1">
-      <c r="A66" s="9" t="inlineStr">
-        <is>
-          <t>MR105</t>
-        </is>
-      </c>
-      <c r="B66" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C66" s="9" t="inlineStr">
-        <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
-        </is>
-      </c>
-      <c r="D66" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E66" s="9" t="inlineStr">
-        <is>
-          <t>AV80 &amp; ~AV150</t>
-        </is>
-      </c>
-      <c r="F66" s="9" t="inlineStr">
-        <is>
-          <t>AV80</t>
-        </is>
-      </c>
-      <c r="G66" s="9" t="inlineStr">
-        <is>
-          <t>No subitem c) do item 2802, não houve declaração afirmativa quanto à prática avaliada: na elaboração do PCA são considerados os demais instrumentos de planejamento da organização</t>
-        </is>
-      </c>
-      <c r="H66" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" ht="30" customHeight="1">
-      <c r="A67" s="9" t="inlineStr">
-        <is>
-          <t>MR106</t>
-        </is>
-      </c>
-      <c r="B67" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C67" s="9" t="inlineStr">
-        <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
-        </is>
-      </c>
-      <c r="D67" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E67" s="9" t="inlineStr">
-        <is>
-          <t>AV150</t>
-        </is>
-      </c>
-      <c r="F67" s="9" t="inlineStr">
-        <is>
-          <t>AV150</t>
-        </is>
-      </c>
-      <c r="G67" s="9" t="inlineStr">
-        <is>
-          <t>No subitem c) do item 2802, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que na elaboração do PCA são considerados os demais instrumentos de planejamento da organização</t>
-        </is>
-      </c>
-      <c r="H67" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68" ht="45" customHeight="1">
-      <c r="A68" s="9" t="inlineStr">
-        <is>
-          <t>MR109</t>
-        </is>
-      </c>
-      <c r="B68" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C68" s="9" t="inlineStr">
-        <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
-        </is>
-      </c>
-      <c r="D68" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="E68" s="9" t="inlineStr">
-        <is>
-          <t>AV82</t>
-        </is>
-      </c>
-      <c r="F68" s="9" t="inlineStr">
-        <is>
-          <t>AV82</t>
-        </is>
-      </c>
-      <c r="G68" s="9" t="inlineStr">
-        <is>
-          <t>No subitem b) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de TI executadas no exercício encontram-se previamente estabelecidas nos instrumentos de planejamento vigentes (PDTI/PEDTIC e PCA)</t>
-        </is>
-      </c>
-      <c r="H68" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69" ht="60" customHeight="1">
-      <c r="A69" s="9" t="inlineStr">
-        <is>
-          <t>MR110</t>
-        </is>
-      </c>
-      <c r="B69" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C69" s="9" t="inlineStr">
-        <is>
-          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
-        </is>
-      </c>
-      <c r="D69" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E69" s="9" t="inlineStr">
-        <is>
-          <t>AV83</t>
-        </is>
-      </c>
-      <c r="F69" s="9" t="inlineStr">
-        <is>
-          <t>AV83</t>
-        </is>
-      </c>
-      <c r="G69" s="9" t="inlineStr">
-        <is>
-          <t>No subitem c) do item 2804, não houve declaração afirmativa quanto à prática avaliada: a fase de planejamento de cada contratação de TI é conduzida por uma Equipe de Planejamento da Contratação formalmente designada (composta, minimamente, por integrante requisitante e integrante técnico da área de TI)</t>
-        </is>
-      </c>
-      <c r="H69" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70" ht="45" customHeight="1">
-      <c r="A70" s="9" t="inlineStr">
-        <is>
-          <t>MR111</t>
-        </is>
-      </c>
-      <c r="B70" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C70" s="9" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="D70" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E70" s="9" t="inlineStr">
-        <is>
-          <t>AV152 &amp; ~AV153</t>
-        </is>
-      </c>
-      <c r="F70" s="9" t="inlineStr">
-        <is>
-          <t>AV152</t>
-        </is>
-      </c>
-      <c r="G70" s="9" t="inlineStr">
-        <is>
-          <t>No subitem b) do item 2801, não houve declaração afirmativa quanto à prática avaliada: são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
-        </is>
-      </c>
-      <c r="H70" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="71" ht="45" customHeight="1">
-      <c r="A71" s="9" t="inlineStr">
-        <is>
-          <t>MR112</t>
-        </is>
-      </c>
-      <c r="B71" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C71" s="9" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="D71" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="E71" s="9" t="inlineStr">
-        <is>
-          <t>AV153</t>
-        </is>
-      </c>
-      <c r="F71" s="9" t="inlineStr">
-        <is>
-          <t>AV153</t>
-        </is>
-      </c>
-      <c r="G71" s="9" t="inlineStr">
-        <is>
-          <t>No subitem b) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
-        </is>
-      </c>
-      <c r="H71" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
+    <row r="66" ht="30" customHeight="1"/>
+    <row r="67" ht="30" customHeight="1"/>
+    <row r="68" ht="45" customHeight="1"/>
+    <row r="69" ht="60" customHeight="1"/>
+    <row r="70" ht="45" customHeight="1"/>
+    <row r="71" ht="45" customHeight="1"/>
     <row r="72" ht="30" customHeight="1"/>
     <row r="73" ht="30" customHeight="1"/>
     <row r="74" ht="30" customHeight="1"/>
@@ -7511,7 +7012,7 @@
     <row r="112" ht="45" customHeight="1"/>
     <row r="113" ht="45" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A3:H71"/>
+  <autoFilter ref="A3:H65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7522,7 +7023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7637,11 +7138,37 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="57" customHeight="1"/>
+    <row r="6" ht="57" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>VT06</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>questionario</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>existe_plano_ti</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>(q2102 == 'Adota parcialmente.') | (q2102 == 'Adota em maior parte ou totalmente.')</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>Indica que a organização declarou possuir plano de TIC vigente, ao menos parcialmente adotado.</t>
+        </is>
+      </c>
+    </row>
     <row r="7" ht="28.5" customHeight="1"/>
     <row r="8" ht="42.75" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A3:E5"/>
+  <autoFilter ref="A3:E6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>

<commit_message>
Revisa a Questão 4 da matriz e do mapa
</commit_message>
<xml_diff>
--- a/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
+++ b/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
@@ -15,8 +15,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Fontes de Informação'!$A$3:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Procedimentos de Auditoria'!$A$3:$E$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ações de Verificação'!$A$3:$P$67</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Motivos do Relatório'!$A$3:$H$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ações de Verificação'!$A$3:$P$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Motivos do Relatório'!$A$3:$H$62</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Variáveis Temporárias'!$A$3:$E$6</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -619,12 +619,12 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>Procedimento para verificar a questão Q4: A organização dispõe de capacidade institucional mínima, em termos de força de trabalho, funções e vínculos, para planejar, gerir, proteger, contratar, fiscalizar e sustentar a TIC e a segurança da informação de forma adequada às suas necessidades institucionais?</t>
+          <t>Procedimento para verificar a questão Q4: A organização dispõe de mecanismos mínimos para estruturar e dimensionar sua força de trabalho de TIC e segurança da informação, formalizar funções e preservar capacidade interna nos modelos de operação predominantemente terceirizados?</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>((AV26 &amp; AV25) | (AV29 | AV103) | ((AV31 | AV105) | (AV33 | AV107)) | (AV45 &amp; AV46))</t>
+          <t>((AV26 &amp; AV25) | AV29 | (AV31 | AV33) | (AV45 &amp; AV46))</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
@@ -632,7 +632,7 @@
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>Capacidade institucional insuficiente para sustentar a gestão de TIC e segurança da informação</t>
+          <t>Capacidade institucional de pessoal de TIC e segurança da informação insuficientemente estruturada ou dimensionada</t>
         </is>
       </c>
     </row>
@@ -699,7 +699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P67"/>
+  <dimension ref="A1:P64"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="K22" s="1" t="inlineStr">
         <is>
-          <t>~(f) Inexistente / Informal: Não há área de TI formalmente instituída no organograma da organização.)</t>
+          <t>(a) Centralizada Interna: Há uma área de TI centralizada e formal que atende toda a organização, utilizando equipe técnica majoritariamente própria (servidores). | b) Centralizada Terceirizada: Há uma área de TI centralizada e formal que faz a gestão, mas a execução operacional/técnica é predominantemente terceirizada (ex: fábricas de software, service desk). | d) Descentralizada: Diferentes secretarias, unidades ou setores possuem autonomia e mantêm suas próprias equipes, contratos ou infraestruturas de TI de forma independente. | e) Híbrida: Existe uma TI central formal para diretrizes e infraestrutura corporativa, mas as áreas de negócio possuem equipes próprias para sustentar sistemas específicos.)</t>
         </is>
       </c>
       <c r="L22" s="1" t="n"/>
@@ -1968,7 +1968,7 @@
       <c r="I23" s="1" t="n"/>
       <c r="J23" s="1" t="inlineStr">
         <is>
-          <t>A organização não definiu o quantitativo necessário de pessoal de TIC e segurança da informação.</t>
+          <t>Ausência ou insuficiência de definição documentada do quantitativo necessário de pessoal de TIC e segurança da informação.</t>
         </is>
       </c>
       <c r="K23" s="1" t="inlineStr">
@@ -2122,7 +2122,7 @@
       <c r="G26" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO07.06 - Gerenciar pessoal contratado: controlar o uso de pessoal terceirizado ou externo, preservando responsabilização, supervisão e retenção de conhecimento.
-Lei nº 14.133/2021, art. 117: dever de acompanhamento e fiscalização da execução contratual por representantes da Administração especialmente designados.</t>
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens I.10.11, III.9.11 e IV.11.3 – Referência para avaliação da estrutura de recursos humanos de TIC quanto à suficiência quantitativa e qualitativa e à preservação de capacidade interna em atividades de planejamento, coordenação, fiscalização e controle.</t>
         </is>
       </c>
       <c r="H26" s="1" t="inlineStr">
@@ -2133,7 +2133,7 @@
       <c r="I26" s="1" t="n"/>
       <c r="J26" s="1" t="inlineStr">
         <is>
-          <t>Dependência externa relevante sem capacidade interna suficiente para coordenar e fiscalizar a TIC.</t>
+          <t>Operação de TIC predominantemente terceirizada sem profissionais internos de TIC.</t>
         </is>
       </c>
       <c r="K26" s="1" t="inlineStr">
@@ -2145,13 +2145,13 @@
       <c r="M26" s="1" t="n"/>
       <c r="N26" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O26" s="1" t="n"/>
       <c r="P26" s="1" t="inlineStr">
         <is>
-          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente para coordenar, aprovar tecnicamente e fiscalizar as atividades e os contratos de TIC executados predominantemente por terceiros, preservando responsabilização e retenção de conhecimento</t>
+          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente para coordenar, supervisionar e fiscalizar as atividades e os contratos de TIC executados predominantemente por terceiros, preservando responsabilização e retenção de conhecimento</t>
         </is>
       </c>
     </row>
@@ -2177,7 +2177,7 @@
       <c r="G27" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO07.06 - Gerenciar pessoal contratado: controlar o uso de pessoal terceirizado ou externo, preservando responsabilização, supervisão e retenção de conhecimento.
-Lei nº 14.133/2021, art. 117: dever de acompanhamento e fiscalização da execução contratual por representantes da Administração especialmente designados.</t>
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens I.10.11, III.9.11 e IV.11.3 – Referência para avaliação da estrutura de recursos humanos de TIC quanto à suficiência quantitativa e qualitativa e à preservação de capacidade interna em atividades de planejamento, coordenação, fiscalização e controle.</t>
         </is>
       </c>
       <c r="H27" s="1" t="inlineStr">
@@ -2188,7 +2188,7 @@
       <c r="I27" s="1" t="n"/>
       <c r="J27" s="1" t="inlineStr">
         <is>
-          <t>Dependência externa relevante sem capacidade interna suficiente para coordenar e fiscalizar a TIC.</t>
+          <t>Operação de TIC predominantemente terceirizada sem profissionais internos de TIC.</t>
         </is>
       </c>
       <c r="K27" s="1" t="inlineStr">
@@ -2200,13 +2200,13 @@
       <c r="M27" s="1" t="n"/>
       <c r="N27" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O27" s="1" t="n"/>
       <c r="P27" s="1" t="inlineStr">
         <is>
-          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente para coordenar, aprovar tecnicamente e fiscalizar as atividades e os contratos de TIC executados predominantemente por terceiros, preservando responsabilização e retenção de conhecimento</t>
+          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente para coordenar, supervisionar e fiscalizar as atividades e os contratos de TIC executados predominantemente por terceiros, preservando responsabilização e retenção de conhecimento</t>
         </is>
       </c>
     </row>
@@ -3204,7 +3204,7 @@
     <row r="46" ht="113.45" customHeight="1">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>AV103</t>
+          <t>AV124</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -3217,13 +3217,13 @@
       <c r="E46" s="1" t="n"/>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>q2703ext[C]</t>
+          <t>q2201ext[A]</t>
         </is>
       </c>
       <c r="G46" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO07.05 - Planejar e monitorar o uso de recursos humanos de TI e de negócio: planejar, alocar e acompanhar capacidade de pessoal para iniciativas, operações e serviços de TIC.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6.5 - O PDTI deve contemplar o quantitativo necessário ou ideal para a força de trabalho em TI.</t>
+          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
+ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.</t>
         </is>
       </c>
       <c r="H46" s="1" t="inlineStr">
@@ -3234,7 +3234,7 @@
       <c r="I46" s="1" t="n"/>
       <c r="J46" s="1" t="inlineStr">
         <is>
-          <t>A organização não definiu o quantitativo necessário de pessoal de TIC e segurança da informação.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="K46" s="1" t="inlineStr">
@@ -3252,14 +3252,14 @@
       <c r="O46" s="1" t="n"/>
       <c r="P46" s="1" t="inlineStr">
         <is>
-          <t>estime e mantenha atualizado o quantitativo necessário de pessoal de TIC e segurança da informação, considerando o porte e a complexidade da organização, os serviços críticos, os sistemas mantidos, as contratações vigentes e os riscos relevantes</t>
+          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
         </is>
       </c>
     </row>
     <row r="47" ht="113.45" customHeight="1">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>AV105</t>
+          <t>AV125</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -3272,13 +3272,13 @@
       <c r="E47" s="1" t="n"/>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>q2708[B]</t>
+          <t>q2201ext[B]</t>
         </is>
       </c>
       <c r="G47" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
-COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
+          <t>ITIL 4, prática de gerenciamento do catálogo de serviços: manter fonte única de informações consistentes sobre serviços e ofertas de serviço, disponível para usuários e equipes de suporte.
+COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.</t>
         </is>
       </c>
       <c r="H47" s="1" t="inlineStr">
@@ -3289,7 +3289,7 @@
       <c r="I47" s="1" t="n"/>
       <c r="J47" s="1" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="K47" s="1" t="inlineStr">
@@ -3307,14 +3307,14 @@
       <c r="O47" s="1" t="n"/>
       <c r="P47" s="1" t="inlineStr">
         <is>
-          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
+          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
         </is>
       </c>
     </row>
     <row r="48" ht="113.45" customHeight="1">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>AV107</t>
+          <t>AV126</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -3327,13 +3327,13 @@
       <c r="E48" s="1" t="n"/>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>q2708[D]</t>
+          <t>q2201ext[C]</t>
         </is>
       </c>
       <c r="G48" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
-COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
+          <t>ITIL 4, prática de gerenciamento do catálogo de serviços: manter fonte única de informações consistentes sobre serviços e ofertas de serviço, disponível para usuários e equipes de suporte.
+COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.</t>
         </is>
       </c>
       <c r="H48" s="1" t="inlineStr">
@@ -3344,7 +3344,7 @@
       <c r="I48" s="1" t="n"/>
       <c r="J48" s="1" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="K48" s="1" t="inlineStr">
@@ -3362,14 +3362,14 @@
       <c r="O48" s="1" t="n"/>
       <c r="P48" s="1" t="inlineStr">
         <is>
-          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
+          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
         </is>
       </c>
     </row>
     <row r="49" ht="113.45" customHeight="1">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>AV124</t>
+          <t>AV127</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -3382,7 +3382,7 @@
       <c r="E49" s="1" t="n"/>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[A]</t>
+          <t>q2201ext[D]</t>
         </is>
       </c>
       <c r="G49" s="1" t="inlineStr">
@@ -3424,7 +3424,7 @@
     <row r="50" ht="113.45" customHeight="1">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>AV125</t>
+          <t>AV128</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -3437,13 +3437,13 @@
       <c r="E50" s="1" t="n"/>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[B]</t>
+          <t>q2201ext[E]</t>
         </is>
       </c>
       <c r="G50" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento do catálogo de serviços: manter fonte única de informações consistentes sobre serviços e ofertas de serviço, disponível para usuários e equipes de suporte.
-COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.</t>
+          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
+ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.</t>
         </is>
       </c>
       <c r="H50" s="1" t="inlineStr">
@@ -3454,7 +3454,7 @@
       <c r="I50" s="1" t="n"/>
       <c r="J50" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="K50" s="1" t="inlineStr">
@@ -3472,14 +3472,14 @@
       <c r="O50" s="1" t="n"/>
       <c r="P50" s="1" t="inlineStr">
         <is>
-          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
+          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
         </is>
       </c>
     </row>
     <row r="51" ht="113.45" customHeight="1">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>AV126</t>
+          <t>AV129</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -3492,13 +3492,13 @@
       <c r="E51" s="1" t="n"/>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[C]</t>
+          <t>q2203ext[A]</t>
         </is>
       </c>
       <c r="G51" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento do catálogo de serviços: manter fonte única de informações consistentes sobre serviços e ofertas de serviço, disponível para usuários e equipes de suporte.
-COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.</t>
+          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
+Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
         </is>
       </c>
       <c r="H51" s="1" t="inlineStr">
@@ -3509,7 +3509,7 @@
       <c r="I51" s="1" t="n"/>
       <c r="J51" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="K51" s="1" t="inlineStr">
@@ -3521,20 +3521,20 @@
       <c r="M51" s="1" t="n"/>
       <c r="N51" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O51" s="1" t="n"/>
       <c r="P51" s="1" t="inlineStr">
         <is>
-          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
+          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
         </is>
       </c>
     </row>
     <row r="52" ht="113.45" customHeight="1">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>AV127</t>
+          <t>AV132</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -3547,13 +3547,13 @@
       <c r="E52" s="1" t="n"/>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[D]</t>
+          <t>q2504ext[A]</t>
         </is>
       </c>
       <c r="G52" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
-ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.</t>
+          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
+Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
         </is>
       </c>
       <c r="H52" s="1" t="inlineStr">
@@ -3564,7 +3564,7 @@
       <c r="I52" s="1" t="n"/>
       <c r="J52" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="K52" s="1" t="inlineStr">
@@ -3576,20 +3576,20 @@
       <c r="M52" s="1" t="n"/>
       <c r="N52" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O52" s="1" t="n"/>
       <c r="P52" s="1" t="inlineStr">
         <is>
-          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
+          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
         </is>
       </c>
     </row>
     <row r="53" ht="113.45" customHeight="1">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>AV128</t>
+          <t>AV133</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -3602,13 +3602,13 @@
       <c r="E53" s="1" t="n"/>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[E]</t>
+          <t>q2504ext[B]</t>
         </is>
       </c>
       <c r="G53" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
-ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.</t>
+          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
+Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
         </is>
       </c>
       <c r="H53" s="1" t="inlineStr">
@@ -3619,7 +3619,7 @@
       <c r="I53" s="1" t="n"/>
       <c r="J53" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="K53" s="1" t="inlineStr">
@@ -3631,20 +3631,20 @@
       <c r="M53" s="1" t="n"/>
       <c r="N53" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O53" s="1" t="n"/>
       <c r="P53" s="1" t="inlineStr">
         <is>
-          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
+          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
         </is>
       </c>
     </row>
     <row r="54" ht="113.45" customHeight="1">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>AV129</t>
+          <t>AV136</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -3657,13 +3657,13 @@
       <c r="E54" s="1" t="n"/>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>q2203ext[A]</t>
+          <t>q2203ext[C]</t>
         </is>
       </c>
       <c r="G54" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
+          <t>ITIL 4, prática de gerenciamento de configuração de serviço: assegurar informações precisas e confiáveis sobre itens de configuração e seus relacionamentos com serviços, sistemas e infraestrutura.
+COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.</t>
         </is>
       </c>
       <c r="H54" s="1" t="inlineStr">
@@ -3674,7 +3674,7 @@
       <c r="I54" s="1" t="n"/>
       <c r="J54" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="K54" s="1" t="inlineStr">
@@ -3686,20 +3686,20 @@
       <c r="M54" s="1" t="n"/>
       <c r="N54" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O54" s="1" t="n"/>
       <c r="P54" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
+          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
         </is>
       </c>
     </row>
     <row r="55" ht="113.45" customHeight="1">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>AV132</t>
+          <t>AV137</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -3712,13 +3712,13 @@
       <c r="E55" s="1" t="n"/>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>q2504ext[A]</t>
+          <t>q2204ext[A]</t>
         </is>
       </c>
       <c r="G55" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
         </is>
       </c>
       <c r="H55" s="1" t="inlineStr">
@@ -3729,7 +3729,7 @@
       <c r="I55" s="1" t="n"/>
       <c r="J55" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="K55" s="1" t="inlineStr">
@@ -3741,20 +3741,20 @@
       <c r="M55" s="1" t="n"/>
       <c r="N55" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O55" s="1" t="n"/>
       <c r="P55" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
     </row>
     <row r="56" ht="113.45" customHeight="1">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>AV133</t>
+          <t>AV140</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -3767,13 +3767,13 @@
       <c r="E56" s="1" t="n"/>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>q2504ext[B]</t>
+          <t>q2204ext[D]</t>
         </is>
       </c>
       <c r="G56" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
         </is>
       </c>
       <c r="H56" s="1" t="inlineStr">
@@ -3784,7 +3784,7 @@
       <c r="I56" s="1" t="n"/>
       <c r="J56" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="K56" s="1" t="inlineStr">
@@ -3796,20 +3796,20 @@
       <c r="M56" s="1" t="n"/>
       <c r="N56" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O56" s="1" t="n"/>
       <c r="P56" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
     </row>
     <row r="57" ht="90.95" customHeight="1">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>AV136</t>
+          <t>AV141</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -3822,13 +3822,13 @@
       <c r="E57" s="1" t="n"/>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>q2203ext[C]</t>
+          <t>q2204ext[E]</t>
         </is>
       </c>
       <c r="G57" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de configuração de serviço: assegurar informações precisas e confiáveis sobre itens de configuração e seus relacionamentos com serviços, sistemas e infraestrutura.
-COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.</t>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
         </is>
       </c>
       <c r="H57" s="1" t="inlineStr">
@@ -3839,7 +3839,7 @@
       <c r="I57" s="1" t="n"/>
       <c r="J57" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="K57" s="1" t="inlineStr">
@@ -3857,14 +3857,14 @@
       <c r="O57" s="1" t="n"/>
       <c r="P57" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
     </row>
     <row r="58" ht="90.95" customHeight="1">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>AV137</t>
+          <t>AV143</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -3877,13 +3877,13 @@
       <c r="E58" s="1" t="n"/>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>q2204ext[A]</t>
+          <t>q2801ext[A]</t>
         </is>
       </c>
       <c r="G58" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
+          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
         </is>
       </c>
       <c r="H58" s="1" t="inlineStr">
@@ -3894,7 +3894,7 @@
       <c r="I58" s="1" t="n"/>
       <c r="J58" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="K58" s="1" t="inlineStr">
@@ -3906,20 +3906,20 @@
       <c r="M58" s="1" t="n"/>
       <c r="N58" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O58" s="1" t="n"/>
       <c r="P58" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
+          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
         </is>
       </c>
     </row>
     <row r="59" ht="90.95" customHeight="1">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>AV140</t>
+          <t>AV148</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -3932,13 +3932,14 @@
       <c r="E59" s="1" t="n"/>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>q2204ext[D]</t>
+          <t>q2804[A]</t>
         </is>
       </c>
       <c r="G59" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
+          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+COBIT 2019, BAI02.04 - Obter aprovação dos requisitos da solução: obter aprovação formal dos requisitos funcionais, técnicos, de segurança e de conformidade antes de prosseguir com a solução.
+Instrução Normativa SGD/ME nº 94, de 23 de dezembro de 2022, art. 1º, § 1º: como referência de boa prática, a aplicação de ritos formais de contratação de TIC pode ser facultada para contratações diretas por dispensa em razão do valor (inciso II do art. 75 da Lei nº 14.133/2021), indicando a possibilidade de fluxos simplificados para aquisições de baixa complexidade ou valor.</t>
         </is>
       </c>
       <c r="H59" s="1" t="inlineStr">
@@ -3949,7 +3950,7 @@
       <c r="I59" s="1" t="n"/>
       <c r="J59" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
         </is>
       </c>
       <c r="K59" s="1" t="inlineStr">
@@ -3967,14 +3968,14 @@
       <c r="O59" s="1" t="n"/>
       <c r="P59" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
+          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo fluxos simplificados para contratações de baixa complexidade ou baixo valor, desde que preservada análise técnica mínima compatível com o risco da contratação</t>
         </is>
       </c>
     </row>
     <row r="60" ht="79.90000000000001" customHeight="1">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>AV141</t>
+          <t>AV150</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -3987,13 +3988,13 @@
       <c r="E60" s="1" t="n"/>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>q2204ext[E]</t>
+          <t>q2802ext[C]</t>
         </is>
       </c>
       <c r="G60" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
+          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Art. 18, caput e §1º, incisos I, IV, V, VIII, IX, X e XIII, da Lei 14.133/2021: fase preparatória caracterizada pelo planejamento, compatibilização com o plano de contratações anual e elementos mínimos do estudo técnico preliminar.</t>
         </is>
       </c>
       <c r="H60" s="1" t="inlineStr">
@@ -4004,7 +4005,7 @@
       <c r="I60" s="1" t="n"/>
       <c r="J60" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
         </is>
       </c>
       <c r="K60" s="1" t="inlineStr">
@@ -4016,25 +4017,25 @@
       <c r="M60" s="1" t="n"/>
       <c r="N60" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O60" s="1" t="n"/>
       <c r="P60" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
+          <t>integre as contratações de TIC com os instrumentos de planejamento da organização e com o Plano de Contratações Anual, quando elaborado, justificando as situações excepcionais</t>
         </is>
       </c>
     </row>
     <row r="61" ht="79.90000000000001" customHeight="1">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>AV143</t>
+          <t>AV152</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
-          <t>avaliacao_evidencias_ajustes</t>
+          <t>questionario</t>
         </is>
       </c>
       <c r="C61" s="1" t="n"/>
@@ -4042,7 +4043,7 @@
       <c r="E61" s="1" t="n"/>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>q2801ext[A]</t>
+          <t>q2801ext[B]</t>
         </is>
       </c>
       <c r="G61" s="1" t="inlineStr">
@@ -4053,7 +4054,7 @@
       </c>
       <c r="H61" s="1" t="inlineStr">
         <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+          <t>Resposta negativa ao detalhamento b) do item 2801 do Questionário, para verificar se são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
         </is>
       </c>
       <c r="I61" s="1" t="n"/>
@@ -4064,7 +4065,7 @@
       </c>
       <c r="K61" s="1" t="inlineStr">
         <is>
-          <t>Não conforme</t>
+          <t>(Não | N/A)</t>
         </is>
       </c>
       <c r="L61" s="1" t="n"/>
@@ -4084,7 +4085,7 @@
     <row r="62" ht="90.95" customHeight="1">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>AV148</t>
+          <t>AV153</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -4097,14 +4098,13 @@
       <c r="E62" s="1" t="n"/>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>q2804[A]</t>
+          <t>q2801ext[B]</t>
         </is>
       </c>
       <c r="G62" s="1" t="inlineStr">
         <is>
           <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-COBIT 2019, BAI02.04 - Obter aprovação dos requisitos da solução: obter aprovação formal dos requisitos funcionais, técnicos, de segurança e de conformidade antes de prosseguir com a solução.
-Instrução Normativa SGD/ME nº 94, de 23 de dezembro de 2022, art. 1º, § 1º: como referência de boa prática, a aplicação de ritos formais de contratação de TIC pode ser facultada para contratações diretas por dispensa em razão do valor (inciso II do art. 75 da Lei nº 14.133/2021), indicando a possibilidade de fluxos simplificados para aquisições de baixa complexidade ou valor.</t>
+Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
         </is>
       </c>
       <c r="H62" s="1" t="inlineStr">
@@ -4115,7 +4115,7 @@
       <c r="I62" s="1" t="n"/>
       <c r="J62" s="1" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="K62" s="1" t="inlineStr">
@@ -4127,25 +4127,25 @@
       <c r="M62" s="1" t="n"/>
       <c r="N62" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O62" s="1" t="n"/>
       <c r="P62" s="1" t="inlineStr">
         <is>
-          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo fluxos simplificados para contratações de baixa complexidade ou baixo valor, desde que preservada análise técnica mínima compatível com o risco da contratação</t>
+          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
         </is>
       </c>
     </row>
     <row r="63" ht="90.95" customHeight="1">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>AV150</t>
+          <t>AV154</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
-          <t>avaliacao_evidencias_ajustes</t>
+          <t>questionario</t>
         </is>
       </c>
       <c r="C63" s="1" t="n"/>
@@ -4153,29 +4153,30 @@
       <c r="E63" s="1" t="n"/>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>q2802ext[C]</t>
+          <t>existe_plano_ti</t>
         </is>
       </c>
       <c r="G63" s="1" t="inlineStr">
         <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 18, caput e §1º, incisos I, IV, V, VIII, IX, X e XIII, da Lei 14.133/2021: fase preparatória caracterizada pelo planejamento, compatibilização com o plano de contratações anual e elementos mínimos do estudo técnico preliminar.</t>
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H63" s="1" t="inlineStr">
         <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+          <t>Resposta ao item 2102 que não caracteriza a existência de plano de TIC vigente, ainda que parcialmente adotado</t>
         </is>
       </c>
       <c r="I63" s="1" t="n"/>
       <c r="J63" s="1" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="K63" s="1" t="inlineStr">
         <is>
-          <t>Não conforme</t>
+          <t>False</t>
         </is>
       </c>
       <c r="L63" s="1" t="n"/>
@@ -4188,14 +4189,14 @@
       <c r="O63" s="1" t="n"/>
       <c r="P63" s="1" t="inlineStr">
         <is>
-          <t>integre as contratações de TIC com os instrumentos de planejamento da organização e com o Plano de Contratações Anual, quando elaborado, justificando as situações excepcionais</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
     <row r="64" ht="90.95" customHeight="1">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>AV152</t>
+          <t>AV155</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -4208,29 +4209,26 @@
       <c r="E64" s="1" t="n"/>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>q2801ext[B]</t>
+          <t>existe_plano_ti</t>
         </is>
       </c>
       <c r="G64" s="1" t="inlineStr">
         <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H64" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento b) do item 2801 do Questionário, para verificar se são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+          <t>Plano de TIC vigente declarado no item 2102, ao menos parcialmente adotado</t>
         </is>
       </c>
       <c r="I64" s="1" t="n"/>
-      <c r="J64" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
+      <c r="J64" s="1" t="n"/>
       <c r="K64" s="1" t="inlineStr">
         <is>
-          <t>(Não | N/A)</t>
+          <t>True</t>
         </is>
       </c>
       <c r="L64" s="1" t="n"/>
@@ -4243,173 +4241,13 @@
       <c r="O64" s="1" t="n"/>
       <c r="P64" s="1" t="inlineStr">
         <is>
-          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="90.95" customHeight="1">
-      <c r="A65" s="1" t="inlineStr">
-        <is>
-          <t>AV153</t>
-        </is>
-      </c>
-      <c r="B65" s="1" t="inlineStr">
-        <is>
-          <t>avaliacao_evidencias_ajustes</t>
-        </is>
-      </c>
-      <c r="C65" s="1" t="n"/>
-      <c r="D65" s="1" t="n"/>
-      <c r="E65" s="1" t="n"/>
-      <c r="F65" s="1" t="inlineStr">
-        <is>
-          <t>q2801ext[B]</t>
-        </is>
-      </c>
-      <c r="G65" s="1" t="inlineStr">
-        <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
-        </is>
-      </c>
-      <c r="H65" s="1" t="inlineStr">
-        <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
-        </is>
-      </c>
-      <c r="I65" s="1" t="n"/>
-      <c r="J65" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="K65" s="1" t="inlineStr">
-        <is>
-          <t>Não conforme</t>
-        </is>
-      </c>
-      <c r="L65" s="1" t="n"/>
-      <c r="M65" s="1" t="n"/>
-      <c r="N65" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O65" s="1" t="n"/>
-      <c r="P65" s="1" t="inlineStr">
-        <is>
-          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="90.95" customHeight="1">
-      <c r="A66" s="1" t="inlineStr">
-        <is>
-          <t>AV154</t>
-        </is>
-      </c>
-      <c r="B66" s="1" t="inlineStr">
-        <is>
-          <t>questionario</t>
-        </is>
-      </c>
-      <c r="C66" s="1" t="n"/>
-      <c r="D66" s="1" t="n"/>
-      <c r="E66" s="1" t="n"/>
-      <c r="F66" s="1" t="inlineStr">
-        <is>
-          <t>existe_plano_ti</t>
-        </is>
-      </c>
-      <c r="G66" s="1" t="inlineStr">
-        <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
-        </is>
-      </c>
-      <c r="H66" s="1" t="inlineStr">
-        <is>
-          <t>Resposta ao item 2102 que não caracteriza a existência de plano de TIC vigente, ainda que parcialmente adotado</t>
-        </is>
-      </c>
-      <c r="I66" s="1" t="n"/>
-      <c r="J66" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
-        </is>
-      </c>
-      <c r="K66" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="L66" s="1" t="n"/>
-      <c r="M66" s="1" t="n"/>
-      <c r="N66" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O66" s="1" t="n"/>
-      <c r="P66" s="1" t="inlineStr">
-        <is>
           <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="79.90000000000001" customHeight="1">
-      <c r="A67" s="1" t="inlineStr">
-        <is>
-          <t>AV155</t>
-        </is>
-      </c>
-      <c r="B67" s="1" t="inlineStr">
-        <is>
-          <t>questionario</t>
-        </is>
-      </c>
-      <c r="C67" s="1" t="n"/>
-      <c r="D67" s="1" t="n"/>
-      <c r="E67" s="1" t="n"/>
-      <c r="F67" s="1" t="inlineStr">
-        <is>
-          <t>existe_plano_ti</t>
-        </is>
-      </c>
-      <c r="G67" s="1" t="inlineStr">
-        <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
-        </is>
-      </c>
-      <c r="H67" s="1" t="inlineStr">
-        <is>
-          <t>Plano de TIC vigente declarado no item 2102, ao menos parcialmente adotado</t>
-        </is>
-      </c>
-      <c r="I67" s="1" t="n"/>
-      <c r="J67" s="1" t="n"/>
-      <c r="K67" s="1" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="L67" s="1" t="n"/>
-      <c r="M67" s="1" t="n"/>
-      <c r="N67" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O67" s="1" t="n"/>
-      <c r="P67" s="1" t="inlineStr">
-        <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
-        </is>
-      </c>
-    </row>
+    <row r="65" ht="90.95" customHeight="1"/>
+    <row r="66" ht="90.95" customHeight="1"/>
+    <row r="67" ht="79.90000000000001" customHeight="1"/>
     <row r="68" ht="79.90000000000001" customHeight="1"/>
     <row r="69" ht="79.90000000000001" customHeight="1"/>
     <row r="70" ht="90.95" customHeight="1"/>
@@ -4498,7 +4336,7 @@
     <row r="153" ht="23.85" customHeight="1"/>
     <row r="154" ht="23.85" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A3:P67"/>
+  <autoFilter ref="A3:P64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -4510,7 +4348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H65"/>
+  <dimension ref="A2:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5342,7 +5180,7 @@
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>A organização não definiu o quantitativo necessário de pessoal de TIC e segurança da informação.</t>
+          <t>Ausência ou insuficiência de definição documentada do quantitativo necessário de pessoal de TIC e segurança da informação.</t>
         </is>
       </c>
       <c r="D23" s="9" t="n">
@@ -5350,7 +5188,7 @@
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>AV29 &amp; ~AV103</t>
+          <t>AV29</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
@@ -5370,7 +5208,7 @@
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>MR046</t>
+          <t>MR047</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
@@ -5380,25 +5218,25 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>A organização não definiu o quantitativo necessário de pessoal de TIC e segurança da informação.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="D24" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>AV103</t>
+          <t>AV31</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>AV103</t>
+          <t>AV31</t>
         </is>
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2703, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu-se, de maneira documentada, um quantitativo necessário de pessoal da área de tecnologia da informação e segurança da informação</t>
+          <t>No subitem b) do item 2708, não houve declaração afirmativa quanto à prática avaliada: possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
         </is>
       </c>
       <c r="H24" s="9" t="b">
@@ -5408,7 +5246,7 @@
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>MR047</t>
+          <t>MR049</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
@@ -5422,21 +5260,21 @@
         </is>
       </c>
       <c r="D25" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>AV31 &amp; ~AV105</t>
+          <t>AV33</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>AV31</t>
+          <t>AV33</t>
         </is>
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2708, não houve declaração afirmativa quanto à prática avaliada: possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
+          <t>No subitem d) do item 2708, não houve declaração afirmativa quanto à prática avaliada: possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
         </is>
       </c>
       <c r="H25" s="9" t="b">
@@ -5446,7 +5284,7 @@
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>MR048</t>
+          <t>MR062</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
@@ -5456,25 +5294,25 @@
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Operação de TIC predominantemente terceirizada sem profissionais internos de TIC.</t>
         </is>
       </c>
       <c r="D26" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>AV105</t>
+          <t>AV45 &amp; AV46</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>AV105</t>
+          <t>AV45</t>
         </is>
       </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2708, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
+          <t>A organização informou modelo de operação de TIC com execução predominantemente terceirizada, o que levou à análise de sua capacidade interna de coordenação e fiscalização</t>
         </is>
       </c>
       <c r="H26" s="9" t="b">
@@ -5484,7 +5322,7 @@
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>MR049</t>
+          <t>MR063</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
@@ -5494,25 +5332,25 @@
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Operação de TIC predominantemente terceirizada sem profissionais internos de TIC.</t>
         </is>
       </c>
       <c r="D27" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>AV33 &amp; ~AV107</t>
+          <t>AV45 &amp; AV46</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>AV33</t>
+          <t>AV46</t>
         </is>
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2708, não houve declaração afirmativa quanto à prática avaliada: possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
+          <t>Não foram identificados profissionais internos de TIC para coordenar e fiscalizar a execução das atividades de tecnologia da informação</t>
         </is>
       </c>
       <c r="H27" s="9" t="b">
@@ -5522,35 +5360,35 @@
     <row r="28" ht="45" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>MR050</t>
+          <t>MR065</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA05</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D28" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>AV107</t>
+          <t>AV54 &amp; ~AV124</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>AV107</t>
+          <t>AV54</t>
         </is>
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2708, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
+          <t>No subitem a) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
         </is>
       </c>
       <c r="H28" s="9" t="b">
@@ -5560,35 +5398,35 @@
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>MR062</t>
+          <t>MR066</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA05</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Dependência externa relevante sem capacidade interna suficiente para coordenar e fiscalizar a TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D29" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>AV45 &amp; AV46</t>
+          <t>AV124</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>AV45</t>
+          <t>AV124</t>
         </is>
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>A organização informou modelo de operação de TIC com execução predominantemente terceirizada, o que levou à análise de sua capacidade interna de coordenação e fiscalização</t>
+          <t>No subitem a) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
         </is>
       </c>
       <c r="H29" s="9" t="b">
@@ -5598,35 +5436,35 @@
     <row r="30" ht="45" customHeight="1">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>MR063</t>
+          <t>MR067</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA05</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>Dependência externa relevante sem capacidade interna suficiente para coordenar e fiscalizar a TIC.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="D30" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>AV45 &amp; AV46</t>
+          <t>AV55 &amp; ~AV125</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>AV46</t>
+          <t>AV55</t>
         </is>
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>Não foram identificados profissionais internos de TIC para coordenar e fiscalizar a execução das atividades de tecnologia da informação</t>
+          <t>No subitem b) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
         </is>
       </c>
       <c r="H30" s="9" t="b">
@@ -5636,7 +5474,7 @@
     <row r="31" ht="45" customHeight="1">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>MR065</t>
+          <t>MR068</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
@@ -5646,25 +5484,25 @@
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="D31" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>AV54 &amp; ~AV124</t>
+          <t>AV125</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>AV54</t>
+          <t>AV125</t>
         </is>
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
+          <t>No subitem b) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
         </is>
       </c>
       <c r="H31" s="9" t="b">
@@ -5674,7 +5512,7 @@
     <row r="32" ht="45" customHeight="1">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>MR066</t>
+          <t>MR069</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
@@ -5684,7 +5522,7 @@
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="D32" s="9" t="n">
@@ -5692,17 +5530,17 @@
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>AV124</t>
+          <t>AV56 &amp; ~AV126</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>AV124</t>
+          <t>AV56</t>
         </is>
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
+          <t>No subitem c) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
         </is>
       </c>
       <c r="H32" s="9" t="b">
@@ -5712,7 +5550,7 @@
     <row r="33" ht="45" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>MR067</t>
+          <t>MR070</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
@@ -5726,21 +5564,21 @@
         </is>
       </c>
       <c r="D33" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>AV55 &amp; ~AV125</t>
+          <t>AV126</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>AV55</t>
+          <t>AV126</t>
         </is>
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
+          <t>No subitem c) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
         </is>
       </c>
       <c r="H33" s="9" t="b">
@@ -5750,7 +5588,7 @@
     <row r="34" ht="45" customHeight="1">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>MR068</t>
+          <t>MR071</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
@@ -5760,7 +5598,7 @@
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D34" s="9" t="n">
@@ -5768,17 +5606,17 @@
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>AV125</t>
+          <t>AV57 &amp; ~AV127</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>AV125</t>
+          <t>AV57</t>
         </is>
       </c>
       <c r="G34" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
+          <t>No subitem d) do item 2201, não houve declaração afirmativa quanto à prática avaliada: são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
         </is>
       </c>
       <c r="H34" s="9" t="b">
@@ -5788,7 +5626,7 @@
     <row r="35" ht="90" customHeight="1">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>MR069</t>
+          <t>MR072</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
@@ -5798,25 +5636,25 @@
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D35" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>AV56 &amp; ~AV126</t>
+          <t>AV127</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>AV56</t>
+          <t>AV127</t>
         </is>
       </c>
       <c r="G35" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
+          <t>No subitem d) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
         </is>
       </c>
       <c r="H35" s="9" t="b">
@@ -5826,7 +5664,7 @@
     <row r="36" ht="105" customHeight="1">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>MR070</t>
+          <t>MR073</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
@@ -5836,25 +5674,25 @@
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D36" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>AV126</t>
+          <t>AV58 &amp; ~AV128</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>AV126</t>
+          <t>AV58</t>
         </is>
       </c>
       <c r="G36" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
+          <t>No subitem e) do item 2201, não houve declaração afirmativa quanto à prática avaliada: a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
         </is>
       </c>
       <c r="H36" s="9" t="b">
@@ -5864,7 +5702,7 @@
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>MR071</t>
+          <t>MR074</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
@@ -5878,21 +5716,21 @@
         </is>
       </c>
       <c r="D37" s="9" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>AV57 &amp; ~AV127</t>
+          <t>AV128</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>AV57</t>
+          <t>AV128</t>
         </is>
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2201, não houve declaração afirmativa quanto à prática avaliada: são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
+          <t>No subitem e) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
         </is>
       </c>
       <c r="H37" s="9" t="b">
@@ -5902,7 +5740,7 @@
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>MR072</t>
+          <t>MR075</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
@@ -5912,25 +5750,25 @@
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="D38" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>AV127</t>
+          <t>AV59 &amp; ~AV129</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>AV127</t>
+          <t>AV59</t>
         </is>
       </c>
       <c r="G38" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
+          <t>No subitem a) do item 2203, não houve declaração afirmativa quanto à prática avaliada: mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
         </is>
       </c>
       <c r="H38" s="9" t="b">
@@ -5940,7 +5778,7 @@
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>MR073</t>
+          <t>MR076</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
@@ -5950,25 +5788,25 @@
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="D39" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>AV58 &amp; ~AV128</t>
+          <t>AV129</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>AV58</t>
+          <t>AV129</t>
         </is>
       </c>
       <c r="G39" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2201, não houve declaração afirmativa quanto à prática avaliada: a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
+          <t>No subitem a) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
         </is>
       </c>
       <c r="H39" s="9" t="b">
@@ -5978,7 +5816,7 @@
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>MR074</t>
+          <t>MR077</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
@@ -5988,25 +5826,25 @@
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
         </is>
       </c>
       <c r="D40" s="9" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>AV128</t>
+          <t>AV62 &amp; ~AV132</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>AV128</t>
+          <t>AV62</t>
         </is>
       </c>
       <c r="G40" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
+          <t>No subitem a) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H40" s="9" t="b">
@@ -6016,7 +5854,7 @@
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>MR075</t>
+          <t>MR078</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
@@ -6030,21 +5868,21 @@
         </is>
       </c>
       <c r="D41" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>AV59 &amp; ~AV129</t>
+          <t>AV132</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>AV59</t>
+          <t>AV132</t>
         </is>
       </c>
       <c r="G41" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2203, não houve declaração afirmativa quanto à prática avaliada: mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
+          <t>No subitem a) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H41" s="9" t="b">
@@ -6054,7 +5892,7 @@
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>MR076</t>
+          <t>MR079</t>
         </is>
       </c>
       <c r="B42" s="9" t="inlineStr">
@@ -6068,21 +5906,21 @@
         </is>
       </c>
       <c r="D42" s="9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>AV129</t>
+          <t>AV63 &amp; ~AV133</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>AV129</t>
+          <t>AV63</t>
         </is>
       </c>
       <c r="G42" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
+          <t>No subitem b) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H42" s="9" t="b">
@@ -6092,7 +5930,7 @@
     <row r="43" ht="45" customHeight="1">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>MR077</t>
+          <t>MR080</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
@@ -6106,21 +5944,21 @@
         </is>
       </c>
       <c r="D43" s="9" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>AV62 &amp; ~AV132</t>
+          <t>AV133</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>AV62</t>
+          <t>AV133</t>
         </is>
       </c>
       <c r="G43" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
+          <t>No subitem b) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H43" s="9" t="b">
@@ -6130,7 +5968,7 @@
     <row r="44" ht="45" customHeight="1">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>MR078</t>
+          <t>MR083</t>
         </is>
       </c>
       <c r="B44" s="9" t="inlineStr">
@@ -6140,25 +5978,25 @@
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="D44" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>AV132</t>
+          <t>AV66 &amp; ~AV136</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>AV132</t>
+          <t>AV66</t>
         </is>
       </c>
       <c r="G44" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
+          <t>No subitem c) do item 2203, não houve declaração afirmativa quanto à prática avaliada: o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H44" s="9" t="b">
@@ -6168,7 +6006,7 @@
     <row r="45" ht="45" customHeight="1">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>MR079</t>
+          <t>MR084</t>
         </is>
       </c>
       <c r="B45" s="9" t="inlineStr">
@@ -6178,25 +6016,25 @@
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="D45" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>AV63 &amp; ~AV133</t>
+          <t>AV136</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>AV63</t>
+          <t>AV136</t>
         </is>
       </c>
       <c r="G45" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
+          <t>No subitem c) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H45" s="9" t="b">
@@ -6206,7 +6044,7 @@
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>MR080</t>
+          <t>MR085</t>
         </is>
       </c>
       <c r="B46" s="9" t="inlineStr">
@@ -6216,25 +6054,25 @@
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="D46" s="9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>AV133</t>
+          <t>AV67 &amp; ~AV137</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>AV133</t>
+          <t>AV67</t>
         </is>
       </c>
       <c r="G46" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
+          <t>No subitem a) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu regras para a priorização e o escalamento de incidentes</t>
         </is>
       </c>
       <c r="H46" s="9" t="b">
@@ -6244,7 +6082,7 @@
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>MR083</t>
+          <t>MR086</t>
         </is>
       </c>
       <c r="B47" s="9" t="inlineStr">
@@ -6254,25 +6092,25 @@
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="D47" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>AV66 &amp; ~AV136</t>
+          <t>AV137</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>AV66</t>
+          <t>AV137</t>
         </is>
       </c>
       <c r="G47" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2203, não houve declaração afirmativa quanto à prática avaliada: o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem a) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu regras para a priorização e o escalamento de incidentes</t>
         </is>
       </c>
       <c r="H47" s="9" t="b">
@@ -6282,7 +6120,7 @@
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>MR084</t>
+          <t>MR087</t>
         </is>
       </c>
       <c r="B48" s="9" t="inlineStr">
@@ -6292,25 +6130,25 @@
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="D48" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>AV136</t>
+          <t>AV70 &amp; ~AV140</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>AV136</t>
+          <t>AV70</t>
         </is>
       </c>
       <c r="G48" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem d) do item 2204, não houve declaração afirmativa quanto à prática avaliada: o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H48" s="9" t="b">
@@ -6320,7 +6158,7 @@
     <row r="49" ht="45" customHeight="1">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>MR085</t>
+          <t>MR088</t>
         </is>
       </c>
       <c r="B49" s="9" t="inlineStr">
@@ -6334,21 +6172,21 @@
         </is>
       </c>
       <c r="D49" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>AV67 &amp; ~AV137</t>
+          <t>AV140</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>AV67</t>
+          <t>AV140</t>
         </is>
       </c>
       <c r="G49" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu regras para a priorização e o escalamento de incidentes</t>
+          <t>No subitem d) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H49" s="9" t="b">
@@ -6358,7 +6196,7 @@
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>MR086</t>
+          <t>MR089</t>
         </is>
       </c>
       <c r="B50" s="9" t="inlineStr">
@@ -6372,21 +6210,21 @@
         </is>
       </c>
       <c r="D50" s="9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>AV137</t>
+          <t>AV71 &amp; ~AV141</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>AV137</t>
+          <t>AV71</t>
         </is>
       </c>
       <c r="G50" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu regras para a priorização e o escalamento de incidentes</t>
+          <t>No subitem e) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
         </is>
       </c>
       <c r="H50" s="9" t="b">
@@ -6396,7 +6234,7 @@
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>MR087</t>
+          <t>MR090</t>
         </is>
       </c>
       <c r="B51" s="9" t="inlineStr">
@@ -6410,21 +6248,21 @@
         </is>
       </c>
       <c r="D51" s="9" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>AV70 &amp; ~AV140</t>
+          <t>AV141</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>AV70</t>
+          <t>AV141</t>
         </is>
       </c>
       <c r="G51" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2204, não houve declaração afirmativa quanto à prática avaliada: o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem e) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
         </is>
       </c>
       <c r="H51" s="9" t="b">
@@ -6434,35 +6272,35 @@
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="9" t="inlineStr">
         <is>
-          <t>MR088</t>
+          <t>MR091</t>
         </is>
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D52" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>AV140</t>
+          <t>AV73 &amp; ~AV143</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>AV140</t>
+          <t>AV73</t>
         </is>
       </c>
       <c r="G52" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem a) do item 2801, não houve declaração afirmativa quanto à prática avaliada: o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
         </is>
       </c>
       <c r="H52" s="9" t="b">
@@ -6472,35 +6310,35 @@
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>MR089</t>
+          <t>MR092</t>
         </is>
       </c>
       <c r="B53" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D53" s="9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>AV71 &amp; ~AV141</t>
+          <t>AV143</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>AV71</t>
+          <t>AV143</t>
         </is>
       </c>
       <c r="G53" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
+          <t>No subitem a) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
         </is>
       </c>
       <c r="H53" s="9" t="b">
@@ -6510,35 +6348,35 @@
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t>MR090</t>
+          <t>MR101</t>
         </is>
       </c>
       <c r="B54" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
         </is>
       </c>
       <c r="D54" s="9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>AV141</t>
+          <t>AV78 &amp; ~AV148</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>AV141</t>
+          <t>AV78</t>
         </is>
       </c>
       <c r="G54" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
+          <t>No subitem a) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
         </is>
       </c>
       <c r="H54" s="9" t="b">
@@ -6548,7 +6386,7 @@
     <row r="55" ht="45" customHeight="1">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>MR091</t>
+          <t>MR102</t>
         </is>
       </c>
       <c r="B55" s="9" t="inlineStr">
@@ -6558,25 +6396,25 @@
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
         </is>
       </c>
       <c r="D55" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>AV73 &amp; ~AV143</t>
+          <t>AV148</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>AV73</t>
+          <t>AV148</t>
         </is>
       </c>
       <c r="G55" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2801, não houve declaração afirmativa quanto à prática avaliada: o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
+          <t>No subitem a) do item 2804, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
         </is>
       </c>
       <c r="H55" s="9" t="b">
@@ -6586,7 +6424,7 @@
     <row r="56" ht="45" customHeight="1">
       <c r="A56" s="9" t="inlineStr">
         <is>
-          <t>MR092</t>
+          <t>MR105</t>
         </is>
       </c>
       <c r="B56" s="9" t="inlineStr">
@@ -6596,25 +6434,25 @@
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
         </is>
       </c>
       <c r="D56" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>AV143</t>
+          <t>AV80 &amp; ~AV150</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>AV143</t>
+          <t>AV80</t>
         </is>
       </c>
       <c r="G56" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
+          <t>No subitem c) do item 2802, não houve declaração afirmativa quanto à prática avaliada: na elaboração do PCA são considerados os demais instrumentos de planejamento da organização</t>
         </is>
       </c>
       <c r="H56" s="9" t="b">
@@ -6624,7 +6462,7 @@
     <row r="57" ht="45" customHeight="1">
       <c r="A57" s="9" t="inlineStr">
         <is>
-          <t>MR101</t>
+          <t>MR106</t>
         </is>
       </c>
       <c r="B57" s="9" t="inlineStr">
@@ -6634,25 +6472,25 @@
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
         </is>
       </c>
       <c r="D57" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>AV78 &amp; ~AV148</t>
+          <t>AV150</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>AV78</t>
+          <t>AV150</t>
         </is>
       </c>
       <c r="G57" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
+          <t>No subitem c) do item 2802, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que na elaboração do PCA são considerados os demais instrumentos de planejamento da organização</t>
         </is>
       </c>
       <c r="H57" s="9" t="b">
@@ -6662,7 +6500,7 @@
     <row r="58" ht="45" customHeight="1">
       <c r="A58" s="9" t="inlineStr">
         <is>
-          <t>MR102</t>
+          <t>MR109</t>
         </is>
       </c>
       <c r="B58" s="9" t="inlineStr">
@@ -6672,25 +6510,25 @@
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
         </is>
       </c>
       <c r="D58" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>AV148</t>
+          <t>AV82</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>AV148</t>
+          <t>AV82</t>
         </is>
       </c>
       <c r="G58" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2804, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
+          <t>No subitem b) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de TI executadas no exercício encontram-se previamente estabelecidas nos instrumentos de planejamento vigentes (PDTI/PEDTIC e PCA)</t>
         </is>
       </c>
       <c r="H58" s="9" t="b">
@@ -6700,7 +6538,7 @@
     <row r="59" ht="45" customHeight="1">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>MR105</t>
+          <t>MR110</t>
         </is>
       </c>
       <c r="B59" s="9" t="inlineStr">
@@ -6710,7 +6548,7 @@
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
+          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
         </is>
       </c>
       <c r="D59" s="9" t="n">
@@ -6718,17 +6556,17 @@
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>AV80 &amp; ~AV150</t>
+          <t>AV83</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>AV80</t>
+          <t>AV83</t>
         </is>
       </c>
       <c r="G59" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2802, não houve declaração afirmativa quanto à prática avaliada: na elaboração do PCA são considerados os demais instrumentos de planejamento da organização</t>
+          <t>No subitem c) do item 2804, não houve declaração afirmativa quanto à prática avaliada: a fase de planejamento de cada contratação de TI é conduzida por uma Equipe de Planejamento da Contratação formalmente designada (composta, minimamente, por integrante requisitante e integrante técnico da área de TI)</t>
         </is>
       </c>
       <c r="H59" s="9" t="b">
@@ -6738,7 +6576,7 @@
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="9" t="inlineStr">
         <is>
-          <t>MR106</t>
+          <t>MR111</t>
         </is>
       </c>
       <c r="B60" s="9" t="inlineStr">
@@ -6748,7 +6586,7 @@
       </c>
       <c r="C60" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D60" s="9" t="n">
@@ -6756,17 +6594,17 @@
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>AV150</t>
+          <t>AV152 &amp; ~AV153</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>AV150</t>
+          <t>AV152</t>
         </is>
       </c>
       <c r="G60" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2802, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que na elaboração do PCA são considerados os demais instrumentos de planejamento da organização</t>
+          <t>No subitem b) do item 2801, não houve declaração afirmativa quanto à prática avaliada: são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
         </is>
       </c>
       <c r="H60" s="9" t="b">
@@ -6776,7 +6614,7 @@
     <row r="61" ht="45" customHeight="1">
       <c r="A61" s="9" t="inlineStr">
         <is>
-          <t>MR109</t>
+          <t>MR112</t>
         </is>
       </c>
       <c r="B61" s="9" t="inlineStr">
@@ -6786,25 +6624,25 @@
       </c>
       <c r="C61" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D61" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>AV82</t>
+          <t>AV153</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>AV82</t>
+          <t>AV153</t>
         </is>
       </c>
       <c r="G61" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de TI executadas no exercício encontram-se previamente estabelecidas nos instrumentos de planejamento vigentes (PDTI/PEDTIC e PCA)</t>
+          <t>No subitem b) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
         </is>
       </c>
       <c r="H61" s="9" t="b">
@@ -6814,155 +6652,44 @@
     <row r="62" ht="45" customHeight="1">
       <c r="A62" s="9" t="inlineStr">
         <is>
-          <t>MR110</t>
+          <t>MR113</t>
         </is>
       </c>
       <c r="B62" s="9" t="inlineStr">
         <is>
-          <t>PA06</t>
+          <t>PA03</t>
         </is>
       </c>
       <c r="C62" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="D62" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>AV83</t>
+          <t>AV154</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>AV83</t>
+          <t>AV154</t>
         </is>
       </c>
       <c r="G62" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2804, não houve declaração afirmativa quanto à prática avaliada: a fase de planejamento de cada contratação de TI é conduzida por uma Equipe de Planejamento da Contratação formalmente designada (composta, minimamente, por integrante requisitante e integrante técnico da área de TI)</t>
+          <t>No item 2102, a organização não declarou possuir plano de tecnologia da informação vigente, ainda que parcialmente adotado</t>
         </is>
       </c>
       <c r="H62" s="9" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="63" ht="30" customHeight="1">
-      <c r="A63" s="9" t="inlineStr">
-        <is>
-          <t>MR111</t>
-        </is>
-      </c>
-      <c r="B63" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C63" s="9" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="D63" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E63" s="9" t="inlineStr">
-        <is>
-          <t>AV152 &amp; ~AV153</t>
-        </is>
-      </c>
-      <c r="F63" s="9" t="inlineStr">
-        <is>
-          <t>AV152</t>
-        </is>
-      </c>
-      <c r="G63" s="9" t="inlineStr">
-        <is>
-          <t>No subitem b) do item 2801, não houve declaração afirmativa quanto à prática avaliada: são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
-        </is>
-      </c>
-      <c r="H63" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64" ht="45" customHeight="1">
-      <c r="A64" s="9" t="inlineStr">
-        <is>
-          <t>MR112</t>
-        </is>
-      </c>
-      <c r="B64" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C64" s="9" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="D64" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="E64" s="9" t="inlineStr">
-        <is>
-          <t>AV153</t>
-        </is>
-      </c>
-      <c r="F64" s="9" t="inlineStr">
-        <is>
-          <t>AV153</t>
-        </is>
-      </c>
-      <c r="G64" s="9" t="inlineStr">
-        <is>
-          <t>No subitem b) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
-        </is>
-      </c>
-      <c r="H64" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65" ht="30" customHeight="1">
-      <c r="A65" s="9" t="inlineStr">
-        <is>
-          <t>MR113</t>
-        </is>
-      </c>
-      <c r="B65" s="9" t="inlineStr">
-        <is>
-          <t>PA03</t>
-        </is>
-      </c>
-      <c r="C65" s="9" t="inlineStr">
-        <is>
-          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
-        </is>
-      </c>
-      <c r="D65" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E65" s="9" t="inlineStr">
-        <is>
-          <t>AV154</t>
-        </is>
-      </c>
-      <c r="F65" s="9" t="inlineStr">
-        <is>
-          <t>AV154</t>
-        </is>
-      </c>
-      <c r="G65" s="9" t="inlineStr">
-        <is>
-          <t>No item 2102, a organização não declarou possuir plano de tecnologia da informação vigente, ainda que parcialmente adotado</t>
-        </is>
-      </c>
-      <c r="H65" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
+    <row r="63" ht="30" customHeight="1"/>
+    <row r="64" ht="45" customHeight="1"/>
+    <row r="65" ht="30" customHeight="1"/>
     <row r="66" ht="30" customHeight="1"/>
     <row r="67" ht="30" customHeight="1"/>
     <row r="68" ht="45" customHeight="1"/>
@@ -7012,7 +6739,7 @@
     <row r="112" ht="45" customHeight="1"/>
     <row r="113" ht="45" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A3:H65"/>
+  <autoFilter ref="A3:H62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Revisa a Questão 5 da matriz e do mapa
</commit_message>
<xml_diff>
--- a/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
+++ b/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
@@ -15,8 +15,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Fontes de Informação'!$A$3:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Procedimentos de Auditoria'!$A$3:$E$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ações de Verificação'!$A$3:$P$64</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Motivos do Relatório'!$A$3:$H$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ações de Verificação'!$A$3:$P$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Motivos do Relatório'!$A$3:$H$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Variáveis Temporárias'!$A$3:$E$6</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -644,12 +644,12 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>Procedimento para verificar a questão Q5: A organização adota práticas mínimas de gestão de serviços de TIC, incluindo catálogo de serviços, níveis de serviço, inventário de ativos, gestão de configuração e tratamento de incidentes, de modo a assegurar eficiência, continuidade, rastreabilidade e qualidade dos serviços prestados?</t>
+          <t>Procedimento para verificar a questão Q5: A organização adota práticas mínimas de gestão de serviços de TIC, incluindo catálogo de serviços, níveis de serviço, inventário de ativos, gestão de configuração e tratamento de incidentes, de modo a assegurar eficiência, rastreabilidade e qualidade dos serviços prestados?</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>(((AV55 | AV125) | (AV56 | AV126)) | ((AV54 | AV124) | (AV57 | AV127) | (AV58 | AV128)) | ((AV59 | AV129) | (AV62 | AV132) | (AV63 | AV133)) | (AV66 | AV136) | ((AV67 | AV137) | (AV70 | AV140) | (AV71 | AV141)))</t>
+          <t>((AV55 | AV56) | (AV54 | AV57 | AV58) | (AV62 | AV63) | (AV59 | AV66) | (AV67 | AV70 | AV71))</t>
         </is>
       </c>
       <c r="D8" s="1" t="n">
@@ -699,7 +699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P64"/>
+  <dimension ref="A1:P52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2231,8 +2231,8 @@
       </c>
       <c r="G28" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
-ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.</t>
+          <t>ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.7, III.9.7 e V.6.4 – Recomendações quanto à definição, pactuação e monitoramento de níveis de serviço.</t>
         </is>
       </c>
       <c r="H28" s="1" t="inlineStr">
@@ -2261,7 +2261,7 @@
       <c r="O28" s="1" t="n"/>
       <c r="P28" s="1" t="inlineStr">
         <is>
-          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
+          <t>defina, acorde e monitore níveis de serviço para os serviços de TIC relevantes, estabelecendo metas e mecanismos de acompanhamento de seu cumprimento</t>
         </is>
       </c>
     </row>
@@ -2286,8 +2286,9 @@
       </c>
       <c r="G29" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento do catálogo de serviços: manter fonte única de informações consistentes sobre serviços e ofertas de serviço, disponível para usuários e equipes de suporte.
-COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.</t>
+          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.4, III.9.4 e V.6.1 – Recomendações quanto à estruturação do catálogo de serviços de TIC, incluindo descrição dos serviços, metas, formas de acesso e disponibilidade aos usuários.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.2.4 – Gerenciamento de catálogo de serviço: orienta que o catálogo descreva os serviços e seus resultados pretendidos, contenha informações relevantes para sua utilização e seja disponibilizado às partes interessadas que necessitem acessá-lo.</t>
         </is>
       </c>
       <c r="H29" s="1" t="inlineStr">
@@ -2341,8 +2342,9 @@
       </c>
       <c r="G30" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento do catálogo de serviços: manter fonte única de informações consistentes sobre serviços e ofertas de serviço, disponível para usuários e equipes de suporte.
-COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.</t>
+          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.4, III.9.4 e V.6.1 – Recomendações quanto à estruturação do catálogo de serviços de TIC, incluindo descrição dos serviços, metas, formas de acesso e disponibilidade aos usuários.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.2.4 – Gerenciamento de catálogo de serviço: orienta que o catálogo descreva os serviços e seus resultados pretendidos, contenha informações relevantes para sua utilização e seja disponibilizado às partes interessadas que necessitem acessá-lo.</t>
         </is>
       </c>
       <c r="H30" s="1" t="inlineStr">
@@ -2396,8 +2398,8 @@
       </c>
       <c r="G31" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
-ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.</t>
+          <t>ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.7, III.9.7 e V.6.4 – Recomendações quanto à definição, pactuação e monitoramento de níveis de serviço.</t>
         </is>
       </c>
       <c r="H31" s="1" t="inlineStr">
@@ -2426,7 +2428,7 @@
       <c r="O31" s="1" t="n"/>
       <c r="P31" s="1" t="inlineStr">
         <is>
-          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
+          <t>defina, acorde e monitore níveis de serviço para os serviços de TIC relevantes, estabelecendo metas e mecanismos de acompanhamento de seu cumprimento</t>
         </is>
       </c>
     </row>
@@ -2451,8 +2453,8 @@
       </c>
       <c r="G32" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
-ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.</t>
+          <t>ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.7, III.9.7 e V.6.4 – Recomendações quanto à definição, pactuação e monitoramento de níveis de serviço.</t>
         </is>
       </c>
       <c r="H32" s="1" t="inlineStr">
@@ -2481,7 +2483,7 @@
       <c r="O32" s="1" t="n"/>
       <c r="P32" s="1" t="inlineStr">
         <is>
-          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
+          <t>defina, acorde e monitore níveis de serviço para os serviços de TIC relevantes, estabelecendo metas e mecanismos de acompanhamento de seu cumprimento</t>
         </is>
       </c>
     </row>
@@ -2506,8 +2508,9 @@
       </c>
       <c r="G33" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
+          <t>COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.2.6 – Gerenciamento de configuração: orienta a identificação, o registro, o controle, o rastreamento e a verificação dos itens de configuração, bem como a manutenção de informações de configuração precisas relacionadas aos serviços.</t>
         </is>
       </c>
       <c r="H33" s="1" t="inlineStr">
@@ -2518,7 +2521,7 @@
       <c r="I33" s="1" t="n"/>
       <c r="J33" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="K33" s="1" t="inlineStr">
@@ -2530,13 +2533,13 @@
       <c r="M33" s="1" t="n"/>
       <c r="N33" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O33" s="1" t="n"/>
       <c r="P33" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
+          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
         </is>
       </c>
     </row>
@@ -2562,7 +2565,7 @@
       <c r="G34" s="1" t="inlineStr">
         <is>
           <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.</t>
         </is>
       </c>
       <c r="H34" s="1" t="inlineStr">
@@ -2573,7 +2576,7 @@
       <c r="I34" s="1" t="n"/>
       <c r="J34" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
         </is>
       </c>
       <c r="K34" s="1" t="inlineStr">
@@ -2585,13 +2588,13 @@
       <c r="M34" s="1" t="n"/>
       <c r="N34" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O34" s="1" t="n"/>
       <c r="P34" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
+          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos sob gestão da organização, contemplando, minimamente, os dispositivos e softwares utilizados, com informações suficientes para sua identificação e controle</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2620,7 @@
       <c r="G35" s="1" t="inlineStr">
         <is>
           <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.</t>
         </is>
       </c>
       <c r="H35" s="1" t="inlineStr">
@@ -2628,7 +2631,7 @@
       <c r="I35" s="1" t="n"/>
       <c r="J35" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
         </is>
       </c>
       <c r="K35" s="1" t="inlineStr">
@@ -2640,13 +2643,13 @@
       <c r="M35" s="1" t="n"/>
       <c r="N35" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O35" s="1" t="n"/>
       <c r="P35" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
+          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos sob gestão da organização, contemplando, minimamente, os dispositivos e softwares utilizados, com informações suficientes para sua identificação e controle</t>
         </is>
       </c>
     </row>
@@ -2671,8 +2674,9 @@
       </c>
       <c r="G36" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de configuração de serviço: assegurar informações precisas e confiáveis sobre itens de configuração e seus relacionamentos com serviços, sistemas e infraestrutura.
-COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.</t>
+          <t>COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.2.6 – Gerenciamento de configuração: orienta a identificação, o registro, o controle, o rastreamento e a verificação dos itens de configuração, bem como a manutenção de informações de configuração precisas relacionadas aos serviços.</t>
         </is>
       </c>
       <c r="H36" s="1" t="inlineStr">
@@ -2727,7 +2731,8 @@
       <c r="G37" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.6, III.9.6 e V.6.3 – Recomendações quanto à formalização e execução do processo de gestão de incidentes, incluindo registros, classificação, escalamento e tratamento.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.6.1 – Gerenciamento de incidente: orienta que os incidentes sejam registrados, classificados e priorizados, que as ações adotadas para sua resolução sejam registradas e rastreáveis e que sejam definidas responsabilidades para seu tratamento, incluindo procedimento documentado para incidentes graves.</t>
         </is>
       </c>
       <c r="H37" s="1" t="inlineStr">
@@ -2782,7 +2787,8 @@
       <c r="G38" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.6, III.9.6 e V.6.3 – Recomendações quanto à formalização e execução do processo de gestão de incidentes, incluindo registros, classificação, escalamento e tratamento.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.6.1 – Gerenciamento de incidente: orienta que os incidentes sejam registrados, classificados e priorizados, que as ações adotadas para sua resolução sejam registradas e rastreáveis e que sejam definidas responsabilidades para seu tratamento, incluindo procedimento documentado para incidentes graves.</t>
         </is>
       </c>
       <c r="H38" s="1" t="inlineStr">
@@ -2837,7 +2843,8 @@
       <c r="G39" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.6, III.9.6 e V.6.3 – Recomendações quanto à formalização e execução do processo de gestão de incidentes, incluindo registros, classificação, escalamento e tratamento.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.6.1 – Gerenciamento de incidente: orienta que os incidentes sejam registrados, classificados e priorizados, que as ações adotadas para sua resolução sejam registradas e rastreáveis e que sejam definidas responsabilidades para seu tratamento, incluindo procedimento documentado para incidentes graves.</t>
         </is>
       </c>
       <c r="H39" s="1" t="inlineStr">
@@ -3204,7 +3211,7 @@
     <row r="46" ht="113.45" customHeight="1">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>AV124</t>
+          <t>AV143</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -3217,13 +3224,13 @@
       <c r="E46" s="1" t="n"/>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[A]</t>
+          <t>q2801ext[A]</t>
         </is>
       </c>
       <c r="G46" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
-ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.</t>
+          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
         </is>
       </c>
       <c r="H46" s="1" t="inlineStr">
@@ -3234,7 +3241,7 @@
       <c r="I46" s="1" t="n"/>
       <c r="J46" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="K46" s="1" t="inlineStr">
@@ -3246,20 +3253,20 @@
       <c r="M46" s="1" t="n"/>
       <c r="N46" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O46" s="1" t="n"/>
       <c r="P46" s="1" t="inlineStr">
         <is>
-          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
+          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
         </is>
       </c>
     </row>
     <row r="47" ht="113.45" customHeight="1">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>AV125</t>
+          <t>AV148</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -3272,13 +3279,14 @@
       <c r="E47" s="1" t="n"/>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[B]</t>
+          <t>q2804[A]</t>
         </is>
       </c>
       <c r="G47" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento do catálogo de serviços: manter fonte única de informações consistentes sobre serviços e ofertas de serviço, disponível para usuários e equipes de suporte.
-COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.</t>
+          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+COBIT 2019, BAI02.04 - Obter aprovação dos requisitos da solução: obter aprovação formal dos requisitos funcionais, técnicos, de segurança e de conformidade antes de prosseguir com a solução.
+Instrução Normativa SGD/ME nº 94, de 23 de dezembro de 2022, art. 1º, § 1º: como referência de boa prática, a aplicação de ritos formais de contratação de TIC pode ser facultada para contratações diretas por dispensa em razão do valor (inciso II do art. 75 da Lei nº 14.133/2021), indicando a possibilidade de fluxos simplificados para aquisições de baixa complexidade ou valor.</t>
         </is>
       </c>
       <c r="H47" s="1" t="inlineStr">
@@ -3289,7 +3297,7 @@
       <c r="I47" s="1" t="n"/>
       <c r="J47" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
         </is>
       </c>
       <c r="K47" s="1" t="inlineStr">
@@ -3307,14 +3315,14 @@
       <c r="O47" s="1" t="n"/>
       <c r="P47" s="1" t="inlineStr">
         <is>
-          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
+          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo fluxos simplificados para contratações de baixa complexidade ou baixo valor, desde que preservada análise técnica mínima compatível com o risco da contratação</t>
         </is>
       </c>
     </row>
     <row r="48" ht="113.45" customHeight="1">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>AV126</t>
+          <t>AV150</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -3327,13 +3335,13 @@
       <c r="E48" s="1" t="n"/>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[C]</t>
+          <t>q2802ext[C]</t>
         </is>
       </c>
       <c r="G48" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento do catálogo de serviços: manter fonte única de informações consistentes sobre serviços e ofertas de serviço, disponível para usuários e equipes de suporte.
-COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.</t>
+          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Art. 18, caput e §1º, incisos I, IV, V, VIII, IX, X e XIII, da Lei 14.133/2021: fase preparatória caracterizada pelo planejamento, compatibilização com o plano de contratações anual e elementos mínimos do estudo técnico preliminar.</t>
         </is>
       </c>
       <c r="H48" s="1" t="inlineStr">
@@ -3344,7 +3352,7 @@
       <c r="I48" s="1" t="n"/>
       <c r="J48" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
         </is>
       </c>
       <c r="K48" s="1" t="inlineStr">
@@ -3356,25 +3364,25 @@
       <c r="M48" s="1" t="n"/>
       <c r="N48" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O48" s="1" t="n"/>
       <c r="P48" s="1" t="inlineStr">
         <is>
-          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
+          <t>integre as contratações de TIC com os instrumentos de planejamento da organização e com o Plano de Contratações Anual, quando elaborado, justificando as situações excepcionais</t>
         </is>
       </c>
     </row>
     <row r="49" ht="113.45" customHeight="1">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>AV127</t>
+          <t>AV152</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
-          <t>avaliacao_evidencias_ajustes</t>
+          <t>questionario</t>
         </is>
       </c>
       <c r="C49" s="1" t="n"/>
@@ -3382,49 +3390,49 @@
       <c r="E49" s="1" t="n"/>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[D]</t>
+          <t>q2801ext[B]</t>
         </is>
       </c>
       <c r="G49" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
-ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.</t>
+          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
         </is>
       </c>
       <c r="H49" s="1" t="inlineStr">
         <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+          <t>Resposta negativa ao detalhamento b) do item 2801 do Questionário, para verificar se são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
         </is>
       </c>
       <c r="I49" s="1" t="n"/>
       <c r="J49" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="K49" s="1" t="inlineStr">
         <is>
-          <t>Não conforme</t>
+          <t>(Não | N/A)</t>
         </is>
       </c>
       <c r="L49" s="1" t="n"/>
       <c r="M49" s="1" t="n"/>
       <c r="N49" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O49" s="1" t="n"/>
       <c r="P49" s="1" t="inlineStr">
         <is>
-          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
+          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
         </is>
       </c>
     </row>
     <row r="50" ht="113.45" customHeight="1">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>AV128</t>
+          <t>AV153</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -3437,13 +3445,13 @@
       <c r="E50" s="1" t="n"/>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[E]</t>
+          <t>q2801ext[B]</t>
         </is>
       </c>
       <c r="G50" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
-ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.</t>
+          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
         </is>
       </c>
       <c r="H50" s="1" t="inlineStr">
@@ -3454,7 +3462,7 @@
       <c r="I50" s="1" t="n"/>
       <c r="J50" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="K50" s="1" t="inlineStr">
@@ -3466,25 +3474,25 @@
       <c r="M50" s="1" t="n"/>
       <c r="N50" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O50" s="1" t="n"/>
       <c r="P50" s="1" t="inlineStr">
         <is>
-          <t>defina e monitore níveis mínimos de serviço ou metas de atendimento para os serviços de TIC relevantes, estabelecendo indicadores, responsáveis, periodicidade de medição e forma de comunicação dos resultados</t>
+          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
         </is>
       </c>
     </row>
     <row r="51" ht="113.45" customHeight="1">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>AV129</t>
+          <t>AV154</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
-          <t>avaliacao_evidencias_ajustes</t>
+          <t>questionario</t>
         </is>
       </c>
       <c r="C51" s="1" t="n"/>
@@ -3492,29 +3500,30 @@
       <c r="E51" s="1" t="n"/>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>q2203ext[A]</t>
+          <t>existe_plano_ti</t>
         </is>
       </c>
       <c r="G51" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H51" s="1" t="inlineStr">
         <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+          <t>Resposta ao item 2102 que não caracteriza a existência de plano de TIC vigente, ainda que parcialmente adotado</t>
         </is>
       </c>
       <c r="I51" s="1" t="n"/>
       <c r="J51" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="K51" s="1" t="inlineStr">
         <is>
-          <t>Não conforme</t>
+          <t>False</t>
         </is>
       </c>
       <c r="L51" s="1" t="n"/>
@@ -3527,19 +3536,19 @@
       <c r="O51" s="1" t="n"/>
       <c r="P51" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
     <row r="52" ht="113.45" customHeight="1">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>AV132</t>
+          <t>AV155</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
-          <t>avaliacao_evidencias_ajustes</t>
+          <t>questionario</t>
         </is>
       </c>
       <c r="C52" s="1" t="n"/>
@@ -3547,29 +3556,26 @@
       <c r="E52" s="1" t="n"/>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>q2504ext[A]</t>
+          <t>existe_plano_ti</t>
         </is>
       </c>
       <c r="G52" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H52" s="1" t="inlineStr">
         <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+          <t>Plano de TIC vigente declarado no item 2102, ao menos parcialmente adotado</t>
         </is>
       </c>
       <c r="I52" s="1" t="n"/>
-      <c r="J52" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
-        </is>
-      </c>
+      <c r="J52" s="1" t="n"/>
       <c r="K52" s="1" t="inlineStr">
         <is>
-          <t>Não conforme</t>
+          <t>True</t>
         </is>
       </c>
       <c r="L52" s="1" t="n"/>
@@ -3582,669 +3588,22 @@
       <c r="O52" s="1" t="n"/>
       <c r="P52" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="113.45" customHeight="1">
-      <c r="A53" s="1" t="inlineStr">
-        <is>
-          <t>AV133</t>
-        </is>
-      </c>
-      <c r="B53" s="1" t="inlineStr">
-        <is>
-          <t>avaliacao_evidencias_ajustes</t>
-        </is>
-      </c>
-      <c r="C53" s="1" t="n"/>
-      <c r="D53" s="1" t="n"/>
-      <c r="E53" s="1" t="n"/>
-      <c r="F53" s="1" t="inlineStr">
-        <is>
-          <t>q2504ext[B]</t>
-        </is>
-      </c>
-      <c r="G53" s="1" t="inlineStr">
-        <is>
-          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-Lei nº 13.709/2018, arts. 46 e 50: medidas técnicas e administrativas de segurança e regras de boas práticas e governança no tratamento de dados pessoais.</t>
-        </is>
-      </c>
-      <c r="H53" s="1" t="inlineStr">
-        <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
-        </is>
-      </c>
-      <c r="I53" s="1" t="n"/>
-      <c r="J53" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
-        </is>
-      </c>
-      <c r="K53" s="1" t="inlineStr">
-        <is>
-          <t>Não conforme</t>
-        </is>
-      </c>
-      <c r="L53" s="1" t="n"/>
-      <c r="M53" s="1" t="n"/>
-      <c r="N53" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O53" s="1" t="n"/>
-      <c r="P53" s="1" t="inlineStr">
-        <is>
-          <t>estabeleça e mantenha atualizado inventário de ativos de TIC, atentando-se, minimamente, em registrar equipamentos, sistemas, softwares, licenças, serviços em nuvem e responsáveis</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="113.45" customHeight="1">
-      <c r="A54" s="1" t="inlineStr">
-        <is>
-          <t>AV136</t>
-        </is>
-      </c>
-      <c r="B54" s="1" t="inlineStr">
-        <is>
-          <t>avaliacao_evidencias_ajustes</t>
-        </is>
-      </c>
-      <c r="C54" s="1" t="n"/>
-      <c r="D54" s="1" t="n"/>
-      <c r="E54" s="1" t="n"/>
-      <c r="F54" s="1" t="inlineStr">
-        <is>
-          <t>q2203ext[C]</t>
-        </is>
-      </c>
-      <c r="G54" s="1" t="inlineStr">
-        <is>
-          <t>ITIL 4, prática de gerenciamento de configuração de serviço: assegurar informações precisas e confiáveis sobre itens de configuração e seus relacionamentos com serviços, sistemas e infraestrutura.
-COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.</t>
-        </is>
-      </c>
-      <c r="H54" s="1" t="inlineStr">
-        <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
-        </is>
-      </c>
-      <c r="I54" s="1" t="n"/>
-      <c r="J54" s="1" t="inlineStr">
-        <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
-        </is>
-      </c>
-      <c r="K54" s="1" t="inlineStr">
-        <is>
-          <t>Não conforme</t>
-        </is>
-      </c>
-      <c r="L54" s="1" t="n"/>
-      <c r="M54" s="1" t="n"/>
-      <c r="N54" s="1" t="inlineStr">
-        <is>
-          <t>Recomendação</t>
-        </is>
-      </c>
-      <c r="O54" s="1" t="n"/>
-      <c r="P54" s="1" t="inlineStr">
-        <is>
-          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="113.45" customHeight="1">
-      <c r="A55" s="1" t="inlineStr">
-        <is>
-          <t>AV137</t>
-        </is>
-      </c>
-      <c r="B55" s="1" t="inlineStr">
-        <is>
-          <t>avaliacao_evidencias_ajustes</t>
-        </is>
-      </c>
-      <c r="C55" s="1" t="n"/>
-      <c r="D55" s="1" t="n"/>
-      <c r="E55" s="1" t="n"/>
-      <c r="F55" s="1" t="inlineStr">
-        <is>
-          <t>q2204ext[A]</t>
-        </is>
-      </c>
-      <c r="G55" s="1" t="inlineStr">
-        <is>
-          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
-        </is>
-      </c>
-      <c r="H55" s="1" t="inlineStr">
-        <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
-        </is>
-      </c>
-      <c r="I55" s="1" t="n"/>
-      <c r="J55" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
-        </is>
-      </c>
-      <c r="K55" s="1" t="inlineStr">
-        <is>
-          <t>Não conforme</t>
-        </is>
-      </c>
-      <c r="L55" s="1" t="n"/>
-      <c r="M55" s="1" t="n"/>
-      <c r="N55" s="1" t="inlineStr">
-        <is>
-          <t>Recomendação</t>
-        </is>
-      </c>
-      <c r="O55" s="1" t="n"/>
-      <c r="P55" s="1" t="inlineStr">
-        <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="113.45" customHeight="1">
-      <c r="A56" s="1" t="inlineStr">
-        <is>
-          <t>AV140</t>
-        </is>
-      </c>
-      <c r="B56" s="1" t="inlineStr">
-        <is>
-          <t>avaliacao_evidencias_ajustes</t>
-        </is>
-      </c>
-      <c r="C56" s="1" t="n"/>
-      <c r="D56" s="1" t="n"/>
-      <c r="E56" s="1" t="n"/>
-      <c r="F56" s="1" t="inlineStr">
-        <is>
-          <t>q2204ext[D]</t>
-        </is>
-      </c>
-      <c r="G56" s="1" t="inlineStr">
-        <is>
-          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
-        </is>
-      </c>
-      <c r="H56" s="1" t="inlineStr">
-        <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
-        </is>
-      </c>
-      <c r="I56" s="1" t="n"/>
-      <c r="J56" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
-        </is>
-      </c>
-      <c r="K56" s="1" t="inlineStr">
-        <is>
-          <t>Não conforme</t>
-        </is>
-      </c>
-      <c r="L56" s="1" t="n"/>
-      <c r="M56" s="1" t="n"/>
-      <c r="N56" s="1" t="inlineStr">
-        <is>
-          <t>Recomendação</t>
-        </is>
-      </c>
-      <c r="O56" s="1" t="n"/>
-      <c r="P56" s="1" t="inlineStr">
-        <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="90.95" customHeight="1">
-      <c r="A57" s="1" t="inlineStr">
-        <is>
-          <t>AV141</t>
-        </is>
-      </c>
-      <c r="B57" s="1" t="inlineStr">
-        <is>
-          <t>avaliacao_evidencias_ajustes</t>
-        </is>
-      </c>
-      <c r="C57" s="1" t="n"/>
-      <c r="D57" s="1" t="n"/>
-      <c r="E57" s="1" t="n"/>
-      <c r="F57" s="1" t="inlineStr">
-        <is>
-          <t>q2204ext[E]</t>
-        </is>
-      </c>
-      <c r="G57" s="1" t="inlineStr">
-        <is>
-          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Lei nº 13.709/2018, arts. 46 e 48: deveres de segurança e comunicação de incidente que possa acarretar risco ou dano relevante aos titulares.</t>
-        </is>
-      </c>
-      <c r="H57" s="1" t="inlineStr">
-        <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
-        </is>
-      </c>
-      <c r="I57" s="1" t="n"/>
-      <c r="J57" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
-        </is>
-      </c>
-      <c r="K57" s="1" t="inlineStr">
-        <is>
-          <t>Não conforme</t>
-        </is>
-      </c>
-      <c r="L57" s="1" t="n"/>
-      <c r="M57" s="1" t="n"/>
-      <c r="N57" s="1" t="inlineStr">
-        <is>
-          <t>Recomendação</t>
-        </is>
-      </c>
-      <c r="O57" s="1" t="n"/>
-      <c r="P57" s="1" t="inlineStr">
-        <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="90.95" customHeight="1">
-      <c r="A58" s="1" t="inlineStr">
-        <is>
-          <t>AV143</t>
-        </is>
-      </c>
-      <c r="B58" s="1" t="inlineStr">
-        <is>
-          <t>avaliacao_evidencias_ajustes</t>
-        </is>
-      </c>
-      <c r="C58" s="1" t="n"/>
-      <c r="D58" s="1" t="n"/>
-      <c r="E58" s="1" t="n"/>
-      <c r="F58" s="1" t="inlineStr">
-        <is>
-          <t>q2801ext[A]</t>
-        </is>
-      </c>
-      <c r="G58" s="1" t="inlineStr">
-        <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
-        </is>
-      </c>
-      <c r="H58" s="1" t="inlineStr">
-        <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
-        </is>
-      </c>
-      <c r="I58" s="1" t="n"/>
-      <c r="J58" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="K58" s="1" t="inlineStr">
-        <is>
-          <t>Não conforme</t>
-        </is>
-      </c>
-      <c r="L58" s="1" t="n"/>
-      <c r="M58" s="1" t="n"/>
-      <c r="N58" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O58" s="1" t="n"/>
-      <c r="P58" s="1" t="inlineStr">
-        <is>
-          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="90.95" customHeight="1">
-      <c r="A59" s="1" t="inlineStr">
-        <is>
-          <t>AV148</t>
-        </is>
-      </c>
-      <c r="B59" s="1" t="inlineStr">
-        <is>
-          <t>avaliacao_evidencias_ajustes</t>
-        </is>
-      </c>
-      <c r="C59" s="1" t="n"/>
-      <c r="D59" s="1" t="n"/>
-      <c r="E59" s="1" t="n"/>
-      <c r="F59" s="1" t="inlineStr">
-        <is>
-          <t>q2804[A]</t>
-        </is>
-      </c>
-      <c r="G59" s="1" t="inlineStr">
-        <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-COBIT 2019, BAI02.04 - Obter aprovação dos requisitos da solução: obter aprovação formal dos requisitos funcionais, técnicos, de segurança e de conformidade antes de prosseguir com a solução.
-Instrução Normativa SGD/ME nº 94, de 23 de dezembro de 2022, art. 1º, § 1º: como referência de boa prática, a aplicação de ritos formais de contratação de TIC pode ser facultada para contratações diretas por dispensa em razão do valor (inciso II do art. 75 da Lei nº 14.133/2021), indicando a possibilidade de fluxos simplificados para aquisições de baixa complexidade ou valor.</t>
-        </is>
-      </c>
-      <c r="H59" s="1" t="inlineStr">
-        <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
-        </is>
-      </c>
-      <c r="I59" s="1" t="n"/>
-      <c r="J59" s="1" t="inlineStr">
-        <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
-        </is>
-      </c>
-      <c r="K59" s="1" t="inlineStr">
-        <is>
-          <t>Não conforme</t>
-        </is>
-      </c>
-      <c r="L59" s="1" t="n"/>
-      <c r="M59" s="1" t="n"/>
-      <c r="N59" s="1" t="inlineStr">
-        <is>
-          <t>Recomendação</t>
-        </is>
-      </c>
-      <c r="O59" s="1" t="n"/>
-      <c r="P59" s="1" t="inlineStr">
-        <is>
-          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo fluxos simplificados para contratações de baixa complexidade ou baixo valor, desde que preservada análise técnica mínima compatível com o risco da contratação</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="79.90000000000001" customHeight="1">
-      <c r="A60" s="1" t="inlineStr">
-        <is>
-          <t>AV150</t>
-        </is>
-      </c>
-      <c r="B60" s="1" t="inlineStr">
-        <is>
-          <t>avaliacao_evidencias_ajustes</t>
-        </is>
-      </c>
-      <c r="C60" s="1" t="n"/>
-      <c r="D60" s="1" t="n"/>
-      <c r="E60" s="1" t="n"/>
-      <c r="F60" s="1" t="inlineStr">
-        <is>
-          <t>q2802ext[C]</t>
-        </is>
-      </c>
-      <c r="G60" s="1" t="inlineStr">
-        <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 18, caput e §1º, incisos I, IV, V, VIII, IX, X e XIII, da Lei 14.133/2021: fase preparatória caracterizada pelo planejamento, compatibilização com o plano de contratações anual e elementos mínimos do estudo técnico preliminar.</t>
-        </is>
-      </c>
-      <c r="H60" s="1" t="inlineStr">
-        <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
-        </is>
-      </c>
-      <c r="I60" s="1" t="n"/>
-      <c r="J60" s="1" t="inlineStr">
-        <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
-        </is>
-      </c>
-      <c r="K60" s="1" t="inlineStr">
-        <is>
-          <t>Não conforme</t>
-        </is>
-      </c>
-      <c r="L60" s="1" t="n"/>
-      <c r="M60" s="1" t="n"/>
-      <c r="N60" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O60" s="1" t="n"/>
-      <c r="P60" s="1" t="inlineStr">
-        <is>
-          <t>integre as contratações de TIC com os instrumentos de planejamento da organização e com o Plano de Contratações Anual, quando elaborado, justificando as situações excepcionais</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="79.90000000000001" customHeight="1">
-      <c r="A61" s="1" t="inlineStr">
-        <is>
-          <t>AV152</t>
-        </is>
-      </c>
-      <c r="B61" s="1" t="inlineStr">
-        <is>
-          <t>questionario</t>
-        </is>
-      </c>
-      <c r="C61" s="1" t="n"/>
-      <c r="D61" s="1" t="n"/>
-      <c r="E61" s="1" t="n"/>
-      <c r="F61" s="1" t="inlineStr">
-        <is>
-          <t>q2801ext[B]</t>
-        </is>
-      </c>
-      <c r="G61" s="1" t="inlineStr">
-        <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
-        </is>
-      </c>
-      <c r="H61" s="1" t="inlineStr">
-        <is>
-          <t>Resposta negativa ao detalhamento b) do item 2801 do Questionário, para verificar se são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
-        </is>
-      </c>
-      <c r="I61" s="1" t="n"/>
-      <c r="J61" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="K61" s="1" t="inlineStr">
-        <is>
-          <t>(Não | N/A)</t>
-        </is>
-      </c>
-      <c r="L61" s="1" t="n"/>
-      <c r="M61" s="1" t="n"/>
-      <c r="N61" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O61" s="1" t="n"/>
-      <c r="P61" s="1" t="inlineStr">
-        <is>
-          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="90.95" customHeight="1">
-      <c r="A62" s="1" t="inlineStr">
-        <is>
-          <t>AV153</t>
-        </is>
-      </c>
-      <c r="B62" s="1" t="inlineStr">
-        <is>
-          <t>avaliacao_evidencias_ajustes</t>
-        </is>
-      </c>
-      <c r="C62" s="1" t="n"/>
-      <c r="D62" s="1" t="n"/>
-      <c r="E62" s="1" t="n"/>
-      <c r="F62" s="1" t="inlineStr">
-        <is>
-          <t>q2801ext[B]</t>
-        </is>
-      </c>
-      <c r="G62" s="1" t="inlineStr">
-        <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
-        </is>
-      </c>
-      <c r="H62" s="1" t="inlineStr">
-        <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
-        </is>
-      </c>
-      <c r="I62" s="1" t="n"/>
-      <c r="J62" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="K62" s="1" t="inlineStr">
-        <is>
-          <t>Não conforme</t>
-        </is>
-      </c>
-      <c r="L62" s="1" t="n"/>
-      <c r="M62" s="1" t="n"/>
-      <c r="N62" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O62" s="1" t="n"/>
-      <c r="P62" s="1" t="inlineStr">
-        <is>
-          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="90.95" customHeight="1">
-      <c r="A63" s="1" t="inlineStr">
-        <is>
-          <t>AV154</t>
-        </is>
-      </c>
-      <c r="B63" s="1" t="inlineStr">
-        <is>
-          <t>questionario</t>
-        </is>
-      </c>
-      <c r="C63" s="1" t="n"/>
-      <c r="D63" s="1" t="n"/>
-      <c r="E63" s="1" t="n"/>
-      <c r="F63" s="1" t="inlineStr">
-        <is>
-          <t>existe_plano_ti</t>
-        </is>
-      </c>
-      <c r="G63" s="1" t="inlineStr">
-        <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
-        </is>
-      </c>
-      <c r="H63" s="1" t="inlineStr">
-        <is>
-          <t>Resposta ao item 2102 que não caracteriza a existência de plano de TIC vigente, ainda que parcialmente adotado</t>
-        </is>
-      </c>
-      <c r="I63" s="1" t="n"/>
-      <c r="J63" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
-        </is>
-      </c>
-      <c r="K63" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="L63" s="1" t="n"/>
-      <c r="M63" s="1" t="n"/>
-      <c r="N63" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O63" s="1" t="n"/>
-      <c r="P63" s="1" t="inlineStr">
-        <is>
           <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="90.95" customHeight="1">
-      <c r="A64" s="1" t="inlineStr">
-        <is>
-          <t>AV155</t>
-        </is>
-      </c>
-      <c r="B64" s="1" t="inlineStr">
-        <is>
-          <t>questionario</t>
-        </is>
-      </c>
-      <c r="C64" s="1" t="n"/>
-      <c r="D64" s="1" t="n"/>
-      <c r="E64" s="1" t="n"/>
-      <c r="F64" s="1" t="inlineStr">
-        <is>
-          <t>existe_plano_ti</t>
-        </is>
-      </c>
-      <c r="G64" s="1" t="inlineStr">
-        <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
-        </is>
-      </c>
-      <c r="H64" s="1" t="inlineStr">
-        <is>
-          <t>Plano de TIC vigente declarado no item 2102, ao menos parcialmente adotado</t>
-        </is>
-      </c>
-      <c r="I64" s="1" t="n"/>
-      <c r="J64" s="1" t="n"/>
-      <c r="K64" s="1" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="L64" s="1" t="n"/>
-      <c r="M64" s="1" t="n"/>
-      <c r="N64" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O64" s="1" t="n"/>
-      <c r="P64" s="1" t="inlineStr">
-        <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
-        </is>
-      </c>
-    </row>
+    <row r="53" ht="113.45" customHeight="1"/>
+    <row r="54" ht="113.45" customHeight="1"/>
+    <row r="55" ht="113.45" customHeight="1"/>
+    <row r="56" ht="113.45" customHeight="1"/>
+    <row r="57" ht="90.95" customHeight="1"/>
+    <row r="58" ht="90.95" customHeight="1"/>
+    <row r="59" ht="90.95" customHeight="1"/>
+    <row r="60" ht="79.90000000000001" customHeight="1"/>
+    <row r="61" ht="79.90000000000001" customHeight="1"/>
+    <row r="62" ht="90.95" customHeight="1"/>
+    <row r="63" ht="90.95" customHeight="1"/>
+    <row r="64" ht="90.95" customHeight="1"/>
     <row r="65" ht="90.95" customHeight="1"/>
     <row r="66" ht="90.95" customHeight="1"/>
     <row r="67" ht="79.90000000000001" customHeight="1"/>
@@ -4336,7 +3695,7 @@
     <row r="153" ht="23.85" customHeight="1"/>
     <row r="154" ht="23.85" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A3:P64"/>
+  <autoFilter ref="A3:P52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -4348,7 +3707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H62"/>
+  <dimension ref="A2:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5378,7 +4737,7 @@
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>AV54 &amp; ~AV124</t>
+          <t>AV54</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
@@ -5398,7 +4757,7 @@
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>MR066</t>
+          <t>MR067</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
@@ -5408,25 +4767,25 @@
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="D29" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>AV124</t>
+          <t>AV55</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>AV124</t>
+          <t>AV55</t>
         </is>
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
+          <t>No subitem b) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
         </is>
       </c>
       <c r="H29" s="9" t="b">
@@ -5436,7 +4795,7 @@
     <row r="30" ht="45" customHeight="1">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>MR067</t>
+          <t>MR069</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
@@ -5450,21 +4809,21 @@
         </is>
       </c>
       <c r="D30" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>AV55 &amp; ~AV125</t>
+          <t>AV56</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>AV55</t>
+          <t>AV56</t>
         </is>
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
+          <t>No subitem c) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
         </is>
       </c>
       <c r="H30" s="9" t="b">
@@ -5474,7 +4833,7 @@
     <row r="31" ht="45" customHeight="1">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>MR068</t>
+          <t>MR071</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
@@ -5484,7 +4843,7 @@
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D31" s="9" t="n">
@@ -5492,17 +4851,17 @@
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>AV125</t>
+          <t>AV57</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>AV125</t>
+          <t>AV57</t>
         </is>
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
+          <t>No subitem d) do item 2201, não houve declaração afirmativa quanto à prática avaliada: são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
         </is>
       </c>
       <c r="H31" s="9" t="b">
@@ -5512,7 +4871,7 @@
     <row r="32" ht="45" customHeight="1">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>MR069</t>
+          <t>MR073</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
@@ -5522,7 +4881,7 @@
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D32" s="9" t="n">
@@ -5530,17 +4889,17 @@
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>AV56 &amp; ~AV126</t>
+          <t>AV58</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>AV56</t>
+          <t>AV58</t>
         </is>
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
+          <t>No subitem e) do item 2201, não houve declaração afirmativa quanto à prática avaliada: a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
         </is>
       </c>
       <c r="H32" s="9" t="b">
@@ -5550,7 +4909,7 @@
     <row r="33" ht="45" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>MR070</t>
+          <t>MR075</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
@@ -5560,25 +4919,25 @@
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="D33" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>AV126</t>
+          <t>AV59</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>AV126</t>
+          <t>AV59</t>
         </is>
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
+          <t>No subitem a) do item 2203, não houve declaração afirmativa quanto à prática avaliada: mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
         </is>
       </c>
       <c r="H33" s="9" t="b">
@@ -5588,7 +4947,7 @@
     <row r="34" ht="45" customHeight="1">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>MR071</t>
+          <t>MR077</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
@@ -5598,25 +4957,25 @@
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
         </is>
       </c>
       <c r="D34" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>AV57 &amp; ~AV127</t>
+          <t>AV62</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>AV57</t>
+          <t>AV62</t>
         </is>
       </c>
       <c r="G34" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2201, não houve declaração afirmativa quanto à prática avaliada: são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
+          <t>No subitem a) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H34" s="9" t="b">
@@ -5626,7 +4985,7 @@
     <row r="35" ht="90" customHeight="1">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>MR072</t>
+          <t>MR079</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
@@ -5636,25 +4995,25 @@
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
         </is>
       </c>
       <c r="D35" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>AV127</t>
+          <t>AV63</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>AV127</t>
+          <t>AV63</t>
         </is>
       </c>
       <c r="G35" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
+          <t>No subitem b) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H35" s="9" t="b">
@@ -5664,7 +5023,7 @@
     <row r="36" ht="105" customHeight="1">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>MR073</t>
+          <t>MR083</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
@@ -5674,25 +5033,25 @@
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="D36" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>AV58 &amp; ~AV128</t>
+          <t>AV66</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>AV58</t>
+          <t>AV66</t>
         </is>
       </c>
       <c r="G36" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2201, não houve declaração afirmativa quanto à prática avaliada: a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
+          <t>No subitem c) do item 2203, não houve declaração afirmativa quanto à prática avaliada: o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H36" s="9" t="b">
@@ -5702,7 +5061,7 @@
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>MR074</t>
+          <t>MR085</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
@@ -5712,25 +5071,25 @@
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="D37" s="9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>AV128</t>
+          <t>AV67</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>AV128</t>
+          <t>AV67</t>
         </is>
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
+          <t>No subitem a) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu regras para a priorização e o escalamento de incidentes</t>
         </is>
       </c>
       <c r="H37" s="9" t="b">
@@ -5740,7 +5099,7 @@
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>MR075</t>
+          <t>MR087</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
@@ -5750,25 +5109,25 @@
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="D38" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>AV59 &amp; ~AV129</t>
+          <t>AV70</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>AV59</t>
+          <t>AV70</t>
         </is>
       </c>
       <c r="G38" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2203, não houve declaração afirmativa quanto à prática avaliada: mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
+          <t>No subitem d) do item 2204, não houve declaração afirmativa quanto à prática avaliada: o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H38" s="9" t="b">
@@ -5778,7 +5137,7 @@
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>MR076</t>
+          <t>MR089</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
@@ -5788,25 +5147,25 @@
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="D39" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>AV129</t>
+          <t>AV71</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>AV129</t>
+          <t>AV71</t>
         </is>
       </c>
       <c r="G39" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
+          <t>No subitem e) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
         </is>
       </c>
       <c r="H39" s="9" t="b">
@@ -5816,35 +5175,35 @@
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>MR077</t>
+          <t>MR091</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D40" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>AV62 &amp; ~AV132</t>
+          <t>AV73 &amp; ~AV143</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>AV62</t>
+          <t>AV73</t>
         </is>
       </c>
       <c r="G40" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
+          <t>No subitem a) do item 2801, não houve declaração afirmativa quanto à prática avaliada: o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
         </is>
       </c>
       <c r="H40" s="9" t="b">
@@ -5854,35 +5213,35 @@
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>MR078</t>
+          <t>MR092</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D41" s="9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>AV132</t>
+          <t>AV143</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>AV132</t>
+          <t>AV143</t>
         </is>
       </c>
       <c r="G41" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
+          <t>No subitem a) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
         </is>
       </c>
       <c r="H41" s="9" t="b">
@@ -5892,35 +5251,35 @@
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>MR079</t>
+          <t>MR101</t>
         </is>
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
         </is>
       </c>
       <c r="D42" s="9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>AV63 &amp; ~AV133</t>
+          <t>AV78 &amp; ~AV148</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>AV63</t>
+          <t>AV78</t>
         </is>
       </c>
       <c r="G42" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
+          <t>No subitem a) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
         </is>
       </c>
       <c r="H42" s="9" t="b">
@@ -5930,35 +5289,35 @@
     <row r="43" ht="45" customHeight="1">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>MR080</t>
+          <t>MR102</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do inventário de ativos de TIC.</t>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
         </is>
       </c>
       <c r="D43" s="9" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>AV133</t>
+          <t>AV148</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>AV133</t>
+          <t>AV148</t>
         </is>
       </c>
       <c r="G43" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
+          <t>No subitem a) do item 2804, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
         </is>
       </c>
       <c r="H43" s="9" t="b">
@@ -5968,17 +5327,17 @@
     <row r="44" ht="45" customHeight="1">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>MR083</t>
+          <t>MR105</t>
         </is>
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
         </is>
       </c>
       <c r="D44" s="9" t="n">
@@ -5986,17 +5345,17 @@
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>AV66 &amp; ~AV136</t>
+          <t>AV80 &amp; ~AV150</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>AV66</t>
+          <t>AV80</t>
         </is>
       </c>
       <c r="G44" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2203, não houve declaração afirmativa quanto à prática avaliada: o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem c) do item 2802, não houve declaração afirmativa quanto à prática avaliada: na elaboração do PCA são considerados os demais instrumentos de planejamento da organização</t>
         </is>
       </c>
       <c r="H44" s="9" t="b">
@@ -6006,17 +5365,17 @@
     <row r="45" ht="45" customHeight="1">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>MR084</t>
+          <t>MR106</t>
         </is>
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
         </is>
       </c>
       <c r="D45" s="9" t="n">
@@ -6024,17 +5383,17 @@
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>AV136</t>
+          <t>AV150</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>AV136</t>
+          <t>AV150</t>
         </is>
       </c>
       <c r="G45" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem c) do item 2802, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que na elaboração do PCA são considerados os demais instrumentos de planejamento da organização</t>
         </is>
       </c>
       <c r="H45" s="9" t="b">
@@ -6044,35 +5403,35 @@
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>MR085</t>
+          <t>MR109</t>
         </is>
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
         </is>
       </c>
       <c r="D46" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>AV67 &amp; ~AV137</t>
+          <t>AV82</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>AV67</t>
+          <t>AV82</t>
         </is>
       </c>
       <c r="G46" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu regras para a priorização e o escalamento de incidentes</t>
+          <t>No subitem b) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de TI executadas no exercício encontram-se previamente estabelecidas nos instrumentos de planejamento vigentes (PDTI/PEDTIC e PCA)</t>
         </is>
       </c>
       <c r="H46" s="9" t="b">
@@ -6082,35 +5441,35 @@
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>MR086</t>
+          <t>MR110</t>
         </is>
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
         </is>
       </c>
       <c r="D47" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>AV137</t>
+          <t>AV83</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>AV137</t>
+          <t>AV83</t>
         </is>
       </c>
       <c r="G47" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu regras para a priorização e o escalamento de incidentes</t>
+          <t>No subitem c) do item 2804, não houve declaração afirmativa quanto à prática avaliada: a fase de planejamento de cada contratação de TI é conduzida por uma Equipe de Planejamento da Contratação formalmente designada (composta, minimamente, por integrante requisitante e integrante técnico da área de TI)</t>
         </is>
       </c>
       <c r="H47" s="9" t="b">
@@ -6120,35 +5479,35 @@
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>MR087</t>
+          <t>MR111</t>
         </is>
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D48" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>AV70 &amp; ~AV140</t>
+          <t>AV152 &amp; ~AV153</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>AV70</t>
+          <t>AV152</t>
         </is>
       </c>
       <c r="G48" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2204, não houve declaração afirmativa quanto à prática avaliada: o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem b) do item 2801, não houve declaração afirmativa quanto à prática avaliada: são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
         </is>
       </c>
       <c r="H48" s="9" t="b">
@@ -6158,17 +5517,17 @@
     <row r="49" ht="45" customHeight="1">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>MR088</t>
+          <t>MR112</t>
         </is>
       </c>
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D49" s="9" t="n">
@@ -6176,17 +5535,17 @@
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>AV140</t>
+          <t>AV153</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>AV140</t>
+          <t>AV153</t>
         </is>
       </c>
       <c r="G49" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem b) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
         </is>
       </c>
       <c r="H49" s="9" t="b">
@@ -6196,497 +5555,53 @@
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>MR089</t>
+          <t>MR113</t>
         </is>
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA03</t>
         </is>
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="D50" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>AV71 &amp; ~AV141</t>
+          <t>AV154</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>AV71</t>
+          <t>AV154</t>
         </is>
       </c>
       <c r="G50" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
+          <t>No item 2102, a organização não declarou possuir plano de tecnologia da informação vigente, ainda que parcialmente adotado</t>
         </is>
       </c>
       <c r="H50" s="9" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="51" ht="30" customHeight="1">
-      <c r="A51" s="9" t="inlineStr">
-        <is>
-          <t>MR090</t>
-        </is>
-      </c>
-      <c r="B51" s="9" t="inlineStr">
-        <is>
-          <t>PA05</t>
-        </is>
-      </c>
-      <c r="C51" s="9" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
-        </is>
-      </c>
-      <c r="D51" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="E51" s="9" t="inlineStr">
-        <is>
-          <t>AV141</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="inlineStr">
-        <is>
-          <t>AV141</t>
-        </is>
-      </c>
-      <c r="G51" s="9" t="inlineStr">
-        <is>
-          <t>No subitem e) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
-        </is>
-      </c>
-      <c r="H51" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" ht="30" customHeight="1">
-      <c r="A52" s="9" t="inlineStr">
-        <is>
-          <t>MR091</t>
-        </is>
-      </c>
-      <c r="B52" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C52" s="9" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="D52" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E52" s="9" t="inlineStr">
-        <is>
-          <t>AV73 &amp; ~AV143</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="inlineStr">
-        <is>
-          <t>AV73</t>
-        </is>
-      </c>
-      <c r="G52" s="9" t="inlineStr">
-        <is>
-          <t>No subitem a) do item 2801, não houve declaração afirmativa quanto à prática avaliada: o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
-        </is>
-      </c>
-      <c r="H52" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" ht="30" customHeight="1">
-      <c r="A53" s="9" t="inlineStr">
-        <is>
-          <t>MR092</t>
-        </is>
-      </c>
-      <c r="B53" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C53" s="9" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="D53" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="E53" s="9" t="inlineStr">
-        <is>
-          <t>AV143</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="inlineStr">
-        <is>
-          <t>AV143</t>
-        </is>
-      </c>
-      <c r="G53" s="9" t="inlineStr">
-        <is>
-          <t>No subitem a) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
-        </is>
-      </c>
-      <c r="H53" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="54" ht="30" customHeight="1">
-      <c r="A54" s="9" t="inlineStr">
-        <is>
-          <t>MR101</t>
-        </is>
-      </c>
-      <c r="B54" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C54" s="9" t="inlineStr">
-        <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
-        </is>
-      </c>
-      <c r="D54" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E54" s="9" t="inlineStr">
-        <is>
-          <t>AV78 &amp; ~AV148</t>
-        </is>
-      </c>
-      <c r="F54" s="9" t="inlineStr">
-        <is>
-          <t>AV78</t>
-        </is>
-      </c>
-      <c r="G54" s="9" t="inlineStr">
-        <is>
-          <t>No subitem a) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
-        </is>
-      </c>
-      <c r="H54" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55" ht="45" customHeight="1">
-      <c r="A55" s="9" t="inlineStr">
-        <is>
-          <t>MR102</t>
-        </is>
-      </c>
-      <c r="B55" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C55" s="9" t="inlineStr">
-        <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
-        </is>
-      </c>
-      <c r="D55" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E55" s="9" t="inlineStr">
-        <is>
-          <t>AV148</t>
-        </is>
-      </c>
-      <c r="F55" s="9" t="inlineStr">
-        <is>
-          <t>AV148</t>
-        </is>
-      </c>
-      <c r="G55" s="9" t="inlineStr">
-        <is>
-          <t>No subitem a) do item 2804, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
-        </is>
-      </c>
-      <c r="H55" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" ht="45" customHeight="1">
-      <c r="A56" s="9" t="inlineStr">
-        <is>
-          <t>MR105</t>
-        </is>
-      </c>
-      <c r="B56" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C56" s="9" t="inlineStr">
-        <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
-        </is>
-      </c>
-      <c r="D56" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E56" s="9" t="inlineStr">
-        <is>
-          <t>AV80 &amp; ~AV150</t>
-        </is>
-      </c>
-      <c r="F56" s="9" t="inlineStr">
-        <is>
-          <t>AV80</t>
-        </is>
-      </c>
-      <c r="G56" s="9" t="inlineStr">
-        <is>
-          <t>No subitem c) do item 2802, não houve declaração afirmativa quanto à prática avaliada: na elaboração do PCA são considerados os demais instrumentos de planejamento da organização</t>
-        </is>
-      </c>
-      <c r="H56" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57" ht="45" customHeight="1">
-      <c r="A57" s="9" t="inlineStr">
-        <is>
-          <t>MR106</t>
-        </is>
-      </c>
-      <c r="B57" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C57" s="9" t="inlineStr">
-        <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
-        </is>
-      </c>
-      <c r="D57" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E57" s="9" t="inlineStr">
-        <is>
-          <t>AV150</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="inlineStr">
-        <is>
-          <t>AV150</t>
-        </is>
-      </c>
-      <c r="G57" s="9" t="inlineStr">
-        <is>
-          <t>No subitem c) do item 2802, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que na elaboração do PCA são considerados os demais instrumentos de planejamento da organização</t>
-        </is>
-      </c>
-      <c r="H57" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58" ht="45" customHeight="1">
-      <c r="A58" s="9" t="inlineStr">
-        <is>
-          <t>MR109</t>
-        </is>
-      </c>
-      <c r="B58" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C58" s="9" t="inlineStr">
-        <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
-        </is>
-      </c>
-      <c r="D58" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="E58" s="9" t="inlineStr">
-        <is>
-          <t>AV82</t>
-        </is>
-      </c>
-      <c r="F58" s="9" t="inlineStr">
-        <is>
-          <t>AV82</t>
-        </is>
-      </c>
-      <c r="G58" s="9" t="inlineStr">
-        <is>
-          <t>No subitem b) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de TI executadas no exercício encontram-se previamente estabelecidas nos instrumentos de planejamento vigentes (PDTI/PEDTIC e PCA)</t>
-        </is>
-      </c>
-      <c r="H58" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" ht="45" customHeight="1">
-      <c r="A59" s="9" t="inlineStr">
-        <is>
-          <t>MR110</t>
-        </is>
-      </c>
-      <c r="B59" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C59" s="9" t="inlineStr">
-        <is>
-          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
-        </is>
-      </c>
-      <c r="D59" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E59" s="9" t="inlineStr">
-        <is>
-          <t>AV83</t>
-        </is>
-      </c>
-      <c r="F59" s="9" t="inlineStr">
-        <is>
-          <t>AV83</t>
-        </is>
-      </c>
-      <c r="G59" s="9" t="inlineStr">
-        <is>
-          <t>No subitem c) do item 2804, não houve declaração afirmativa quanto à prática avaliada: a fase de planejamento de cada contratação de TI é conduzida por uma Equipe de Planejamento da Contratação formalmente designada (composta, minimamente, por integrante requisitante e integrante técnico da área de TI)</t>
-        </is>
-      </c>
-      <c r="H59" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60" ht="30" customHeight="1">
-      <c r="A60" s="9" t="inlineStr">
-        <is>
-          <t>MR111</t>
-        </is>
-      </c>
-      <c r="B60" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C60" s="9" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="D60" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E60" s="9" t="inlineStr">
-        <is>
-          <t>AV152 &amp; ~AV153</t>
-        </is>
-      </c>
-      <c r="F60" s="9" t="inlineStr">
-        <is>
-          <t>AV152</t>
-        </is>
-      </c>
-      <c r="G60" s="9" t="inlineStr">
-        <is>
-          <t>No subitem b) do item 2801, não houve declaração afirmativa quanto à prática avaliada: são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
-        </is>
-      </c>
-      <c r="H60" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="61" ht="45" customHeight="1">
-      <c r="A61" s="9" t="inlineStr">
-        <is>
-          <t>MR112</t>
-        </is>
-      </c>
-      <c r="B61" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C61" s="9" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="D61" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="E61" s="9" t="inlineStr">
-        <is>
-          <t>AV153</t>
-        </is>
-      </c>
-      <c r="F61" s="9" t="inlineStr">
-        <is>
-          <t>AV153</t>
-        </is>
-      </c>
-      <c r="G61" s="9" t="inlineStr">
-        <is>
-          <t>No subitem b) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
-        </is>
-      </c>
-      <c r="H61" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" ht="45" customHeight="1">
-      <c r="A62" s="9" t="inlineStr">
-        <is>
-          <t>MR113</t>
-        </is>
-      </c>
-      <c r="B62" s="9" t="inlineStr">
-        <is>
-          <t>PA03</t>
-        </is>
-      </c>
-      <c r="C62" s="9" t="inlineStr">
-        <is>
-          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
-        </is>
-      </c>
-      <c r="D62" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E62" s="9" t="inlineStr">
-        <is>
-          <t>AV154</t>
-        </is>
-      </c>
-      <c r="F62" s="9" t="inlineStr">
-        <is>
-          <t>AV154</t>
-        </is>
-      </c>
-      <c r="G62" s="9" t="inlineStr">
-        <is>
-          <t>No item 2102, a organização não declarou possuir plano de tecnologia da informação vigente, ainda que parcialmente adotado</t>
-        </is>
-      </c>
-      <c r="H62" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
+    <row r="51" ht="30" customHeight="1"/>
+    <row r="52" ht="30" customHeight="1"/>
+    <row r="53" ht="30" customHeight="1"/>
+    <row r="54" ht="30" customHeight="1"/>
+    <row r="55" ht="45" customHeight="1"/>
+    <row r="56" ht="45" customHeight="1"/>
+    <row r="57" ht="45" customHeight="1"/>
+    <row r="58" ht="45" customHeight="1"/>
+    <row r="59" ht="45" customHeight="1"/>
+    <row r="60" ht="30" customHeight="1"/>
+    <row r="61" ht="45" customHeight="1"/>
+    <row r="62" ht="45" customHeight="1"/>
     <row r="63" ht="30" customHeight="1"/>
     <row r="64" ht="45" customHeight="1"/>
     <row r="65" ht="30" customHeight="1"/>
@@ -6739,7 +5654,7 @@
     <row r="112" ht="45" customHeight="1"/>
     <row r="113" ht="45" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A3:H62"/>
+  <autoFilter ref="A3:H50"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Revisa a Questão 6 da matriz e do mapa
</commit_message>
<xml_diff>
--- a/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
+++ b/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
@@ -15,8 +15,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Fontes de Informação'!$A$3:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Procedimentos de Auditoria'!$A$3:$E$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ações de Verificação'!$A$3:$P$52</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Motivos do Relatório'!$A$3:$H$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ações de Verificação'!$A$3:$P$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Motivos do Relatório'!$A$3:$H$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Variáveis Temporárias'!$A$3:$E$6</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -674,7 +674,7 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>(((AV73 | AV143) | (AV152 | AV153)) | (AV78 | AV148) | (AV82 | (AV80 | AV150)) | AV83)</t>
+          <t>((AV73 | AV152) | AV78 | AV82 | AV83)</t>
         </is>
       </c>
       <c r="D9" s="1" t="n">
@@ -699,7 +699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P52"/>
+  <dimension ref="A1:P47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2898,8 +2898,9 @@
       </c>
       <c r="G40" s="1" t="inlineStr">
         <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
+          <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Lei nº 14.133/2021, art. 19, inciso IV: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.
+Acórdão nº 2.342/2016-TCU-Plenário, item 9.1.7 – Precedente quanto à definição, aprovação e formalização de processo de trabalho para o planejamento de cada contratação, com controles internos mínimos.</t>
         </is>
       </c>
       <c r="H40" s="1" t="inlineStr">
@@ -2922,13 +2923,13 @@
       <c r="M40" s="1" t="n"/>
       <c r="N40" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O40" s="1" t="n"/>
       <c r="P40" s="1" t="inlineStr">
         <is>
-          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
+          <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
         </is>
       </c>
     </row>
@@ -2953,9 +2954,9 @@
       </c>
       <c r="G41" s="1" t="inlineStr">
         <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+          <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
 COBIT 2019, BAI02.04 - Obter aprovação dos requisitos da solução: obter aprovação formal dos requisitos funcionais, técnicos, de segurança e de conformidade antes de prosseguir com a solução.
-Instrução Normativa SGD/ME nº 94, de 23 de dezembro de 2022, art. 1º, § 1º: como referência de boa prática, a aplicação de ritos formais de contratação de TIC pode ser facultada para contratações diretas por dispensa em razão do valor (inciso II do art. 75 da Lei nº 14.133/2021), indicando a possibilidade de fluxos simplificados para aquisições de baixa complexidade ou valor.</t>
+Instrução Normativa SGD/ME nº 94/2022, arts. 1º, §1º, 10, II, 11, §2º, e 12, §6º – referência de boa prática para estruturação da fase de planejamento das contratações de TIC, participação da área técnica e instituição da Equipe de Planejamento, observada sua aplicação direta aos integrantes do SISP e a possibilidade de procedimentos simplificados.</t>
         </is>
       </c>
       <c r="H41" s="1" t="inlineStr">
@@ -2984,14 +2985,14 @@
       <c r="O41" s="1" t="n"/>
       <c r="P41" s="1" t="inlineStr">
         <is>
-          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo fluxos simplificados para contratações de baixa complexidade ou baixo valor, desde que preservada análise técnica mínima compatível com o risco da contratação</t>
+          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo procedimentos simplificados e proporcionais à natureza, ao risco e ao valor da contratação, preservada análise técnica compatível</t>
         </is>
       </c>
     </row>
     <row r="42" ht="113.45" customHeight="1">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>AV80</t>
+          <t>AV82</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -3004,18 +3005,19 @@
       <c r="E42" s="1" t="n"/>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>q2802ext[C]</t>
+          <t>q2804[B]</t>
         </is>
       </c>
       <c r="G42" s="1" t="inlineStr">
         <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 18, caput e §1º, incisos I, IV, V, VIII, IX, X e XIII, da Lei 14.133/2021: fase preparatória caracterizada pelo planejamento, compatibilização com o plano de contratações anual e elementos mínimos do estudo técnico preliminar.</t>
+          <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Lei nº 14.133/2021, arts. 12, VII e §1º, e 18, caput e §1º, II – a fase preparatória deve compatibilizar-se com o Plano de Contratações Anual, quando elaborado, e deve ser demonstrado o alinhamento da contratação com o planejamento da Administração.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens III.7 e IV.9 – Determinações para estruturação do processo de planejamento anual das contratações, contemplando consolidação das demandas, participação das áreas, aprovação e publicidade do plano.</t>
         </is>
       </c>
       <c r="H42" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento c) do item 2802 do Questionário, para verificar se na elaboração do PCA são considerados os demais instrumentos de planejamento da organização</t>
+          <t>Resposta negativa ao subitem b) do item 2804 do Questionário, para verificar se as contratações de TI executadas no exercício encontram-se previamente estabelecidas nos instrumentos de planejamento vigentes (PDTI/PEDTIC e PCA)</t>
         </is>
       </c>
       <c r="I42" s="1" t="n"/>
@@ -3026,7 +3028,7 @@
       </c>
       <c r="K42" s="1" t="inlineStr">
         <is>
-          <t>(Não | N/A)</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="L42" s="1" t="n"/>
@@ -3039,14 +3041,14 @@
       <c r="O42" s="1" t="n"/>
       <c r="P42" s="1" t="inlineStr">
         <is>
-          <t>integre as contratações de TIC com os instrumentos de planejamento da organização e com o Plano de Contratações Anual, quando elaborado, justificando as situações excepcionais</t>
+          <t>assegure que as contratações de TIC sejam compatíveis com os instrumentos de planejamento de TIC e, quando elaborado, com o Plano de Contratações Anual, promovendo os ajustes ou justificativas cabíveis nos casos excepcionais</t>
         </is>
       </c>
     </row>
     <row r="43" ht="113.45" customHeight="1">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>AV82</t>
+          <t>AV83</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -3059,24 +3061,25 @@
       <c r="E43" s="1" t="n"/>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>q2804[B]</t>
+          <t>q2804[C]</t>
         </is>
       </c>
       <c r="G43" s="1" t="inlineStr">
         <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 18, caput e §1º, incisos I, IV, V, VIII, IX, X e XIII, da Lei 14.133/2021: fase preparatória caracterizada pelo planejamento, compatibilização com o plano de contratações anual e elementos mínimos do estudo técnico preliminar.</t>
+          <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Lei nº 14.133/2021, art. 7º, caput, incisos I a III e §1º: designação de agentes públicos para funções essenciais, observados atribuições, formação, segregação de funções e inexistência de vínculos que comprometam a atuação.
+Instrução Normativa SGD/ME nº 94/2022, arts. 1º, §1º, 10, II, 11, §2º, e 12, §6º – referência de boa prática para estruturação da fase de planejamento das contratações de TIC, participação da área técnica e instituição da Equipe de Planejamento, observada sua aplicação direta aos integrantes do SISP e a possibilidade de procedimentos simplificados.</t>
         </is>
       </c>
       <c r="H43" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao subitem b) do item 2804 do Questionário, para verificar se as contratações de TI executadas no exercício encontram-se previamente estabelecidas nos instrumentos de planejamento vigentes (PDTI/PEDTIC e PCA)</t>
+          <t>Resposta negativa ao subitem c) do item 2804 do Questionário, para verificar se a fase de planejamento de cada contratação de TI é conduzida por uma Equipe de Planejamento da Contratação formalmente designada (composta, minimamente, por integrante requisitante e integrante técnico da área de TI)</t>
         </is>
       </c>
       <c r="I43" s="1" t="n"/>
       <c r="J43" s="1" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
+          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
         </is>
       </c>
       <c r="K43" s="1" t="inlineStr">
@@ -3088,25 +3091,25 @@
       <c r="M43" s="1" t="n"/>
       <c r="N43" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O43" s="1" t="n"/>
       <c r="P43" s="1" t="inlineStr">
         <is>
-          <t>integre as contratações de TIC com os instrumentos de planejamento da organização e com o Plano de Contratações Anual, quando elaborado, justificando as situações excepcionais</t>
+          <t>designe formalmente equipe de planejamento para as contratações de TIC, atentando-se, minimamente, em assegurar a participação de integrante da área requisitante e da área técnica de TIC, com definição das responsabilidades de seus integrantes</t>
         </is>
       </c>
     </row>
     <row r="44" ht="113.45" customHeight="1">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>AV83</t>
+          <t>AV84</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
-          <t>questionario</t>
+          <t>avaliacao_evidencias_ajustes</t>
         </is>
       </c>
       <c r="C44" s="1" t="n"/>
@@ -3114,29 +3117,29 @@
       <c r="E44" s="1" t="n"/>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>q2804[C]</t>
+          <t>q0103[D]</t>
         </is>
       </c>
       <c r="G44" s="1" t="inlineStr">
         <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 7º, caput, incisos I a III e §1º, da Lei 14.133/2021: designação de agentes públicos para funções essenciais, observados atribuições, formação, segregação de funções e inexistência de vínculos que comprometam a atuação.</t>
+          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TI.
+Constituição Federal, art. 37, caput - Princípio da eficiência.</t>
         </is>
       </c>
       <c r="H44" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao subitem c) do item 2804 do Questionário, para verificar se a fase de planejamento de cada contratação de TI é conduzida por uma Equipe de Planejamento da Contratação formalmente designada (composta, minimamente, por integrante requisitante e integrante técnico da área de TI)</t>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
         </is>
       </c>
       <c r="I44" s="1" t="n"/>
       <c r="J44" s="1" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
+          <t>Área de TIC sem atribuições formalmente definidas ou sem atribuições formais de gestão de TIC.</t>
         </is>
       </c>
       <c r="K44" s="1" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Não conforme</t>
         </is>
       </c>
       <c r="L44" s="1" t="n"/>
@@ -3149,19 +3152,19 @@
       <c r="O44" s="1" t="n"/>
       <c r="P44" s="1" t="inlineStr">
         <is>
-          <t>designe formalmente equipe de planejamento para as contratações de TIC, atentando-se, minimamente, em assegurar a participação de integrante da área requisitante e da área técnica de TIC, com definição das responsabilidades de seus integrantes</t>
+          <t>defina formalmente as atribuições da área de TIC, atentando-se, minimamente, em abranger as atividades de planejamento, coordenação, gestão e controle da TIC</t>
         </is>
       </c>
     </row>
     <row r="45" ht="113.45" customHeight="1">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>AV84</t>
+          <t>AV152</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
-          <t>avaliacao_evidencias_ajustes</t>
+          <t>questionario</t>
         </is>
       </c>
       <c r="C45" s="1" t="n"/>
@@ -3169,29 +3172,30 @@
       <c r="E45" s="1" t="n"/>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>q0103[D]</t>
+          <t>q2801ext[B]</t>
         </is>
       </c>
       <c r="G45" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TI.
-Constituição Federal, art. 37, caput - Princípio da eficiência.</t>
+          <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Lei nº 14.133/2021, art. 19, inciso IV: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.
+Acórdão nº 2.342/2016-TCU-Plenário, item 9.1.7 – Precedente quanto à definição, aprovação e formalização de processo de trabalho para o planejamento de cada contratação, com controles internos mínimos.</t>
         </is>
       </c>
       <c r="H45" s="1" t="inlineStr">
         <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+          <t>Resposta negativa ao detalhamento b) do item 2801 do Questionário, para verificar se são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
         </is>
       </c>
       <c r="I45" s="1" t="n"/>
       <c r="J45" s="1" t="inlineStr">
         <is>
-          <t>Área de TIC sem atribuições formalmente definidas ou sem atribuições formais de gestão de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="K45" s="1" t="inlineStr">
         <is>
-          <t>Não conforme</t>
+          <t>(Não | N/A)</t>
         </is>
       </c>
       <c r="L45" s="1" t="n"/>
@@ -3204,19 +3208,19 @@
       <c r="O45" s="1" t="n"/>
       <c r="P45" s="1" t="inlineStr">
         <is>
-          <t>defina formalmente as atribuições da área de TIC, atentando-se, minimamente, em abranger as atividades de planejamento, coordenação, gestão e controle da TIC</t>
+          <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
         </is>
       </c>
     </row>
     <row r="46" ht="113.45" customHeight="1">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>AV143</t>
+          <t>AV154</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
-          <t>avaliacao_evidencias_ajustes</t>
+          <t>questionario</t>
         </is>
       </c>
       <c r="C46" s="1" t="n"/>
@@ -3224,29 +3228,30 @@
       <c r="E46" s="1" t="n"/>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>q2801ext[A]</t>
+          <t>existe_plano_ti</t>
         </is>
       </c>
       <c r="G46" s="1" t="inlineStr">
         <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H46" s="1" t="inlineStr">
         <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+          <t>Resposta ao item 2102 que não caracteriza a existência de plano de TIC vigente, ainda que parcialmente adotado</t>
         </is>
       </c>
       <c r="I46" s="1" t="n"/>
       <c r="J46" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="K46" s="1" t="inlineStr">
         <is>
-          <t>Não conforme</t>
+          <t>False</t>
         </is>
       </c>
       <c r="L46" s="1" t="n"/>
@@ -3259,19 +3264,19 @@
       <c r="O46" s="1" t="n"/>
       <c r="P46" s="1" t="inlineStr">
         <is>
-          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
     <row r="47" ht="113.45" customHeight="1">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>AV148</t>
+          <t>AV155</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
-          <t>avaliacao_evidencias_ajustes</t>
+          <t>questionario</t>
         </is>
       </c>
       <c r="C47" s="1" t="n"/>
@@ -3279,319 +3284,47 @@
       <c r="E47" s="1" t="n"/>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>q2804[A]</t>
+          <t>existe_plano_ti</t>
         </is>
       </c>
       <c r="G47" s="1" t="inlineStr">
         <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-COBIT 2019, BAI02.04 - Obter aprovação dos requisitos da solução: obter aprovação formal dos requisitos funcionais, técnicos, de segurança e de conformidade antes de prosseguir com a solução.
-Instrução Normativa SGD/ME nº 94, de 23 de dezembro de 2022, art. 1º, § 1º: como referência de boa prática, a aplicação de ritos formais de contratação de TIC pode ser facultada para contratações diretas por dispensa em razão do valor (inciso II do art. 75 da Lei nº 14.133/2021), indicando a possibilidade de fluxos simplificados para aquisições de baixa complexidade ou valor.</t>
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H47" s="1" t="inlineStr">
         <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+          <t>Plano de TIC vigente declarado no item 2102, ao menos parcialmente adotado</t>
         </is>
       </c>
       <c r="I47" s="1" t="n"/>
-      <c r="J47" s="1" t="inlineStr">
-        <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
-        </is>
-      </c>
+      <c r="J47" s="1" t="n"/>
       <c r="K47" s="1" t="inlineStr">
         <is>
-          <t>Não conforme</t>
+          <t>True</t>
         </is>
       </c>
       <c r="L47" s="1" t="n"/>
       <c r="M47" s="1" t="n"/>
       <c r="N47" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O47" s="1" t="n"/>
       <c r="P47" s="1" t="inlineStr">
         <is>
-          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo fluxos simplificados para contratações de baixa complexidade ou baixo valor, desde que preservada análise técnica mínima compatível com o risco da contratação</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="113.45" customHeight="1">
-      <c r="A48" s="1" t="inlineStr">
-        <is>
-          <t>AV150</t>
-        </is>
-      </c>
-      <c r="B48" s="1" t="inlineStr">
-        <is>
-          <t>avaliacao_evidencias_ajustes</t>
-        </is>
-      </c>
-      <c r="C48" s="1" t="n"/>
-      <c r="D48" s="1" t="n"/>
-      <c r="E48" s="1" t="n"/>
-      <c r="F48" s="1" t="inlineStr">
-        <is>
-          <t>q2802ext[C]</t>
-        </is>
-      </c>
-      <c r="G48" s="1" t="inlineStr">
-        <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 18, caput e §1º, incisos I, IV, V, VIII, IX, X e XIII, da Lei 14.133/2021: fase preparatória caracterizada pelo planejamento, compatibilização com o plano de contratações anual e elementos mínimos do estudo técnico preliminar.</t>
-        </is>
-      </c>
-      <c r="H48" s="1" t="inlineStr">
-        <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
-        </is>
-      </c>
-      <c r="I48" s="1" t="n"/>
-      <c r="J48" s="1" t="inlineStr">
-        <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
-        </is>
-      </c>
-      <c r="K48" s="1" t="inlineStr">
-        <is>
-          <t>Não conforme</t>
-        </is>
-      </c>
-      <c r="L48" s="1" t="n"/>
-      <c r="M48" s="1" t="n"/>
-      <c r="N48" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O48" s="1" t="n"/>
-      <c r="P48" s="1" t="inlineStr">
-        <is>
-          <t>integre as contratações de TIC com os instrumentos de planejamento da organização e com o Plano de Contratações Anual, quando elaborado, justificando as situações excepcionais</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="113.45" customHeight="1">
-      <c r="A49" s="1" t="inlineStr">
-        <is>
-          <t>AV152</t>
-        </is>
-      </c>
-      <c r="B49" s="1" t="inlineStr">
-        <is>
-          <t>questionario</t>
-        </is>
-      </c>
-      <c r="C49" s="1" t="n"/>
-      <c r="D49" s="1" t="n"/>
-      <c r="E49" s="1" t="n"/>
-      <c r="F49" s="1" t="inlineStr">
-        <is>
-          <t>q2801ext[B]</t>
-        </is>
-      </c>
-      <c r="G49" s="1" t="inlineStr">
-        <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
-        </is>
-      </c>
-      <c r="H49" s="1" t="inlineStr">
-        <is>
-          <t>Resposta negativa ao detalhamento b) do item 2801 do Questionário, para verificar se são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
-        </is>
-      </c>
-      <c r="I49" s="1" t="n"/>
-      <c r="J49" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="K49" s="1" t="inlineStr">
-        <is>
-          <t>(Não | N/A)</t>
-        </is>
-      </c>
-      <c r="L49" s="1" t="n"/>
-      <c r="M49" s="1" t="n"/>
-      <c r="N49" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O49" s="1" t="n"/>
-      <c r="P49" s="1" t="inlineStr">
-        <is>
-          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="113.45" customHeight="1">
-      <c r="A50" s="1" t="inlineStr">
-        <is>
-          <t>AV153</t>
-        </is>
-      </c>
-      <c r="B50" s="1" t="inlineStr">
-        <is>
-          <t>avaliacao_evidencias_ajustes</t>
-        </is>
-      </c>
-      <c r="C50" s="1" t="n"/>
-      <c r="D50" s="1" t="n"/>
-      <c r="E50" s="1" t="n"/>
-      <c r="F50" s="1" t="inlineStr">
-        <is>
-          <t>q2801ext[B]</t>
-        </is>
-      </c>
-      <c r="G50" s="1" t="inlineStr">
-        <is>
-          <t>Art. 11, parágrafo único, da Lei 14.133/2021: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Art. 19, inciso IV, da Lei 14.133/2021: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.</t>
-        </is>
-      </c>
-      <c r="H50" s="1" t="inlineStr">
-        <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
-        </is>
-      </c>
-      <c r="I50" s="1" t="n"/>
-      <c r="J50" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="K50" s="1" t="inlineStr">
-        <is>
-          <t>Não conforme</t>
-        </is>
-      </c>
-      <c r="L50" s="1" t="n"/>
-      <c r="M50" s="1" t="n"/>
-      <c r="N50" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O50" s="1" t="n"/>
-      <c r="P50" s="1" t="inlineStr">
-        <is>
-          <t>formalize e padronize o processo de planejamento das contratações de TIC, com etapas, responsabilidades e artefatos padronizados, admitidos fluxos proporcionais à complexidade e ao risco</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="113.45" customHeight="1">
-      <c r="A51" s="1" t="inlineStr">
-        <is>
-          <t>AV154</t>
-        </is>
-      </c>
-      <c r="B51" s="1" t="inlineStr">
-        <is>
-          <t>questionario</t>
-        </is>
-      </c>
-      <c r="C51" s="1" t="n"/>
-      <c r="D51" s="1" t="n"/>
-      <c r="E51" s="1" t="n"/>
-      <c r="F51" s="1" t="inlineStr">
-        <is>
-          <t>existe_plano_ti</t>
-        </is>
-      </c>
-      <c r="G51" s="1" t="inlineStr">
-        <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
-        </is>
-      </c>
-      <c r="H51" s="1" t="inlineStr">
-        <is>
-          <t>Resposta ao item 2102 que não caracteriza a existência de plano de TIC vigente, ainda que parcialmente adotado</t>
-        </is>
-      </c>
-      <c r="I51" s="1" t="n"/>
-      <c r="J51" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
-        </is>
-      </c>
-      <c r="K51" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="L51" s="1" t="n"/>
-      <c r="M51" s="1" t="n"/>
-      <c r="N51" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O51" s="1" t="n"/>
-      <c r="P51" s="1" t="inlineStr">
-        <is>
           <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="113.45" customHeight="1">
-      <c r="A52" s="1" t="inlineStr">
-        <is>
-          <t>AV155</t>
-        </is>
-      </c>
-      <c r="B52" s="1" t="inlineStr">
-        <is>
-          <t>questionario</t>
-        </is>
-      </c>
-      <c r="C52" s="1" t="n"/>
-      <c r="D52" s="1" t="n"/>
-      <c r="E52" s="1" t="n"/>
-      <c r="F52" s="1" t="inlineStr">
-        <is>
-          <t>existe_plano_ti</t>
-        </is>
-      </c>
-      <c r="G52" s="1" t="inlineStr">
-        <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
-        </is>
-      </c>
-      <c r="H52" s="1" t="inlineStr">
-        <is>
-          <t>Plano de TIC vigente declarado no item 2102, ao menos parcialmente adotado</t>
-        </is>
-      </c>
-      <c r="I52" s="1" t="n"/>
-      <c r="J52" s="1" t="n"/>
-      <c r="K52" s="1" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="L52" s="1" t="n"/>
-      <c r="M52" s="1" t="n"/>
-      <c r="N52" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O52" s="1" t="n"/>
-      <c r="P52" s="1" t="inlineStr">
-        <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
-        </is>
-      </c>
-    </row>
+    <row r="48" ht="113.45" customHeight="1"/>
+    <row r="49" ht="113.45" customHeight="1"/>
+    <row r="50" ht="113.45" customHeight="1"/>
+    <row r="51" ht="113.45" customHeight="1"/>
+    <row r="52" ht="113.45" customHeight="1"/>
     <row r="53" ht="113.45" customHeight="1"/>
     <row r="54" ht="113.45" customHeight="1"/>
     <row r="55" ht="113.45" customHeight="1"/>
@@ -3695,7 +3428,7 @@
     <row r="153" ht="23.85" customHeight="1"/>
     <row r="154" ht="23.85" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A3:P52"/>
+  <autoFilter ref="A3:P47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -3707,7 +3440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H50"/>
+  <dimension ref="A2:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5193,7 +4926,7 @@
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>AV73 &amp; ~AV143</t>
+          <t>AV73</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
@@ -5213,7 +4946,7 @@
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>MR092</t>
+          <t>MR101</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
@@ -5223,25 +4956,25 @@
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
         </is>
       </c>
       <c r="D41" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>AV143</t>
+          <t>AV78</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>AV143</t>
+          <t>AV78</t>
         </is>
       </c>
       <c r="G41" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
+          <t>No subitem a) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
         </is>
       </c>
       <c r="H41" s="9" t="b">
@@ -5251,7 +4984,7 @@
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>MR101</t>
+          <t>MR109</t>
         </is>
       </c>
       <c r="B42" s="9" t="inlineStr">
@@ -5261,7 +4994,7 @@
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
         </is>
       </c>
       <c r="D42" s="9" t="n">
@@ -5269,17 +5002,17 @@
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>AV78 &amp; ~AV148</t>
+          <t>AV82</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>AV78</t>
+          <t>AV82</t>
         </is>
       </c>
       <c r="G42" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
+          <t>No subitem b) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de TI executadas no exercício encontram-se previamente estabelecidas nos instrumentos de planejamento vigentes (PDTI/PEDTIC e PCA)</t>
         </is>
       </c>
       <c r="H42" s="9" t="b">
@@ -5289,7 +5022,7 @@
     <row r="43" ht="45" customHeight="1">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>MR102</t>
+          <t>MR110</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
@@ -5299,25 +5032,25 @@
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
+          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
         </is>
       </c>
       <c r="D43" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>AV148</t>
+          <t>AV83</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>AV148</t>
+          <t>AV83</t>
         </is>
       </c>
       <c r="G43" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2804, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
+          <t>No subitem c) do item 2804, não houve declaração afirmativa quanto à prática avaliada: a fase de planejamento de cada contratação de TI é conduzida por uma Equipe de Planejamento da Contratação formalmente designada (composta, minimamente, por integrante requisitante e integrante técnico da área de TI)</t>
         </is>
       </c>
       <c r="H43" s="9" t="b">
@@ -5327,7 +5060,7 @@
     <row r="44" ht="45" customHeight="1">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>MR105</t>
+          <t>MR111</t>
         </is>
       </c>
       <c r="B44" s="9" t="inlineStr">
@@ -5337,25 +5070,25 @@
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D44" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>AV80 &amp; ~AV150</t>
+          <t>AV152</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>AV80</t>
+          <t>AV152</t>
         </is>
       </c>
       <c r="G44" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2802, não houve declaração afirmativa quanto à prática avaliada: na elaboração do PCA são considerados os demais instrumentos de planejamento da organização</t>
+          <t>No subitem b) do item 2801, não houve declaração afirmativa quanto à prática avaliada: são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
         </is>
       </c>
       <c r="H44" s="9" t="b">
@@ -5365,17 +5098,17 @@
     <row r="45" ht="45" customHeight="1">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>MR106</t>
+          <t>MR113</t>
         </is>
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>PA06</t>
+          <t>PA03</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="D45" s="9" t="n">
@@ -5383,213 +5116,28 @@
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>AV150</t>
+          <t>AV154</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>AV150</t>
+          <t>AV154</t>
         </is>
       </c>
       <c r="G45" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2802, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que na elaboração do PCA são considerados os demais instrumentos de planejamento da organização</t>
+          <t>No item 2102, a organização não declarou possuir plano de tecnologia da informação vigente, ainda que parcialmente adotado</t>
         </is>
       </c>
       <c r="H45" s="9" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="46" ht="30" customHeight="1">
-      <c r="A46" s="9" t="inlineStr">
-        <is>
-          <t>MR109</t>
-        </is>
-      </c>
-      <c r="B46" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C46" s="9" t="inlineStr">
-        <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
-        </is>
-      </c>
-      <c r="D46" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="E46" s="9" t="inlineStr">
-        <is>
-          <t>AV82</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="inlineStr">
-        <is>
-          <t>AV82</t>
-        </is>
-      </c>
-      <c r="G46" s="9" t="inlineStr">
-        <is>
-          <t>No subitem b) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de TI executadas no exercício encontram-se previamente estabelecidas nos instrumentos de planejamento vigentes (PDTI/PEDTIC e PCA)</t>
-        </is>
-      </c>
-      <c r="H46" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="9" t="inlineStr">
-        <is>
-          <t>MR110</t>
-        </is>
-      </c>
-      <c r="B47" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C47" s="9" t="inlineStr">
-        <is>
-          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
-        </is>
-      </c>
-      <c r="D47" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E47" s="9" t="inlineStr">
-        <is>
-          <t>AV83</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="inlineStr">
-        <is>
-          <t>AV83</t>
-        </is>
-      </c>
-      <c r="G47" s="9" t="inlineStr">
-        <is>
-          <t>No subitem c) do item 2804, não houve declaração afirmativa quanto à prática avaliada: a fase de planejamento de cada contratação de TI é conduzida por uma Equipe de Planejamento da Contratação formalmente designada (composta, minimamente, por integrante requisitante e integrante técnico da área de TI)</t>
-        </is>
-      </c>
-      <c r="H47" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="9" t="inlineStr">
-        <is>
-          <t>MR111</t>
-        </is>
-      </c>
-      <c r="B48" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C48" s="9" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="D48" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E48" s="9" t="inlineStr">
-        <is>
-          <t>AV152 &amp; ~AV153</t>
-        </is>
-      </c>
-      <c r="F48" s="9" t="inlineStr">
-        <is>
-          <t>AV152</t>
-        </is>
-      </c>
-      <c r="G48" s="9" t="inlineStr">
-        <is>
-          <t>No subitem b) do item 2801, não houve declaração afirmativa quanto à prática avaliada: são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
-        </is>
-      </c>
-      <c r="H48" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49" ht="45" customHeight="1">
-      <c r="A49" s="9" t="inlineStr">
-        <is>
-          <t>MR112</t>
-        </is>
-      </c>
-      <c r="B49" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C49" s="9" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="D49" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="E49" s="9" t="inlineStr">
-        <is>
-          <t>AV153</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="inlineStr">
-        <is>
-          <t>AV153</t>
-        </is>
-      </c>
-      <c r="G49" s="9" t="inlineStr">
-        <is>
-          <t>No subitem b) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
-        </is>
-      </c>
-      <c r="H49" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" ht="30" customHeight="1">
-      <c r="A50" s="9" t="inlineStr">
-        <is>
-          <t>MR113</t>
-        </is>
-      </c>
-      <c r="B50" s="9" t="inlineStr">
-        <is>
-          <t>PA03</t>
-        </is>
-      </c>
-      <c r="C50" s="9" t="inlineStr">
-        <is>
-          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
-        </is>
-      </c>
-      <c r="D50" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E50" s="9" t="inlineStr">
-        <is>
-          <t>AV154</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="inlineStr">
-        <is>
-          <t>AV154</t>
-        </is>
-      </c>
-      <c r="G50" s="9" t="inlineStr">
-        <is>
-          <t>No item 2102, a organização não declarou possuir plano de tecnologia da informação vigente, ainda que parcialmente adotado</t>
-        </is>
-      </c>
-      <c r="H50" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
+    <row r="46" ht="30" customHeight="1"/>
+    <row r="47" ht="30" customHeight="1"/>
+    <row r="48" ht="30" customHeight="1"/>
+    <row r="49" ht="45" customHeight="1"/>
+    <row r="50" ht="30" customHeight="1"/>
     <row r="51" ht="30" customHeight="1"/>
     <row r="52" ht="30" customHeight="1"/>
     <row r="53" ht="30" customHeight="1"/>
@@ -5654,7 +5202,7 @@
     <row r="112" ht="45" customHeight="1"/>
     <row r="113" ht="45" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A3:H50"/>
+  <autoFilter ref="A3:H45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Restaura avaliações documentais e documenta variáveis derivadas
</commit_message>
<xml_diff>
--- a/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
+++ b/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
@@ -15,8 +15,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Fontes de Informação'!$A$3:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Procedimentos de Auditoria'!$A$3:$E$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ações de Verificação'!$A$3:$P$47</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Motivos do Relatório'!$A$3:$H$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ações de Verificação'!$A$3:$P$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Motivos do Relatório'!$A$3:$H$74</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Variáveis Temporárias'!$A$3:$E$6</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -574,7 +574,7 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>(AV08 | AV11 | (AV12 &amp; AV13))</t>
+          <t>((AV08 | AV86) | (AV11 | AV89) | ((AV12 &amp; ~AV90) &amp; (AV13 | AV91)))</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
@@ -599,7 +599,7 @@
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>((AV14 | AV15 | AV17 | AV154) | (AV155 &amp; (AV18 | AV19 | AV20 | AV24)))</t>
+          <t>(((AV14 | AV92) | (AV15 | AV93) | (AV17 | AV95) | AV154) | (AV155 &amp; ((AV18 | AV96) | (AV19 | AV97) | (AV20 | AV98) | (AV24 | AV101))))</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
@@ -624,7 +624,7 @@
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>((AV26 &amp; AV25) | AV29 | (AV31 | AV33) | (AV45 &amp; AV46))</t>
+          <t>((AV26 &amp; AV25) | (AV29 | AV103) | ((AV31 | AV105) | (AV33 | AV107)) | (AV45 &amp; AV46))</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
@@ -649,7 +649,7 @@
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>((AV55 | AV56) | (AV54 | AV57 | AV58) | (AV62 | AV63) | (AV59 | AV66) | (AV67 | AV70 | AV71))</t>
+          <t>(((AV55 | AV125) | (AV56 | AV126)) | ((AV54 | AV124) | (AV57 | AV127) | (AV58 | AV128)) | (AV129 | (AV62 | AV132) | (AV63 | AV133)) | ((AV59 | AV134) | (AV66 | AV136)) | ((AV67 | AV137) | (AV70 | AV140) | (AV71 | AV141)))</t>
         </is>
       </c>
       <c r="D8" s="1" t="n">
@@ -674,7 +674,7 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>((AV73 | AV152) | AV78 | AV82 | AV83)</t>
+          <t>(((AV73 | AV143) | (AV152 | AV153)) | (AV78 | AV148) | AV82 | AV83)</t>
         </is>
       </c>
       <c r="D9" s="1" t="n">
@@ -699,7 +699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P47"/>
+  <dimension ref="A1:P77"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2576,7 +2576,7 @@
       <c r="I34" s="1" t="n"/>
       <c r="J34" s="1" t="inlineStr">
         <is>
-          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
+          <t>Inventário e controle de ativos e configurações de TIC inexistente ou insuficiente.</t>
         </is>
       </c>
       <c r="K34" s="1" t="inlineStr">
@@ -2594,7 +2594,7 @@
       <c r="O34" s="1" t="n"/>
       <c r="P34" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos sob gestão da organização, contemplando, minimamente, os dispositivos e softwares utilizados, com informações suficientes para sua identificação e controle</t>
+          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos e base consolidada das configurações relevantes, contemplando, minimamente, dispositivos, softwares e seus relacionamentos, com informações suficientes para identificação e controle</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2631,7 @@
       <c r="I35" s="1" t="n"/>
       <c r="J35" s="1" t="inlineStr">
         <is>
-          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
+          <t>Inventário e controle de ativos e configurações de TIC inexistente ou insuficiente.</t>
         </is>
       </c>
       <c r="K35" s="1" t="inlineStr">
@@ -2649,7 +2649,7 @@
       <c r="O35" s="1" t="n"/>
       <c r="P35" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos sob gestão da organização, contemplando, minimamente, os dispositivos e softwares utilizados, com informações suficientes para sua identificação e controle</t>
+          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos e base consolidada das configurações relevantes, contemplando, minimamente, dispositivos, softwares e seus relacionamentos, com informações suficientes para identificação e controle</t>
         </is>
       </c>
     </row>
@@ -3159,12 +3159,12 @@
     <row r="45" ht="113.45" customHeight="1">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>AV152</t>
+          <t>AV86</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
-          <t>questionario</t>
+          <t>avaliacao_evidencias_ajustes</t>
         </is>
       </c>
       <c r="C45" s="1" t="n"/>
@@ -3172,30 +3172,28 @@
       <c r="E45" s="1" t="n"/>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>q2801ext[B]</t>
+          <t>q1001ext[H]</t>
         </is>
       </c>
       <c r="G45" s="1" t="inlineStr">
         <is>
-          <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Lei nº 14.133/2021, art. 19, inciso IV: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.
-Acórdão nº 2.342/2016-TCU-Plenário, item 9.1.7 – Precedente quanto à definição, aprovação e formalização de processo de trabalho para o planejamento de cada contratação, com controles internos mínimos.</t>
+          <t>COBIT 2019, MEA01.04 - Avaliar o desempenho: monitorar e avaliar periodicamente o desempenho e a conformidade da TI em relação a objetivos, indicadores, metas e expectativas das partes interessadas.</t>
         </is>
       </c>
       <c r="H45" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento b) do item 2801 do Questionário, para verificar se são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
         </is>
       </c>
       <c r="I45" s="1" t="n"/>
       <c r="J45" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+          <t>Ausência de objetivos, indicadores ou metas para a gestão de TIC.</t>
         </is>
       </c>
       <c r="K45" s="1" t="inlineStr">
         <is>
-          <t>(Não | N/A)</t>
+          <t>Não conforme</t>
         </is>
       </c>
       <c r="L45" s="1" t="n"/>
@@ -3208,19 +3206,19 @@
       <c r="O45" s="1" t="n"/>
       <c r="P45" s="1" t="inlineStr">
         <is>
-          <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
+          <t>estabeleça objetivos, indicadores e metas para a gestão de TIC, de modo a possibilitar o acompanhamento periódico do desempenho da TIC pela alta administração</t>
         </is>
       </c>
     </row>
     <row r="46" ht="113.45" customHeight="1">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>AV154</t>
+          <t>AV89</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
-          <t>questionario</t>
+          <t>avaliacao_evidencias_ajustes</t>
         </is>
       </c>
       <c r="C46" s="1" t="n"/>
@@ -3228,30 +3226,30 @@
       <c r="E46" s="1" t="n"/>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>existe_plano_ti</t>
+          <t>q1001ext[E]</t>
         </is>
       </c>
       <c r="G46" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
+          <t>COBIT 2019, EDM01.02 - Dirigir o sistema de governança: orientar estruturas, princípios, processos e práticas de governança para assegurar que a TI apoie os objetivos organizacionais.
+Decreto nº 12.198/2024, arts. 5º e 6º, § 2º – Referência de governança digital: instituição, no âmbito da Administração Pública federal direta, autárquica e fundacional, de Comitê de Governança Digital ou colegiado equivalente com função deliberativa sobre ações de governo digital e uso de recursos de TIC, incluindo a aprovação dos instrumentos de planejamento previstos no Decreto.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.1, III.1 e V.1 – Precedente pela instituição e atuação efetiva de instância colegiada de governança de TIC, com responsabilidade pelo alinhamento das ações de TIC aos objetivos institucionais, priorização dos investimentos e monitoramento do desempenho da TIC.</t>
         </is>
       </c>
       <c r="H46" s="1" t="inlineStr">
         <is>
-          <t>Resposta ao item 2102 que não caracteriza a existência de plano de TIC vigente, ainda que parcialmente adotado</t>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
         </is>
       </c>
       <c r="I46" s="1" t="n"/>
       <c r="J46" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
+          <t>Comitê de TIC ou instância equivalente não instituído formalmente ou sem representação de áreas relevantes da organização.</t>
         </is>
       </c>
       <c r="K46" s="1" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>Não conforme</t>
         </is>
       </c>
       <c r="L46" s="1" t="n"/>
@@ -3264,19 +3262,19 @@
       <c r="O46" s="1" t="n"/>
       <c r="P46" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>institua formalmente Comitê de TIC ou instância colegiada equivalente, compatível com o porte e a estrutura decisória da organização, definindo em seu ato constitutivo, minimamente, a participação de representantes de áreas relevantes da organização, suas competências, a periodicidade de reuniões, a forma de registro das deliberações e os mecanismos de acompanhamento dos encaminhamentos</t>
         </is>
       </c>
     </row>
     <row r="47" ht="113.45" customHeight="1">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>AV155</t>
+          <t>AV90</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
-          <t>questionario</t>
+          <t>avaliacao_evidencias_ajustes</t>
         </is>
       </c>
       <c r="C47" s="1" t="n"/>
@@ -3284,72 +3282,1709 @@
       <c r="E47" s="1" t="n"/>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>existe_plano_ti</t>
+          <t>q1001ext[E]</t>
         </is>
       </c>
       <c r="G47" s="1" t="inlineStr">
+        <is>
+          <t>COBIT 2019, EDM01.02 - Dirigir o sistema de governança: orientar estruturas, princípios, processos e práticas de governança para assegurar que a TI apoie os objetivos organizacionais.
+Decreto nº 12.198/2024, arts. 5º e 6º, § 2º – Referência de governança digital: instituição, no âmbito da Administração Pública federal direta, autárquica e fundacional, de Comitê de Governança Digital ou colegiado equivalente com função deliberativa sobre ações de governo digital e uso de recursos de TIC, incluindo a aprovação dos instrumentos de planejamento previstos no Decreto.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.1, III.1 e V.1 – Precedente pela instituição e atuação efetiva de instância colegiada de governança de TIC, com responsabilidade pelo alinhamento das ações de TIC aos objetivos institucionais, priorização dos investimentos e monitoramento do desempenho da TIC.</t>
+        </is>
+      </c>
+      <c r="H47" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I47" s="1" t="n"/>
+      <c r="J47" s="1" t="inlineStr">
+        <is>
+          <t>Comitê de TIC ou instância equivalente sem atuação efetiva comprovada.</t>
+        </is>
+      </c>
+      <c r="K47" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L47" s="1" t="n"/>
+      <c r="M47" s="1" t="n"/>
+      <c r="N47" s="1" t="inlineStr">
+        <is>
+          <t>Determinação</t>
+        </is>
+      </c>
+      <c r="O47" s="1" t="n"/>
+      <c r="P47" s="1" t="inlineStr">
+        <is>
+          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância colegiada equivalente, mediante o exercício das competências previstas em seu ato constitutivo, com registro das deliberações e acompanhamento dos respectivos encaminhamentos</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="113.45" customHeight="1">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>AV91</t>
+        </is>
+      </c>
+      <c r="B48" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C48" s="1" t="n"/>
+      <c r="D48" s="1" t="n"/>
+      <c r="E48" s="1" t="n"/>
+      <c r="F48" s="1" t="inlineStr">
+        <is>
+          <t>q1001ext[F]</t>
+        </is>
+      </c>
+      <c r="G48" s="1" t="inlineStr">
+        <is>
+          <t>COBIT 2019, EDM01.02 - Dirigir o sistema de governança: orientar estruturas, princípios, processos e práticas de governança para assegurar que a TI apoie os objetivos organizacionais.
+Decreto nº 12.198/2024, arts. 5º e 6º, § 2º – Referência de governança digital: instituição, no âmbito da Administração Pública federal direta, autárquica e fundacional, de Comitê de Governança Digital ou colegiado equivalente com função deliberativa sobre ações de governo digital e uso de recursos de TIC, incluindo a aprovação dos instrumentos de planejamento previstos no Decreto.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.1, III.1 e V.1 – Precedente pela instituição e atuação efetiva de instância colegiada de governança de TIC, com responsabilidade pelo alinhamento das ações de TIC aos objetivos institucionais, priorização dos investimentos e monitoramento do desempenho da TIC.</t>
+        </is>
+      </c>
+      <c r="H48" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I48" s="1" t="n"/>
+      <c r="J48" s="1" t="inlineStr">
+        <is>
+          <t>Comitê de TIC ou instância equivalente sem atuação efetiva comprovada.</t>
+        </is>
+      </c>
+      <c r="K48" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L48" s="1" t="n"/>
+      <c r="M48" s="1" t="n"/>
+      <c r="N48" s="1" t="inlineStr">
+        <is>
+          <t>Determinação</t>
+        </is>
+      </c>
+      <c r="O48" s="1" t="n"/>
+      <c r="P48" s="1" t="inlineStr">
+        <is>
+          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância colegiada equivalente, mediante o exercício das competências previstas em seu ato constitutivo, com registro das deliberações e acompanhamento dos respectivos encaminhamentos</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="113.45" customHeight="1">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>AV92</t>
+        </is>
+      </c>
+      <c r="B49" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C49" s="1" t="n"/>
+      <c r="D49" s="1" t="n"/>
+      <c r="E49" s="1" t="n"/>
+      <c r="F49" s="1" t="inlineStr">
+        <is>
+          <t>q2101ext[A]</t>
+        </is>
+      </c>
+      <c r="G49" s="1" t="inlineStr">
         <is>
           <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
 Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
 Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
-      <c r="H47" s="1" t="inlineStr">
+      <c r="H49" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I49" s="1" t="n"/>
+      <c r="J49" s="1" t="inlineStr">
+        <is>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
+        </is>
+      </c>
+      <c r="K49" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L49" s="1" t="n"/>
+      <c r="M49" s="1" t="n"/>
+      <c r="N49" s="1" t="inlineStr">
+        <is>
+          <t>Determinação</t>
+        </is>
+      </c>
+      <c r="O49" s="1" t="n"/>
+      <c r="P49" s="1" t="inlineStr">
+        <is>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="113.45" customHeight="1">
+      <c r="A50" s="1" t="inlineStr">
+        <is>
+          <t>AV93</t>
+        </is>
+      </c>
+      <c r="B50" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C50" s="1" t="n"/>
+      <c r="D50" s="1" t="n"/>
+      <c r="E50" s="1" t="n"/>
+      <c r="F50" s="1" t="inlineStr">
+        <is>
+          <t>q2101ext[B]</t>
+        </is>
+      </c>
+      <c r="G50" s="1" t="inlineStr">
+        <is>
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
+        </is>
+      </c>
+      <c r="H50" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I50" s="1" t="n"/>
+      <c r="J50" s="1" t="inlineStr">
+        <is>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
+        </is>
+      </c>
+      <c r="K50" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L50" s="1" t="n"/>
+      <c r="M50" s="1" t="n"/>
+      <c r="N50" s="1" t="inlineStr">
+        <is>
+          <t>Determinação</t>
+        </is>
+      </c>
+      <c r="O50" s="1" t="n"/>
+      <c r="P50" s="1" t="inlineStr">
+        <is>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="113.45" customHeight="1">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>AV95</t>
+        </is>
+      </c>
+      <c r="B51" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C51" s="1" t="n"/>
+      <c r="D51" s="1" t="n"/>
+      <c r="E51" s="1" t="n"/>
+      <c r="F51" s="1" t="inlineStr">
+        <is>
+          <t>q2101ext[D]</t>
+        </is>
+      </c>
+      <c r="G51" s="1" t="inlineStr">
+        <is>
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
+        </is>
+      </c>
+      <c r="H51" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I51" s="1" t="n"/>
+      <c r="J51" s="1" t="inlineStr">
+        <is>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
+        </is>
+      </c>
+      <c r="K51" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L51" s="1" t="n"/>
+      <c r="M51" s="1" t="n"/>
+      <c r="N51" s="1" t="inlineStr">
+        <is>
+          <t>Determinação</t>
+        </is>
+      </c>
+      <c r="O51" s="1" t="n"/>
+      <c r="P51" s="1" t="inlineStr">
+        <is>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="113.45" customHeight="1">
+      <c r="A52" s="1" t="inlineStr">
+        <is>
+          <t>AV96</t>
+        </is>
+      </c>
+      <c r="B52" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C52" s="1" t="n"/>
+      <c r="D52" s="1" t="n"/>
+      <c r="E52" s="1" t="n"/>
+      <c r="F52" s="1" t="inlineStr">
+        <is>
+          <t>q2102ext[A]</t>
+        </is>
+      </c>
+      <c r="G52" s="1" t="inlineStr">
+        <is>
+          <t>Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
+        </is>
+      </c>
+      <c r="H52" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I52" s="1" t="n"/>
+      <c r="J52" s="1" t="inlineStr">
+        <is>
+          <t>Ausência de aprovação formal do plano de TIC.</t>
+        </is>
+      </c>
+      <c r="K52" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L52" s="1" t="n"/>
+      <c r="M52" s="1" t="n"/>
+      <c r="N52" s="1" t="inlineStr">
+        <is>
+          <t>Determinação</t>
+        </is>
+      </c>
+      <c r="O52" s="1" t="n"/>
+      <c r="P52" s="1" t="inlineStr">
+        <is>
+          <t>submeta o plano de TIC à aprovação formal do dirigente máximo ou de instância competente da alta administração, mantendo registro do respectivo ato de aprovação</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="113.45" customHeight="1">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>AV97</t>
+        </is>
+      </c>
+      <c r="B53" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C53" s="1" t="n"/>
+      <c r="D53" s="1" t="n"/>
+      <c r="E53" s="1" t="n"/>
+      <c r="F53" s="1" t="inlineStr">
+        <is>
+          <t>q2102ext[D]</t>
+        </is>
+      </c>
+      <c r="G53" s="1" t="inlineStr">
+        <is>
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
+        </is>
+      </c>
+      <c r="H53" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I53" s="1" t="n"/>
+      <c r="J53" s="1" t="inlineStr">
+        <is>
+          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
+        </is>
+      </c>
+      <c r="K53" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L53" s="1" t="n"/>
+      <c r="M53" s="1" t="n"/>
+      <c r="N53" s="1" t="inlineStr">
+        <is>
+          <t>Determinação</t>
+        </is>
+      </c>
+      <c r="O53" s="1" t="n"/>
+      <c r="P53" s="1" t="inlineStr">
+        <is>
+          <t>revise o plano de TIC para explicitar seu alinhamento ao planejamento institucional, às diretrizes superiores e às necessidades das áreas finalísticas e administrativas, relacionando objetivos, iniciativas, indicadores e metas de TIC aos resultados institucionais pretendidos</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="113.45" customHeight="1">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>AV98</t>
+        </is>
+      </c>
+      <c r="B54" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C54" s="1" t="n"/>
+      <c r="D54" s="1" t="n"/>
+      <c r="E54" s="1" t="n"/>
+      <c r="F54" s="1" t="inlineStr">
+        <is>
+          <t>q2102ext[C]</t>
+        </is>
+      </c>
+      <c r="G54" s="1" t="inlineStr">
+        <is>
+          <t>COBIT 2019, APO06.03 - Criar e manter orçamentos: elaborar e manter orçamento de TIC alinhado ao portfólio, ao planejamento e às prioridades aprovadas.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
+        </is>
+      </c>
+      <c r="H54" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I54" s="1" t="n"/>
+      <c r="J54" s="1" t="inlineStr">
+        <is>
+          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
+        </is>
+      </c>
+      <c r="K54" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L54" s="1" t="n"/>
+      <c r="M54" s="1" t="n"/>
+      <c r="N54" s="1" t="inlineStr">
+        <is>
+          <t>Determinação</t>
+        </is>
+      </c>
+      <c r="O54" s="1" t="n"/>
+      <c r="P54" s="1" t="inlineStr">
+        <is>
+          <t>integre o plano de TIC à elaboração da proposta orçamentária e do plano de contratações, de maneira proporcional ao porte, à estrutura e à capacidade de planejamento da organização</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="113.45" customHeight="1">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>AV101</t>
+        </is>
+      </c>
+      <c r="B55" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C55" s="1" t="n"/>
+      <c r="D55" s="1" t="n"/>
+      <c r="E55" s="1" t="n"/>
+      <c r="F55" s="1" t="inlineStr">
+        <is>
+          <t>q2102ext[E]</t>
+        </is>
+      </c>
+      <c r="G55" s="1" t="inlineStr">
+        <is>
+          <t>Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
+        </is>
+      </c>
+      <c r="H55" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I55" s="1" t="n"/>
+      <c r="J55" s="1" t="inlineStr">
+        <is>
+          <t>Ausência de acompanhamento da execução do plano de TIC.</t>
+        </is>
+      </c>
+      <c r="K55" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L55" s="1" t="n"/>
+      <c r="M55" s="1" t="n"/>
+      <c r="N55" s="1" t="inlineStr">
+        <is>
+          <t>Determinação</t>
+        </is>
+      </c>
+      <c r="O55" s="1" t="n"/>
+      <c r="P55" s="1" t="inlineStr">
+        <is>
+          <t>estabeleça e execute rotina periódica de acompanhamento da execução do plano de TIC, promovendo sua revisão periódica e os ajustes ou atualizações necessários, com registro das principais decisões e reprogramações</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="113.45" customHeight="1">
+      <c r="A56" s="1" t="inlineStr">
+        <is>
+          <t>AV103</t>
+        </is>
+      </c>
+      <c r="B56" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C56" s="1" t="n"/>
+      <c r="D56" s="1" t="n"/>
+      <c r="E56" s="1" t="n"/>
+      <c r="F56" s="1" t="inlineStr">
+        <is>
+          <t>q2703ext[C]</t>
+        </is>
+      </c>
+      <c r="G56" s="1" t="inlineStr">
+        <is>
+          <t>COBIT 2019, APO07.05 - Planejar e monitorar o uso de recursos humanos de TI e de negócio: planejar, alocar e acompanhar capacidade de pessoal para iniciativas, operações e serviços de TIC.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6.5 - O PDTI deve contemplar o quantitativo necessário ou ideal para a força de trabalho em TI.</t>
+        </is>
+      </c>
+      <c r="H56" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I56" s="1" t="n"/>
+      <c r="J56" s="1" t="inlineStr">
+        <is>
+          <t>Ausência ou insuficiência de definição documentada do quantitativo necessário de pessoal de TIC e segurança da informação.</t>
+        </is>
+      </c>
+      <c r="K56" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L56" s="1" t="n"/>
+      <c r="M56" s="1" t="n"/>
+      <c r="N56" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="O56" s="1" t="n"/>
+      <c r="P56" s="1" t="inlineStr">
+        <is>
+          <t>estime e mantenha atualizado o quantitativo necessário de pessoal de TIC e segurança da informação, considerando o porte e a complexidade da organização, os serviços críticos, os sistemas mantidos, as contratações vigentes e os riscos relevantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="90.95" customHeight="1">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>AV105</t>
+        </is>
+      </c>
+      <c r="B57" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C57" s="1" t="n"/>
+      <c r="D57" s="1" t="n"/>
+      <c r="E57" s="1" t="n"/>
+      <c r="F57" s="1" t="inlineStr">
+        <is>
+          <t>q2708[B]</t>
+        </is>
+      </c>
+      <c r="G57" s="1" t="inlineStr">
+        <is>
+          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
+COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
+        </is>
+      </c>
+      <c r="H57" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I57" s="1" t="n"/>
+      <c r="J57" s="1" t="inlineStr">
+        <is>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+        </is>
+      </c>
+      <c r="K57" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L57" s="1" t="n"/>
+      <c r="M57" s="1" t="n"/>
+      <c r="N57" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="O57" s="1" t="n"/>
+      <c r="P57" s="1" t="inlineStr">
+        <is>
+          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="90.95" customHeight="1">
+      <c r="A58" s="1" t="inlineStr">
+        <is>
+          <t>AV107</t>
+        </is>
+      </c>
+      <c r="B58" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C58" s="1" t="n"/>
+      <c r="D58" s="1" t="n"/>
+      <c r="E58" s="1" t="n"/>
+      <c r="F58" s="1" t="inlineStr">
+        <is>
+          <t>q2708[D]</t>
+        </is>
+      </c>
+      <c r="G58" s="1" t="inlineStr">
+        <is>
+          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
+COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
+        </is>
+      </c>
+      <c r="H58" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I58" s="1" t="n"/>
+      <c r="J58" s="1" t="inlineStr">
+        <is>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+        </is>
+      </c>
+      <c r="K58" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L58" s="1" t="n"/>
+      <c r="M58" s="1" t="n"/>
+      <c r="N58" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="O58" s="1" t="n"/>
+      <c r="P58" s="1" t="inlineStr">
+        <is>
+          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="90.95" customHeight="1">
+      <c r="A59" s="1" t="inlineStr">
+        <is>
+          <t>AV124</t>
+        </is>
+      </c>
+      <c r="B59" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C59" s="1" t="n"/>
+      <c r="D59" s="1" t="n"/>
+      <c r="E59" s="1" t="n"/>
+      <c r="F59" s="1" t="inlineStr">
+        <is>
+          <t>q2201ext[A]</t>
+        </is>
+      </c>
+      <c r="G59" s="1" t="inlineStr">
+        <is>
+          <t>ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.7, III.9.7 e V.6.4 – Recomendações quanto à definição, pactuação e monitoramento de níveis de serviço.</t>
+        </is>
+      </c>
+      <c r="H59" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I59" s="1" t="n"/>
+      <c r="J59" s="1" t="inlineStr">
+        <is>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+        </is>
+      </c>
+      <c r="K59" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L59" s="1" t="n"/>
+      <c r="M59" s="1" t="n"/>
+      <c r="N59" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="O59" s="1" t="n"/>
+      <c r="P59" s="1" t="inlineStr">
+        <is>
+          <t>defina, acorde e monitore níveis de serviço para os serviços de TIC relevantes, estabelecendo metas e mecanismos de acompanhamento de seu cumprimento</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="79.90000000000001" customHeight="1">
+      <c r="A60" s="1" t="inlineStr">
+        <is>
+          <t>AV125</t>
+        </is>
+      </c>
+      <c r="B60" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C60" s="1" t="n"/>
+      <c r="D60" s="1" t="n"/>
+      <c r="E60" s="1" t="n"/>
+      <c r="F60" s="1" t="inlineStr">
+        <is>
+          <t>q2201ext[B]</t>
+        </is>
+      </c>
+      <c r="G60" s="1" t="inlineStr">
+        <is>
+          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.4, III.9.4 e V.6.1 – Recomendações quanto à estruturação do catálogo de serviços de TIC, incluindo descrição dos serviços, metas, formas de acesso e disponibilidade aos usuários.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.2.4 – Gerenciamento de catálogo de serviço: orienta que o catálogo descreva os serviços e seus resultados pretendidos, contenha informações relevantes para sua utilização e seja disponibilizado às partes interessadas que necessitem acessá-lo.</t>
+        </is>
+      </c>
+      <c r="H60" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I60" s="1" t="n"/>
+      <c r="J60" s="1" t="inlineStr">
+        <is>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+        </is>
+      </c>
+      <c r="K60" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L60" s="1" t="n"/>
+      <c r="M60" s="1" t="n"/>
+      <c r="N60" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="O60" s="1" t="n"/>
+      <c r="P60" s="1" t="inlineStr">
+        <is>
+          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="79.90000000000001" customHeight="1">
+      <c r="A61" s="1" t="inlineStr">
+        <is>
+          <t>AV126</t>
+        </is>
+      </c>
+      <c r="B61" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C61" s="1" t="n"/>
+      <c r="D61" s="1" t="n"/>
+      <c r="E61" s="1" t="n"/>
+      <c r="F61" s="1" t="inlineStr">
+        <is>
+          <t>q2201ext[C]</t>
+        </is>
+      </c>
+      <c r="G61" s="1" t="inlineStr">
+        <is>
+          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.4, III.9.4 e V.6.1 – Recomendações quanto à estruturação do catálogo de serviços de TIC, incluindo descrição dos serviços, metas, formas de acesso e disponibilidade aos usuários.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.2.4 – Gerenciamento de catálogo de serviço: orienta que o catálogo descreva os serviços e seus resultados pretendidos, contenha informações relevantes para sua utilização e seja disponibilizado às partes interessadas que necessitem acessá-lo.</t>
+        </is>
+      </c>
+      <c r="H61" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I61" s="1" t="n"/>
+      <c r="J61" s="1" t="inlineStr">
+        <is>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+        </is>
+      </c>
+      <c r="K61" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L61" s="1" t="n"/>
+      <c r="M61" s="1" t="n"/>
+      <c r="N61" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="O61" s="1" t="n"/>
+      <c r="P61" s="1" t="inlineStr">
+        <is>
+          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="90.95" customHeight="1">
+      <c r="A62" s="1" t="inlineStr">
+        <is>
+          <t>AV127</t>
+        </is>
+      </c>
+      <c r="B62" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C62" s="1" t="n"/>
+      <c r="D62" s="1" t="n"/>
+      <c r="E62" s="1" t="n"/>
+      <c r="F62" s="1" t="inlineStr">
+        <is>
+          <t>q2201ext[D]</t>
+        </is>
+      </c>
+      <c r="G62" s="1" t="inlineStr">
+        <is>
+          <t>ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.7, III.9.7 e V.6.4 – Recomendações quanto à definição, pactuação e monitoramento de níveis de serviço.</t>
+        </is>
+      </c>
+      <c r="H62" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I62" s="1" t="n"/>
+      <c r="J62" s="1" t="inlineStr">
+        <is>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+        </is>
+      </c>
+      <c r="K62" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L62" s="1" t="n"/>
+      <c r="M62" s="1" t="n"/>
+      <c r="N62" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="O62" s="1" t="n"/>
+      <c r="P62" s="1" t="inlineStr">
+        <is>
+          <t>defina, acorde e monitore níveis de serviço para os serviços de TIC relevantes, estabelecendo metas e mecanismos de acompanhamento de seu cumprimento</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="90.95" customHeight="1">
+      <c r="A63" s="1" t="inlineStr">
+        <is>
+          <t>AV128</t>
+        </is>
+      </c>
+      <c r="B63" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C63" s="1" t="n"/>
+      <c r="D63" s="1" t="n"/>
+      <c r="E63" s="1" t="n"/>
+      <c r="F63" s="1" t="inlineStr">
+        <is>
+          <t>q2201ext[E]</t>
+        </is>
+      </c>
+      <c r="G63" s="1" t="inlineStr">
+        <is>
+          <t>ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.7, III.9.7 e V.6.4 – Recomendações quanto à definição, pactuação e monitoramento de níveis de serviço.</t>
+        </is>
+      </c>
+      <c r="H63" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I63" s="1" t="n"/>
+      <c r="J63" s="1" t="inlineStr">
+        <is>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+        </is>
+      </c>
+      <c r="K63" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L63" s="1" t="n"/>
+      <c r="M63" s="1" t="n"/>
+      <c r="N63" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="O63" s="1" t="n"/>
+      <c r="P63" s="1" t="inlineStr">
+        <is>
+          <t>defina, acorde e monitore níveis de serviço para os serviços de TIC relevantes, estabelecendo metas e mecanismos de acompanhamento de seu cumprimento</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="90.95" customHeight="1">
+      <c r="A64" s="1" t="inlineStr">
+        <is>
+          <t>AV129</t>
+        </is>
+      </c>
+      <c r="B64" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C64" s="1" t="n"/>
+      <c r="D64" s="1" t="n"/>
+      <c r="E64" s="1" t="n"/>
+      <c r="F64" s="1" t="inlineStr">
+        <is>
+          <t>q2203ext[A]</t>
+        </is>
+      </c>
+      <c r="G64" s="1" t="inlineStr">
+        <is>
+          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.</t>
+        </is>
+      </c>
+      <c r="H64" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I64" s="1" t="n"/>
+      <c r="J64" s="1" t="inlineStr">
+        <is>
+          <t>Inventário e controle de ativos e configurações de TIC inexistente ou insuficiente.</t>
+        </is>
+      </c>
+      <c r="K64" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L64" s="1" t="n"/>
+      <c r="M64" s="1" t="n"/>
+      <c r="N64" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="O64" s="1" t="n"/>
+      <c r="P64" s="1" t="inlineStr">
+        <is>
+          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos e base consolidada das configurações relevantes, contemplando, minimamente, dispositivos, softwares e seus relacionamentos, com informações suficientes para identificação e controle</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="90.95" customHeight="1">
+      <c r="A65" s="1" t="inlineStr">
+        <is>
+          <t>AV132</t>
+        </is>
+      </c>
+      <c r="B65" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C65" s="1" t="n"/>
+      <c r="D65" s="1" t="n"/>
+      <c r="E65" s="1" t="n"/>
+      <c r="F65" s="1" t="inlineStr">
+        <is>
+          <t>q2504ext[A]</t>
+        </is>
+      </c>
+      <c r="G65" s="1" t="inlineStr">
+        <is>
+          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.</t>
+        </is>
+      </c>
+      <c r="H65" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I65" s="1" t="n"/>
+      <c r="J65" s="1" t="inlineStr">
+        <is>
+          <t>Inventário e controle de ativos e configurações de TIC inexistente ou insuficiente.</t>
+        </is>
+      </c>
+      <c r="K65" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L65" s="1" t="n"/>
+      <c r="M65" s="1" t="n"/>
+      <c r="N65" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="O65" s="1" t="n"/>
+      <c r="P65" s="1" t="inlineStr">
+        <is>
+          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos e base consolidada das configurações relevantes, contemplando, minimamente, dispositivos, softwares e seus relacionamentos, com informações suficientes para identificação e controle</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="90.95" customHeight="1">
+      <c r="A66" s="1" t="inlineStr">
+        <is>
+          <t>AV133</t>
+        </is>
+      </c>
+      <c r="B66" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C66" s="1" t="n"/>
+      <c r="D66" s="1" t="n"/>
+      <c r="E66" s="1" t="n"/>
+      <c r="F66" s="1" t="inlineStr">
+        <is>
+          <t>q2504ext[B]</t>
+        </is>
+      </c>
+      <c r="G66" s="1" t="inlineStr">
+        <is>
+          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.</t>
+        </is>
+      </c>
+      <c r="H66" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I66" s="1" t="n"/>
+      <c r="J66" s="1" t="inlineStr">
+        <is>
+          <t>Inventário e controle de ativos e configurações de TIC inexistente ou insuficiente.</t>
+        </is>
+      </c>
+      <c r="K66" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L66" s="1" t="n"/>
+      <c r="M66" s="1" t="n"/>
+      <c r="N66" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="O66" s="1" t="n"/>
+      <c r="P66" s="1" t="inlineStr">
+        <is>
+          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos e base consolidada das configurações relevantes, contemplando, minimamente, dispositivos, softwares e seus relacionamentos, com informações suficientes para identificação e controle</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="79.90000000000001" customHeight="1">
+      <c r="A67" s="1" t="inlineStr">
+        <is>
+          <t>AV134</t>
+        </is>
+      </c>
+      <c r="B67" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C67" s="1" t="n"/>
+      <c r="D67" s="1" t="n"/>
+      <c r="E67" s="1" t="n"/>
+      <c r="F67" s="1" t="inlineStr">
+        <is>
+          <t>q2203ext[A]</t>
+        </is>
+      </c>
+      <c r="G67" s="1" t="inlineStr">
+        <is>
+          <t>COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.2.6 – Gerenciamento de configuração: orienta a identificação, o registro, o controle, o rastreamento e a verificação dos itens de configuração, bem como a manutenção de informações de configuração precisas relacionadas aos serviços.</t>
+        </is>
+      </c>
+      <c r="H67" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I67" s="1" t="n"/>
+      <c r="J67" s="1" t="inlineStr">
+        <is>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+        </is>
+      </c>
+      <c r="K67" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L67" s="1" t="n"/>
+      <c r="M67" s="1" t="n"/>
+      <c r="N67" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="O67" s="1" t="n"/>
+      <c r="P67" s="1" t="inlineStr">
+        <is>
+          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="79.90000000000001" customHeight="1">
+      <c r="A68" s="1" t="inlineStr">
+        <is>
+          <t>AV136</t>
+        </is>
+      </c>
+      <c r="B68" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C68" s="1" t="n"/>
+      <c r="D68" s="1" t="n"/>
+      <c r="E68" s="1" t="n"/>
+      <c r="F68" s="1" t="inlineStr">
+        <is>
+          <t>q2203ext[C]</t>
+        </is>
+      </c>
+      <c r="G68" s="1" t="inlineStr">
+        <is>
+          <t>COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.2.6 – Gerenciamento de configuração: orienta a identificação, o registro, o controle, o rastreamento e a verificação dos itens de configuração, bem como a manutenção de informações de configuração precisas relacionadas aos serviços.</t>
+        </is>
+      </c>
+      <c r="H68" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I68" s="1" t="n"/>
+      <c r="J68" s="1" t="inlineStr">
+        <is>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+        </is>
+      </c>
+      <c r="K68" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L68" s="1" t="n"/>
+      <c r="M68" s="1" t="n"/>
+      <c r="N68" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="O68" s="1" t="n"/>
+      <c r="P68" s="1" t="inlineStr">
+        <is>
+          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="79.90000000000001" customHeight="1">
+      <c r="A69" s="1" t="inlineStr">
+        <is>
+          <t>AV137</t>
+        </is>
+      </c>
+      <c r="B69" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C69" s="1" t="n"/>
+      <c r="D69" s="1" t="n"/>
+      <c r="E69" s="1" t="n"/>
+      <c r="F69" s="1" t="inlineStr">
+        <is>
+          <t>q2204ext[A]</t>
+        </is>
+      </c>
+      <c r="G69" s="1" t="inlineStr">
+        <is>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.6, III.9.6 e V.6.3 – Recomendações quanto à formalização e execução do processo de gestão de incidentes, incluindo registros, classificação, escalamento e tratamento.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.6.1 – Gerenciamento de incidente: orienta que os incidentes sejam registrados, classificados e priorizados, que as ações adotadas para sua resolução sejam registradas e rastreáveis e que sejam definidas responsabilidades para seu tratamento, incluindo procedimento documentado para incidentes graves.</t>
+        </is>
+      </c>
+      <c r="H69" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I69" s="1" t="n"/>
+      <c r="J69" s="1" t="inlineStr">
+        <is>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+        </is>
+      </c>
+      <c r="K69" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L69" s="1" t="n"/>
+      <c r="M69" s="1" t="n"/>
+      <c r="N69" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="O69" s="1" t="n"/>
+      <c r="P69" s="1" t="inlineStr">
+        <is>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="90.95" customHeight="1">
+      <c r="A70" s="1" t="inlineStr">
+        <is>
+          <t>AV140</t>
+        </is>
+      </c>
+      <c r="B70" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C70" s="1" t="n"/>
+      <c r="D70" s="1" t="n"/>
+      <c r="E70" s="1" t="n"/>
+      <c r="F70" s="1" t="inlineStr">
+        <is>
+          <t>q2204ext[D]</t>
+        </is>
+      </c>
+      <c r="G70" s="1" t="inlineStr">
+        <is>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.6, III.9.6 e V.6.3 – Recomendações quanto à formalização e execução do processo de gestão de incidentes, incluindo registros, classificação, escalamento e tratamento.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.6.1 – Gerenciamento de incidente: orienta que os incidentes sejam registrados, classificados e priorizados, que as ações adotadas para sua resolução sejam registradas e rastreáveis e que sejam definidas responsabilidades para seu tratamento, incluindo procedimento documentado para incidentes graves.</t>
+        </is>
+      </c>
+      <c r="H70" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I70" s="1" t="n"/>
+      <c r="J70" s="1" t="inlineStr">
+        <is>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+        </is>
+      </c>
+      <c r="K70" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L70" s="1" t="n"/>
+      <c r="M70" s="1" t="n"/>
+      <c r="N70" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="O70" s="1" t="n"/>
+      <c r="P70" s="1" t="inlineStr">
+        <is>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="90.95" customHeight="1">
+      <c r="A71" s="1" t="inlineStr">
+        <is>
+          <t>AV141</t>
+        </is>
+      </c>
+      <c r="B71" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C71" s="1" t="n"/>
+      <c r="D71" s="1" t="n"/>
+      <c r="E71" s="1" t="n"/>
+      <c r="F71" s="1" t="inlineStr">
+        <is>
+          <t>q2204ext[E]</t>
+        </is>
+      </c>
+      <c r="G71" s="1" t="inlineStr">
+        <is>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.6, III.9.6 e V.6.3 – Recomendações quanto à formalização e execução do processo de gestão de incidentes, incluindo registros, classificação, escalamento e tratamento.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.6.1 – Gerenciamento de incidente: orienta que os incidentes sejam registrados, classificados e priorizados, que as ações adotadas para sua resolução sejam registradas e rastreáveis e que sejam definidas responsabilidades para seu tratamento, incluindo procedimento documentado para incidentes graves.</t>
+        </is>
+      </c>
+      <c r="H71" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I71" s="1" t="n"/>
+      <c r="J71" s="1" t="inlineStr">
+        <is>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+        </is>
+      </c>
+      <c r="K71" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L71" s="1" t="n"/>
+      <c r="M71" s="1" t="n"/>
+      <c r="N71" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="O71" s="1" t="n"/>
+      <c r="P71" s="1" t="inlineStr">
+        <is>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="90.95" customHeight="1">
+      <c r="A72" s="1" t="inlineStr">
+        <is>
+          <t>AV143</t>
+        </is>
+      </c>
+      <c r="B72" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C72" s="1" t="n"/>
+      <c r="D72" s="1" t="n"/>
+      <c r="E72" s="1" t="n"/>
+      <c r="F72" s="1" t="inlineStr">
+        <is>
+          <t>q2801ext[A]</t>
+        </is>
+      </c>
+      <c r="G72" s="1" t="inlineStr">
+        <is>
+          <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Lei nº 14.133/2021, art. 19, inciso IV: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.
+Acórdão nº 2.342/2016-TCU-Plenário, item 9.1.7 – Precedente quanto à definição, aprovação e formalização de processo de trabalho para o planejamento de cada contratação, com controles internos mínimos.</t>
+        </is>
+      </c>
+      <c r="H72" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I72" s="1" t="n"/>
+      <c r="J72" s="1" t="inlineStr">
+        <is>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+        </is>
+      </c>
+      <c r="K72" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L72" s="1" t="n"/>
+      <c r="M72" s="1" t="n"/>
+      <c r="N72" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="O72" s="1" t="n"/>
+      <c r="P72" s="1" t="inlineStr">
+        <is>
+          <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="90.95" customHeight="1">
+      <c r="A73" s="1" t="inlineStr">
+        <is>
+          <t>AV148</t>
+        </is>
+      </c>
+      <c r="B73" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C73" s="1" t="n"/>
+      <c r="D73" s="1" t="n"/>
+      <c r="E73" s="1" t="n"/>
+      <c r="F73" s="1" t="inlineStr">
+        <is>
+          <t>q2804[A]</t>
+        </is>
+      </c>
+      <c r="G73" s="1" t="inlineStr">
+        <is>
+          <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+COBIT 2019, BAI02.04 - Obter aprovação dos requisitos da solução: obter aprovação formal dos requisitos funcionais, técnicos, de segurança e de conformidade antes de prosseguir com a solução.
+Instrução Normativa SGD/ME nº 94/2022, arts. 1º, §1º, 10, II, 11, §2º, e 12, §6º – referência de boa prática para estruturação da fase de planejamento das contratações de TIC, participação da área técnica e instituição da Equipe de Planejamento, observada sua aplicação direta aos integrantes do SISP e a possibilidade de procedimentos simplificados.</t>
+        </is>
+      </c>
+      <c r="H73" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I73" s="1" t="n"/>
+      <c r="J73" s="1" t="inlineStr">
+        <is>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
+        </is>
+      </c>
+      <c r="K73" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L73" s="1" t="n"/>
+      <c r="M73" s="1" t="n"/>
+      <c r="N73" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="O73" s="1" t="n"/>
+      <c r="P73" s="1" t="inlineStr">
+        <is>
+          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo procedimentos simplificados e proporcionais à natureza, ao risco e ao valor da contratação, preservada análise técnica compatível</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="90.95" customHeight="1">
+      <c r="A74" s="1" t="inlineStr">
+        <is>
+          <t>AV152</t>
+        </is>
+      </c>
+      <c r="B74" s="1" t="inlineStr">
+        <is>
+          <t>questionario</t>
+        </is>
+      </c>
+      <c r="C74" s="1" t="n"/>
+      <c r="D74" s="1" t="n"/>
+      <c r="E74" s="1" t="n"/>
+      <c r="F74" s="1" t="inlineStr">
+        <is>
+          <t>q2801ext[B]</t>
+        </is>
+      </c>
+      <c r="G74" s="1" t="inlineStr">
+        <is>
+          <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Lei nº 14.133/2021, art. 19, inciso IV: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.
+Acórdão nº 2.342/2016-TCU-Plenário, item 9.1.7 – Precedente quanto à definição, aprovação e formalização de processo de trabalho para o planejamento de cada contratação, com controles internos mínimos.</t>
+        </is>
+      </c>
+      <c r="H74" s="1" t="inlineStr">
+        <is>
+          <t>Resposta negativa ao detalhamento b) do item 2801 do Questionário, para verificar se são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
+      <c r="I74" s="1" t="n"/>
+      <c r="J74" s="1" t="inlineStr">
+        <is>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+        </is>
+      </c>
+      <c r="K74" s="1" t="inlineStr">
+        <is>
+          <t>(Não | N/A)</t>
+        </is>
+      </c>
+      <c r="L74" s="1" t="n"/>
+      <c r="M74" s="1" t="n"/>
+      <c r="N74" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="O74" s="1" t="n"/>
+      <c r="P74" s="1" t="inlineStr">
+        <is>
+          <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="90.95" customHeight="1">
+      <c r="A75" s="1" t="inlineStr">
+        <is>
+          <t>AV153</t>
+        </is>
+      </c>
+      <c r="B75" s="1" t="inlineStr">
+        <is>
+          <t>avaliacao_evidencias_ajustes</t>
+        </is>
+      </c>
+      <c r="C75" s="1" t="n"/>
+      <c r="D75" s="1" t="n"/>
+      <c r="E75" s="1" t="n"/>
+      <c r="F75" s="1" t="inlineStr">
+        <is>
+          <t>q2801ext[B]</t>
+        </is>
+      </c>
+      <c r="G75" s="1" t="inlineStr">
+        <is>
+          <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Lei nº 14.133/2021, art. 19, inciso IV: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.
+Acórdão nº 2.342/2016-TCU-Plenário, item 9.1.7 – Precedente quanto à definição, aprovação e formalização de processo de trabalho para o planejamento de cada contratação, com controles internos mínimos.</t>
+        </is>
+      </c>
+      <c r="H75" s="1" t="inlineStr">
+        <is>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+        </is>
+      </c>
+      <c r="I75" s="1" t="n"/>
+      <c r="J75" s="1" t="inlineStr">
+        <is>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+        </is>
+      </c>
+      <c r="K75" s="1" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="L75" s="1" t="n"/>
+      <c r="M75" s="1" t="n"/>
+      <c r="N75" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="O75" s="1" t="n"/>
+      <c r="P75" s="1" t="inlineStr">
+        <is>
+          <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="102.2" customHeight="1">
+      <c r="A76" s="1" t="inlineStr">
+        <is>
+          <t>AV154</t>
+        </is>
+      </c>
+      <c r="B76" s="1" t="inlineStr">
+        <is>
+          <t>questionario</t>
+        </is>
+      </c>
+      <c r="C76" s="1" t="n"/>
+      <c r="D76" s="1" t="n"/>
+      <c r="E76" s="1" t="n"/>
+      <c r="F76" s="1" t="inlineStr">
+        <is>
+          <t>existe_plano_ti</t>
+        </is>
+      </c>
+      <c r="G76" s="1" t="inlineStr">
+        <is>
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
+        </is>
+      </c>
+      <c r="H76" s="1" t="inlineStr">
+        <is>
+          <t>Resposta ao item 2102 que não caracteriza a existência de plano de TIC vigente, ainda que parcialmente adotado</t>
+        </is>
+      </c>
+      <c r="I76" s="1" t="n"/>
+      <c r="J76" s="1" t="inlineStr">
+        <is>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
+        </is>
+      </c>
+      <c r="K76" s="1" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L76" s="1" t="n"/>
+      <c r="M76" s="1" t="n"/>
+      <c r="N76" s="1" t="inlineStr">
+        <is>
+          <t>Determinação</t>
+        </is>
+      </c>
+      <c r="O76" s="1" t="n"/>
+      <c r="P76" s="1" t="inlineStr">
+        <is>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="102.2" customHeight="1">
+      <c r="A77" s="1" t="inlineStr">
+        <is>
+          <t>AV155</t>
+        </is>
+      </c>
+      <c r="B77" s="1" t="inlineStr">
+        <is>
+          <t>questionario</t>
+        </is>
+      </c>
+      <c r="C77" s="1" t="n"/>
+      <c r="D77" s="1" t="n"/>
+      <c r="E77" s="1" t="n"/>
+      <c r="F77" s="1" t="inlineStr">
+        <is>
+          <t>existe_plano_ti</t>
+        </is>
+      </c>
+      <c r="G77" s="1" t="inlineStr">
+        <is>
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
+        </is>
+      </c>
+      <c r="H77" s="1" t="inlineStr">
         <is>
           <t>Plano de TIC vigente declarado no item 2102, ao menos parcialmente adotado</t>
         </is>
       </c>
-      <c r="I47" s="1" t="n"/>
-      <c r="J47" s="1" t="n"/>
-      <c r="K47" s="1" t="inlineStr">
+      <c r="I77" s="1" t="n"/>
+      <c r="J77" s="1" t="n"/>
+      <c r="K77" s="1" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="L47" s="1" t="n"/>
-      <c r="M47" s="1" t="n"/>
-      <c r="N47" s="1" t="inlineStr">
+      <c r="L77" s="1" t="n"/>
+      <c r="M77" s="1" t="n"/>
+      <c r="N77" s="1" t="inlineStr">
         <is>
           <t>Determinação</t>
         </is>
       </c>
-      <c r="O47" s="1" t="n"/>
-      <c r="P47" s="1" t="inlineStr">
+      <c r="O77" s="1" t="n"/>
+      <c r="P77" s="1" t="inlineStr">
         <is>
           <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="113.45" customHeight="1"/>
-    <row r="49" ht="113.45" customHeight="1"/>
-    <row r="50" ht="113.45" customHeight="1"/>
-    <row r="51" ht="113.45" customHeight="1"/>
-    <row r="52" ht="113.45" customHeight="1"/>
-    <row r="53" ht="113.45" customHeight="1"/>
-    <row r="54" ht="113.45" customHeight="1"/>
-    <row r="55" ht="113.45" customHeight="1"/>
-    <row r="56" ht="113.45" customHeight="1"/>
-    <row r="57" ht="90.95" customHeight="1"/>
-    <row r="58" ht="90.95" customHeight="1"/>
-    <row r="59" ht="90.95" customHeight="1"/>
-    <row r="60" ht="79.90000000000001" customHeight="1"/>
-    <row r="61" ht="79.90000000000001" customHeight="1"/>
-    <row r="62" ht="90.95" customHeight="1"/>
-    <row r="63" ht="90.95" customHeight="1"/>
-    <row r="64" ht="90.95" customHeight="1"/>
-    <row r="65" ht="90.95" customHeight="1"/>
-    <row r="66" ht="90.95" customHeight="1"/>
-    <row r="67" ht="79.90000000000001" customHeight="1"/>
-    <row r="68" ht="79.90000000000001" customHeight="1"/>
-    <row r="69" ht="79.90000000000001" customHeight="1"/>
-    <row r="70" ht="90.95" customHeight="1"/>
-    <row r="71" ht="90.95" customHeight="1"/>
-    <row r="72" ht="90.95" customHeight="1"/>
-    <row r="73" ht="90.95" customHeight="1"/>
-    <row r="74" ht="90.95" customHeight="1"/>
-    <row r="75" ht="90.95" customHeight="1"/>
-    <row r="76" ht="102.2" customHeight="1"/>
-    <row r="77" ht="102.2" customHeight="1"/>
     <row r="78" ht="102.2" customHeight="1"/>
     <row r="79" ht="102.2" customHeight="1"/>
     <row r="80" ht="102.2" customHeight="1"/>
@@ -3428,7 +5063,7 @@
     <row r="153" ht="23.85" customHeight="1"/>
     <row r="154" ht="23.85" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A3:P47"/>
+  <autoFilter ref="A3:P77"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -3440,7 +5075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H45"/>
+  <dimension ref="A2:H74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3824,7 +5459,7 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>AV08</t>
+          <t>AV08 &amp; ~AV86</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
@@ -3844,7 +5479,7 @@
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>MR016</t>
+          <t>MR011</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
@@ -3854,25 +5489,25 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Comitê de TIC ou instância equivalente não instituído formalmente ou sem representação de áreas relevantes da organização.</t>
+          <t>Ausência de objetivos, indicadores ou metas para a gestão de TIC.</t>
         </is>
       </c>
       <c r="D12" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>AV11</t>
+          <t>AV86</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>AV11</t>
+          <t>AV86</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 1001, não houve declaração afirmativa quanto à prática avaliada: dispõe de comitê de tecnologia da informação composto por representantes de áreas relevantes da organização</t>
+          <t>No subitem h) do item 1001, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que estabeleceu objetivos, indicadores e metas para a gestão de tecnologia da informação</t>
         </is>
       </c>
       <c r="H12" s="9" t="b">
@@ -3882,7 +5517,7 @@
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>MR018</t>
+          <t>MR016</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
@@ -3892,7 +5527,7 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>Comitê de TIC ou instância equivalente sem atuação efetiva comprovada.</t>
+          <t>Comitê de TIC ou instância equivalente não instituído formalmente ou sem representação de áreas relevantes da organização.</t>
         </is>
       </c>
       <c r="D13" s="9" t="n">
@@ -3900,17 +5535,17 @@
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>AV12 &amp; AV13</t>
+          <t>AV11 &amp; ~AV89</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>AV12</t>
+          <t>AV11</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 1001, a organização declarou dispor de comitê de tecnologia da informação composto por representantes de áreas relevantes, o que levou à análise de sua atuação efetiva</t>
+          <t>No subitem e) do item 1001, não houve declaração afirmativa quanto à prática avaliada: dispõe de comitê de tecnologia da informação composto por representantes de áreas relevantes da organização</t>
         </is>
       </c>
       <c r="H13" s="9" t="b">
@@ -3920,7 +5555,7 @@
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>MR020</t>
+          <t>MR017</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
@@ -3930,7 +5565,7 @@
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Comitê de TIC ou instância equivalente sem atuação efetiva comprovada.</t>
+          <t>Comitê de TIC ou instância equivalente não instituído formalmente ou sem representação de áreas relevantes da organização.</t>
         </is>
       </c>
       <c r="D14" s="9" t="n">
@@ -3938,17 +5573,17 @@
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>AV12 &amp; AV13</t>
+          <t>AV89</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>AV13</t>
+          <t>AV89</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>No subitem f) do item 1001, não houve declaração afirmativa quanto à atuação do comitê de tecnologia da informação nas atividades previstas em ato constitutivo</t>
+          <t>No subitem e) do item 1001, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que dispõe de comitê de tecnologia da informação composto por representantes de áreas relevantes da organização</t>
         </is>
       </c>
       <c r="H14" s="9" t="b">
@@ -3958,17 +5593,17 @@
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>MR022</t>
+          <t>MR018</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>PA03</t>
+          <t>PA02</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
+          <t>Comitê de TIC ou instância equivalente sem atuação efetiva comprovada.</t>
         </is>
       </c>
       <c r="D15" s="9" t="n">
@@ -3976,17 +5611,17 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>AV14</t>
+          <t>AV12 &amp; ~AV90 &amp; (AV13 | AV91)</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>AV14</t>
+          <t>AV12</t>
         </is>
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2101, não houve declaração afirmativa quanto à prática avaliada: as áreas demandantes de soluções de TI participam do processo de planejamento de tecnologia da informação</t>
+          <t>No subitem e) do item 1001, a organização declarou dispor de comitê de tecnologia da informação composto por representantes de áreas relevantes, o que levou à análise de sua atuação efetiva</t>
         </is>
       </c>
       <c r="H15" s="9" t="b">
@@ -3996,35 +5631,35 @@
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>MR024</t>
+          <t>MR019</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>PA03</t>
+          <t>PA02</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
+          <t>Comitê de TIC ou instância equivalente sem atuação efetiva comprovada.</t>
         </is>
       </c>
       <c r="D16" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>AV15</t>
+          <t>AV90 &amp; (AV13 | AV91)</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>AV15</t>
+          <t>AV90</t>
         </is>
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2101, não houve declaração afirmativa quanto à prática avaliada: estabeleceu critérios para orientar a seleção e a priorização das iniciativas de TI (projetos e ações) e os mantêm atualizados</t>
+          <t>No subitem e) do item 1001, a organização declarou dispor de comitê de tecnologia da informação composto por representantes de áreas relevantes, mas a evidência foi insuficiente para comprovar a prática declarada</t>
         </is>
       </c>
       <c r="H16" s="9" t="b">
@@ -4034,35 +5669,35 @@
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>MR028</t>
+          <t>MR020</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>PA03</t>
+          <t>PA02</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
+          <t>Comitê de TIC ou instância equivalente sem atuação efetiva comprovada.</t>
         </is>
       </c>
       <c r="D17" s="9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>AV17</t>
+          <t>AV13 &amp; ~AV91 &amp; AV12 &amp; ~AV90</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>AV17</t>
+          <t>AV13</t>
         </is>
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2101, não houve declaração afirmativa quanto à prática avaliada: o processo de planejamento de TI está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem f) do item 1001, não houve declaração afirmativa quanto à atuação do comitê de tecnologia da informação nas atividades previstas em ato constitutivo</t>
         </is>
       </c>
       <c r="H17" s="9" t="b">
@@ -4072,35 +5707,35 @@
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>MR030</t>
+          <t>MR021</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>PA03</t>
+          <t>PA02</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Ausência de aprovação formal do plano de TIC.</t>
+          <t>Comitê de TIC ou instância equivalente sem atuação efetiva comprovada.</t>
         </is>
       </c>
       <c r="D18" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>AV155 &amp; AV18</t>
+          <t>AV91 &amp; (AV12 | AV90)</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>AV18</t>
+          <t>AV91</t>
         </is>
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2102, não houve declaração afirmativa quanto à prática avaliada: o plano de tecnologia da informação (plano de TI) é aprovado pelo dirigente máximo da organização ou por dirigente ou colegiado que integra a alta administração</t>
+          <t>No subitem f) do item 1001, a organização declarou atuação do comitê de tecnologia da informação, mas a evidência foi insuficiente para comprovar a prática declarada</t>
         </is>
       </c>
       <c r="H18" s="9" t="b">
@@ -4110,7 +5745,7 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>MR032</t>
+          <t>MR022</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
@@ -4120,7 +5755,7 @@
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="D19" s="9" t="n">
@@ -4128,17 +5763,17 @@
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>AV155 &amp; AV19</t>
+          <t>AV14 &amp; ~AV92</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>AV19</t>
+          <t>AV14</t>
         </is>
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2102, não houve declaração afirmativa quanto à prática avaliada: as iniciativas de TI (projetos e ações) constantes do plano de TI alinham-se aos objetivos e iniciativas definidos no planejamento institucional (como PPA, planos estratégicos, planos setoriais e plano de governo, no caso de municípios), bem como, quando aplicável, às estratégias e diretrizes estabelecidas por instâncias superiores de governança (como a Estratégia Nacional de Tecnologia da Informação e Comunicação do Poder Judiciário - ENTIC-JUD, normas e orientações do SETIC/PRODERJ (para órgãos estaduais) ou instâncias de governança equivalentes no âmbito municipal)</t>
+          <t>No subitem a) do item 2101, não houve declaração afirmativa quanto à prática avaliada: as áreas demandantes de soluções de TI participam do processo de planejamento de tecnologia da informação</t>
         </is>
       </c>
       <c r="H19" s="9" t="b">
@@ -4148,7 +5783,7 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>MR034</t>
+          <t>MR023</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
@@ -4158,25 +5793,25 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="D20" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>AV155 &amp; AV20</t>
+          <t>AV92</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>AV20</t>
+          <t>AV92</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2102, não houve declaração afirmativa quanto à prática avaliada: o plano de TI fundamenta a proposta orçamentária da área de TI e o plano de contratações</t>
+          <t>No subitem a) do item 2101, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as áreas demandantes de soluções de TI participam do processo de planejamento de tecnologia da informação</t>
         </is>
       </c>
       <c r="H20" s="9" t="b">
@@ -4186,7 +5821,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>MR041</t>
+          <t>MR024</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
@@ -4196,25 +5831,25 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Ausência de acompanhamento da execução do plano de TIC.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="D21" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>AV155 &amp; AV24</t>
+          <t>AV15 &amp; ~AV93</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>AV24</t>
+          <t>AV15</t>
         </is>
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2102, não houve declaração afirmativa quanto à prática avaliada: é feito acompanhamento concomitante à execução do plano de TI, com vistas a assegurar sua observância e possibilitar a realização de ajustes que se fizerem necessário</t>
+          <t>No subitem b) do item 2101, não houve declaração afirmativa quanto à prática avaliada: estabeleceu critérios para orientar a seleção e a priorização das iniciativas de TI (projetos e ações) e os mantêm atualizados</t>
         </is>
       </c>
       <c r="H21" s="9" t="b">
@@ -4224,35 +5859,35 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>MR043</t>
+          <t>MR025</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA03</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Ausência de força de trabalho dedicada à TIC.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="D22" s="9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>AV26 &amp; AV25</t>
+          <t>AV93</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>AV25</t>
+          <t>AV93</t>
         </is>
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>Item 0105: embora a organização tenha declarado estrutura formal de TIC no item 0101, informou não possuir profissionais atuando regularmente em tecnologia da informação</t>
+          <t>No subitem b) do item 2101, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que estabeleceu critérios para orientar a seleção e a priorização das iniciativas de TI (projetos e ações) e os mantêm atualizados</t>
         </is>
       </c>
       <c r="H22" s="9" t="b">
@@ -4262,35 +5897,35 @@
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>MR045</t>
+          <t>MR028</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA03</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou insuficiência de definição documentada do quantitativo necessário de pessoal de TIC e segurança da informação.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="D23" s="9" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>AV29</t>
+          <t>AV17 &amp; ~AV95</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>AV29</t>
+          <t>AV17</t>
         </is>
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2703, não houve declaração afirmativa quanto à prática avaliada: definiu-se, de maneira documentada, um quantitativo necessário de pessoal da área de tecnologia da informação e segurança da informação</t>
+          <t>No subitem d) do item 2101, não houve declaração afirmativa quanto à prática avaliada: o processo de planejamento de TI está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H23" s="9" t="b">
@@ -4300,35 +5935,35 @@
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>MR047</t>
+          <t>MR029</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA03</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="D24" s="9" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>AV31</t>
+          <t>AV95</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>AV31</t>
+          <t>AV95</t>
         </is>
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2708, não houve declaração afirmativa quanto à prática avaliada: possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
+          <t>No subitem d) do item 2101, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de planejamento de TI está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H24" s="9" t="b">
@@ -4338,35 +5973,35 @@
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>MR049</t>
+          <t>MR030</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA03</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Ausência de aprovação formal do plano de TIC.</t>
         </is>
       </c>
       <c r="D25" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>AV33</t>
+          <t>AV155 &amp; AV18 &amp; ~AV96</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>AV33</t>
+          <t>AV18</t>
         </is>
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2708, não houve declaração afirmativa quanto à prática avaliada: possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
+          <t>No subitem a) do item 2102, não houve declaração afirmativa quanto à prática avaliada: o plano de tecnologia da informação (plano de TI) é aprovado pelo dirigente máximo da organização ou por dirigente ou colegiado que integra a alta administração</t>
         </is>
       </c>
       <c r="H25" s="9" t="b">
@@ -4376,35 +6011,35 @@
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>MR062</t>
+          <t>MR031</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA03</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Operação de TIC predominantemente terceirizada sem profissionais internos de TIC.</t>
+          <t>Ausência de aprovação formal do plano de TIC.</t>
         </is>
       </c>
       <c r="D26" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>AV45 &amp; AV46</t>
+          <t>AV96</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>AV45</t>
+          <t>AV96</t>
         </is>
       </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>A organização informou modelo de operação de TIC com execução predominantemente terceirizada, o que levou à análise de sua capacidade interna de coordenação e fiscalização</t>
+          <t>No subitem a) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o plano de tecnologia da informação (plano de TI) é aprovado pelo dirigente máximo da organização ou por dirigente ou colegiado que integra a alta administração</t>
         </is>
       </c>
       <c r="H26" s="9" t="b">
@@ -4414,35 +6049,35 @@
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>MR063</t>
+          <t>MR032</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA03</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>Operação de TIC predominantemente terceirizada sem profissionais internos de TIC.</t>
+          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
         </is>
       </c>
       <c r="D27" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>AV45 &amp; AV46</t>
+          <t>AV155 &amp; AV19 &amp; ~AV97</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>AV46</t>
+          <t>AV19</t>
         </is>
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t>Não foram identificados profissionais internos de TIC para coordenar e fiscalizar a execução das atividades de tecnologia da informação</t>
+          <t>No subitem d) do item 2102, não houve declaração afirmativa quanto à prática avaliada: as iniciativas de TI (projetos e ações) constantes do plano de TI alinham-se aos objetivos e iniciativas definidos no planejamento institucional (como PPA, planos estratégicos, planos setoriais e plano de governo, no caso de municípios), bem como, quando aplicável, às estratégias e diretrizes estabelecidas por instâncias superiores de governança (como a Estratégia Nacional de Tecnologia da Informação e Comunicação do Poder Judiciário - ENTIC-JUD, normas e orientações do SETIC/PRODERJ (para órgãos estaduais) ou instâncias de governança equivalentes no âmbito municipal)</t>
         </is>
       </c>
       <c r="H27" s="9" t="b">
@@ -4452,35 +6087,35 @@
     <row r="28" ht="45" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>MR065</t>
+          <t>MR033</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA03</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
         </is>
       </c>
       <c r="D28" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>AV54</t>
+          <t>AV97</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>AV54</t>
+          <t>AV97</t>
         </is>
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
+          <t>No subitem d) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as iniciativas de TI (projetos e ações) constantes do plano de TI alinham-se aos objetivos e iniciativas definidos no planejamento institucional (como PPA, planos estratégicos, planos setoriais e plano de governo, no caso de municípios), bem como, quando aplicável, às estratégias e diretrizes estabelecidas por instâncias superiores de governança (como a Estratégia Nacional de Tecnologia da Informação e Comunicação do Poder Judiciário - ENTIC-JUD, normas e orientações do SETIC/PRODERJ (para órgãos estaduais) ou instâncias de governança equivalentes no âmbito municipal)</t>
         </is>
       </c>
       <c r="H28" s="9" t="b">
@@ -4490,17 +6125,17 @@
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>MR067</t>
+          <t>MR034</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA03</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
         </is>
       </c>
       <c r="D29" s="9" t="n">
@@ -4508,17 +6143,17 @@
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>AV55</t>
+          <t>AV155 &amp; AV20 &amp; ~AV98</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>AV55</t>
+          <t>AV20</t>
         </is>
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
+          <t>No subitem c) do item 2102, não houve declaração afirmativa quanto à prática avaliada: o plano de TI fundamenta a proposta orçamentária da área de TI e o plano de contratações</t>
         </is>
       </c>
       <c r="H29" s="9" t="b">
@@ -4528,17 +6163,17 @@
     <row r="30" ht="45" customHeight="1">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>MR069</t>
+          <t>MR035</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA03</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
         </is>
       </c>
       <c r="D30" s="9" t="n">
@@ -4546,17 +6181,17 @@
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>AV56</t>
+          <t>AV98</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>AV56</t>
+          <t>AV98</t>
         </is>
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
+          <t>No subitem c) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o plano de TI fundamenta a proposta orçamentária da área de TI e o plano de contratações</t>
         </is>
       </c>
       <c r="H30" s="9" t="b">
@@ -4566,35 +6201,35 @@
     <row r="31" ht="45" customHeight="1">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>MR071</t>
+          <t>MR041</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA03</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Ausência de acompanhamento da execução do plano de TIC.</t>
         </is>
       </c>
       <c r="D31" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>AV57</t>
+          <t>AV155 &amp; AV24 &amp; ~AV101</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>AV57</t>
+          <t>AV24</t>
         </is>
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2201, não houve declaração afirmativa quanto à prática avaliada: são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
+          <t>No subitem e) do item 2102, não houve declaração afirmativa quanto à prática avaliada: é feito acompanhamento concomitante à execução do plano de TI, com vistas a assegurar sua observância e possibilitar a realização de ajustes que se fizerem necessário</t>
         </is>
       </c>
       <c r="H31" s="9" t="b">
@@ -4604,35 +6239,35 @@
     <row r="32" ht="45" customHeight="1">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>MR073</t>
+          <t>MR042</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA03</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Ausência de acompanhamento da execução do plano de TIC.</t>
         </is>
       </c>
       <c r="D32" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>AV58</t>
+          <t>AV101</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>AV58</t>
+          <t>AV101</t>
         </is>
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2201, não houve declaração afirmativa quanto à prática avaliada: a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
+          <t>No subitem e) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que é feito acompanhamento concomitante à execução do plano de TI, com vistas a assegurar sua observância e possibilitar a realização de ajustes que se fizerem necessário</t>
         </is>
       </c>
       <c r="H32" s="9" t="b">
@@ -4642,17 +6277,17 @@
     <row r="33" ht="45" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>MR075</t>
+          <t>MR043</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Ausência de força de trabalho dedicada à TIC.</t>
         </is>
       </c>
       <c r="D33" s="9" t="n">
@@ -4660,17 +6295,17 @@
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>AV59</t>
+          <t>AV26 &amp; AV25</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>AV59</t>
+          <t>AV25</t>
         </is>
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2203, não houve declaração afirmativa quanto à prática avaliada: mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
+          <t>Item 0105: embora a organização tenha declarado estrutura formal de TIC no item 0101, informou não possuir profissionais atuando regularmente em tecnologia da informação</t>
         </is>
       </c>
       <c r="H33" s="9" t="b">
@@ -4680,17 +6315,17 @@
     <row r="34" ht="45" customHeight="1">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>MR077</t>
+          <t>MR045</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
+          <t>Ausência ou insuficiência de definição documentada do quantitativo necessário de pessoal de TIC e segurança da informação.</t>
         </is>
       </c>
       <c r="D34" s="9" t="n">
@@ -4698,17 +6333,17 @@
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>AV62</t>
+          <t>AV29 &amp; ~AV103</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>AV62</t>
+          <t>AV29</t>
         </is>
       </c>
       <c r="G34" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
+          <t>No subitem c) do item 2703, não houve declaração afirmativa quanto à prática avaliada: definiu-se, de maneira documentada, um quantitativo necessário de pessoal da área de tecnologia da informação e segurança da informação</t>
         </is>
       </c>
       <c r="H34" s="9" t="b">
@@ -4718,17 +6353,17 @@
     <row r="35" ht="90" customHeight="1">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>MR079</t>
+          <t>MR046</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
+          <t>Ausência ou insuficiência de definição documentada do quantitativo necessário de pessoal de TIC e segurança da informação.</t>
         </is>
       </c>
       <c r="D35" s="9" t="n">
@@ -4736,17 +6371,17 @@
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>AV63</t>
+          <t>AV103</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>AV63</t>
+          <t>AV103</t>
         </is>
       </c>
       <c r="G35" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
+          <t>No subitem c) do item 2703, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu-se, de maneira documentada, um quantitativo necessário de pessoal da área de tecnologia da informação e segurança da informação</t>
         </is>
       </c>
       <c r="H35" s="9" t="b">
@@ -4756,35 +6391,35 @@
     <row r="36" ht="105" customHeight="1">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>MR083</t>
+          <t>MR047</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="D36" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>AV66</t>
+          <t>AV31 &amp; ~AV105</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>AV66</t>
+          <t>AV31</t>
         </is>
       </c>
       <c r="G36" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2203, não houve declaração afirmativa quanto à prática avaliada: o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem b) do item 2708, não houve declaração afirmativa quanto à prática avaliada: possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
         </is>
       </c>
       <c r="H36" s="9" t="b">
@@ -4794,35 +6429,35 @@
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>MR085</t>
+          <t>MR048</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="D37" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>AV67</t>
+          <t>AV105</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>AV67</t>
+          <t>AV105</t>
         </is>
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu regras para a priorização e o escalamento de incidentes</t>
+          <t>No subitem b) do item 2708, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
         </is>
       </c>
       <c r="H37" s="9" t="b">
@@ -4832,35 +6467,35 @@
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>MR087</t>
+          <t>MR049</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="D38" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>AV70</t>
+          <t>AV33 &amp; ~AV107</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>AV70</t>
+          <t>AV33</t>
         </is>
       </c>
       <c r="G38" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2204, não houve declaração afirmativa quanto à prática avaliada: o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem d) do item 2708, não houve declaração afirmativa quanto à prática avaliada: possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
         </is>
       </c>
       <c r="H38" s="9" t="b">
@@ -4870,35 +6505,35 @@
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>MR089</t>
+          <t>MR050</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="D39" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>AV71</t>
+          <t>AV107</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>AV71</t>
+          <t>AV107</t>
         </is>
       </c>
       <c r="G39" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
+          <t>No subitem d) do item 2708, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
         </is>
       </c>
       <c r="H39" s="9" t="b">
@@ -4908,17 +6543,17 @@
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>MR091</t>
+          <t>MR062</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>PA06</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+          <t>Operação de TIC predominantemente terceirizada sem profissionais internos de TIC.</t>
         </is>
       </c>
       <c r="D40" s="9" t="n">
@@ -4926,17 +6561,17 @@
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>AV73</t>
+          <t>AV45 &amp; AV46</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>AV73</t>
+          <t>AV45</t>
         </is>
       </c>
       <c r="G40" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2801, não houve declaração afirmativa quanto à prática avaliada: o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
+          <t>A organização informou modelo de operação de TIC com execução predominantemente terceirizada, o que levou à análise de sua capacidade interna de coordenação e fiscalização</t>
         </is>
       </c>
       <c r="H40" s="9" t="b">
@@ -4946,35 +6581,35 @@
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>MR101</t>
+          <t>MR063</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
         <is>
-          <t>PA06</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
+          <t>Operação de TIC predominantemente terceirizada sem profissionais internos de TIC.</t>
         </is>
       </c>
       <c r="D41" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>AV78</t>
+          <t>AV45 &amp; AV46</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>AV78</t>
+          <t>AV46</t>
         </is>
       </c>
       <c r="G41" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
+          <t>Não foram identificados profissionais internos de TIC para coordenar e fiscalizar a execução das atividades de tecnologia da informação</t>
         </is>
       </c>
       <c r="H41" s="9" t="b">
@@ -4984,17 +6619,17 @@
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>MR109</t>
+          <t>MR065</t>
         </is>
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>PA06</t>
+          <t>PA05</t>
         </is>
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D42" s="9" t="n">
@@ -5002,17 +6637,17 @@
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>AV82</t>
+          <t>AV54 &amp; ~AV124</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>AV82</t>
+          <t>AV54</t>
         </is>
       </c>
       <c r="G42" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de TI executadas no exercício encontram-se previamente estabelecidas nos instrumentos de planejamento vigentes (PDTI/PEDTIC e PCA)</t>
+          <t>No subitem a) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
         </is>
       </c>
       <c r="H42" s="9" t="b">
@@ -5022,35 +6657,35 @@
     <row r="43" ht="45" customHeight="1">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>MR110</t>
+          <t>MR066</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>PA06</t>
+          <t>PA05</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D43" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>AV83</t>
+          <t>AV124</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>AV83</t>
+          <t>AV124</t>
         </is>
       </c>
       <c r="G43" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2804, não houve declaração afirmativa quanto à prática avaliada: a fase de planejamento de cada contratação de TI é conduzida por uma Equipe de Planejamento da Contratação formalmente designada (composta, minimamente, por integrante requisitante e integrante técnico da área de TI)</t>
+          <t>No subitem a) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
         </is>
       </c>
       <c r="H43" s="9" t="b">
@@ -5060,35 +6695,35 @@
     <row r="44" ht="45" customHeight="1">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>MR111</t>
+          <t>MR067</t>
         </is>
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>PA06</t>
+          <t>PA05</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="D44" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>AV152</t>
+          <t>AV55 &amp; ~AV125</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>AV152</t>
+          <t>AV55</t>
         </is>
       </c>
       <c r="G44" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2801, não houve declaração afirmativa quanto à prática avaliada: são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
+          <t>No subitem b) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
         </is>
       </c>
       <c r="H44" s="9" t="b">
@@ -5098,17 +6733,17 @@
     <row r="45" ht="45" customHeight="1">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>MR113</t>
+          <t>MR068</t>
         </is>
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>PA03</t>
+          <t>PA05</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="D45" s="9" t="n">
@@ -5116,52 +6751,1125 @@
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
+          <t>AV125</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="inlineStr">
+        <is>
+          <t>AV125</t>
+        </is>
+      </c>
+      <c r="G45" s="9" t="inlineStr">
+        <is>
+          <t>No subitem b) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
+        </is>
+      </c>
+      <c r="H45" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>MR069</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>AV56 &amp; ~AV126</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="inlineStr">
+        <is>
+          <t>AV56</t>
+        </is>
+      </c>
+      <c r="G46" s="9" t="inlineStr">
+        <is>
+          <t>No subitem c) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
+        </is>
+      </c>
+      <c r="H46" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>MR070</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>AV126</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="inlineStr">
+        <is>
+          <t>AV126</t>
+        </is>
+      </c>
+      <c r="G47" s="9" t="inlineStr">
+        <is>
+          <t>No subitem c) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
+        </is>
+      </c>
+      <c r="H47" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>MR071</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>AV57 &amp; ~AV127</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="inlineStr">
+        <is>
+          <t>AV57</t>
+        </is>
+      </c>
+      <c r="G48" s="9" t="inlineStr">
+        <is>
+          <t>No subitem d) do item 2201, não houve declaração afirmativa quanto à prática avaliada: são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
+        </is>
+      </c>
+      <c r="H48" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" ht="45" customHeight="1">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>MR072</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+        </is>
+      </c>
+      <c r="D49" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>AV127</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="inlineStr">
+        <is>
+          <t>AV127</t>
+        </is>
+      </c>
+      <c r="G49" s="9" t="inlineStr">
+        <is>
+          <t>No subitem d) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
+        </is>
+      </c>
+      <c r="H49" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>MR073</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>AV58 &amp; ~AV128</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="inlineStr">
+        <is>
+          <t>AV58</t>
+        </is>
+      </c>
+      <c r="G50" s="9" t="inlineStr">
+        <is>
+          <t>No subitem e) do item 2201, não houve declaração afirmativa quanto à prática avaliada: a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
+        </is>
+      </c>
+      <c r="H50" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>MR074</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E51" s="9" t="inlineStr">
+        <is>
+          <t>AV128</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>AV128</t>
+        </is>
+      </c>
+      <c r="G51" s="9" t="inlineStr">
+        <is>
+          <t>No subitem e) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
+        </is>
+      </c>
+      <c r="H51" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>MR075</t>
+        </is>
+      </c>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+        </is>
+      </c>
+      <c r="D52" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>AV59 &amp; ~AV134</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="inlineStr">
+        <is>
+          <t>AV59</t>
+        </is>
+      </c>
+      <c r="G52" s="9" t="inlineStr">
+        <is>
+          <t>No subitem a) do item 2203, não houve declaração afirmativa quanto à prática avaliada: mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
+        </is>
+      </c>
+      <c r="H52" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="9" t="inlineStr">
+        <is>
+          <t>MR076</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>Inventário e controle de ativos e configurações de TIC inexistente ou insuficiente.</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="9" t="inlineStr">
+        <is>
+          <t>AV129</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="inlineStr">
+        <is>
+          <t>AV129</t>
+        </is>
+      </c>
+      <c r="G53" s="9" t="inlineStr">
+        <is>
+          <t>No subitem a) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
+        </is>
+      </c>
+      <c r="H53" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="9" t="inlineStr">
+        <is>
+          <t>MR077</t>
+        </is>
+      </c>
+      <c r="B54" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>Inventário e controle de ativos e configurações de TIC inexistente ou insuficiente.</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E54" s="9" t="inlineStr">
+        <is>
+          <t>AV62 &amp; ~AV132</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="inlineStr">
+        <is>
+          <t>AV62</t>
+        </is>
+      </c>
+      <c r="G54" s="9" t="inlineStr">
+        <is>
+          <t>No subitem a) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
+        </is>
+      </c>
+      <c r="H54" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" ht="45" customHeight="1">
+      <c r="A55" s="9" t="inlineStr">
+        <is>
+          <t>MR078</t>
+        </is>
+      </c>
+      <c r="B55" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr">
+        <is>
+          <t>Inventário e controle de ativos e configurações de TIC inexistente ou insuficiente.</t>
+        </is>
+      </c>
+      <c r="D55" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t>AV132</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="inlineStr">
+        <is>
+          <t>AV132</t>
+        </is>
+      </c>
+      <c r="G55" s="9" t="inlineStr">
+        <is>
+          <t>No subitem a) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
+        </is>
+      </c>
+      <c r="H55" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" ht="45" customHeight="1">
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>MR079</t>
+        </is>
+      </c>
+      <c r="B56" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>Inventário e controle de ativos e configurações de TIC inexistente ou insuficiente.</t>
+        </is>
+      </c>
+      <c r="D56" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E56" s="9" t="inlineStr">
+        <is>
+          <t>AV63 &amp; ~AV133</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="inlineStr">
+        <is>
+          <t>AV63</t>
+        </is>
+      </c>
+      <c r="G56" s="9" t="inlineStr">
+        <is>
+          <t>No subitem b) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
+        </is>
+      </c>
+      <c r="H56" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" ht="45" customHeight="1">
+      <c r="A57" s="9" t="inlineStr">
+        <is>
+          <t>MR080</t>
+        </is>
+      </c>
+      <c r="B57" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="inlineStr">
+        <is>
+          <t>Inventário e controle de ativos e configurações de TIC inexistente ou insuficiente.</t>
+        </is>
+      </c>
+      <c r="D57" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E57" s="9" t="inlineStr">
+        <is>
+          <t>AV133</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="inlineStr">
+        <is>
+          <t>AV133</t>
+        </is>
+      </c>
+      <c r="G57" s="9" t="inlineStr">
+        <is>
+          <t>No subitem b) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
+        </is>
+      </c>
+      <c r="H57" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" ht="45" customHeight="1">
+      <c r="A58" s="9" t="inlineStr">
+        <is>
+          <t>MR082</t>
+        </is>
+      </c>
+      <c r="B58" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C58" s="9" t="inlineStr">
+        <is>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+        </is>
+      </c>
+      <c r="D58" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E58" s="9" t="inlineStr">
+        <is>
+          <t>AV134</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="inlineStr">
+        <is>
+          <t>AV134</t>
+        </is>
+      </c>
+      <c r="G58" s="9" t="inlineStr">
+        <is>
+          <t>No subitem a) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
+        </is>
+      </c>
+      <c r="H58" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" ht="45" customHeight="1">
+      <c r="A59" s="9" t="inlineStr">
+        <is>
+          <t>MR083</t>
+        </is>
+      </c>
+      <c r="B59" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+        </is>
+      </c>
+      <c r="D59" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E59" s="9" t="inlineStr">
+        <is>
+          <t>AV66 &amp; ~AV136</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="inlineStr">
+        <is>
+          <t>AV66</t>
+        </is>
+      </c>
+      <c r="G59" s="9" t="inlineStr">
+        <is>
+          <t>No subitem c) do item 2203, não houve declaração afirmativa quanto à prática avaliada: o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+        </is>
+      </c>
+      <c r="H59" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" ht="30" customHeight="1">
+      <c r="A60" s="9" t="inlineStr">
+        <is>
+          <t>MR084</t>
+        </is>
+      </c>
+      <c r="B60" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+        </is>
+      </c>
+      <c r="D60" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E60" s="9" t="inlineStr">
+        <is>
+          <t>AV136</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="inlineStr">
+        <is>
+          <t>AV136</t>
+        </is>
+      </c>
+      <c r="G60" s="9" t="inlineStr">
+        <is>
+          <t>No subitem c) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+        </is>
+      </c>
+      <c r="H60" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" ht="45" customHeight="1">
+      <c r="A61" s="9" t="inlineStr">
+        <is>
+          <t>MR085</t>
+        </is>
+      </c>
+      <c r="B61" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C61" s="9" t="inlineStr">
+        <is>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+        </is>
+      </c>
+      <c r="D61" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" s="9" t="inlineStr">
+        <is>
+          <t>AV67 &amp; ~AV137</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="inlineStr">
+        <is>
+          <t>AV67</t>
+        </is>
+      </c>
+      <c r="G61" s="9" t="inlineStr">
+        <is>
+          <t>No subitem a) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu regras para a priorização e o escalamento de incidentes</t>
+        </is>
+      </c>
+      <c r="H61" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" ht="45" customHeight="1">
+      <c r="A62" s="9" t="inlineStr">
+        <is>
+          <t>MR086</t>
+        </is>
+      </c>
+      <c r="B62" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C62" s="9" t="inlineStr">
+        <is>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+        </is>
+      </c>
+      <c r="D62" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E62" s="9" t="inlineStr">
+        <is>
+          <t>AV137</t>
+        </is>
+      </c>
+      <c r="F62" s="9" t="inlineStr">
+        <is>
+          <t>AV137</t>
+        </is>
+      </c>
+      <c r="G62" s="9" t="inlineStr">
+        <is>
+          <t>No subitem a) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu regras para a priorização e o escalamento de incidentes</t>
+        </is>
+      </c>
+      <c r="H62" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" ht="30" customHeight="1">
+      <c r="A63" s="9" t="inlineStr">
+        <is>
+          <t>MR087</t>
+        </is>
+      </c>
+      <c r="B63" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C63" s="9" t="inlineStr">
+        <is>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+        </is>
+      </c>
+      <c r="D63" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E63" s="9" t="inlineStr">
+        <is>
+          <t>AV70 &amp; ~AV140</t>
+        </is>
+      </c>
+      <c r="F63" s="9" t="inlineStr">
+        <is>
+          <t>AV70</t>
+        </is>
+      </c>
+      <c r="G63" s="9" t="inlineStr">
+        <is>
+          <t>No subitem d) do item 2204, não houve declaração afirmativa quanto à prática avaliada: o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+        </is>
+      </c>
+      <c r="H63" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" ht="45" customHeight="1">
+      <c r="A64" s="9" t="inlineStr">
+        <is>
+          <t>MR088</t>
+        </is>
+      </c>
+      <c r="B64" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C64" s="9" t="inlineStr">
+        <is>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+        </is>
+      </c>
+      <c r="D64" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E64" s="9" t="inlineStr">
+        <is>
+          <t>AV140</t>
+        </is>
+      </c>
+      <c r="F64" s="9" t="inlineStr">
+        <is>
+          <t>AV140</t>
+        </is>
+      </c>
+      <c r="G64" s="9" t="inlineStr">
+        <is>
+          <t>No subitem d) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+        </is>
+      </c>
+      <c r="H64" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" ht="30" customHeight="1">
+      <c r="A65" s="9" t="inlineStr">
+        <is>
+          <t>MR089</t>
+        </is>
+      </c>
+      <c r="B65" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C65" s="9" t="inlineStr">
+        <is>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+        </is>
+      </c>
+      <c r="D65" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E65" s="9" t="inlineStr">
+        <is>
+          <t>AV71 &amp; ~AV141</t>
+        </is>
+      </c>
+      <c r="F65" s="9" t="inlineStr">
+        <is>
+          <t>AV71</t>
+        </is>
+      </c>
+      <c r="G65" s="9" t="inlineStr">
+        <is>
+          <t>No subitem e) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
+        </is>
+      </c>
+      <c r="H65" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" ht="30" customHeight="1">
+      <c r="A66" s="9" t="inlineStr">
+        <is>
+          <t>MR090</t>
+        </is>
+      </c>
+      <c r="B66" s="9" t="inlineStr">
+        <is>
+          <t>PA05</t>
+        </is>
+      </c>
+      <c r="C66" s="9" t="inlineStr">
+        <is>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+        </is>
+      </c>
+      <c r="D66" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E66" s="9" t="inlineStr">
+        <is>
+          <t>AV141</t>
+        </is>
+      </c>
+      <c r="F66" s="9" t="inlineStr">
+        <is>
+          <t>AV141</t>
+        </is>
+      </c>
+      <c r="G66" s="9" t="inlineStr">
+        <is>
+          <t>No subitem e) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
+        </is>
+      </c>
+      <c r="H66" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" ht="30" customHeight="1">
+      <c r="A67" s="9" t="inlineStr">
+        <is>
+          <t>MR091</t>
+        </is>
+      </c>
+      <c r="B67" s="9" t="inlineStr">
+        <is>
+          <t>PA06</t>
+        </is>
+      </c>
+      <c r="C67" s="9" t="inlineStr">
+        <is>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+        </is>
+      </c>
+      <c r="D67" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" s="9" t="inlineStr">
+        <is>
+          <t>AV73 &amp; ~AV143</t>
+        </is>
+      </c>
+      <c r="F67" s="9" t="inlineStr">
+        <is>
+          <t>AV73</t>
+        </is>
+      </c>
+      <c r="G67" s="9" t="inlineStr">
+        <is>
+          <t>No subitem a) do item 2801, não houve declaração afirmativa quanto à prática avaliada: o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
+        </is>
+      </c>
+      <c r="H67" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" ht="45" customHeight="1">
+      <c r="A68" s="9" t="inlineStr">
+        <is>
+          <t>MR092</t>
+        </is>
+      </c>
+      <c r="B68" s="9" t="inlineStr">
+        <is>
+          <t>PA06</t>
+        </is>
+      </c>
+      <c r="C68" s="9" t="inlineStr">
+        <is>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+        </is>
+      </c>
+      <c r="D68" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E68" s="9" t="inlineStr">
+        <is>
+          <t>AV143</t>
+        </is>
+      </c>
+      <c r="F68" s="9" t="inlineStr">
+        <is>
+          <t>AV143</t>
+        </is>
+      </c>
+      <c r="G68" s="9" t="inlineStr">
+        <is>
+          <t>No subitem a) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
+        </is>
+      </c>
+      <c r="H68" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" ht="60" customHeight="1">
+      <c r="A69" s="9" t="inlineStr">
+        <is>
+          <t>MR101</t>
+        </is>
+      </c>
+      <c r="B69" s="9" t="inlineStr">
+        <is>
+          <t>PA06</t>
+        </is>
+      </c>
+      <c r="C69" s="9" t="inlineStr">
+        <is>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
+        </is>
+      </c>
+      <c r="D69" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E69" s="9" t="inlineStr">
+        <is>
+          <t>AV78 &amp; ~AV148</t>
+        </is>
+      </c>
+      <c r="F69" s="9" t="inlineStr">
+        <is>
+          <t>AV78</t>
+        </is>
+      </c>
+      <c r="G69" s="9" t="inlineStr">
+        <is>
+          <t>No subitem a) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
+        </is>
+      </c>
+      <c r="H69" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" ht="45" customHeight="1">
+      <c r="A70" s="9" t="inlineStr">
+        <is>
+          <t>MR102</t>
+        </is>
+      </c>
+      <c r="B70" s="9" t="inlineStr">
+        <is>
+          <t>PA06</t>
+        </is>
+      </c>
+      <c r="C70" s="9" t="inlineStr">
+        <is>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
+        </is>
+      </c>
+      <c r="D70" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E70" s="9" t="inlineStr">
+        <is>
+          <t>AV148</t>
+        </is>
+      </c>
+      <c r="F70" s="9" t="inlineStr">
+        <is>
+          <t>AV148</t>
+        </is>
+      </c>
+      <c r="G70" s="9" t="inlineStr">
+        <is>
+          <t>No subitem a) do item 2804, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
+        </is>
+      </c>
+      <c r="H70" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" ht="45" customHeight="1">
+      <c r="A71" s="9" t="inlineStr">
+        <is>
+          <t>MR109</t>
+        </is>
+      </c>
+      <c r="B71" s="9" t="inlineStr">
+        <is>
+          <t>PA06</t>
+        </is>
+      </c>
+      <c r="C71" s="9" t="inlineStr">
+        <is>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
+        </is>
+      </c>
+      <c r="D71" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E71" s="9" t="inlineStr">
+        <is>
+          <t>AV82</t>
+        </is>
+      </c>
+      <c r="F71" s="9" t="inlineStr">
+        <is>
+          <t>AV82</t>
+        </is>
+      </c>
+      <c r="G71" s="9" t="inlineStr">
+        <is>
+          <t>No subitem b) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de TI executadas no exercício encontram-se previamente estabelecidas nos instrumentos de planejamento vigentes (PDTI/PEDTIC e PCA)</t>
+        </is>
+      </c>
+      <c r="H71" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" ht="30" customHeight="1">
+      <c r="A72" s="9" t="inlineStr">
+        <is>
+          <t>MR110</t>
+        </is>
+      </c>
+      <c r="B72" s="9" t="inlineStr">
+        <is>
+          <t>PA06</t>
+        </is>
+      </c>
+      <c r="C72" s="9" t="inlineStr">
+        <is>
+          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
+        </is>
+      </c>
+      <c r="D72" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E72" s="9" t="inlineStr">
+        <is>
+          <t>AV83</t>
+        </is>
+      </c>
+      <c r="F72" s="9" t="inlineStr">
+        <is>
+          <t>AV83</t>
+        </is>
+      </c>
+      <c r="G72" s="9" t="inlineStr">
+        <is>
+          <t>No subitem c) do item 2804, não houve declaração afirmativa quanto à prática avaliada: a fase de planejamento de cada contratação de TI é conduzida por uma Equipe de Planejamento da Contratação formalmente designada (composta, minimamente, por integrante requisitante e integrante técnico da área de TI)</t>
+        </is>
+      </c>
+      <c r="H72" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" ht="30" customHeight="1">
+      <c r="A73" s="9" t="inlineStr">
+        <is>
+          <t>MR111</t>
+        </is>
+      </c>
+      <c r="B73" s="9" t="inlineStr">
+        <is>
+          <t>PA06</t>
+        </is>
+      </c>
+      <c r="C73" s="9" t="inlineStr">
+        <is>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+        </is>
+      </c>
+      <c r="D73" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E73" s="9" t="inlineStr">
+        <is>
+          <t>AV152 &amp; ~AV153</t>
+        </is>
+      </c>
+      <c r="F73" s="9" t="inlineStr">
+        <is>
+          <t>AV152</t>
+        </is>
+      </c>
+      <c r="G73" s="9" t="inlineStr">
+        <is>
+          <t>No subitem b) do item 2801, não houve declaração afirmativa quanto à prática avaliada: são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
+        </is>
+      </c>
+      <c r="H73" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" ht="30" customHeight="1">
+      <c r="A74" s="9" t="inlineStr">
+        <is>
+          <t>MR113</t>
+        </is>
+      </c>
+      <c r="B74" s="9" t="inlineStr">
+        <is>
+          <t>PA03</t>
+        </is>
+      </c>
+      <c r="C74" s="9" t="inlineStr">
+        <is>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
+        </is>
+      </c>
+      <c r="D74" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E74" s="9" t="inlineStr">
+        <is>
           <t>AV154</t>
         </is>
       </c>
-      <c r="F45" s="9" t="inlineStr">
+      <c r="F74" s="9" t="inlineStr">
         <is>
           <t>AV154</t>
         </is>
       </c>
-      <c r="G45" s="9" t="inlineStr">
+      <c r="G74" s="9" t="inlineStr">
         <is>
           <t>No item 2102, a organização não declarou possuir plano de tecnologia da informação vigente, ainda que parcialmente adotado</t>
         </is>
       </c>
-      <c r="H45" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" ht="30" customHeight="1"/>
-    <row r="47" ht="30" customHeight="1"/>
-    <row r="48" ht="30" customHeight="1"/>
-    <row r="49" ht="45" customHeight="1"/>
-    <row r="50" ht="30" customHeight="1"/>
-    <row r="51" ht="30" customHeight="1"/>
-    <row r="52" ht="30" customHeight="1"/>
-    <row r="53" ht="30" customHeight="1"/>
-    <row r="54" ht="30" customHeight="1"/>
-    <row r="55" ht="45" customHeight="1"/>
-    <row r="56" ht="45" customHeight="1"/>
-    <row r="57" ht="45" customHeight="1"/>
-    <row r="58" ht="45" customHeight="1"/>
-    <row r="59" ht="45" customHeight="1"/>
-    <row r="60" ht="30" customHeight="1"/>
-    <row r="61" ht="45" customHeight="1"/>
-    <row r="62" ht="45" customHeight="1"/>
-    <row r="63" ht="30" customHeight="1"/>
-    <row r="64" ht="45" customHeight="1"/>
-    <row r="65" ht="30" customHeight="1"/>
-    <row r="66" ht="30" customHeight="1"/>
-    <row r="67" ht="30" customHeight="1"/>
-    <row r="68" ht="45" customHeight="1"/>
-    <row r="69" ht="60" customHeight="1"/>
-    <row r="70" ht="45" customHeight="1"/>
-    <row r="71" ht="45" customHeight="1"/>
-    <row r="72" ht="30" customHeight="1"/>
-    <row r="73" ht="30" customHeight="1"/>
-    <row r="74" ht="30" customHeight="1"/>
+      <c r="H74" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
     <row r="75" ht="45" customHeight="1"/>
     <row r="76" ht="30" customHeight="1"/>
     <row r="77" ht="45" customHeight="1"/>
@@ -5202,7 +7910,7 @@
     <row r="112" ht="45" customHeight="1"/>
     <row r="113" ht="45" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A3:H45"/>
+  <autoFilter ref="A3:H74"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Aprimora matriz e mapa pós-comentários
</commit_message>
<xml_diff>
--- a/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
+++ b/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
@@ -649,7 +649,7 @@
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>(((AV55 | AV125) | (AV56 | AV126)) | ((AV54 | AV124) | (AV57 | AV127) | (AV58 | AV128)) | (AV129 | (AV62 | AV132) | (AV63 | AV133)) | ((AV59 | AV134) | (AV66 | AV136)) | ((AV67 | AV137) | (AV70 | AV140) | (AV71 | AV141)))</t>
+          <t>(((AV55 | AV125) | (AV56 | AV126)) | ((AV54 | AV124) | (AV57 | AV127) | (AV58 | AV128)) | ((AV62 | AV132) | (AV63 | AV133)) | ((AV59 | AV134) | (AV66 | AV136)) | ((AV67 | AV137) | (AV70 | AV140) | (AV71 | AV141)))</t>
         </is>
       </c>
       <c r="D8" s="1" t="n">
@@ -699,7 +699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P77"/>
+  <dimension ref="A1:P76"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1143,7 +1143,7 @@
       </c>
       <c r="K8" s="1" t="inlineStr">
         <is>
-          <t>~(f) Inexistente / Informal: Não há área de TI formalmente instituída no organograma da organização.)</t>
+          <t>(a) Centralizada Interna: Há uma área de TI centralizada e formal que atende toda a organização, utilizando equipe técnica majoritariamente própria (servidores). | b) Centralizada Terceirizada: Há uma área de TI centralizada e formal que faz a gestão, mas a execução operacional/técnica é predominantemente terceirizada (ex: fábricas de software, service desk). | e) Híbrida: Existe uma TI central formal para diretrizes e infraestrutura corporativa, mas as áreas de negócio possuem equipes próprias para sustentar sistemas específicos.)</t>
         </is>
       </c>
       <c r="L8" s="1" t="n"/>
@@ -2576,7 +2576,7 @@
       <c r="I34" s="1" t="n"/>
       <c r="J34" s="1" t="inlineStr">
         <is>
-          <t>Inventário e controle de ativos e configurações de TIC inexistente ou insuficiente.</t>
+          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
         </is>
       </c>
       <c r="K34" s="1" t="inlineStr">
@@ -2594,7 +2594,7 @@
       <c r="O34" s="1" t="n"/>
       <c r="P34" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos e base consolidada das configurações relevantes, contemplando, minimamente, dispositivos, softwares e seus relacionamentos, com informações suficientes para identificação e controle</t>
+          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos sob gestão da organização, contemplando, minimamente, os dispositivos e softwares utilizados, com informações suficientes para sua identificação e controle</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2631,7 @@
       <c r="I35" s="1" t="n"/>
       <c r="J35" s="1" t="inlineStr">
         <is>
-          <t>Inventário e controle de ativos e configurações de TIC inexistente ou insuficiente.</t>
+          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
         </is>
       </c>
       <c r="K35" s="1" t="inlineStr">
@@ -2649,7 +2649,7 @@
       <c r="O35" s="1" t="n"/>
       <c r="P35" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos e base consolidada das configurações relevantes, contemplando, minimamente, dispositivos, softwares e seus relacionamentos, com informações suficientes para identificação e controle</t>
+          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos sob gestão da organização, contemplando, minimamente, os dispositivos e softwares utilizados, com informações suficientes para sua identificação e controle</t>
         </is>
       </c>
     </row>
@@ -2956,7 +2956,7 @@
         <is>
           <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
 COBIT 2019, BAI02.04 - Obter aprovação dos requisitos da solução: obter aprovação formal dos requisitos funcionais, técnicos, de segurança e de conformidade antes de prosseguir com a solução.
-Instrução Normativa SGD/ME nº 94/2022, arts. 1º, §1º, 10, II, 11, §2º, e 12, §6º – referência de boa prática para estruturação da fase de planejamento das contratações de TIC, participação da área técnica e instituição da Equipe de Planejamento, observada sua aplicação direta aos integrantes do SISP e a possibilidade de procedimentos simplificados.</t>
+Instrução Normativa SGD/ME nº 94/2022, arts. 2º, IV, 9º, 10, 11 e 12, §6º – referência de boa prática para estruturação da fase de planejamento das contratações de TIC, instituição da Equipe de Planejamento da Contratação e participação do integrante técnico da área de TIC, observada sua aplicação direta aos integrantes do SISP e as hipóteses de simplificação de procedimentos previstas na norma.</t>
         </is>
       </c>
       <c r="H41" s="1" t="inlineStr">
@@ -3068,7 +3068,7 @@
         <is>
           <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
 Lei nº 14.133/2021, art. 7º, caput, incisos I a III e §1º: designação de agentes públicos para funções essenciais, observados atribuições, formação, segregação de funções e inexistência de vínculos que comprometam a atuação.
-Instrução Normativa SGD/ME nº 94/2022, arts. 1º, §1º, 10, II, 11, §2º, e 12, §6º – referência de boa prática para estruturação da fase de planejamento das contratações de TIC, participação da área técnica e instituição da Equipe de Planejamento, observada sua aplicação direta aos integrantes do SISP e a possibilidade de procedimentos simplificados.</t>
+Instrução Normativa SGD/ME nº 94/2022, arts. 2º, IV, 9º, 10, 11 e 12, §6º – referência de boa prática para estruturação da fase de planejamento das contratações de TIC, instituição da Equipe de Planejamento da Contratação e participação do integrante técnico da área de TIC, observada sua aplicação direta aos integrantes do SISP e as hipóteses de simplificação de procedimentos previstas na norma.</t>
         </is>
       </c>
       <c r="H43" s="1" t="inlineStr">
@@ -4211,7 +4211,7 @@
     <row r="64" ht="90.95" customHeight="1">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>AV129</t>
+          <t>AV132</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -4224,7 +4224,7 @@
       <c r="E64" s="1" t="n"/>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>q2203ext[A]</t>
+          <t>q2504ext[A]</t>
         </is>
       </c>
       <c r="G64" s="1" t="inlineStr">
@@ -4241,7 +4241,7 @@
       <c r="I64" s="1" t="n"/>
       <c r="J64" s="1" t="inlineStr">
         <is>
-          <t>Inventário e controle de ativos e configurações de TIC inexistente ou insuficiente.</t>
+          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
         </is>
       </c>
       <c r="K64" s="1" t="inlineStr">
@@ -4259,14 +4259,14 @@
       <c r="O64" s="1" t="n"/>
       <c r="P64" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos e base consolidada das configurações relevantes, contemplando, minimamente, dispositivos, softwares e seus relacionamentos, com informações suficientes para identificação e controle</t>
+          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos sob gestão da organização, contemplando, minimamente, os dispositivos e softwares utilizados, com informações suficientes para sua identificação e controle</t>
         </is>
       </c>
     </row>
     <row r="65" ht="90.95" customHeight="1">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>AV132</t>
+          <t>AV133</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -4279,7 +4279,7 @@
       <c r="E65" s="1" t="n"/>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>q2504ext[A]</t>
+          <t>q2504ext[B]</t>
         </is>
       </c>
       <c r="G65" s="1" t="inlineStr">
@@ -4296,7 +4296,7 @@
       <c r="I65" s="1" t="n"/>
       <c r="J65" s="1" t="inlineStr">
         <is>
-          <t>Inventário e controle de ativos e configurações de TIC inexistente ou insuficiente.</t>
+          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
         </is>
       </c>
       <c r="K65" s="1" t="inlineStr">
@@ -4314,14 +4314,14 @@
       <c r="O65" s="1" t="n"/>
       <c r="P65" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos e base consolidada das configurações relevantes, contemplando, minimamente, dispositivos, softwares e seus relacionamentos, com informações suficientes para identificação e controle</t>
+          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos sob gestão da organização, contemplando, minimamente, os dispositivos e softwares utilizados, com informações suficientes para sua identificação e controle</t>
         </is>
       </c>
     </row>
     <row r="66" ht="90.95" customHeight="1">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>AV133</t>
+          <t>AV134</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -4334,13 +4334,14 @@
       <c r="E66" s="1" t="n"/>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>q2504ext[B]</t>
+          <t>q2203ext[A]</t>
         </is>
       </c>
       <c r="G66" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.</t>
+          <t>COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.2.6 – Gerenciamento de configuração: orienta a identificação, o registro, o controle, o rastreamento e a verificação dos itens de configuração, bem como a manutenção de informações de configuração precisas relacionadas aos serviços.</t>
         </is>
       </c>
       <c r="H66" s="1" t="inlineStr">
@@ -4351,7 +4352,7 @@
       <c r="I66" s="1" t="n"/>
       <c r="J66" s="1" t="inlineStr">
         <is>
-          <t>Inventário e controle de ativos e configurações de TIC inexistente ou insuficiente.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="K66" s="1" t="inlineStr">
@@ -4369,14 +4370,14 @@
       <c r="O66" s="1" t="n"/>
       <c r="P66" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos e base consolidada das configurações relevantes, contemplando, minimamente, dispositivos, softwares e seus relacionamentos, com informações suficientes para identificação e controle</t>
+          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
         </is>
       </c>
     </row>
     <row r="67" ht="79.90000000000001" customHeight="1">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>AV134</t>
+          <t>AV136</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -4389,7 +4390,7 @@
       <c r="E67" s="1" t="n"/>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>q2203ext[A]</t>
+          <t>q2203ext[C]</t>
         </is>
       </c>
       <c r="G67" s="1" t="inlineStr">
@@ -4432,7 +4433,7 @@
     <row r="68" ht="79.90000000000001" customHeight="1">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>AV136</t>
+          <t>AV137</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -4445,14 +4446,14 @@
       <c r="E68" s="1" t="n"/>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>q2203ext[C]</t>
+          <t>q2204ext[A]</t>
         </is>
       </c>
       <c r="G68" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.
-ABNT NBR ISO/IEC 20000-2:2021, item 8.2.6 – Gerenciamento de configuração: orienta a identificação, o registro, o controle, o rastreamento e a verificação dos itens de configuração, bem como a manutenção de informações de configuração precisas relacionadas aos serviços.</t>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.6, III.9.6 e V.6.3 – Recomendações quanto à formalização e execução do processo de gestão de incidentes, incluindo registros, classificação, escalamento e tratamento.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.6.1 – Gerenciamento de incidente: orienta que os incidentes sejam registrados, classificados e priorizados, que as ações adotadas para sua resolução sejam registradas e rastreáveis e que sejam definidas responsabilidades para seu tratamento, incluindo procedimento documentado para incidentes graves.</t>
         </is>
       </c>
       <c r="H68" s="1" t="inlineStr">
@@ -4463,7 +4464,7 @@
       <c r="I68" s="1" t="n"/>
       <c r="J68" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="K68" s="1" t="inlineStr">
@@ -4481,14 +4482,14 @@
       <c r="O68" s="1" t="n"/>
       <c r="P68" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
     </row>
     <row r="69" ht="79.90000000000001" customHeight="1">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>AV137</t>
+          <t>AV140</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -4501,7 +4502,7 @@
       <c r="E69" s="1" t="n"/>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>q2204ext[A]</t>
+          <t>q2204ext[D]</t>
         </is>
       </c>
       <c r="G69" s="1" t="inlineStr">
@@ -4544,7 +4545,7 @@
     <row r="70" ht="90.95" customHeight="1">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>AV140</t>
+          <t>AV141</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -4557,7 +4558,7 @@
       <c r="E70" s="1" t="n"/>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>q2204ext[D]</t>
+          <t>q2204ext[E]</t>
         </is>
       </c>
       <c r="G70" s="1" t="inlineStr">
@@ -4600,7 +4601,7 @@
     <row r="71" ht="90.95" customHeight="1">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>AV141</t>
+          <t>AV143</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -4613,14 +4614,14 @@
       <c r="E71" s="1" t="n"/>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>q2204ext[E]</t>
+          <t>q2801ext[A]</t>
         </is>
       </c>
       <c r="G71" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.6, III.9.6 e V.6.3 – Recomendações quanto à formalização e execução do processo de gestão de incidentes, incluindo registros, classificação, escalamento e tratamento.
-ABNT NBR ISO/IEC 20000-2:2021, item 8.6.1 – Gerenciamento de incidente: orienta que os incidentes sejam registrados, classificados e priorizados, que as ações adotadas para sua resolução sejam registradas e rastreáveis e que sejam definidas responsabilidades para seu tratamento, incluindo procedimento documentado para incidentes graves.</t>
+          <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Lei nº 14.133/2021, art. 19, inciso IV: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.
+Acórdão nº 2.342/2016-TCU-Plenário, item 9.1.7 – Precedente quanto à definição, aprovação e formalização de processo de trabalho para o planejamento de cada contratação, com controles internos mínimos.</t>
         </is>
       </c>
       <c r="H71" s="1" t="inlineStr">
@@ -4631,7 +4632,7 @@
       <c r="I71" s="1" t="n"/>
       <c r="J71" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="K71" s="1" t="inlineStr">
@@ -4649,14 +4650,14 @@
       <c r="O71" s="1" t="n"/>
       <c r="P71" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
+          <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
         </is>
       </c>
     </row>
     <row r="72" ht="90.95" customHeight="1">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>AV143</t>
+          <t>AV148</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -4669,14 +4670,14 @@
       <c r="E72" s="1" t="n"/>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>q2801ext[A]</t>
+          <t>q2804[A]</t>
         </is>
       </c>
       <c r="G72" s="1" t="inlineStr">
         <is>
           <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Lei nº 14.133/2021, art. 19, inciso IV: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.
-Acórdão nº 2.342/2016-TCU-Plenário, item 9.1.7 – Precedente quanto à definição, aprovação e formalização de processo de trabalho para o planejamento de cada contratação, com controles internos mínimos.</t>
+COBIT 2019, BAI02.04 - Obter aprovação dos requisitos da solução: obter aprovação formal dos requisitos funcionais, técnicos, de segurança e de conformidade antes de prosseguir com a solução.
+Instrução Normativa SGD/ME nº 94/2022, arts. 2º, IV, 9º, 10, 11 e 12, §6º – referência de boa prática para estruturação da fase de planejamento das contratações de TIC, instituição da Equipe de Planejamento da Contratação e participação do integrante técnico da área de TIC, observada sua aplicação direta aos integrantes do SISP e as hipóteses de simplificação de procedimentos previstas na norma.</t>
         </is>
       </c>
       <c r="H72" s="1" t="inlineStr">
@@ -4687,7 +4688,7 @@
       <c r="I72" s="1" t="n"/>
       <c r="J72" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
         </is>
       </c>
       <c r="K72" s="1" t="inlineStr">
@@ -4705,19 +4706,19 @@
       <c r="O72" s="1" t="n"/>
       <c r="P72" s="1" t="inlineStr">
         <is>
-          <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
+          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo procedimentos simplificados e proporcionais à natureza, ao risco e ao valor da contratação, preservada análise técnica compatível</t>
         </is>
       </c>
     </row>
     <row r="73" ht="90.95" customHeight="1">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>AV148</t>
+          <t>AV152</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
         <is>
-          <t>avaliacao_evidencias_ajustes</t>
+          <t>questionario</t>
         </is>
       </c>
       <c r="C73" s="1" t="n"/>
@@ -4725,30 +4726,30 @@
       <c r="E73" s="1" t="n"/>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>q2804[A]</t>
+          <t>q2801ext[B]</t>
         </is>
       </c>
       <c r="G73" s="1" t="inlineStr">
         <is>
           <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-COBIT 2019, BAI02.04 - Obter aprovação dos requisitos da solução: obter aprovação formal dos requisitos funcionais, técnicos, de segurança e de conformidade antes de prosseguir com a solução.
-Instrução Normativa SGD/ME nº 94/2022, arts. 1º, §1º, 10, II, 11, §2º, e 12, §6º – referência de boa prática para estruturação da fase de planejamento das contratações de TIC, participação da área técnica e instituição da Equipe de Planejamento, observada sua aplicação direta aos integrantes do SISP e a possibilidade de procedimentos simplificados.</t>
+Lei nº 14.133/2021, art. 19, inciso IV: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.
+Acórdão nº 2.342/2016-TCU-Plenário, item 9.1.7 – Precedente quanto à definição, aprovação e formalização de processo de trabalho para o planejamento de cada contratação, com controles internos mínimos.</t>
         </is>
       </c>
       <c r="H73" s="1" t="inlineStr">
         <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+          <t>Resposta negativa ao detalhamento b) do item 2801 do Questionário, para verificar se são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
         </is>
       </c>
       <c r="I73" s="1" t="n"/>
       <c r="J73" s="1" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="K73" s="1" t="inlineStr">
         <is>
-          <t>Não conforme</t>
+          <t>(Não | N/A)</t>
         </is>
       </c>
       <c r="L73" s="1" t="n"/>
@@ -4761,19 +4762,19 @@
       <c r="O73" s="1" t="n"/>
       <c r="P73" s="1" t="inlineStr">
         <is>
-          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo procedimentos simplificados e proporcionais à natureza, ao risco e ao valor da contratação, preservada análise técnica compatível</t>
+          <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
         </is>
       </c>
     </row>
     <row r="74" ht="90.95" customHeight="1">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>AV152</t>
+          <t>AV153</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
         <is>
-          <t>questionario</t>
+          <t>avaliacao_evidencias_ajustes</t>
         </is>
       </c>
       <c r="C74" s="1" t="n"/>
@@ -4793,7 +4794,7 @@
       </c>
       <c r="H74" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento b) do item 2801 do Questionário, para verificar se são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
         </is>
       </c>
       <c r="I74" s="1" t="n"/>
@@ -4804,7 +4805,7 @@
       </c>
       <c r="K74" s="1" t="inlineStr">
         <is>
-          <t>(Não | N/A)</t>
+          <t>Não conforme</t>
         </is>
       </c>
       <c r="L74" s="1" t="n"/>
@@ -4824,12 +4825,12 @@
     <row r="75" ht="90.95" customHeight="1">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>AV153</t>
+          <t>AV154</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
         <is>
-          <t>avaliacao_evidencias_ajustes</t>
+          <t>questionario</t>
         </is>
       </c>
       <c r="C75" s="1" t="n"/>
@@ -4837,50 +4838,50 @@
       <c r="E75" s="1" t="n"/>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>q2801ext[B]</t>
+          <t>existe_plano_ti</t>
         </is>
       </c>
       <c r="G75" s="1" t="inlineStr">
         <is>
-          <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Lei nº 14.133/2021, art. 19, inciso IV: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.
-Acórdão nº 2.342/2016-TCU-Plenário, item 9.1.7 – Precedente quanto à definição, aprovação e formalização de processo de trabalho para o planejamento de cada contratação, com controles internos mínimos.</t>
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H75" s="1" t="inlineStr">
         <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+          <t>Resposta ao item 2102 que não caracteriza a existência de plano de TIC vigente, ainda que parcialmente adotado</t>
         </is>
       </c>
       <c r="I75" s="1" t="n"/>
       <c r="J75" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="K75" s="1" t="inlineStr">
         <is>
-          <t>Não conforme</t>
+          <t>False</t>
         </is>
       </c>
       <c r="L75" s="1" t="n"/>
       <c r="M75" s="1" t="n"/>
       <c r="N75" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O75" s="1" t="n"/>
       <c r="P75" s="1" t="inlineStr">
         <is>
-          <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
     <row r="76" ht="102.2" customHeight="1">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>AV154</t>
+          <t>AV155</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -4905,18 +4906,14 @@
       </c>
       <c r="H76" s="1" t="inlineStr">
         <is>
-          <t>Resposta ao item 2102 que não caracteriza a existência de plano de TIC vigente, ainda que parcialmente adotado</t>
+          <t>Plano de TIC vigente declarado no item 2102, ao menos parcialmente adotado</t>
         </is>
       </c>
       <c r="I76" s="1" t="n"/>
-      <c r="J76" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
-        </is>
-      </c>
+      <c r="J76" s="1" t="n"/>
       <c r="K76" s="1" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="L76" s="1" t="n"/>
@@ -4933,58 +4930,7 @@
         </is>
       </c>
     </row>
-    <row r="77" ht="102.2" customHeight="1">
-      <c r="A77" s="1" t="inlineStr">
-        <is>
-          <t>AV155</t>
-        </is>
-      </c>
-      <c r="B77" s="1" t="inlineStr">
-        <is>
-          <t>questionario</t>
-        </is>
-      </c>
-      <c r="C77" s="1" t="n"/>
-      <c r="D77" s="1" t="n"/>
-      <c r="E77" s="1" t="n"/>
-      <c r="F77" s="1" t="inlineStr">
-        <is>
-          <t>existe_plano_ti</t>
-        </is>
-      </c>
-      <c r="G77" s="1" t="inlineStr">
-        <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
-        </is>
-      </c>
-      <c r="H77" s="1" t="inlineStr">
-        <is>
-          <t>Plano de TIC vigente declarado no item 2102, ao menos parcialmente adotado</t>
-        </is>
-      </c>
-      <c r="I77" s="1" t="n"/>
-      <c r="J77" s="1" t="n"/>
-      <c r="K77" s="1" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="L77" s="1" t="n"/>
-      <c r="M77" s="1" t="n"/>
-      <c r="N77" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O77" s="1" t="n"/>
-      <c r="P77" s="1" t="inlineStr">
-        <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
-        </is>
-      </c>
-    </row>
+    <row r="77" ht="102.2" customHeight="1"/>
     <row r="78" ht="102.2" customHeight="1"/>
     <row r="79" ht="102.2" customHeight="1"/>
     <row r="80" ht="102.2" customHeight="1"/>
@@ -5075,7 +5021,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H74"/>
+  <dimension ref="A2:H73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5393,7 +5339,7 @@
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>Item 0101: a organização informou possuir área ou modelo de operação de TI, o que levou à análise do seu posicionamento organizacional</t>
+          <t>Item 0101: a organização informou modelo de operação com área de TI formal interna, predominantemente terceirizada ou híbrida, o que levou à análise do seu posicionamento organizacional</t>
         </is>
       </c>
       <c r="H9" s="9" t="b">
@@ -7037,7 +6983,7 @@
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>MR076</t>
+          <t>MR077</t>
         </is>
       </c>
       <c r="B53" s="9" t="inlineStr">
@@ -7047,7 +6993,7 @@
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>Inventário e controle de ativos e configurações de TIC inexistente ou insuficiente.</t>
+          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
         </is>
       </c>
       <c r="D53" s="9" t="n">
@@ -7055,17 +7001,17 @@
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>AV129</t>
+          <t>AV62 &amp; ~AV132</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>AV129</t>
+          <t>AV62</t>
         </is>
       </c>
       <c r="G53" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
+          <t>No subitem a) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H53" s="9" t="b">
@@ -7075,7 +7021,7 @@
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t>MR077</t>
+          <t>MR078</t>
         </is>
       </c>
       <c r="B54" s="9" t="inlineStr">
@@ -7085,7 +7031,7 @@
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>Inventário e controle de ativos e configurações de TIC inexistente ou insuficiente.</t>
+          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
         </is>
       </c>
       <c r="D54" s="9" t="n">
@@ -7093,17 +7039,17 @@
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>AV62 &amp; ~AV132</t>
+          <t>AV132</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>AV62</t>
+          <t>AV132</t>
         </is>
       </c>
       <c r="G54" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
+          <t>No subitem a) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H54" s="9" t="b">
@@ -7113,7 +7059,7 @@
     <row r="55" ht="45" customHeight="1">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>MR078</t>
+          <t>MR079</t>
         </is>
       </c>
       <c r="B55" s="9" t="inlineStr">
@@ -7123,7 +7069,7 @@
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>Inventário e controle de ativos e configurações de TIC inexistente ou insuficiente.</t>
+          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
         </is>
       </c>
       <c r="D55" s="9" t="n">
@@ -7131,17 +7077,17 @@
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>AV132</t>
+          <t>AV63 &amp; ~AV133</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>AV132</t>
+          <t>AV63</t>
         </is>
       </c>
       <c r="G55" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
+          <t>No subitem b) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H55" s="9" t="b">
@@ -7151,7 +7097,7 @@
     <row r="56" ht="45" customHeight="1">
       <c r="A56" s="9" t="inlineStr">
         <is>
-          <t>MR079</t>
+          <t>MR080</t>
         </is>
       </c>
       <c r="B56" s="9" t="inlineStr">
@@ -7161,7 +7107,7 @@
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>Inventário e controle de ativos e configurações de TIC inexistente ou insuficiente.</t>
+          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
         </is>
       </c>
       <c r="D56" s="9" t="n">
@@ -7169,17 +7115,17 @@
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>AV63 &amp; ~AV133</t>
+          <t>AV133</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>AV63</t>
+          <t>AV133</t>
         </is>
       </c>
       <c r="G56" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
+          <t>No subitem b) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H56" s="9" t="b">
@@ -7189,7 +7135,7 @@
     <row r="57" ht="45" customHeight="1">
       <c r="A57" s="9" t="inlineStr">
         <is>
-          <t>MR080</t>
+          <t>MR082</t>
         </is>
       </c>
       <c r="B57" s="9" t="inlineStr">
@@ -7199,25 +7145,25 @@
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>Inventário e controle de ativos e configurações de TIC inexistente ou insuficiente.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="D57" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>AV133</t>
+          <t>AV134</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>AV133</t>
+          <t>AV134</t>
         </is>
       </c>
       <c r="G57" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
+          <t>No subitem a) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
         </is>
       </c>
       <c r="H57" s="9" t="b">
@@ -7227,7 +7173,7 @@
     <row r="58" ht="45" customHeight="1">
       <c r="A58" s="9" t="inlineStr">
         <is>
-          <t>MR082</t>
+          <t>MR083</t>
         </is>
       </c>
       <c r="B58" s="9" t="inlineStr">
@@ -7241,21 +7187,21 @@
         </is>
       </c>
       <c r="D58" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>AV134</t>
+          <t>AV66 &amp; ~AV136</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>AV134</t>
+          <t>AV66</t>
         </is>
       </c>
       <c r="G58" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
+          <t>No subitem c) do item 2203, não houve declaração afirmativa quanto à prática avaliada: o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H58" s="9" t="b">
@@ -7265,7 +7211,7 @@
     <row r="59" ht="45" customHeight="1">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>MR083</t>
+          <t>MR084</t>
         </is>
       </c>
       <c r="B59" s="9" t="inlineStr">
@@ -7279,21 +7225,21 @@
         </is>
       </c>
       <c r="D59" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>AV66 &amp; ~AV136</t>
+          <t>AV136</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>AV66</t>
+          <t>AV136</t>
         </is>
       </c>
       <c r="G59" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2203, não houve declaração afirmativa quanto à prática avaliada: o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem c) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H59" s="9" t="b">
@@ -7303,7 +7249,7 @@
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="9" t="inlineStr">
         <is>
-          <t>MR084</t>
+          <t>MR085</t>
         </is>
       </c>
       <c r="B60" s="9" t="inlineStr">
@@ -7313,25 +7259,25 @@
       </c>
       <c r="C60" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="D60" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>AV136</t>
+          <t>AV67 &amp; ~AV137</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>AV136</t>
+          <t>AV67</t>
         </is>
       </c>
       <c r="G60" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem a) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu regras para a priorização e o escalamento de incidentes</t>
         </is>
       </c>
       <c r="H60" s="9" t="b">
@@ -7341,7 +7287,7 @@
     <row r="61" ht="45" customHeight="1">
       <c r="A61" s="9" t="inlineStr">
         <is>
-          <t>MR085</t>
+          <t>MR086</t>
         </is>
       </c>
       <c r="B61" s="9" t="inlineStr">
@@ -7355,21 +7301,21 @@
         </is>
       </c>
       <c r="D61" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>AV67 &amp; ~AV137</t>
+          <t>AV137</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>AV67</t>
+          <t>AV137</t>
         </is>
       </c>
       <c r="G61" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu regras para a priorização e o escalamento de incidentes</t>
+          <t>No subitem a) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu regras para a priorização e o escalamento de incidentes</t>
         </is>
       </c>
       <c r="H61" s="9" t="b">
@@ -7379,7 +7325,7 @@
     <row r="62" ht="45" customHeight="1">
       <c r="A62" s="9" t="inlineStr">
         <is>
-          <t>MR086</t>
+          <t>MR087</t>
         </is>
       </c>
       <c r="B62" s="9" t="inlineStr">
@@ -7393,21 +7339,21 @@
         </is>
       </c>
       <c r="D62" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>AV137</t>
+          <t>AV70 &amp; ~AV140</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>AV137</t>
+          <t>AV70</t>
         </is>
       </c>
       <c r="G62" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu regras para a priorização e o escalamento de incidentes</t>
+          <t>No subitem d) do item 2204, não houve declaração afirmativa quanto à prática avaliada: o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H62" s="9" t="b">
@@ -7417,7 +7363,7 @@
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>MR087</t>
+          <t>MR088</t>
         </is>
       </c>
       <c r="B63" s="9" t="inlineStr">
@@ -7431,21 +7377,21 @@
         </is>
       </c>
       <c r="D63" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>AV70 &amp; ~AV140</t>
+          <t>AV140</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>AV70</t>
+          <t>AV140</t>
         </is>
       </c>
       <c r="G63" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2204, não houve declaração afirmativa quanto à prática avaliada: o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem d) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H63" s="9" t="b">
@@ -7455,7 +7401,7 @@
     <row r="64" ht="45" customHeight="1">
       <c r="A64" s="9" t="inlineStr">
         <is>
-          <t>MR088</t>
+          <t>MR089</t>
         </is>
       </c>
       <c r="B64" s="9" t="inlineStr">
@@ -7469,21 +7415,21 @@
         </is>
       </c>
       <c r="D64" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>AV140</t>
+          <t>AV71 &amp; ~AV141</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>AV140</t>
+          <t>AV71</t>
         </is>
       </c>
       <c r="G64" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem e) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
         </is>
       </c>
       <c r="H64" s="9" t="b">
@@ -7493,7 +7439,7 @@
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="9" t="inlineStr">
         <is>
-          <t>MR089</t>
+          <t>MR090</t>
         </is>
       </c>
       <c r="B65" s="9" t="inlineStr">
@@ -7507,21 +7453,21 @@
         </is>
       </c>
       <c r="D65" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>AV71 &amp; ~AV141</t>
+          <t>AV141</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>AV71</t>
+          <t>AV141</t>
         </is>
       </c>
       <c r="G65" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
+          <t>No subitem e) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
         </is>
       </c>
       <c r="H65" s="9" t="b">
@@ -7531,35 +7477,35 @@
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="9" t="inlineStr">
         <is>
-          <t>MR090</t>
+          <t>MR091</t>
         </is>
       </c>
       <c r="B66" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C66" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D66" s="9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>AV141</t>
+          <t>AV73 &amp; ~AV143</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>AV141</t>
+          <t>AV73</t>
         </is>
       </c>
       <c r="G66" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
+          <t>No subitem a) do item 2801, não houve declaração afirmativa quanto à prática avaliada: o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
         </is>
       </c>
       <c r="H66" s="9" t="b">
@@ -7569,7 +7515,7 @@
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="9" t="inlineStr">
         <is>
-          <t>MR091</t>
+          <t>MR092</t>
         </is>
       </c>
       <c r="B67" s="9" t="inlineStr">
@@ -7583,21 +7529,21 @@
         </is>
       </c>
       <c r="D67" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>AV73 &amp; ~AV143</t>
+          <t>AV143</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>AV73</t>
+          <t>AV143</t>
         </is>
       </c>
       <c r="G67" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2801, não houve declaração afirmativa quanto à prática avaliada: o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
+          <t>No subitem a) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
         </is>
       </c>
       <c r="H67" s="9" t="b">
@@ -7607,7 +7553,7 @@
     <row r="68" ht="45" customHeight="1">
       <c r="A68" s="9" t="inlineStr">
         <is>
-          <t>MR092</t>
+          <t>MR101</t>
         </is>
       </c>
       <c r="B68" s="9" t="inlineStr">
@@ -7617,25 +7563,25 @@
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
         </is>
       </c>
       <c r="D68" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>AV143</t>
+          <t>AV78 &amp; ~AV148</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>AV143</t>
+          <t>AV78</t>
         </is>
       </c>
       <c r="G68" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
+          <t>No subitem a) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
         </is>
       </c>
       <c r="H68" s="9" t="b">
@@ -7645,7 +7591,7 @@
     <row r="69" ht="60" customHeight="1">
       <c r="A69" s="9" t="inlineStr">
         <is>
-          <t>MR101</t>
+          <t>MR102</t>
         </is>
       </c>
       <c r="B69" s="9" t="inlineStr">
@@ -7659,21 +7605,21 @@
         </is>
       </c>
       <c r="D69" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>AV78 &amp; ~AV148</t>
+          <t>AV148</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>AV78</t>
+          <t>AV148</t>
         </is>
       </c>
       <c r="G69" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
+          <t>No subitem a) do item 2804, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
         </is>
       </c>
       <c r="H69" s="9" t="b">
@@ -7683,7 +7629,7 @@
     <row r="70" ht="45" customHeight="1">
       <c r="A70" s="9" t="inlineStr">
         <is>
-          <t>MR102</t>
+          <t>MR109</t>
         </is>
       </c>
       <c r="B70" s="9" t="inlineStr">
@@ -7693,25 +7639,25 @@
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
         </is>
       </c>
       <c r="D70" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>AV148</t>
+          <t>AV82</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>AV148</t>
+          <t>AV82</t>
         </is>
       </c>
       <c r="G70" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2804, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
+          <t>No subitem b) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de TI executadas no exercício encontram-se previamente estabelecidas nos instrumentos de planejamento vigentes (PDTI/PEDTIC e PCA)</t>
         </is>
       </c>
       <c r="H70" s="9" t="b">
@@ -7721,7 +7667,7 @@
     <row r="71" ht="45" customHeight="1">
       <c r="A71" s="9" t="inlineStr">
         <is>
-          <t>MR109</t>
+          <t>MR110</t>
         </is>
       </c>
       <c r="B71" s="9" t="inlineStr">
@@ -7731,7 +7677,7 @@
       </c>
       <c r="C71" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
+          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
         </is>
       </c>
       <c r="D71" s="9" t="n">
@@ -7739,17 +7685,17 @@
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>AV82</t>
+          <t>AV83</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>AV82</t>
+          <t>AV83</t>
         </is>
       </c>
       <c r="G71" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de TI executadas no exercício encontram-se previamente estabelecidas nos instrumentos de planejamento vigentes (PDTI/PEDTIC e PCA)</t>
+          <t>No subitem c) do item 2804, não houve declaração afirmativa quanto à prática avaliada: a fase de planejamento de cada contratação de TI é conduzida por uma Equipe de Planejamento da Contratação formalmente designada (composta, minimamente, por integrante requisitante e integrante técnico da área de TI)</t>
         </is>
       </c>
       <c r="H71" s="9" t="b">
@@ -7759,7 +7705,7 @@
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="9" t="inlineStr">
         <is>
-          <t>MR110</t>
+          <t>MR111</t>
         </is>
       </c>
       <c r="B72" s="9" t="inlineStr">
@@ -7769,25 +7715,25 @@
       </c>
       <c r="C72" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D72" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>AV83</t>
+          <t>AV152 &amp; ~AV153</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>AV83</t>
+          <t>AV152</t>
         </is>
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2804, não houve declaração afirmativa quanto à prática avaliada: a fase de planejamento de cada contratação de TI é conduzida por uma Equipe de Planejamento da Contratação formalmente designada (composta, minimamente, por integrante requisitante e integrante técnico da área de TI)</t>
+          <t>No subitem b) do item 2801, não houve declaração afirmativa quanto à prática avaliada: são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
         </is>
       </c>
       <c r="H72" s="9" t="b">
@@ -7797,17 +7743,17 @@
     <row r="73" ht="30" customHeight="1">
       <c r="A73" s="9" t="inlineStr">
         <is>
-          <t>MR111</t>
+          <t>MR113</t>
         </is>
       </c>
       <c r="B73" s="9" t="inlineStr">
         <is>
-          <t>PA06</t>
+          <t>PA03</t>
         </is>
       </c>
       <c r="C73" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="D73" s="9" t="n">
@@ -7815,61 +7761,24 @@
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>AV152 &amp; ~AV153</t>
+          <t>AV154</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>AV152</t>
+          <t>AV154</t>
         </is>
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2801, não houve declaração afirmativa quanto à prática avaliada: são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
+          <t>No item 2102, a organização não declarou possuir plano de tecnologia da informação vigente, ainda que parcialmente adotado</t>
         </is>
       </c>
       <c r="H73" s="9" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="74" ht="30" customHeight="1">
-      <c r="A74" s="9" t="inlineStr">
-        <is>
-          <t>MR113</t>
-        </is>
-      </c>
-      <c r="B74" s="9" t="inlineStr">
-        <is>
-          <t>PA03</t>
-        </is>
-      </c>
-      <c r="C74" s="9" t="inlineStr">
-        <is>
-          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
-        </is>
-      </c>
-      <c r="D74" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E74" s="9" t="inlineStr">
-        <is>
-          <t>AV154</t>
-        </is>
-      </c>
-      <c r="F74" s="9" t="inlineStr">
-        <is>
-          <t>AV154</t>
-        </is>
-      </c>
-      <c r="G74" s="9" t="inlineStr">
-        <is>
-          <t>No item 2102, a organização não declarou possuir plano de tecnologia da informação vigente, ainda que parcialmente adotado</t>
-        </is>
-      </c>
-      <c r="H74" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
+    <row r="74" ht="30" customHeight="1"/>
     <row r="75" ht="45" customHeight="1"/>
     <row r="76" ht="30" customHeight="1"/>
     <row r="77" ht="45" customHeight="1"/>

</xml_diff>

<commit_message>
Ajusta regras de S3.1 e S4.6
</commit_message>
<xml_diff>
--- a/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
+++ b/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
@@ -599,7 +599,7 @@
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>(((AV14 | AV92) | (AV15 | AV93) | (AV17 | AV95) | AV154) | (AV155 &amp; ((AV18 | AV96) | (AV19 | AV97) | (AV20 | AV98) | (AV24 | AV101))))</t>
+          <t>(((AV14 | AV92) | (AV17 | AV95) | AV154) | (AV155 &amp; ((AV18 | AV96) | (AV19 | AV97) | (AV20 | AV98) | (AV24 | AV101))))</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
@@ -624,7 +624,7 @@
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>((AV26 &amp; AV25) | (AV29 | AV103) | ((AV31 | AV105) | (AV33 | AV107)) | (AV45 &amp; AV46))</t>
+          <t>((AV26 &amp; AV25) | (AV29 | AV103) | ((AV31 | AV105) | (AV33 | AV107)) | (AV45 &amp; AV46 &amp; ~AV25))</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
@@ -699,7 +699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P76"/>
+  <dimension ref="A1:P74"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1489,14 +1489,14 @@
       <c r="O14" s="1" t="n"/>
       <c r="P14" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades e participação das áreas demandantes</t>
         </is>
       </c>
     </row>
     <row r="15" ht="169.35" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>AV15</t>
+          <t>AV17</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -1509,7 +1509,7 @@
       <c r="E15" s="1" t="n"/>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>q2101ext[B]</t>
+          <t>q2101ext[D]</t>
         </is>
       </c>
       <c r="G15" s="1" t="inlineStr">
@@ -1521,7 +1521,7 @@
       </c>
       <c r="H15" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento b) do item 2101 do Questionário, para verificar se a organização estabeleceu critérios para orientar a seleção e a priorização das iniciativas de TI (projetos e ações) e os mantêm atualizados</t>
+          <t>Resposta negativa ao detalhamento d) do item 2101 do Questionário, para verificar se o processo de planejamento de TI está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="I15" s="1" t="n"/>
@@ -1545,14 +1545,14 @@
       <c r="O15" s="1" t="n"/>
       <c r="P15" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades e participação das áreas demandantes</t>
         </is>
       </c>
     </row>
     <row r="16" ht="169.35" customHeight="1">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>AV17</t>
+          <t>AV18</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -1565,25 +1565,24 @@
       <c r="E16" s="1" t="n"/>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>q2101ext[D]</t>
+          <t>q2102ext[A]</t>
         </is>
       </c>
       <c r="G16" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+          <t>Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
 Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H16" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento d) do item 2101 do Questionário, para verificar se o processo de planejamento de TI está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>Resposta negativa ao detalhamento a) do item 2102 do Questionário, para verificar se o plano de tecnologia da informação (plano de TI) é aprovado pelo dirigente máximo da organização ou por dirigente ou colegiado que integra a alta administração</t>
         </is>
       </c>
       <c r="I16" s="1" t="n"/>
       <c r="J16" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
+          <t>Ausência de aprovação formal do plano de TIC.</t>
         </is>
       </c>
       <c r="K16" s="1" t="inlineStr">
@@ -1601,14 +1600,14 @@
       <c r="O16" s="1" t="n"/>
       <c r="P16" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>submeta o plano de TIC à aprovação formal do dirigente máximo ou de instância competente da alta administração, mantendo registro do respectivo ato de aprovação</t>
         </is>
       </c>
     </row>
     <row r="17" ht="225.4" customHeight="1">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>AV18</t>
+          <t>AV19</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -1621,24 +1620,25 @@
       <c r="E17" s="1" t="n"/>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>q2102ext[A]</t>
+          <t>q2102ext[D]</t>
         </is>
       </c>
       <c r="G17" s="1" t="inlineStr">
         <is>
-          <t>Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
 Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H17" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento a) do item 2102 do Questionário, para verificar se o plano de tecnologia da informação (plano de TI) é aprovado pelo dirigente máximo da organização ou por dirigente ou colegiado que integra a alta administração</t>
+          <t>Resposta negativa ao detalhamento d) do item 2102 do Questionário, para verificar se as iniciativas de TI (projetos e ações) constantes do plano de TI alinham-se aos objetivos e iniciativas definidos no planejamento institucional (como PPA, planos estratégicos, planos setoriais e plano de governo, no caso de municípios), bem como, quando aplicável, às estratégias e diretrizes estabelecidas por instâncias superiores de governança (como a Estratégia Nacional de Tecnologia da Informação e Comunicação do Poder Judiciário - ENTIC-JUD, normas e orientações do SETIC/PRODERJ (para órgãos estaduais) ou instâncias de governança equivalentes no âmbito municipal)</t>
         </is>
       </c>
       <c r="I17" s="1" t="n"/>
       <c r="J17" s="1" t="inlineStr">
         <is>
-          <t>Ausência de aprovação formal do plano de TIC.</t>
+          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
         </is>
       </c>
       <c r="K17" s="1" t="inlineStr">
@@ -1656,14 +1656,14 @@
       <c r="O17" s="1" t="n"/>
       <c r="P17" s="1" t="inlineStr">
         <is>
-          <t>submeta o plano de TIC à aprovação formal do dirigente máximo ou de instância competente da alta administração, mantendo registro do respectivo ato de aprovação</t>
+          <t>revise o plano de TIC para explicitar seu alinhamento ao planejamento institucional, às diretrizes superiores e às necessidades das áreas finalísticas e administrativas, relacionando objetivos, iniciativas, indicadores e metas de TIC aos resultados institucionais pretendidos</t>
         </is>
       </c>
     </row>
     <row r="18" ht="225.4" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>AV19</t>
+          <t>AV20</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -1676,25 +1676,24 @@
       <c r="E18" s="1" t="n"/>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>q2102ext[D]</t>
+          <t>q2102ext[C]</t>
         </is>
       </c>
       <c r="G18" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+          <t>COBIT 2019, APO06.03 - Criar e manter orçamentos: elaborar e manter orçamento de TIC alinhado ao portfólio, ao planejamento e às prioridades aprovadas.
 Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H18" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento d) do item 2102 do Questionário, para verificar se as iniciativas de TI (projetos e ações) constantes do plano de TI alinham-se aos objetivos e iniciativas definidos no planejamento institucional (como PPA, planos estratégicos, planos setoriais e plano de governo, no caso de municípios), bem como, quando aplicável, às estratégias e diretrizes estabelecidas por instâncias superiores de governança (como a Estratégia Nacional de Tecnologia da Informação e Comunicação do Poder Judiciário - ENTIC-JUD, normas e orientações do SETIC/PRODERJ (para órgãos estaduais) ou instâncias de governança equivalentes no âmbito municipal)</t>
+          <t>Resposta negativa ao detalhamento c) do item 2102 do Questionário, para verificar se o plano de TI fundamenta a proposta orçamentária da área de TI e o plano de contratações</t>
         </is>
       </c>
       <c r="I18" s="1" t="n"/>
       <c r="J18" s="1" t="inlineStr">
         <is>
-          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
+          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
         </is>
       </c>
       <c r="K18" s="1" t="inlineStr">
@@ -1712,14 +1711,14 @@
       <c r="O18" s="1" t="n"/>
       <c r="P18" s="1" t="inlineStr">
         <is>
-          <t>revise o plano de TIC para explicitar seu alinhamento ao planejamento institucional, às diretrizes superiores e às necessidades das áreas finalísticas e administrativas, relacionando objetivos, iniciativas, indicadores e metas de TIC aos resultados institucionais pretendidos</t>
+          <t>integre o plano de TIC à elaboração da proposta orçamentária e do plano de contratações, de maneira proporcional ao porte, à estrutura e à capacidade de planejamento da organização</t>
         </is>
       </c>
     </row>
     <row r="19" ht="225.4" customHeight="1">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>AV20</t>
+          <t>AV24</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1732,24 +1731,23 @@
       <c r="E19" s="1" t="n"/>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>q2102ext[C]</t>
+          <t>q2102ext[E]</t>
         </is>
       </c>
       <c r="G19" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO06.03 - Criar e manter orçamentos: elaborar e manter orçamento de TIC alinhado ao portfólio, ao planejamento e às prioridades aprovadas.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
+          <t>Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H19" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento c) do item 2102 do Questionário, para verificar se o plano de TI fundamenta a proposta orçamentária da área de TI e o plano de contratações</t>
+          <t>Resposta negativa ao detalhamento e) do item 2102 do Questionário, para verificar se é feito acompanhamento concomitante à execução do plano de TI, com vistas a assegurar sua observância e possibilitar a realização de ajustes que se fizerem necessário</t>
         </is>
       </c>
       <c r="I19" s="1" t="n"/>
       <c r="J19" s="1" t="inlineStr">
         <is>
-          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
+          <t>Ausência de acompanhamento da execução do plano de TIC.</t>
         </is>
       </c>
       <c r="K19" s="1" t="inlineStr">
@@ -1767,14 +1765,14 @@
       <c r="O19" s="1" t="n"/>
       <c r="P19" s="1" t="inlineStr">
         <is>
-          <t>integre o plano de TIC à elaboração da proposta orçamentária e do plano de contratações, de maneira proporcional ao porte, à estrutura e à capacidade de planejamento da organização</t>
+          <t>estabeleça e execute rotina periódica de acompanhamento da execução do plano de TIC, promovendo sua revisão periódica e os ajustes ou atualizações necessários, com registro das principais decisões e reprogramações</t>
         </is>
       </c>
     </row>
     <row r="20" ht="225.4" customHeight="1">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>AV24</t>
+          <t>AV25</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1787,48 +1785,49 @@
       <c r="E20" s="1" t="n"/>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>q2102ext[E]</t>
+          <t>total_TI</t>
         </is>
       </c>
       <c r="G20" s="1" t="inlineStr">
         <is>
-          <t>Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
+          <t>COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.7 - A organização deve adotar providências para dotar o setor de TI de quantitativo adequado às necessidades de trabalho em TI, consideradas as necessidades das demais áreas.</t>
         </is>
       </c>
       <c r="H20" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento e) do item 2102 do Questionário, para verificar se é feito acompanhamento concomitante à execução do plano de TI, com vistas a assegurar sua observância e possibilitar a realização de ajustes que se fizerem necessário</t>
+          <t>Ausência de profissionais que atuam regularmente em tecnologia da informação, conforme informado em resposta ao item 0105</t>
         </is>
       </c>
       <c r="I20" s="1" t="n"/>
       <c r="J20" s="1" t="inlineStr">
         <is>
-          <t>Ausência de acompanhamento da execução do plano de TIC.</t>
+          <t>Ausência de força de trabalho dedicada à TIC.</t>
         </is>
       </c>
       <c r="K20" s="1" t="inlineStr">
         <is>
-          <t>(Não | N/A)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L20" s="1" t="n"/>
       <c r="M20" s="1" t="n"/>
       <c r="N20" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O20" s="1" t="n"/>
       <c r="P20" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e execute rotina periódica de acompanhamento da execução do plano de TIC, promovendo sua revisão periódica e os ajustes ou atualizações necessários, com registro das principais decisões e reprogramações</t>
+          <t>avalie a força de trabalho dedicada à TIC e adote medidas proporcionais para assegurar capacidade mínima de planejamento, gestão, proteção, contratação, fiscalização e sustentação dos serviços e ativos de TIC</t>
         </is>
       </c>
     </row>
     <row r="21" ht="225.4" customHeight="1">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>AV25</t>
+          <t>AV26</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1841,7 +1840,7 @@
       <c r="E21" s="1" t="n"/>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>total_TI</t>
+          <t>q0101</t>
         </is>
       </c>
       <c r="G21" s="1" t="inlineStr">
@@ -1852,7 +1851,7 @@
       </c>
       <c r="H21" s="1" t="inlineStr">
         <is>
-          <t>Ausência de profissionais que atuam regularmente em tecnologia da informação, conforme informado em resposta ao item 0105</t>
+          <t>Resposta "@" ao item 0101 do Questionário, para verificar qual alternativa melhor descreve a formalização e o modelo de operação predominante da Tecnologia da Informação (TI) na organização</t>
         </is>
       </c>
       <c r="I21" s="1" t="n"/>
@@ -1863,7 +1862,7 @@
       </c>
       <c r="K21" s="1" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>(a) Centralizada Interna: Há uma área de TI centralizada e formal que atende toda a organização, utilizando equipe técnica majoritariamente própria (servidores). | b) Centralizada Terceirizada: Há uma área de TI centralizada e formal que faz a gestão, mas a execução operacional/técnica é predominantemente terceirizada (ex: fábricas de software, service desk). | d) Descentralizada: Diferentes secretarias, unidades ou setores possuem autonomia e mantêm suas próprias equipes, contratos ou infraestruturas de TI de forma independente. | e) Híbrida: Existe uma TI central formal para diretrizes e infraestrutura corporativa, mas as áreas de negócio possuem equipes próprias para sustentar sistemas específicos.)</t>
         </is>
       </c>
       <c r="L21" s="1" t="n"/>
@@ -1883,7 +1882,7 @@
     <row r="22" ht="225.4" customHeight="1">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>AV26</t>
+          <t>AV29</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1896,29 +1895,29 @@
       <c r="E22" s="1" t="n"/>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>q0101</t>
+          <t>q2703ext[C]</t>
         </is>
       </c>
       <c r="G22" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.7 - A organização deve adotar providências para dotar o setor de TI de quantitativo adequado às necessidades de trabalho em TI, consideradas as necessidades das demais áreas.</t>
+          <t>COBIT 2019, APO07.05 - Planejar e monitorar o uso de recursos humanos de TI e de negócio: planejar, alocar e acompanhar capacidade de pessoal para iniciativas, operações e serviços de TIC.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6.5 - O PDTI deve contemplar o quantitativo necessário ou ideal para a força de trabalho em TI.</t>
         </is>
       </c>
       <c r="H22" s="1" t="inlineStr">
         <is>
-          <t>Resposta "@" ao item 0101 do Questionário, para verificar qual alternativa melhor descreve a formalização e o modelo de operação predominante da Tecnologia da Informação (TI) na organização</t>
+          <t>Resposta negativa ao detalhamento c) do item 2703 do Questionário, para verificar se definiu-se, de maneira documentada, um quantitativo necessário de pessoal da área de tecnologia da informação e segurança da informação</t>
         </is>
       </c>
       <c r="I22" s="1" t="n"/>
       <c r="J22" s="1" t="inlineStr">
         <is>
-          <t>Ausência de força de trabalho dedicada à TIC.</t>
+          <t>Ausência ou insuficiência de definição documentada do quantitativo necessário de pessoal de TIC e segurança da informação.</t>
         </is>
       </c>
       <c r="K22" s="1" t="inlineStr">
         <is>
-          <t>(a) Centralizada Interna: Há uma área de TI centralizada e formal que atende toda a organização, utilizando equipe técnica majoritariamente própria (servidores). | b) Centralizada Terceirizada: Há uma área de TI centralizada e formal que faz a gestão, mas a execução operacional/técnica é predominantemente terceirizada (ex: fábricas de software, service desk). | d) Descentralizada: Diferentes secretarias, unidades ou setores possuem autonomia e mantêm suas próprias equipes, contratos ou infraestruturas de TI de forma independente. | e) Híbrida: Existe uma TI central formal para diretrizes e infraestrutura corporativa, mas as áreas de negócio possuem equipes próprias para sustentar sistemas específicos.)</t>
+          <t>(Não | N/A)</t>
         </is>
       </c>
       <c r="L22" s="1" t="n"/>
@@ -1931,14 +1930,14 @@
       <c r="O22" s="1" t="n"/>
       <c r="P22" s="1" t="inlineStr">
         <is>
-          <t>avalie a força de trabalho dedicada à TIC e adote medidas proporcionais para assegurar capacidade mínima de planejamento, gestão, proteção, contratação, fiscalização e sustentação dos serviços e ativos de TIC</t>
+          <t>estime e mantenha atualizado o quantitativo necessário de pessoal de TIC e segurança da informação, considerando o porte e a complexidade da organização, os serviços críticos, os sistemas mantidos, as contratações vigentes e os riscos relevantes</t>
         </is>
       </c>
     </row>
     <row r="23" ht="214.15" customHeight="1">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>AV29</t>
+          <t>AV31</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1951,29 +1950,29 @@
       <c r="E23" s="1" t="n"/>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>q2703ext[C]</t>
+          <t>q2708[B]</t>
         </is>
       </c>
       <c r="G23" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO07.05 - Planejar e monitorar o uso de recursos humanos de TI e de negócio: planejar, alocar e acompanhar capacidade de pessoal para iniciativas, operações e serviços de TIC.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6.5 - O PDTI deve contemplar o quantitativo necessário ou ideal para a força de trabalho em TI.</t>
+          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
+COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
         </is>
       </c>
       <c r="H23" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento c) do item 2703 do Questionário, para verificar se definiu-se, de maneira documentada, um quantitativo necessário de pessoal da área de tecnologia da informação e segurança da informação</t>
+          <t>Resposta negativa ao subitem b) do item 2708 do Questionário, para verificar se a organização possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
         </is>
       </c>
       <c r="I23" s="1" t="n"/>
       <c r="J23" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou insuficiência de definição documentada do quantitativo necessário de pessoal de TIC e segurança da informação.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="K23" s="1" t="inlineStr">
         <is>
-          <t>(Não | N/A)</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="L23" s="1" t="n"/>
@@ -1986,14 +1985,14 @@
       <c r="O23" s="1" t="n"/>
       <c r="P23" s="1" t="inlineStr">
         <is>
-          <t>estime e mantenha atualizado o quantitativo necessário de pessoal de TIC e segurança da informação, considerando o porte e a complexidade da organização, os serviços críticos, os sistemas mantidos, as contratações vigentes e os riscos relevantes</t>
+          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
         </is>
       </c>
     </row>
     <row r="24" ht="214.15" customHeight="1">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>AV31</t>
+          <t>AV33</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -2006,7 +2005,7 @@
       <c r="E24" s="1" t="n"/>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>q2708[B]</t>
+          <t>q2708[D]</t>
         </is>
       </c>
       <c r="G24" s="1" t="inlineStr">
@@ -2017,7 +2016,7 @@
       </c>
       <c r="H24" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao subitem b) do item 2708 do Questionário, para verificar se a organização possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
+          <t>Resposta negativa ao subitem d) do item 2708 do Questionário, para verificar se a organização possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
         </is>
       </c>
       <c r="I24" s="1" t="n"/>
@@ -2048,7 +2047,7 @@
     <row r="25" ht="214.15" customHeight="1">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>AV33</t>
+          <t>AV45</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -2061,29 +2060,29 @@
       <c r="E25" s="1" t="n"/>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>q2708[D]</t>
+          <t>q0101</t>
         </is>
       </c>
       <c r="G25" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
-COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
+          <t>COBIT 2019, APO07.06 - Gerenciar pessoal contratado: controlar o uso de pessoal terceirizado ou externo, preservando responsabilização, supervisão e retenção de conhecimento.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens I.10.11, III.9.11 e IV.11.3 – Referência para avaliação da estrutura de recursos humanos de TIC quanto à suficiência quantitativa e qualitativa e à preservação de capacidade interna em atividades de planejamento, coordenação, fiscalização e controle.</t>
         </is>
       </c>
       <c r="H25" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao subitem d) do item 2708 do Questionário, para verificar se a organização possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
+          <t>Resposta "@" ao item 0101 do Questionário, para verificar qual alternativa melhor descreve a formalização e o modelo de operação predominante da Tecnologia da Informação (TI) na organização</t>
         </is>
       </c>
       <c r="I25" s="1" t="n"/>
       <c r="J25" s="1" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Operação de TIC predominantemente terceirizada sem profissionais internos de TIC.</t>
         </is>
       </c>
       <c r="K25" s="1" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>b) Centralizada Terceirizada: Há uma área de TI centralizada e formal que faz a gestão, mas a execução operacional/técnica é predominantemente terceirizada (ex: fábricas de software, service desk).</t>
         </is>
       </c>
       <c r="L25" s="1" t="n"/>
@@ -2096,14 +2095,14 @@
       <c r="O25" s="1" t="n"/>
       <c r="P25" s="1" t="inlineStr">
         <is>
-          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
+          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente para coordenar, supervisionar e fiscalizar as atividades e os contratos de TIC executados predominantemente por terceiros, preservando responsabilização e retenção de conhecimento</t>
         </is>
       </c>
     </row>
     <row r="26" ht="214.15" customHeight="1">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>AV45</t>
+          <t>AV46</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -2116,7 +2115,7 @@
       <c r="E26" s="1" t="n"/>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>q0101</t>
+          <t>total_TI_interno</t>
         </is>
       </c>
       <c r="G26" s="1" t="inlineStr">
@@ -2127,7 +2126,7 @@
       </c>
       <c r="H26" s="1" t="inlineStr">
         <is>
-          <t>Resposta "@" ao item 0101 do Questionário, para verificar qual alternativa melhor descreve a formalização e o modelo de operação predominante da Tecnologia da Informação (TI) na organização</t>
+          <t>Ausência de profissionais internos da organização que atuam regularmente em tecnologia da informação, conforme informado em resposta ao item 0105</t>
         </is>
       </c>
       <c r="I26" s="1" t="n"/>
@@ -2138,7 +2137,7 @@
       </c>
       <c r="K26" s="1" t="inlineStr">
         <is>
-          <t>b) Centralizada Terceirizada: Há uma área de TI centralizada e formal que faz a gestão, mas a execução operacional/técnica é predominantemente terceirizada (ex: fábricas de software, service desk).</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L26" s="1" t="n"/>
@@ -2158,7 +2157,7 @@
     <row r="27" ht="225.4" customHeight="1">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>AV46</t>
+          <t>AV54</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -2171,29 +2170,29 @@
       <c r="E27" s="1" t="n"/>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>total_TI_interno</t>
+          <t>q2201ext[A]</t>
         </is>
       </c>
       <c r="G27" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO07.06 - Gerenciar pessoal contratado: controlar o uso de pessoal terceirizado ou externo, preservando responsabilização, supervisão e retenção de conhecimento.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens I.10.11, III.9.11 e IV.11.3 – Referência para avaliação da estrutura de recursos humanos de TIC quanto à suficiência quantitativa e qualitativa e à preservação de capacidade interna em atividades de planejamento, coordenação, fiscalização e controle.</t>
+          <t>ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.7, III.9.7 e V.6.4 – Recomendações quanto à definição, pactuação e monitoramento de níveis de serviço.</t>
         </is>
       </c>
       <c r="H27" s="1" t="inlineStr">
         <is>
-          <t>Ausência de profissionais internos da organização que atuam regularmente em tecnologia da informação, conforme informado em resposta ao item 0105</t>
+          <t>Resposta negativa ao detalhamento a) do item 2201 do Questionário, para verificar se o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
         </is>
       </c>
       <c r="I27" s="1" t="n"/>
       <c r="J27" s="1" t="inlineStr">
         <is>
-          <t>Operação de TIC predominantemente terceirizada sem profissionais internos de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="K27" s="1" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>(Não | N/A)</t>
         </is>
       </c>
       <c r="L27" s="1" t="n"/>
@@ -2206,14 +2205,14 @@
       <c r="O27" s="1" t="n"/>
       <c r="P27" s="1" t="inlineStr">
         <is>
-          <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente para coordenar, supervisionar e fiscalizar as atividades e os contratos de TIC executados predominantemente por terceiros, preservando responsabilização e retenção de conhecimento</t>
+          <t>defina, acorde e monitore níveis de serviço para os serviços de TIC relevantes, estabelecendo metas e mecanismos de acompanhamento de seu cumprimento</t>
         </is>
       </c>
     </row>
     <row r="28" ht="113.45" customHeight="1">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>AV54</t>
+          <t>AV55</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -2226,24 +2225,25 @@
       <c r="E28" s="1" t="n"/>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[A]</t>
+          <t>q2201ext[B]</t>
         </is>
       </c>
       <c r="G28" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.7, III.9.7 e V.6.4 – Recomendações quanto à definição, pactuação e monitoramento de níveis de serviço.</t>
+          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.4, III.9.4 e V.6.1 – Recomendações quanto à estruturação do catálogo de serviços de TIC, incluindo descrição dos serviços, metas, formas de acesso e disponibilidade aos usuários.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.2.4 – Gerenciamento de catálogo de serviço: orienta que o catálogo descreva os serviços e seus resultados pretendidos, contenha informações relevantes para sua utilização e seja disponibilizado às partes interessadas que necessitem acessá-lo.</t>
         </is>
       </c>
       <c r="H28" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento a) do item 2201 do Questionário, para verificar se o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
+          <t>Resposta negativa ao detalhamento b) do item 2201 do Questionário, para verificar se o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
         </is>
       </c>
       <c r="I28" s="1" t="n"/>
       <c r="J28" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="K28" s="1" t="inlineStr">
@@ -2261,14 +2261,14 @@
       <c r="O28" s="1" t="n"/>
       <c r="P28" s="1" t="inlineStr">
         <is>
-          <t>defina, acorde e monitore níveis de serviço para os serviços de TIC relevantes, estabelecendo metas e mecanismos de acompanhamento de seu cumprimento</t>
+          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
         </is>
       </c>
     </row>
     <row r="29" ht="113.45" customHeight="1">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>AV55</t>
+          <t>AV56</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -2281,7 +2281,7 @@
       <c r="E29" s="1" t="n"/>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[B]</t>
+          <t>q2201ext[C]</t>
         </is>
       </c>
       <c r="G29" s="1" t="inlineStr">
@@ -2293,7 +2293,7 @@
       </c>
       <c r="H29" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento b) do item 2201 do Questionário, para verificar se o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
+          <t>Resposta negativa ao detalhamento c) do item 2201 do Questionário, para verificar se o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
         </is>
       </c>
       <c r="I29" s="1" t="n"/>
@@ -2324,7 +2324,7 @@
     <row r="30" ht="113.45" customHeight="1">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>AV56</t>
+          <t>AV57</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -2337,25 +2337,24 @@
       <c r="E30" s="1" t="n"/>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[C]</t>
+          <t>q2201ext[D]</t>
         </is>
       </c>
       <c r="G30" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.4, III.9.4 e V.6.1 – Recomendações quanto à estruturação do catálogo de serviços de TIC, incluindo descrição dos serviços, metas, formas de acesso e disponibilidade aos usuários.
-ABNT NBR ISO/IEC 20000-2:2021, item 8.2.4 – Gerenciamento de catálogo de serviço: orienta que o catálogo descreva os serviços e seus resultados pretendidos, contenha informações relevantes para sua utilização e seja disponibilizado às partes interessadas que necessitem acessá-lo.</t>
+          <t>ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.7, III.9.7 e V.6.4 – Recomendações quanto à definição, pactuação e monitoramento de níveis de serviço.</t>
         </is>
       </c>
       <c r="H30" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento c) do item 2201 do Questionário, para verificar se o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
+          <t>Resposta negativa ao detalhamento d) do item 2201 do Questionário, para verificar se são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
         </is>
       </c>
       <c r="I30" s="1" t="n"/>
       <c r="J30" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="K30" s="1" t="inlineStr">
@@ -2373,14 +2372,14 @@
       <c r="O30" s="1" t="n"/>
       <c r="P30" s="1" t="inlineStr">
         <is>
-          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
+          <t>defina, acorde e monitore níveis de serviço para os serviços de TIC relevantes, estabelecendo metas e mecanismos de acompanhamento de seu cumprimento</t>
         </is>
       </c>
     </row>
     <row r="31" ht="113.45" customHeight="1">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>AV57</t>
+          <t>AV58</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -2393,7 +2392,7 @@
       <c r="E31" s="1" t="n"/>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[D]</t>
+          <t>q2201ext[E]</t>
         </is>
       </c>
       <c r="G31" s="1" t="inlineStr">
@@ -2404,7 +2403,7 @@
       </c>
       <c r="H31" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento d) do item 2201 do Questionário, para verificar se são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
+          <t>Resposta negativa ao detalhamento e) do item 2201 do Questionário, para verificar se a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
         </is>
       </c>
       <c r="I31" s="1" t="n"/>
@@ -2435,7 +2434,7 @@
     <row r="32" ht="113.45" customHeight="1">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>AV58</t>
+          <t>AV59</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -2448,24 +2447,25 @@
       <c r="E32" s="1" t="n"/>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[E]</t>
+          <t>q2203ext[A]</t>
         </is>
       </c>
       <c r="G32" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.7, III.9.7 e V.6.4 – Recomendações quanto à definição, pactuação e monitoramento de níveis de serviço.</t>
+          <t>COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.2.6 – Gerenciamento de configuração: orienta a identificação, o registro, o controle, o rastreamento e a verificação dos itens de configuração, bem como a manutenção de informações de configuração precisas relacionadas aos serviços.</t>
         </is>
       </c>
       <c r="H32" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento e) do item 2201 do Questionário, para verificar se a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
+          <t>Resposta negativa ao detalhamento a) do item 2203 do Questionário, para verificar se a organização mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
         </is>
       </c>
       <c r="I32" s="1" t="n"/>
       <c r="J32" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="K32" s="1" t="inlineStr">
@@ -2483,14 +2483,14 @@
       <c r="O32" s="1" t="n"/>
       <c r="P32" s="1" t="inlineStr">
         <is>
-          <t>defina, acorde e monitore níveis de serviço para os serviços de TIC relevantes, estabelecendo metas e mecanismos de acompanhamento de seu cumprimento</t>
+          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
         </is>
       </c>
     </row>
     <row r="33" ht="102.2" customHeight="1">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>AV59</t>
+          <t>AV62</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -2503,25 +2503,24 @@
       <c r="E33" s="1" t="n"/>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>q2203ext[A]</t>
+          <t>q2504ext[A]</t>
         </is>
       </c>
       <c r="G33" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.
-ABNT NBR ISO/IEC 20000-2:2021, item 8.2.6 – Gerenciamento de configuração: orienta a identificação, o registro, o controle, o rastreamento e a verificação dos itens de configuração, bem como a manutenção de informações de configuração precisas relacionadas aos serviços.</t>
+          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.</t>
         </is>
       </c>
       <c r="H33" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento a) do item 2203 do Questionário, para verificar se a organização mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
+          <t>Resposta negativa ao detalhamento a) do item 2504 do Questionário, para verificar se a organização gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="I33" s="1" t="n"/>
       <c r="J33" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
         </is>
       </c>
       <c r="K33" s="1" t="inlineStr">
@@ -2539,14 +2538,14 @@
       <c r="O33" s="1" t="n"/>
       <c r="P33" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
+          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos sob gestão da organização, contemplando, minimamente, os dispositivos e softwares utilizados, com informações suficientes para sua identificação e controle</t>
         </is>
       </c>
     </row>
     <row r="34" ht="102.2" customHeight="1">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>AV62</t>
+          <t>AV63</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -2559,7 +2558,7 @@
       <c r="E34" s="1" t="n"/>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>q2504ext[A]</t>
+          <t>q2504ext[B]</t>
         </is>
       </c>
       <c r="G34" s="1" t="inlineStr">
@@ -2570,7 +2569,7 @@
       </c>
       <c r="H34" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento a) do item 2504 do Questionário, para verificar se a organização gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
+          <t>Resposta negativa ao detalhamento b) do item 2504 do Questionário, para verificar se a organização gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="I34" s="1" t="n"/>
@@ -2601,7 +2600,7 @@
     <row r="35" ht="102.2" customHeight="1">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>AV63</t>
+          <t>AV66</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -2614,24 +2613,25 @@
       <c r="E35" s="1" t="n"/>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>q2504ext[B]</t>
+          <t>q2203ext[C]</t>
         </is>
       </c>
       <c r="G35" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.</t>
+          <t>COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.2.6 – Gerenciamento de configuração: orienta a identificação, o registro, o controle, o rastreamento e a verificação dos itens de configuração, bem como a manutenção de informações de configuração precisas relacionadas aos serviços.</t>
         </is>
       </c>
       <c r="H35" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento b) do item 2504 do Questionário, para verificar se a organização gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
+          <t>Resposta negativa ao detalhamento c) do item 2203 do Questionário, para verificar se o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="I35" s="1" t="n"/>
       <c r="J35" s="1" t="inlineStr">
         <is>
-          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="K35" s="1" t="inlineStr">
@@ -2649,14 +2649,14 @@
       <c r="O35" s="1" t="n"/>
       <c r="P35" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos sob gestão da organização, contemplando, minimamente, os dispositivos e softwares utilizados, com informações suficientes para sua identificação e controle</t>
+          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
         </is>
       </c>
     </row>
     <row r="36" ht="102.2" customHeight="1">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>AV66</t>
+          <t>AV67</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -2669,25 +2669,25 @@
       <c r="E36" s="1" t="n"/>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>q2203ext[C]</t>
+          <t>q2204ext[A]</t>
         </is>
       </c>
       <c r="G36" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.
-ABNT NBR ISO/IEC 20000-2:2021, item 8.2.6 – Gerenciamento de configuração: orienta a identificação, o registro, o controle, o rastreamento e a verificação dos itens de configuração, bem como a manutenção de informações de configuração precisas relacionadas aos serviços.</t>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.6, III.9.6 e V.6.3 – Recomendações quanto à formalização e execução do processo de gestão de incidentes, incluindo registros, classificação, escalamento e tratamento.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.6.1 – Gerenciamento de incidente: orienta que os incidentes sejam registrados, classificados e priorizados, que as ações adotadas para sua resolução sejam registradas e rastreáveis e que sejam definidas responsabilidades para seu tratamento, incluindo procedimento documentado para incidentes graves.</t>
         </is>
       </c>
       <c r="H36" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento c) do item 2203 do Questionário, para verificar se o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>Resposta negativa ao detalhamento a) do item 2204 do Questionário, para verificar se a organização definiu regras para a priorização e o escalamento de incidentes</t>
         </is>
       </c>
       <c r="I36" s="1" t="n"/>
       <c r="J36" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="K36" s="1" t="inlineStr">
@@ -2705,14 +2705,14 @@
       <c r="O36" s="1" t="n"/>
       <c r="P36" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
     </row>
     <row r="37" ht="102.2" customHeight="1">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>AV67</t>
+          <t>AV70</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -2725,7 +2725,7 @@
       <c r="E37" s="1" t="n"/>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>q2204ext[A]</t>
+          <t>q2204ext[D]</t>
         </is>
       </c>
       <c r="G37" s="1" t="inlineStr">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="H37" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento a) do item 2204 do Questionário, para verificar se a organização definiu regras para a priorização e o escalamento de incidentes</t>
+          <t>Resposta negativa ao detalhamento d) do item 2204 do Questionário, para verificar se o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="I37" s="1" t="n"/>
@@ -2768,7 +2768,7 @@
     <row r="38" ht="102.2" customHeight="1">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>AV70</t>
+          <t>AV71</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -2781,7 +2781,7 @@
       <c r="E38" s="1" t="n"/>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>q2204ext[D]</t>
+          <t>q2204ext[E]</t>
         </is>
       </c>
       <c r="G38" s="1" t="inlineStr">
@@ -2793,7 +2793,7 @@
       </c>
       <c r="H38" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento d) do item 2204 do Questionário, para verificar se o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>Resposta negativa ao detalhamento e) do item 2204 do Questionário, para verificar se a organização definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
         </is>
       </c>
       <c r="I38" s="1" t="n"/>
@@ -2824,7 +2824,7 @@
     <row r="39" ht="102.2" customHeight="1">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>AV71</t>
+          <t>AV73</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -2837,25 +2837,25 @@
       <c r="E39" s="1" t="n"/>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>q2204ext[E]</t>
+          <t>q2801ext[A]</t>
         </is>
       </c>
       <c r="G39" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.6, III.9.6 e V.6.3 – Recomendações quanto à formalização e execução do processo de gestão de incidentes, incluindo registros, classificação, escalamento e tratamento.
-ABNT NBR ISO/IEC 20000-2:2021, item 8.6.1 – Gerenciamento de incidente: orienta que os incidentes sejam registrados, classificados e priorizados, que as ações adotadas para sua resolução sejam registradas e rastreáveis e que sejam definidas responsabilidades para seu tratamento, incluindo procedimento documentado para incidentes graves.</t>
+          <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Lei nº 14.133/2021, art. 19, inciso IV: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.
+Acórdão nº 2.342/2016-TCU-Plenário, item 9.1.7 – Precedente quanto à definição, aprovação e formalização de processo de trabalho para o planejamento de cada contratação, com controles internos mínimos.</t>
         </is>
       </c>
       <c r="H39" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento e) do item 2204 do Questionário, para verificar se a organização definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
+          <t>Resposta negativa ao detalhamento a) do item 2801 do Questionário, para verificar se o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
         </is>
       </c>
       <c r="I39" s="1" t="n"/>
       <c r="J39" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="K39" s="1" t="inlineStr">
@@ -2873,14 +2873,14 @@
       <c r="O39" s="1" t="n"/>
       <c r="P39" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
+          <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
         </is>
       </c>
     </row>
     <row r="40" ht="102.2" customHeight="1">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>AV73</t>
+          <t>AV78</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -2893,30 +2893,30 @@
       <c r="E40" s="1" t="n"/>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>q2801ext[A]</t>
+          <t>q2804[A]</t>
         </is>
       </c>
       <c r="G40" s="1" t="inlineStr">
         <is>
           <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Lei nº 14.133/2021, art. 19, inciso IV: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.
-Acórdão nº 2.342/2016-TCU-Plenário, item 9.1.7 – Precedente quanto à definição, aprovação e formalização de processo de trabalho para o planejamento de cada contratação, com controles internos mínimos.</t>
+COBIT 2019, BAI02.04 - Obter aprovação dos requisitos da solução: obter aprovação formal dos requisitos funcionais, técnicos, de segurança e de conformidade antes de prosseguir com a solução.
+Instrução Normativa SGD/ME nº 94/2022, arts. 2º, IV, 9º, 10, 11 e 12, §6º – referência de boa prática para estruturação da fase de planejamento das contratações de TIC, instituição da Equipe de Planejamento da Contratação e participação do integrante técnico da área de TIC, observada sua aplicação direta aos integrantes do SISP e as hipóteses de simplificação de procedimentos previstas na norma.</t>
         </is>
       </c>
       <c r="H40" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento a) do item 2801 do Questionário, para verificar se o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
+          <t>Resposta negativa ao subitem a) do item 2804 do Questionário, para verificar se as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
         </is>
       </c>
       <c r="I40" s="1" t="n"/>
       <c r="J40" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
         </is>
       </c>
       <c r="K40" s="1" t="inlineStr">
         <is>
-          <t>(Não | N/A)</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="L40" s="1" t="n"/>
@@ -2929,14 +2929,14 @@
       <c r="O40" s="1" t="n"/>
       <c r="P40" s="1" t="inlineStr">
         <is>
-          <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
+          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo procedimentos simplificados e proporcionais à natureza, ao risco e ao valor da contratação, preservada análise técnica compatível</t>
         </is>
       </c>
     </row>
     <row r="41" ht="102.2" customHeight="1">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>AV78</t>
+          <t>AV82</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -2949,25 +2949,25 @@
       <c r="E41" s="1" t="n"/>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>q2804[A]</t>
+          <t>q2804[B]</t>
         </is>
       </c>
       <c r="G41" s="1" t="inlineStr">
         <is>
           <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-COBIT 2019, BAI02.04 - Obter aprovação dos requisitos da solução: obter aprovação formal dos requisitos funcionais, técnicos, de segurança e de conformidade antes de prosseguir com a solução.
-Instrução Normativa SGD/ME nº 94/2022, arts. 2º, IV, 9º, 10, 11 e 12, §6º – referência de boa prática para estruturação da fase de planejamento das contratações de TIC, instituição da Equipe de Planejamento da Contratação e participação do integrante técnico da área de TIC, observada sua aplicação direta aos integrantes do SISP e as hipóteses de simplificação de procedimentos previstas na norma.</t>
+Lei nº 14.133/2021, arts. 12, VII e §1º, e 18, caput e §1º, II – a fase preparatória deve compatibilizar-se com o Plano de Contratações Anual, quando elaborado, e deve ser demonstrado o alinhamento da contratação com o planejamento da Administração.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens III.7 e IV.9 – Determinações para estruturação do processo de planejamento anual das contratações, contemplando consolidação das demandas, participação das áreas, aprovação e publicidade do plano.</t>
         </is>
       </c>
       <c r="H41" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao subitem a) do item 2804 do Questionário, para verificar se as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
+          <t>Resposta negativa ao subitem b) do item 2804 do Questionário, para verificar se as contratações de TI executadas no exercício encontram-se previamente estabelecidas nos instrumentos de planejamento vigentes (PDTI/PEDTIC e PCA)</t>
         </is>
       </c>
       <c r="I41" s="1" t="n"/>
       <c r="J41" s="1" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
         </is>
       </c>
       <c r="K41" s="1" t="inlineStr">
@@ -2979,20 +2979,20 @@
       <c r="M41" s="1" t="n"/>
       <c r="N41" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O41" s="1" t="n"/>
       <c r="P41" s="1" t="inlineStr">
         <is>
-          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo procedimentos simplificados e proporcionais à natureza, ao risco e ao valor da contratação, preservada análise técnica compatível</t>
+          <t>assegure que as contratações de TIC sejam compatíveis com os instrumentos de planejamento de TIC e, quando elaborado, com o Plano de Contratações Anual, promovendo os ajustes ou justificativas cabíveis nos casos excepcionais</t>
         </is>
       </c>
     </row>
     <row r="42" ht="113.45" customHeight="1">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>AV82</t>
+          <t>AV83</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -3005,25 +3005,25 @@
       <c r="E42" s="1" t="n"/>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>q2804[B]</t>
+          <t>q2804[C]</t>
         </is>
       </c>
       <c r="G42" s="1" t="inlineStr">
         <is>
           <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Lei nº 14.133/2021, arts. 12, VII e §1º, e 18, caput e §1º, II – a fase preparatória deve compatibilizar-se com o Plano de Contratações Anual, quando elaborado, e deve ser demonstrado o alinhamento da contratação com o planejamento da Administração.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens III.7 e IV.9 – Determinações para estruturação do processo de planejamento anual das contratações, contemplando consolidação das demandas, participação das áreas, aprovação e publicidade do plano.</t>
+Lei nº 14.133/2021, art. 7º, caput, incisos I a III e §1º: designação de agentes públicos para funções essenciais, observados atribuições, formação, segregação de funções e inexistência de vínculos que comprometam a atuação.
+Instrução Normativa SGD/ME nº 94/2022, arts. 2º, IV, 9º, 10, 11 e 12, §6º – referência de boa prática para estruturação da fase de planejamento das contratações de TIC, instituição da Equipe de Planejamento da Contratação e participação do integrante técnico da área de TIC, observada sua aplicação direta aos integrantes do SISP e as hipóteses de simplificação de procedimentos previstas na norma.</t>
         </is>
       </c>
       <c r="H42" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao subitem b) do item 2804 do Questionário, para verificar se as contratações de TI executadas no exercício encontram-se previamente estabelecidas nos instrumentos de planejamento vigentes (PDTI/PEDTIC e PCA)</t>
+          <t>Resposta negativa ao subitem c) do item 2804 do Questionário, para verificar se a fase de planejamento de cada contratação de TI é conduzida por uma Equipe de Planejamento da Contratação formalmente designada (composta, minimamente, por integrante requisitante e integrante técnico da área de TI)</t>
         </is>
       </c>
       <c r="I42" s="1" t="n"/>
       <c r="J42" s="1" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
+          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
         </is>
       </c>
       <c r="K42" s="1" t="inlineStr">
@@ -3035,25 +3035,25 @@
       <c r="M42" s="1" t="n"/>
       <c r="N42" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O42" s="1" t="n"/>
       <c r="P42" s="1" t="inlineStr">
         <is>
-          <t>assegure que as contratações de TIC sejam compatíveis com os instrumentos de planejamento de TIC e, quando elaborado, com o Plano de Contratações Anual, promovendo os ajustes ou justificativas cabíveis nos casos excepcionais</t>
+          <t>designe formalmente equipe de planejamento para as contratações de TIC, atentando-se, minimamente, em assegurar a participação de integrante da área requisitante e da área técnica de TIC, com definição das responsabilidades de seus integrantes</t>
         </is>
       </c>
     </row>
     <row r="43" ht="113.45" customHeight="1">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>AV83</t>
+          <t>AV84</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
-          <t>questionario</t>
+          <t>avaliacao_evidencias_ajustes</t>
         </is>
       </c>
       <c r="C43" s="1" t="n"/>
@@ -3061,30 +3061,29 @@
       <c r="E43" s="1" t="n"/>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>q2804[C]</t>
+          <t>q0103[D]</t>
         </is>
       </c>
       <c r="G43" s="1" t="inlineStr">
         <is>
-          <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Lei nº 14.133/2021, art. 7º, caput, incisos I a III e §1º: designação de agentes públicos para funções essenciais, observados atribuições, formação, segregação de funções e inexistência de vínculos que comprometam a atuação.
-Instrução Normativa SGD/ME nº 94/2022, arts. 2º, IV, 9º, 10, 11 e 12, §6º – referência de boa prática para estruturação da fase de planejamento das contratações de TIC, instituição da Equipe de Planejamento da Contratação e participação do integrante técnico da área de TIC, observada sua aplicação direta aos integrantes do SISP e as hipóteses de simplificação de procedimentos previstas na norma.</t>
+          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TI.
+Constituição Federal, art. 37, caput - Princípio da eficiência.</t>
         </is>
       </c>
       <c r="H43" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao subitem c) do item 2804 do Questionário, para verificar se a fase de planejamento de cada contratação de TI é conduzida por uma Equipe de Planejamento da Contratação formalmente designada (composta, minimamente, por integrante requisitante e integrante técnico da área de TI)</t>
+          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
         </is>
       </c>
       <c r="I43" s="1" t="n"/>
       <c r="J43" s="1" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
+          <t>Área de TIC sem atribuições formalmente definidas ou sem atribuições formais de gestão de TIC.</t>
         </is>
       </c>
       <c r="K43" s="1" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Não conforme</t>
         </is>
       </c>
       <c r="L43" s="1" t="n"/>
@@ -3097,14 +3096,14 @@
       <c r="O43" s="1" t="n"/>
       <c r="P43" s="1" t="inlineStr">
         <is>
-          <t>designe formalmente equipe de planejamento para as contratações de TIC, atentando-se, minimamente, em assegurar a participação de integrante da área requisitante e da área técnica de TIC, com definição das responsabilidades de seus integrantes</t>
+          <t>defina formalmente as atribuições da área de TIC, atentando-se, minimamente, em abranger as atividades de planejamento, coordenação, gestão e controle da TIC</t>
         </is>
       </c>
     </row>
     <row r="44" ht="113.45" customHeight="1">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>AV84</t>
+          <t>AV86</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -3117,13 +3116,12 @@
       <c r="E44" s="1" t="n"/>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>q0103[D]</t>
+          <t>q1001ext[H]</t>
         </is>
       </c>
       <c r="G44" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TI.
-Constituição Federal, art. 37, caput - Princípio da eficiência.</t>
+          <t>COBIT 2019, MEA01.04 - Avaliar o desempenho: monitorar e avaliar periodicamente o desempenho e a conformidade da TI em relação a objetivos, indicadores, metas e expectativas das partes interessadas.</t>
         </is>
       </c>
       <c r="H44" s="1" t="inlineStr">
@@ -3134,7 +3132,7 @@
       <c r="I44" s="1" t="n"/>
       <c r="J44" s="1" t="inlineStr">
         <is>
-          <t>Área de TIC sem atribuições formalmente definidas ou sem atribuições formais de gestão de TIC.</t>
+          <t>Ausência de objetivos, indicadores ou metas para a gestão de TIC.</t>
         </is>
       </c>
       <c r="K44" s="1" t="inlineStr">
@@ -3152,14 +3150,14 @@
       <c r="O44" s="1" t="n"/>
       <c r="P44" s="1" t="inlineStr">
         <is>
-          <t>defina formalmente as atribuições da área de TIC, atentando-se, minimamente, em abranger as atividades de planejamento, coordenação, gestão e controle da TIC</t>
+          <t>estabeleça objetivos, indicadores e metas para a gestão de TIC, de modo a possibilitar o acompanhamento periódico do desempenho da TIC pela alta administração</t>
         </is>
       </c>
     </row>
     <row r="45" ht="113.45" customHeight="1">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>AV86</t>
+          <t>AV89</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -3172,12 +3170,14 @@
       <c r="E45" s="1" t="n"/>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>q1001ext[H]</t>
+          <t>q1001ext[E]</t>
         </is>
       </c>
       <c r="G45" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, MEA01.04 - Avaliar o desempenho: monitorar e avaliar periodicamente o desempenho e a conformidade da TI em relação a objetivos, indicadores, metas e expectativas das partes interessadas.</t>
+          <t>COBIT 2019, EDM01.02 - Dirigir o sistema de governança: orientar estruturas, princípios, processos e práticas de governança para assegurar que a TI apoie os objetivos organizacionais.
+Decreto nº 12.198/2024, arts. 5º e 6º, § 2º – Referência de governança digital: instituição, no âmbito da Administração Pública federal direta, autárquica e fundacional, de Comitê de Governança Digital ou colegiado equivalente com função deliberativa sobre ações de governo digital e uso de recursos de TIC, incluindo a aprovação dos instrumentos de planejamento previstos no Decreto.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.1, III.1 e V.1 – Precedente pela instituição e atuação efetiva de instância colegiada de governança de TIC, com responsabilidade pelo alinhamento das ações de TIC aos objetivos institucionais, priorização dos investimentos e monitoramento do desempenho da TIC.</t>
         </is>
       </c>
       <c r="H45" s="1" t="inlineStr">
@@ -3188,7 +3188,7 @@
       <c r="I45" s="1" t="n"/>
       <c r="J45" s="1" t="inlineStr">
         <is>
-          <t>Ausência de objetivos, indicadores ou metas para a gestão de TIC.</t>
+          <t>Comitê de TIC ou instância equivalente não instituído formalmente ou sem representação de áreas relevantes da organização.</t>
         </is>
       </c>
       <c r="K45" s="1" t="inlineStr">
@@ -3200,20 +3200,20 @@
       <c r="M45" s="1" t="n"/>
       <c r="N45" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O45" s="1" t="n"/>
       <c r="P45" s="1" t="inlineStr">
         <is>
-          <t>estabeleça objetivos, indicadores e metas para a gestão de TIC, de modo a possibilitar o acompanhamento periódico do desempenho da TIC pela alta administração</t>
+          <t>institua formalmente Comitê de TIC ou instância colegiada equivalente, compatível com o porte e a estrutura decisória da organização, definindo em seu ato constitutivo, minimamente, a participação de representantes de áreas relevantes da organização, suas competências, a periodicidade de reuniões, a forma de registro das deliberações e os mecanismos de acompanhamento dos encaminhamentos</t>
         </is>
       </c>
     </row>
     <row r="46" ht="113.45" customHeight="1">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>AV89</t>
+          <t>AV90</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -3244,7 +3244,7 @@
       <c r="I46" s="1" t="n"/>
       <c r="J46" s="1" t="inlineStr">
         <is>
-          <t>Comitê de TIC ou instância equivalente não instituído formalmente ou sem representação de áreas relevantes da organização.</t>
+          <t>Comitê de TIC ou instância equivalente sem atuação efetiva comprovada.</t>
         </is>
       </c>
       <c r="K46" s="1" t="inlineStr">
@@ -3262,14 +3262,14 @@
       <c r="O46" s="1" t="n"/>
       <c r="P46" s="1" t="inlineStr">
         <is>
-          <t>institua formalmente Comitê de TIC ou instância colegiada equivalente, compatível com o porte e a estrutura decisória da organização, definindo em seu ato constitutivo, minimamente, a participação de representantes de áreas relevantes da organização, suas competências, a periodicidade de reuniões, a forma de registro das deliberações e os mecanismos de acompanhamento dos encaminhamentos</t>
+          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância colegiada equivalente, mediante o exercício das competências previstas em seu ato constitutivo, com registro das deliberações e acompanhamento dos respectivos encaminhamentos</t>
         </is>
       </c>
     </row>
     <row r="47" ht="113.45" customHeight="1">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>AV90</t>
+          <t>AV91</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -3282,7 +3282,7 @@
       <c r="E47" s="1" t="n"/>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>q1001ext[E]</t>
+          <t>q1001ext[F]</t>
         </is>
       </c>
       <c r="G47" s="1" t="inlineStr">
@@ -3325,7 +3325,7 @@
     <row r="48" ht="113.45" customHeight="1">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>AV91</t>
+          <t>AV92</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -3338,14 +3338,14 @@
       <c r="E48" s="1" t="n"/>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>q1001ext[F]</t>
+          <t>q2101ext[A]</t>
         </is>
       </c>
       <c r="G48" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, EDM01.02 - Dirigir o sistema de governança: orientar estruturas, princípios, processos e práticas de governança para assegurar que a TI apoie os objetivos organizacionais.
-Decreto nº 12.198/2024, arts. 5º e 6º, § 2º – Referência de governança digital: instituição, no âmbito da Administração Pública federal direta, autárquica e fundacional, de Comitê de Governança Digital ou colegiado equivalente com função deliberativa sobre ações de governo digital e uso de recursos de TIC, incluindo a aprovação dos instrumentos de planejamento previstos no Decreto.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.1, III.1 e V.1 – Precedente pela instituição e atuação efetiva de instância colegiada de governança de TIC, com responsabilidade pelo alinhamento das ações de TIC aos objetivos institucionais, priorização dos investimentos e monitoramento do desempenho da TIC.</t>
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H48" s="1" t="inlineStr">
@@ -3356,7 +3356,7 @@
       <c r="I48" s="1" t="n"/>
       <c r="J48" s="1" t="inlineStr">
         <is>
-          <t>Comitê de TIC ou instância equivalente sem atuação efetiva comprovada.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="K48" s="1" t="inlineStr">
@@ -3374,14 +3374,14 @@
       <c r="O48" s="1" t="n"/>
       <c r="P48" s="1" t="inlineStr">
         <is>
-          <t>assegure o funcionamento efetivo do Comitê de TIC ou instância colegiada equivalente, mediante o exercício das competências previstas em seu ato constitutivo, com registro das deliberações e acompanhamento dos respectivos encaminhamentos</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades e participação das áreas demandantes</t>
         </is>
       </c>
     </row>
     <row r="49" ht="113.45" customHeight="1">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>AV92</t>
+          <t>AV95</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -3394,7 +3394,7 @@
       <c r="E49" s="1" t="n"/>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>q2101ext[A]</t>
+          <t>q2101ext[D]</t>
         </is>
       </c>
       <c r="G49" s="1" t="inlineStr">
@@ -3430,14 +3430,14 @@
       <c r="O49" s="1" t="n"/>
       <c r="P49" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades e participação das áreas demandantes</t>
         </is>
       </c>
     </row>
     <row r="50" ht="113.45" customHeight="1">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>AV93</t>
+          <t>AV96</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -3450,13 +3450,12 @@
       <c r="E50" s="1" t="n"/>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>q2101ext[B]</t>
+          <t>q2102ext[A]</t>
         </is>
       </c>
       <c r="G50" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+          <t>Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
 Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
@@ -3468,7 +3467,7 @@
       <c r="I50" s="1" t="n"/>
       <c r="J50" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
+          <t>Ausência de aprovação formal do plano de TIC.</t>
         </is>
       </c>
       <c r="K50" s="1" t="inlineStr">
@@ -3486,14 +3485,14 @@
       <c r="O50" s="1" t="n"/>
       <c r="P50" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>submeta o plano de TIC à aprovação formal do dirigente máximo ou de instância competente da alta administração, mantendo registro do respectivo ato de aprovação</t>
         </is>
       </c>
     </row>
     <row r="51" ht="113.45" customHeight="1">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>AV95</t>
+          <t>AV97</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -3506,7 +3505,7 @@
       <c r="E51" s="1" t="n"/>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>q2101ext[D]</t>
+          <t>q2102ext[D]</t>
         </is>
       </c>
       <c r="G51" s="1" t="inlineStr">
@@ -3524,7 +3523,7 @@
       <c r="I51" s="1" t="n"/>
       <c r="J51" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
+          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
         </is>
       </c>
       <c r="K51" s="1" t="inlineStr">
@@ -3542,14 +3541,14 @@
       <c r="O51" s="1" t="n"/>
       <c r="P51" s="1" t="inlineStr">
         <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
+          <t>revise o plano de TIC para explicitar seu alinhamento ao planejamento institucional, às diretrizes superiores e às necessidades das áreas finalísticas e administrativas, relacionando objetivos, iniciativas, indicadores e metas de TIC aos resultados institucionais pretendidos</t>
         </is>
       </c>
     </row>
     <row r="52" ht="113.45" customHeight="1">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>AV96</t>
+          <t>AV98</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -3562,12 +3561,12 @@
       <c r="E52" s="1" t="n"/>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>q2102ext[A]</t>
+          <t>q2102ext[C]</t>
         </is>
       </c>
       <c r="G52" s="1" t="inlineStr">
         <is>
-          <t>Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+          <t>COBIT 2019, APO06.03 - Criar e manter orçamentos: elaborar e manter orçamento de TIC alinhado ao portfólio, ao planejamento e às prioridades aprovadas.
 Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
@@ -3579,7 +3578,7 @@
       <c r="I52" s="1" t="n"/>
       <c r="J52" s="1" t="inlineStr">
         <is>
-          <t>Ausência de aprovação formal do plano de TIC.</t>
+          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
         </is>
       </c>
       <c r="K52" s="1" t="inlineStr">
@@ -3597,14 +3596,14 @@
       <c r="O52" s="1" t="n"/>
       <c r="P52" s="1" t="inlineStr">
         <is>
-          <t>submeta o plano de TIC à aprovação formal do dirigente máximo ou de instância competente da alta administração, mantendo registro do respectivo ato de aprovação</t>
+          <t>integre o plano de TIC à elaboração da proposta orçamentária e do plano de contratações, de maneira proporcional ao porte, à estrutura e à capacidade de planejamento da organização</t>
         </is>
       </c>
     </row>
     <row r="53" ht="113.45" customHeight="1">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>AV97</t>
+          <t>AV101</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -3617,14 +3616,12 @@
       <c r="E53" s="1" t="n"/>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>q2102ext[D]</t>
+          <t>q2102ext[E]</t>
         </is>
       </c>
       <c r="G53" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
+          <t>Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H53" s="1" t="inlineStr">
@@ -3635,7 +3632,7 @@
       <c r="I53" s="1" t="n"/>
       <c r="J53" s="1" t="inlineStr">
         <is>
-          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
+          <t>Ausência de acompanhamento da execução do plano de TIC.</t>
         </is>
       </c>
       <c r="K53" s="1" t="inlineStr">
@@ -3653,14 +3650,14 @@
       <c r="O53" s="1" t="n"/>
       <c r="P53" s="1" t="inlineStr">
         <is>
-          <t>revise o plano de TIC para explicitar seu alinhamento ao planejamento institucional, às diretrizes superiores e às necessidades das áreas finalísticas e administrativas, relacionando objetivos, iniciativas, indicadores e metas de TIC aos resultados institucionais pretendidos</t>
+          <t>estabeleça e execute rotina periódica de acompanhamento da execução do plano de TIC, promovendo sua revisão periódica e os ajustes ou atualizações necessários, com registro das principais decisões e reprogramações</t>
         </is>
       </c>
     </row>
     <row r="54" ht="113.45" customHeight="1">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>AV98</t>
+          <t>AV103</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -3673,13 +3670,13 @@
       <c r="E54" s="1" t="n"/>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>q2102ext[C]</t>
+          <t>q2703ext[C]</t>
         </is>
       </c>
       <c r="G54" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO06.03 - Criar e manter orçamentos: elaborar e manter orçamento de TIC alinhado ao portfólio, ao planejamento e às prioridades aprovadas.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
+          <t>COBIT 2019, APO07.05 - Planejar e monitorar o uso de recursos humanos de TI e de negócio: planejar, alocar e acompanhar capacidade de pessoal para iniciativas, operações e serviços de TIC.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6.5 - O PDTI deve contemplar o quantitativo necessário ou ideal para a força de trabalho em TI.</t>
         </is>
       </c>
       <c r="H54" s="1" t="inlineStr">
@@ -3690,7 +3687,7 @@
       <c r="I54" s="1" t="n"/>
       <c r="J54" s="1" t="inlineStr">
         <is>
-          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
+          <t>Ausência ou insuficiência de definição documentada do quantitativo necessário de pessoal de TIC e segurança da informação.</t>
         </is>
       </c>
       <c r="K54" s="1" t="inlineStr">
@@ -3702,20 +3699,20 @@
       <c r="M54" s="1" t="n"/>
       <c r="N54" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O54" s="1" t="n"/>
       <c r="P54" s="1" t="inlineStr">
         <is>
-          <t>integre o plano de TIC à elaboração da proposta orçamentária e do plano de contratações, de maneira proporcional ao porte, à estrutura e à capacidade de planejamento da organização</t>
+          <t>estime e mantenha atualizado o quantitativo necessário de pessoal de TIC e segurança da informação, considerando o porte e a complexidade da organização, os serviços críticos, os sistemas mantidos, as contratações vigentes e os riscos relevantes</t>
         </is>
       </c>
     </row>
     <row r="55" ht="113.45" customHeight="1">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>AV101</t>
+          <t>AV105</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -3728,12 +3725,13 @@
       <c r="E55" s="1" t="n"/>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>q2102ext[E]</t>
+          <t>q2708[B]</t>
         </is>
       </c>
       <c r="G55" s="1" t="inlineStr">
         <is>
-          <t>Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
+          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
+COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
         </is>
       </c>
       <c r="H55" s="1" t="inlineStr">
@@ -3744,7 +3742,7 @@
       <c r="I55" s="1" t="n"/>
       <c r="J55" s="1" t="inlineStr">
         <is>
-          <t>Ausência de acompanhamento da execução do plano de TIC.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="K55" s="1" t="inlineStr">
@@ -3756,20 +3754,20 @@
       <c r="M55" s="1" t="n"/>
       <c r="N55" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="O55" s="1" t="n"/>
       <c r="P55" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e execute rotina periódica de acompanhamento da execução do plano de TIC, promovendo sua revisão periódica e os ajustes ou atualizações necessários, com registro das principais decisões e reprogramações</t>
+          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
         </is>
       </c>
     </row>
     <row r="56" ht="113.45" customHeight="1">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>AV103</t>
+          <t>AV107</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -3782,13 +3780,13 @@
       <c r="E56" s="1" t="n"/>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>q2703ext[C]</t>
+          <t>q2708[D]</t>
         </is>
       </c>
       <c r="G56" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO07.05 - Planejar e monitorar o uso de recursos humanos de TI e de negócio: planejar, alocar e acompanhar capacidade de pessoal para iniciativas, operações e serviços de TIC.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6.5 - O PDTI deve contemplar o quantitativo necessário ou ideal para a força de trabalho em TI.</t>
+          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
+COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
         </is>
       </c>
       <c r="H56" s="1" t="inlineStr">
@@ -3799,7 +3797,7 @@
       <c r="I56" s="1" t="n"/>
       <c r="J56" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou insuficiência de definição documentada do quantitativo necessário de pessoal de TIC e segurança da informação.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="K56" s="1" t="inlineStr">
@@ -3817,14 +3815,14 @@
       <c r="O56" s="1" t="n"/>
       <c r="P56" s="1" t="inlineStr">
         <is>
-          <t>estime e mantenha atualizado o quantitativo necessário de pessoal de TIC e segurança da informação, considerando o porte e a complexidade da organização, os serviços críticos, os sistemas mantidos, as contratações vigentes e os riscos relevantes</t>
+          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
         </is>
       </c>
     </row>
     <row r="57" ht="90.95" customHeight="1">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>AV105</t>
+          <t>AV124</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -3837,13 +3835,13 @@
       <c r="E57" s="1" t="n"/>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>q2708[B]</t>
+          <t>q2201ext[A]</t>
         </is>
       </c>
       <c r="G57" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
-COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
+          <t>ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.7, III.9.7 e V.6.4 – Recomendações quanto à definição, pactuação e monitoramento de níveis de serviço.</t>
         </is>
       </c>
       <c r="H57" s="1" t="inlineStr">
@@ -3854,7 +3852,7 @@
       <c r="I57" s="1" t="n"/>
       <c r="J57" s="1" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="K57" s="1" t="inlineStr">
@@ -3872,14 +3870,14 @@
       <c r="O57" s="1" t="n"/>
       <c r="P57" s="1" t="inlineStr">
         <is>
-          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
+          <t>defina, acorde e monitore níveis de serviço para os serviços de TIC relevantes, estabelecendo metas e mecanismos de acompanhamento de seu cumprimento</t>
         </is>
       </c>
     </row>
     <row r="58" ht="90.95" customHeight="1">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>AV107</t>
+          <t>AV125</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -3892,13 +3890,14 @@
       <c r="E58" s="1" t="n"/>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>q2708[D]</t>
+          <t>q2201ext[B]</t>
         </is>
       </c>
       <c r="G58" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO01.05 - Estabelecer papéis e responsabilidades: definir, comunicar e manter papéis e responsabilidades relacionados à governança e gestão de TIC.
-COBIT 2019, APO07.01 - Adquirir e manter pessoal adequado e apropriado: assegurar quantidade e perfil de profissionais compatíveis com as necessidades de TIC.</t>
+          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.4, III.9.4 e V.6.1 – Recomendações quanto à estruturação do catálogo de serviços de TIC, incluindo descrição dos serviços, metas, formas de acesso e disponibilidade aos usuários.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.2.4 – Gerenciamento de catálogo de serviço: orienta que o catálogo descreva os serviços e seus resultados pretendidos, contenha informações relevantes para sua utilização e seja disponibilizado às partes interessadas que necessitem acessá-lo.</t>
         </is>
       </c>
       <c r="H58" s="1" t="inlineStr">
@@ -3909,7 +3908,7 @@
       <c r="I58" s="1" t="n"/>
       <c r="J58" s="1" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="K58" s="1" t="inlineStr">
@@ -3927,14 +3926,14 @@
       <c r="O58" s="1" t="n"/>
       <c r="P58" s="1" t="inlineStr">
         <is>
-          <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
+          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
         </is>
       </c>
     </row>
     <row r="59" ht="90.95" customHeight="1">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>AV124</t>
+          <t>AV126</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -3947,13 +3946,14 @@
       <c r="E59" s="1" t="n"/>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[A]</t>
+          <t>q2201ext[C]</t>
         </is>
       </c>
       <c r="G59" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.7, III.9.7 e V.6.4 – Recomendações quanto à definição, pactuação e monitoramento de níveis de serviço.</t>
+          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.4, III.9.4 e V.6.1 – Recomendações quanto à estruturação do catálogo de serviços de TIC, incluindo descrição dos serviços, metas, formas de acesso e disponibilidade aos usuários.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.2.4 – Gerenciamento de catálogo de serviço: orienta que o catálogo descreva os serviços e seus resultados pretendidos, contenha informações relevantes para sua utilização e seja disponibilizado às partes interessadas que necessitem acessá-lo.</t>
         </is>
       </c>
       <c r="H59" s="1" t="inlineStr">
@@ -3964,7 +3964,7 @@
       <c r="I59" s="1" t="n"/>
       <c r="J59" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="K59" s="1" t="inlineStr">
@@ -3982,14 +3982,14 @@
       <c r="O59" s="1" t="n"/>
       <c r="P59" s="1" t="inlineStr">
         <is>
-          <t>defina, acorde e monitore níveis de serviço para os serviços de TIC relevantes, estabelecendo metas e mecanismos de acompanhamento de seu cumprimento</t>
+          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
         </is>
       </c>
     </row>
     <row r="60" ht="79.90000000000001" customHeight="1">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>AV125</t>
+          <t>AV127</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -4002,14 +4002,13 @@
       <c r="E60" s="1" t="n"/>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[B]</t>
+          <t>q2201ext[D]</t>
         </is>
       </c>
       <c r="G60" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.4, III.9.4 e V.6.1 – Recomendações quanto à estruturação do catálogo de serviços de TIC, incluindo descrição dos serviços, metas, formas de acesso e disponibilidade aos usuários.
-ABNT NBR ISO/IEC 20000-2:2021, item 8.2.4 – Gerenciamento de catálogo de serviço: orienta que o catálogo descreva os serviços e seus resultados pretendidos, contenha informações relevantes para sua utilização e seja disponibilizado às partes interessadas que necessitem acessá-lo.</t>
+          <t>ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.7, III.9.7 e V.6.4 – Recomendações quanto à definição, pactuação e monitoramento de níveis de serviço.</t>
         </is>
       </c>
       <c r="H60" s="1" t="inlineStr">
@@ -4020,7 +4019,7 @@
       <c r="I60" s="1" t="n"/>
       <c r="J60" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="K60" s="1" t="inlineStr">
@@ -4038,14 +4037,14 @@
       <c r="O60" s="1" t="n"/>
       <c r="P60" s="1" t="inlineStr">
         <is>
-          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
+          <t>defina, acorde e monitore níveis de serviço para os serviços de TIC relevantes, estabelecendo metas e mecanismos de acompanhamento de seu cumprimento</t>
         </is>
       </c>
     </row>
     <row r="61" ht="79.90000000000001" customHeight="1">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>AV126</t>
+          <t>AV128</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -4058,14 +4057,13 @@
       <c r="E61" s="1" t="n"/>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[C]</t>
+          <t>q2201ext[E]</t>
         </is>
       </c>
       <c r="G61" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, APO09.02 - Catalogar serviços facilitados por TI: definir, manter e comunicar catálogo de serviços, incluindo serviços prestados, características, requisitos e níveis de serviço esperados.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.4, III.9.4 e V.6.1 – Recomendações quanto à estruturação do catálogo de serviços de TIC, incluindo descrição dos serviços, metas, formas de acesso e disponibilidade aos usuários.
-ABNT NBR ISO/IEC 20000-2:2021, item 8.2.4 – Gerenciamento de catálogo de serviço: orienta que o catálogo descreva os serviços e seus resultados pretendidos, contenha informações relevantes para sua utilização e seja disponibilizado às partes interessadas que necessitem acessá-lo.</t>
+          <t>ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.7, III.9.7 e V.6.4 – Recomendações quanto à definição, pactuação e monitoramento de níveis de serviço.</t>
         </is>
       </c>
       <c r="H61" s="1" t="inlineStr">
@@ -4076,7 +4074,7 @@
       <c r="I61" s="1" t="n"/>
       <c r="J61" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="K61" s="1" t="inlineStr">
@@ -4094,14 +4092,14 @@
       <c r="O61" s="1" t="n"/>
       <c r="P61" s="1" t="inlineStr">
         <is>
-          <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
+          <t>defina, acorde e monitore níveis de serviço para os serviços de TIC relevantes, estabelecendo metas e mecanismos de acompanhamento de seu cumprimento</t>
         </is>
       </c>
     </row>
     <row r="62" ht="90.95" customHeight="1">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>AV127</t>
+          <t>AV132</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -4114,13 +4112,13 @@
       <c r="E62" s="1" t="n"/>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[D]</t>
+          <t>q2504ext[A]</t>
         </is>
       </c>
       <c r="G62" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.7, III.9.7 e V.6.4 – Recomendações quanto à definição, pactuação e monitoramento de níveis de serviço.</t>
+          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.</t>
         </is>
       </c>
       <c r="H62" s="1" t="inlineStr">
@@ -4131,7 +4129,7 @@
       <c r="I62" s="1" t="n"/>
       <c r="J62" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
         </is>
       </c>
       <c r="K62" s="1" t="inlineStr">
@@ -4149,14 +4147,14 @@
       <c r="O62" s="1" t="n"/>
       <c r="P62" s="1" t="inlineStr">
         <is>
-          <t>defina, acorde e monitore níveis de serviço para os serviços de TIC relevantes, estabelecendo metas e mecanismos de acompanhamento de seu cumprimento</t>
+          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos sob gestão da organização, contemplando, minimamente, os dispositivos e softwares utilizados, com informações suficientes para sua identificação e controle</t>
         </is>
       </c>
     </row>
     <row r="63" ht="90.95" customHeight="1">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>AV128</t>
+          <t>AV133</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -4169,13 +4167,13 @@
       <c r="E63" s="1" t="n"/>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>q2201ext[E]</t>
+          <t>q2504ext[B]</t>
         </is>
       </c>
       <c r="G63" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de nível de serviço: definir, acordar, monitorar, avaliar e reportar metas e níveis de serviço alinhados às necessidades das áreas usuárias.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.7, III.9.7 e V.6.4 – Recomendações quanto à definição, pactuação e monitoramento de níveis de serviço.</t>
+          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.</t>
         </is>
       </c>
       <c r="H63" s="1" t="inlineStr">
@@ -4186,7 +4184,7 @@
       <c r="I63" s="1" t="n"/>
       <c r="J63" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
         </is>
       </c>
       <c r="K63" s="1" t="inlineStr">
@@ -4204,14 +4202,14 @@
       <c r="O63" s="1" t="n"/>
       <c r="P63" s="1" t="inlineStr">
         <is>
-          <t>defina, acorde e monitore níveis de serviço para os serviços de TIC relevantes, estabelecendo metas e mecanismos de acompanhamento de seu cumprimento</t>
+          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos sob gestão da organização, contemplando, minimamente, os dispositivos e softwares utilizados, com informações suficientes para sua identificação e controle</t>
         </is>
       </c>
     </row>
     <row r="64" ht="90.95" customHeight="1">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>AV132</t>
+          <t>AV134</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -4224,13 +4222,14 @@
       <c r="E64" s="1" t="n"/>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>q2504ext[A]</t>
+          <t>q2203ext[A]</t>
         </is>
       </c>
       <c r="G64" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.</t>
+          <t>COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.2.6 – Gerenciamento de configuração: orienta a identificação, o registro, o controle, o rastreamento e a verificação dos itens de configuração, bem como a manutenção de informações de configuração precisas relacionadas aos serviços.</t>
         </is>
       </c>
       <c r="H64" s="1" t="inlineStr">
@@ -4241,7 +4240,7 @@
       <c r="I64" s="1" t="n"/>
       <c r="J64" s="1" t="inlineStr">
         <is>
-          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="K64" s="1" t="inlineStr">
@@ -4259,14 +4258,14 @@
       <c r="O64" s="1" t="n"/>
       <c r="P64" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos sob gestão da organização, contemplando, minimamente, os dispositivos e softwares utilizados, com informações suficientes para sua identificação e controle</t>
+          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
         </is>
       </c>
     </row>
     <row r="65" ht="90.95" customHeight="1">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>AV133</t>
+          <t>AV136</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -4279,13 +4278,14 @@
       <c r="E65" s="1" t="n"/>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>q2504ext[B]</t>
+          <t>q2203ext[C]</t>
         </is>
       </c>
       <c r="G65" s="1" t="inlineStr">
         <is>
-          <t>ITIL 4, prática de gerenciamento de ativos de TI: planejar e gerenciar o ciclo de vida dos ativos de TI, mantendo informações suficientes para apoiar controle, custo, risco, valor e tomada de decisão.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.</t>
+          <t>COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.2.6 – Gerenciamento de configuração: orienta a identificação, o registro, o controle, o rastreamento e a verificação dos itens de configuração, bem como a manutenção de informações de configuração precisas relacionadas aos serviços.</t>
         </is>
       </c>
       <c r="H65" s="1" t="inlineStr">
@@ -4296,7 +4296,7 @@
       <c r="I65" s="1" t="n"/>
       <c r="J65" s="1" t="inlineStr">
         <is>
-          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="K65" s="1" t="inlineStr">
@@ -4314,14 +4314,14 @@
       <c r="O65" s="1" t="n"/>
       <c r="P65" s="1" t="inlineStr">
         <is>
-          <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos sob gestão da organização, contemplando, minimamente, os dispositivos e softwares utilizados, com informações suficientes para sua identificação e controle</t>
+          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
         </is>
       </c>
     </row>
     <row r="66" ht="90.95" customHeight="1">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>AV134</t>
+          <t>AV137</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -4334,14 +4334,14 @@
       <c r="E66" s="1" t="n"/>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>q2203ext[A]</t>
+          <t>q2204ext[A]</t>
         </is>
       </c>
       <c r="G66" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.
-ABNT NBR ISO/IEC 20000-2:2021, item 8.2.6 – Gerenciamento de configuração: orienta a identificação, o registro, o controle, o rastreamento e a verificação dos itens de configuração, bem como a manutenção de informações de configuração precisas relacionadas aos serviços.</t>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.6, III.9.6 e V.6.3 – Recomendações quanto à formalização e execução do processo de gestão de incidentes, incluindo registros, classificação, escalamento e tratamento.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.6.1 – Gerenciamento de incidente: orienta que os incidentes sejam registrados, classificados e priorizados, que as ações adotadas para sua resolução sejam registradas e rastreáveis e que sejam definidas responsabilidades para seu tratamento, incluindo procedimento documentado para incidentes graves.</t>
         </is>
       </c>
       <c r="H66" s="1" t="inlineStr">
@@ -4352,7 +4352,7 @@
       <c r="I66" s="1" t="n"/>
       <c r="J66" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="K66" s="1" t="inlineStr">
@@ -4370,14 +4370,14 @@
       <c r="O66" s="1" t="n"/>
       <c r="P66" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
     </row>
     <row r="67" ht="79.90000000000001" customHeight="1">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>AV136</t>
+          <t>AV140</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -4390,14 +4390,14 @@
       <c r="E67" s="1" t="n"/>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>q2203ext[C]</t>
+          <t>q2204ext[D]</t>
         </is>
       </c>
       <c r="G67" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, BAI10.01 - Estabelecer e manter um modelo de configuração: definir escopo, granularidade, atributos, relacionamentos e responsáveis pela base de configuração.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.5, III.9.5 e V.6.2 – Recomendações quanto à gestão de configuração e ativos de TIC, incluindo formalização do processo e manutenção de base consolidada de ativos e itens de configuração.
-ABNT NBR ISO/IEC 20000-2:2021, item 8.2.6 – Gerenciamento de configuração: orienta a identificação, o registro, o controle, o rastreamento e a verificação dos itens de configuração, bem como a manutenção de informações de configuração precisas relacionadas aos serviços.</t>
+          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.6, III.9.6 e V.6.3 – Recomendações quanto à formalização e execução do processo de gestão de incidentes, incluindo registros, classificação, escalamento e tratamento.
+ABNT NBR ISO/IEC 20000-2:2021, item 8.6.1 – Gerenciamento de incidente: orienta que os incidentes sejam registrados, classificados e priorizados, que as ações adotadas para sua resolução sejam registradas e rastreáveis e que sejam definidas responsabilidades para seu tratamento, incluindo procedimento documentado para incidentes graves.</t>
         </is>
       </c>
       <c r="H67" s="1" t="inlineStr">
@@ -4408,7 +4408,7 @@
       <c r="I67" s="1" t="n"/>
       <c r="J67" s="1" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="K67" s="1" t="inlineStr">
@@ -4426,14 +4426,14 @@
       <c r="O67" s="1" t="n"/>
       <c r="P67" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
+          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
     </row>
     <row r="68" ht="79.90000000000001" customHeight="1">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>AV137</t>
+          <t>AV141</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -4446,7 +4446,7 @@
       <c r="E68" s="1" t="n"/>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>q2204ext[A]</t>
+          <t>q2204ext[E]</t>
         </is>
       </c>
       <c r="G68" s="1" t="inlineStr">
@@ -4489,7 +4489,7 @@
     <row r="69" ht="79.90000000000001" customHeight="1">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>AV140</t>
+          <t>AV143</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -4502,14 +4502,14 @@
       <c r="E69" s="1" t="n"/>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>q2204ext[D]</t>
+          <t>q2801ext[A]</t>
         </is>
       </c>
       <c r="G69" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.6, III.9.6 e V.6.3 – Recomendações quanto à formalização e execução do processo de gestão de incidentes, incluindo registros, classificação, escalamento e tratamento.
-ABNT NBR ISO/IEC 20000-2:2021, item 8.6.1 – Gerenciamento de incidente: orienta que os incidentes sejam registrados, classificados e priorizados, que as ações adotadas para sua resolução sejam registradas e rastreáveis e que sejam definidas responsabilidades para seu tratamento, incluindo procedimento documentado para incidentes graves.</t>
+          <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+Lei nº 14.133/2021, art. 19, inciso IV: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.
+Acórdão nº 2.342/2016-TCU-Plenário, item 9.1.7 – Precedente quanto à definição, aprovação e formalização de processo de trabalho para o planejamento de cada contratação, com controles internos mínimos.</t>
         </is>
       </c>
       <c r="H69" s="1" t="inlineStr">
@@ -4520,7 +4520,7 @@
       <c r="I69" s="1" t="n"/>
       <c r="J69" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="K69" s="1" t="inlineStr">
@@ -4538,14 +4538,14 @@
       <c r="O69" s="1" t="n"/>
       <c r="P69" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
+          <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
         </is>
       </c>
     </row>
     <row r="70" ht="90.95" customHeight="1">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>AV141</t>
+          <t>AV148</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -4558,14 +4558,14 @@
       <c r="E70" s="1" t="n"/>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>q2204ext[E]</t>
+          <t>q2804[A]</t>
         </is>
       </c>
       <c r="G70" s="1" t="inlineStr">
         <is>
-          <t>COBIT 2019, DSS02.02, DSS02.04 e DSS02.07 - Requisições de serviço e incidentes gerenciados: registrar, classificar, priorizar, investigar, diagnosticar, resolver, acompanhar e reportar incidentes e requisições de serviço.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.7.6, III.9.6 e V.6.3 – Recomendações quanto à formalização e execução do processo de gestão de incidentes, incluindo registros, classificação, escalamento e tratamento.
-ABNT NBR ISO/IEC 20000-2:2021, item 8.6.1 – Gerenciamento de incidente: orienta que os incidentes sejam registrados, classificados e priorizados, que as ações adotadas para sua resolução sejam registradas e rastreáveis e que sejam definidas responsabilidades para seu tratamento, incluindo procedimento documentado para incidentes graves.</t>
+          <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
+COBIT 2019, BAI02.04 - Obter aprovação dos requisitos da solução: obter aprovação formal dos requisitos funcionais, técnicos, de segurança e de conformidade antes de prosseguir com a solução.
+Instrução Normativa SGD/ME nº 94/2022, arts. 2º, IV, 9º, 10, 11 e 12, §6º – referência de boa prática para estruturação da fase de planejamento das contratações de TIC, instituição da Equipe de Planejamento da Contratação e participação do integrante técnico da área de TIC, observada sua aplicação direta aos integrantes do SISP e as hipóteses de simplificação de procedimentos previstas na norma.</t>
         </is>
       </c>
       <c r="H70" s="1" t="inlineStr">
@@ -4576,7 +4576,7 @@
       <c r="I70" s="1" t="n"/>
       <c r="J70" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
         </is>
       </c>
       <c r="K70" s="1" t="inlineStr">
@@ -4594,19 +4594,19 @@
       <c r="O70" s="1" t="n"/>
       <c r="P70" s="1" t="inlineStr">
         <is>
-          <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
+          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo procedimentos simplificados e proporcionais à natureza, ao risco e ao valor da contratação, preservada análise técnica compatível</t>
         </is>
       </c>
     </row>
     <row r="71" ht="90.95" customHeight="1">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>AV143</t>
+          <t>AV152</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
-          <t>avaliacao_evidencias_ajustes</t>
+          <t>questionario</t>
         </is>
       </c>
       <c r="C71" s="1" t="n"/>
@@ -4614,7 +4614,7 @@
       <c r="E71" s="1" t="n"/>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>q2801ext[A]</t>
+          <t>q2801ext[B]</t>
         </is>
       </c>
       <c r="G71" s="1" t="inlineStr">
@@ -4626,7 +4626,7 @@
       </c>
       <c r="H71" s="1" t="inlineStr">
         <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+          <t>Resposta negativa ao detalhamento b) do item 2801 do Questionário, para verificar se são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
         </is>
       </c>
       <c r="I71" s="1" t="n"/>
@@ -4637,7 +4637,7 @@
       </c>
       <c r="K71" s="1" t="inlineStr">
         <is>
-          <t>Não conforme</t>
+          <t>(Não | N/A)</t>
         </is>
       </c>
       <c r="L71" s="1" t="n"/>
@@ -4657,7 +4657,7 @@
     <row r="72" ht="90.95" customHeight="1">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>AV148</t>
+          <t>AV153</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -4670,14 +4670,14 @@
       <c r="E72" s="1" t="n"/>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>q2804[A]</t>
+          <t>q2801ext[B]</t>
         </is>
       </c>
       <c r="G72" s="1" t="inlineStr">
         <is>
           <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-COBIT 2019, BAI02.04 - Obter aprovação dos requisitos da solução: obter aprovação formal dos requisitos funcionais, técnicos, de segurança e de conformidade antes de prosseguir com a solução.
-Instrução Normativa SGD/ME nº 94/2022, arts. 2º, IV, 9º, 10, 11 e 12, §6º – referência de boa prática para estruturação da fase de planejamento das contratações de TIC, instituição da Equipe de Planejamento da Contratação e participação do integrante técnico da área de TIC, observada sua aplicação direta aos integrantes do SISP e as hipóteses de simplificação de procedimentos previstas na norma.</t>
+Lei nº 14.133/2021, art. 19, inciso IV: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.
+Acórdão nº 2.342/2016-TCU-Plenário, item 9.1.7 – Precedente quanto à definição, aprovação e formalização de processo de trabalho para o planejamento de cada contratação, com controles internos mínimos.</t>
         </is>
       </c>
       <c r="H72" s="1" t="inlineStr">
@@ -4688,7 +4688,7 @@
       <c r="I72" s="1" t="n"/>
       <c r="J72" s="1" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="K72" s="1" t="inlineStr">
@@ -4706,14 +4706,14 @@
       <c r="O72" s="1" t="n"/>
       <c r="P72" s="1" t="inlineStr">
         <is>
-          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo procedimentos simplificados e proporcionais à natureza, ao risco e ao valor da contratação, preservada análise técnica compatível</t>
+          <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
         </is>
       </c>
     </row>
     <row r="73" ht="90.95" customHeight="1">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>AV152</t>
+          <t>AV154</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -4726,55 +4726,55 @@
       <c r="E73" s="1" t="n"/>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>q2801ext[B]</t>
+          <t>existe_plano_ti</t>
         </is>
       </c>
       <c r="G73" s="1" t="inlineStr">
         <is>
-          <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Lei nº 14.133/2021, art. 19, inciso IV: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.
-Acórdão nº 2.342/2016-TCU-Plenário, item 9.1.7 – Precedente quanto à definição, aprovação e formalização de processo de trabalho para o planejamento de cada contratação, com controles internos mínimos.</t>
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H73" s="1" t="inlineStr">
         <is>
-          <t>Resposta negativa ao detalhamento b) do item 2801 do Questionário, para verificar se são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+          <t>Resposta ao item 2102 que não caracteriza a existência de plano de TIC vigente, ainda que parcialmente adotado</t>
         </is>
       </c>
       <c r="I73" s="1" t="n"/>
       <c r="J73" s="1" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="K73" s="1" t="inlineStr">
         <is>
-          <t>(Não | N/A)</t>
+          <t>False</t>
         </is>
       </c>
       <c r="L73" s="1" t="n"/>
       <c r="M73" s="1" t="n"/>
       <c r="N73" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O73" s="1" t="n"/>
       <c r="P73" s="1" t="inlineStr">
         <is>
-          <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
+          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades e participação das áreas demandantes</t>
         </is>
       </c>
     </row>
     <row r="74" ht="90.95" customHeight="1">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>AV153</t>
+          <t>AV155</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
         <is>
-          <t>avaliacao_evidencias_ajustes</t>
+          <t>questionario</t>
         </is>
       </c>
       <c r="C74" s="1" t="n"/>
@@ -4782,154 +4782,44 @@
       <c r="E74" s="1" t="n"/>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>q2801ext[B]</t>
+          <t>existe_plano_ti</t>
         </is>
       </c>
       <c r="G74" s="1" t="inlineStr">
         <is>
-          <t>Lei nº 14.133/2021, art. 11, parágrafo único: responsabilidade da alta administração pela governança das contratações, com processos, estruturas, gestão de riscos e controles internos.
-Lei nº 14.133/2021, art. 19, inciso IV: instituição de modelos de minutas de editais, termos de referência, contratos padronizados e demais documentos.
-Acórdão nº 2.342/2016-TCU-Plenário, item 9.1.7 – Precedente quanto à definição, aprovação e formalização de processo de trabalho para o planejamento de cada contratação, com controles internos mínimos.</t>
+          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
+Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
+Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
         </is>
       </c>
       <c r="H74" s="1" t="inlineStr">
         <is>
-          <t>A organização declarou "{resposta_afirmada}" no {item_avaliado}, mas a evidência encaminhada foi considerada insuficiente para comprovar que {pratica}. Justificativa da avaliação: {avaliacao_justificativa}</t>
+          <t>Plano de TIC vigente declarado no item 2102, ao menos parcialmente adotado</t>
         </is>
       </c>
       <c r="I74" s="1" t="n"/>
-      <c r="J74" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
+      <c r="J74" s="1" t="n"/>
       <c r="K74" s="1" t="inlineStr">
         <is>
-          <t>Não conforme</t>
+          <t>True</t>
         </is>
       </c>
       <c r="L74" s="1" t="n"/>
       <c r="M74" s="1" t="n"/>
       <c r="N74" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="O74" s="1" t="n"/>
       <c r="P74" s="1" t="inlineStr">
         <is>
-          <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="90.95" customHeight="1">
-      <c r="A75" s="1" t="inlineStr">
-        <is>
-          <t>AV154</t>
-        </is>
-      </c>
-      <c r="B75" s="1" t="inlineStr">
-        <is>
-          <t>questionario</t>
-        </is>
-      </c>
-      <c r="C75" s="1" t="n"/>
-      <c r="D75" s="1" t="n"/>
-      <c r="E75" s="1" t="n"/>
-      <c r="F75" s="1" t="inlineStr">
-        <is>
-          <t>existe_plano_ti</t>
-        </is>
-      </c>
-      <c r="G75" s="1" t="inlineStr">
-        <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
-        </is>
-      </c>
-      <c r="H75" s="1" t="inlineStr">
-        <is>
-          <t>Resposta ao item 2102 que não caracteriza a existência de plano de TIC vigente, ainda que parcialmente adotado</t>
-        </is>
-      </c>
-      <c r="I75" s="1" t="n"/>
-      <c r="J75" s="1" t="inlineStr">
-        <is>
-          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
-        </is>
-      </c>
-      <c r="K75" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="L75" s="1" t="n"/>
-      <c r="M75" s="1" t="n"/>
-      <c r="N75" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O75" s="1" t="n"/>
-      <c r="P75" s="1" t="inlineStr">
-        <is>
           <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="102.2" customHeight="1">
-      <c r="A76" s="1" t="inlineStr">
-        <is>
-          <t>AV155</t>
-        </is>
-      </c>
-      <c r="B76" s="1" t="inlineStr">
-        <is>
-          <t>questionario</t>
-        </is>
-      </c>
-      <c r="C76" s="1" t="n"/>
-      <c r="D76" s="1" t="n"/>
-      <c r="E76" s="1" t="n"/>
-      <c r="F76" s="1" t="inlineStr">
-        <is>
-          <t>existe_plano_ti</t>
-        </is>
-      </c>
-      <c r="G76" s="1" t="inlineStr">
-        <is>
-          <t>COBIT 2019, APO02.05 - Definir o plano e o roteiro estratégico: estabelecer plano e roteiro de TIC que traduzam a estratégia em iniciativas, prioridades, recursos, dependências, prazos e benefícios esperados.
-Acórdão 1.411/2014-TCU-Plenário, item 9.1.6 e subitens 9.1.6.1 a 9.1.6.4: necessidade de instituir formalmente plano diretor de TI, contemplando desdobramento de diretrizes estratégicas, vinculação das ações de TI a indicadores e metas de negócio, vinculação das ações de TI a indicadores e metas de serviços ao cidadão e vinculação das ações priorizadas ao orçamento de TI.
-Acórdão TCE-RJ nº 44.490/2024-PLEN, itens II.3 e III.3 e respectivos subitens – Precedentes quanto ao estabelecimento formal de processo estruturado de planejamento de TIC, com participação das áreas relevantes, elaboração, manutenção e revisão periódica de PDTI, contemplando objetivos, indicadores e metas alinhados aos objetivos institucionais, riscos, projetos, aquisições, recursos necessários e ações de monitoramento após aprovação pela alta administração.</t>
-        </is>
-      </c>
-      <c r="H76" s="1" t="inlineStr">
-        <is>
-          <t>Plano de TIC vigente declarado no item 2102, ao menos parcialmente adotado</t>
-        </is>
-      </c>
-      <c r="I76" s="1" t="n"/>
-      <c r="J76" s="1" t="n"/>
-      <c r="K76" s="1" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="L76" s="1" t="n"/>
-      <c r="M76" s="1" t="n"/>
-      <c r="N76" s="1" t="inlineStr">
-        <is>
-          <t>Determinação</t>
-        </is>
-      </c>
-      <c r="O76" s="1" t="n"/>
-      <c r="P76" s="1" t="inlineStr">
-        <is>
-          <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades, participação das áreas demandantes e critérios de priorização das necessidades e iniciativas de TIC</t>
-        </is>
-      </c>
-    </row>
+    <row r="75" ht="90.95" customHeight="1"/>
+    <row r="76" ht="102.2" customHeight="1"/>
     <row r="77" ht="102.2" customHeight="1"/>
     <row r="78" ht="102.2" customHeight="1"/>
     <row r="79" ht="102.2" customHeight="1"/>
@@ -5021,7 +4911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H73"/>
+  <dimension ref="A2:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5767,7 +5657,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>MR024</t>
+          <t>MR028</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
@@ -5785,17 +5675,17 @@
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>AV15 &amp; ~AV93</t>
+          <t>AV17 &amp; ~AV95</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>AV15</t>
+          <t>AV17</t>
         </is>
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2101, não houve declaração afirmativa quanto à prática avaliada: estabeleceu critérios para orientar a seleção e a priorização das iniciativas de TI (projetos e ações) e os mantêm atualizados</t>
+          <t>No subitem d) do item 2101, não houve declaração afirmativa quanto à prática avaliada: o processo de planejamento de TI está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H21" s="9" t="b">
@@ -5805,7 +5695,7 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>MR025</t>
+          <t>MR029</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
@@ -5823,17 +5713,17 @@
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>AV93</t>
+          <t>AV95</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>AV93</t>
+          <t>AV95</t>
         </is>
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2101, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que estabeleceu critérios para orientar a seleção e a priorização das iniciativas de TI (projetos e ações) e os mantêm atualizados</t>
+          <t>No subitem d) do item 2101, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de planejamento de TI está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H22" s="9" t="b">
@@ -5843,7 +5733,7 @@
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>MR028</t>
+          <t>MR030</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
@@ -5853,25 +5743,25 @@
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
+          <t>Ausência de aprovação formal do plano de TIC.</t>
         </is>
       </c>
       <c r="D23" s="9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>AV17 &amp; ~AV95</t>
+          <t>AV155 &amp; AV18 &amp; ~AV96</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>AV17</t>
+          <t>AV18</t>
         </is>
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2101, não houve declaração afirmativa quanto à prática avaliada: o processo de planejamento de TI está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem a) do item 2102, não houve declaração afirmativa quanto à prática avaliada: o plano de tecnologia da informação (plano de TI) é aprovado pelo dirigente máximo da organização ou por dirigente ou colegiado que integra a alta administração</t>
         </is>
       </c>
       <c r="H23" s="9" t="b">
@@ -5881,7 +5771,7 @@
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>MR029</t>
+          <t>MR031</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
@@ -5891,25 +5781,25 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
+          <t>Ausência de aprovação formal do plano de TIC.</t>
         </is>
       </c>
       <c r="D24" s="9" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>AV95</t>
+          <t>AV96</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>AV95</t>
+          <t>AV96</t>
         </is>
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2101, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de planejamento de TI está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem a) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o plano de tecnologia da informação (plano de TI) é aprovado pelo dirigente máximo da organização ou por dirigente ou colegiado que integra a alta administração</t>
         </is>
       </c>
       <c r="H24" s="9" t="b">
@@ -5919,7 +5809,7 @@
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>MR030</t>
+          <t>MR032</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
@@ -5929,7 +5819,7 @@
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>Ausência de aprovação formal do plano de TIC.</t>
+          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
         </is>
       </c>
       <c r="D25" s="9" t="n">
@@ -5937,17 +5827,17 @@
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>AV155 &amp; AV18 &amp; ~AV96</t>
+          <t>AV155 &amp; AV19 &amp; ~AV97</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>AV18</t>
+          <t>AV19</t>
         </is>
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2102, não houve declaração afirmativa quanto à prática avaliada: o plano de tecnologia da informação (plano de TI) é aprovado pelo dirigente máximo da organização ou por dirigente ou colegiado que integra a alta administração</t>
+          <t>No subitem d) do item 2102, não houve declaração afirmativa quanto à prática avaliada: as iniciativas de TI (projetos e ações) constantes do plano de TI alinham-se aos objetivos e iniciativas definidos no planejamento institucional (como PPA, planos estratégicos, planos setoriais e plano de governo, no caso de municípios), bem como, quando aplicável, às estratégias e diretrizes estabelecidas por instâncias superiores de governança (como a Estratégia Nacional de Tecnologia da Informação e Comunicação do Poder Judiciário - ENTIC-JUD, normas e orientações do SETIC/PRODERJ (para órgãos estaduais) ou instâncias de governança equivalentes no âmbito municipal)</t>
         </is>
       </c>
       <c r="H25" s="9" t="b">
@@ -5957,7 +5847,7 @@
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>MR031</t>
+          <t>MR033</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
@@ -5967,7 +5857,7 @@
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Ausência de aprovação formal do plano de TIC.</t>
+          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
         </is>
       </c>
       <c r="D26" s="9" t="n">
@@ -5975,17 +5865,17 @@
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>AV96</t>
+          <t>AV97</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>AV96</t>
+          <t>AV97</t>
         </is>
       </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o plano de tecnologia da informação (plano de TI) é aprovado pelo dirigente máximo da organização ou por dirigente ou colegiado que integra a alta administração</t>
+          <t>No subitem d) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as iniciativas de TI (projetos e ações) constantes do plano de TI alinham-se aos objetivos e iniciativas definidos no planejamento institucional (como PPA, planos estratégicos, planos setoriais e plano de governo, no caso de municípios), bem como, quando aplicável, às estratégias e diretrizes estabelecidas por instâncias superiores de governança (como a Estratégia Nacional de Tecnologia da Informação e Comunicação do Poder Judiciário - ENTIC-JUD, normas e orientações do SETIC/PRODERJ (para órgãos estaduais) ou instâncias de governança equivalentes no âmbito municipal)</t>
         </is>
       </c>
       <c r="H26" s="9" t="b">
@@ -5995,7 +5885,7 @@
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>MR032</t>
+          <t>MR034</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
@@ -6005,7 +5895,7 @@
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
+          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
         </is>
       </c>
       <c r="D27" s="9" t="n">
@@ -6013,17 +5903,17 @@
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>AV155 &amp; AV19 &amp; ~AV97</t>
+          <t>AV155 &amp; AV20 &amp; ~AV98</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>AV19</t>
+          <t>AV20</t>
         </is>
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2102, não houve declaração afirmativa quanto à prática avaliada: as iniciativas de TI (projetos e ações) constantes do plano de TI alinham-se aos objetivos e iniciativas definidos no planejamento institucional (como PPA, planos estratégicos, planos setoriais e plano de governo, no caso de municípios), bem como, quando aplicável, às estratégias e diretrizes estabelecidas por instâncias superiores de governança (como a Estratégia Nacional de Tecnologia da Informação e Comunicação do Poder Judiciário - ENTIC-JUD, normas e orientações do SETIC/PRODERJ (para órgãos estaduais) ou instâncias de governança equivalentes no âmbito municipal)</t>
+          <t>No subitem c) do item 2102, não houve declaração afirmativa quanto à prática avaliada: o plano de TI fundamenta a proposta orçamentária da área de TI e o plano de contratações</t>
         </is>
       </c>
       <c r="H27" s="9" t="b">
@@ -6033,7 +5923,7 @@
     <row r="28" ht="45" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>MR033</t>
+          <t>MR035</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
@@ -6043,7 +5933,7 @@
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Plano de TIC sem alinhamento adequado ao planejamento institucional.</t>
+          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
         </is>
       </c>
       <c r="D28" s="9" t="n">
@@ -6051,17 +5941,17 @@
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>AV97</t>
+          <t>AV98</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>AV97</t>
+          <t>AV98</t>
         </is>
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as iniciativas de TI (projetos e ações) constantes do plano de TI alinham-se aos objetivos e iniciativas definidos no planejamento institucional (como PPA, planos estratégicos, planos setoriais e plano de governo, no caso de municípios), bem como, quando aplicável, às estratégias e diretrizes estabelecidas por instâncias superiores de governança (como a Estratégia Nacional de Tecnologia da Informação e Comunicação do Poder Judiciário - ENTIC-JUD, normas e orientações do SETIC/PRODERJ (para órgãos estaduais) ou instâncias de governança equivalentes no âmbito municipal)</t>
+          <t>No subitem c) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o plano de TI fundamenta a proposta orçamentária da área de TI e o plano de contratações</t>
         </is>
       </c>
       <c r="H28" s="9" t="b">
@@ -6071,7 +5961,7 @@
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>MR034</t>
+          <t>MR041</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
@@ -6081,7 +5971,7 @@
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
+          <t>Ausência de acompanhamento da execução do plano de TIC.</t>
         </is>
       </c>
       <c r="D29" s="9" t="n">
@@ -6089,17 +5979,17 @@
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>AV155 &amp; AV20 &amp; ~AV98</t>
+          <t>AV155 &amp; AV24 &amp; ~AV101</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>AV20</t>
+          <t>AV24</t>
         </is>
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2102, não houve declaração afirmativa quanto à prática avaliada: o plano de TI fundamenta a proposta orçamentária da área de TI e o plano de contratações</t>
+          <t>No subitem e) do item 2102, não houve declaração afirmativa quanto à prática avaliada: é feito acompanhamento concomitante à execução do plano de TI, com vistas a assegurar sua observância e possibilitar a realização de ajustes que se fizerem necessário</t>
         </is>
       </c>
       <c r="H29" s="9" t="b">
@@ -6109,7 +5999,7 @@
     <row r="30" ht="45" customHeight="1">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>MR035</t>
+          <t>MR042</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
@@ -6119,7 +6009,7 @@
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>Plano de TIC não utilizado como referência para a elaboração da proposta orçamentária e do plano de contratações.</t>
+          <t>Ausência de acompanhamento da execução do plano de TIC.</t>
         </is>
       </c>
       <c r="D30" s="9" t="n">
@@ -6127,17 +6017,17 @@
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>AV98</t>
+          <t>AV101</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>AV98</t>
+          <t>AV101</t>
         </is>
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o plano de TI fundamenta a proposta orçamentária da área de TI e o plano de contratações</t>
+          <t>No subitem e) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que é feito acompanhamento concomitante à execução do plano de TI, com vistas a assegurar sua observância e possibilitar a realização de ajustes que se fizerem necessário</t>
         </is>
       </c>
       <c r="H30" s="9" t="b">
@@ -6147,17 +6037,17 @@
     <row r="31" ht="45" customHeight="1">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>MR041</t>
+          <t>MR043</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>PA03</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>Ausência de acompanhamento da execução do plano de TIC.</t>
+          <t>Ausência de força de trabalho dedicada à TIC.</t>
         </is>
       </c>
       <c r="D31" s="9" t="n">
@@ -6165,17 +6055,17 @@
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>AV155 &amp; AV24 &amp; ~AV101</t>
+          <t>AV26 &amp; AV25</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>AV24</t>
+          <t>AV25</t>
         </is>
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2102, não houve declaração afirmativa quanto à prática avaliada: é feito acompanhamento concomitante à execução do plano de TI, com vistas a assegurar sua observância e possibilitar a realização de ajustes que se fizerem necessário</t>
+          <t>Item 0105: embora a organização tenha declarado estrutura formal de TIC no item 0101, informou não possuir profissionais atuando regularmente em tecnologia da informação</t>
         </is>
       </c>
       <c r="H31" s="9" t="b">
@@ -6185,35 +6075,35 @@
     <row r="32" ht="45" customHeight="1">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>MR042</t>
+          <t>MR045</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>PA03</t>
+          <t>PA04</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Ausência de acompanhamento da execução do plano de TIC.</t>
+          <t>Ausência ou insuficiência de definição documentada do quantitativo necessário de pessoal de TIC e segurança da informação.</t>
         </is>
       </c>
       <c r="D32" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>AV101</t>
+          <t>AV29 &amp; ~AV103</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>AV101</t>
+          <t>AV29</t>
         </is>
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2102, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que é feito acompanhamento concomitante à execução do plano de TI, com vistas a assegurar sua observância e possibilitar a realização de ajustes que se fizerem necessário</t>
+          <t>No subitem c) do item 2703, não houve declaração afirmativa quanto à prática avaliada: definiu-se, de maneira documentada, um quantitativo necessário de pessoal da área de tecnologia da informação e segurança da informação</t>
         </is>
       </c>
       <c r="H32" s="9" t="b">
@@ -6223,7 +6113,7 @@
     <row r="33" ht="45" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>MR043</t>
+          <t>MR046</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
@@ -6233,25 +6123,25 @@
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>Ausência de força de trabalho dedicada à TIC.</t>
+          <t>Ausência ou insuficiência de definição documentada do quantitativo necessário de pessoal de TIC e segurança da informação.</t>
         </is>
       </c>
       <c r="D33" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>AV26 &amp; AV25</t>
+          <t>AV103</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>AV25</t>
+          <t>AV103</t>
         </is>
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
-          <t>Item 0105: embora a organização tenha declarado estrutura formal de TIC no item 0101, informou não possuir profissionais atuando regularmente em tecnologia da informação</t>
+          <t>No subitem c) do item 2703, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu-se, de maneira documentada, um quantitativo necessário de pessoal da área de tecnologia da informação e segurança da informação</t>
         </is>
       </c>
       <c r="H33" s="9" t="b">
@@ -6261,7 +6151,7 @@
     <row r="34" ht="45" customHeight="1">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>MR045</t>
+          <t>MR047</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
@@ -6271,7 +6161,7 @@
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou insuficiência de definição documentada do quantitativo necessário de pessoal de TIC e segurança da informação.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="D34" s="9" t="n">
@@ -6279,17 +6169,17 @@
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>AV29 &amp; ~AV103</t>
+          <t>AV31 &amp; ~AV105</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>AV29</t>
+          <t>AV31</t>
         </is>
       </c>
       <c r="G34" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2703, não houve declaração afirmativa quanto à prática avaliada: definiu-se, de maneira documentada, um quantitativo necessário de pessoal da área de tecnologia da informação e segurança da informação</t>
+          <t>No subitem b) do item 2708, não houve declaração afirmativa quanto à prática avaliada: possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
         </is>
       </c>
       <c r="H34" s="9" t="b">
@@ -6299,7 +6189,7 @@
     <row r="35" ht="90" customHeight="1">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>MR046</t>
+          <t>MR048</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
@@ -6309,7 +6199,7 @@
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou insuficiência de definição documentada do quantitativo necessário de pessoal de TIC e segurança da informação.</t>
+          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
         </is>
       </c>
       <c r="D35" s="9" t="n">
@@ -6317,17 +6207,17 @@
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>AV103</t>
+          <t>AV105</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>AV103</t>
+          <t>AV105</t>
         </is>
       </c>
       <c r="G35" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2703, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu-se, de maneira documentada, um quantitativo necessário de pessoal da área de tecnologia da informação e segurança da informação</t>
+          <t>No subitem b) do item 2708, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
         </is>
       </c>
       <c r="H35" s="9" t="b">
@@ -6337,7 +6227,7 @@
     <row r="36" ht="105" customHeight="1">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>MR047</t>
+          <t>MR049</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
@@ -6351,21 +6241,21 @@
         </is>
       </c>
       <c r="D36" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>AV31 &amp; ~AV105</t>
+          <t>AV33 &amp; ~AV107</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>AV31</t>
+          <t>AV33</t>
         </is>
       </c>
       <c r="G36" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2708, não houve declaração afirmativa quanto à prática avaliada: possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
+          <t>No subitem d) do item 2708, não houve declaração afirmativa quanto à prática avaliada: possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
         </is>
       </c>
       <c r="H36" s="9" t="b">
@@ -6375,7 +6265,7 @@
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>MR048</t>
+          <t>MR050</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
@@ -6389,21 +6279,21 @@
         </is>
       </c>
       <c r="D37" s="9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>AV105</t>
+          <t>AV107</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>AV105</t>
+          <t>AV107</t>
         </is>
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2708, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
+          <t>No subitem d) do item 2708, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
         </is>
       </c>
       <c r="H37" s="9" t="b">
@@ -6413,7 +6303,7 @@
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>MR049</t>
+          <t>MR062</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
@@ -6423,25 +6313,25 @@
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Operação de TIC predominantemente terceirizada sem profissionais internos de TIC.</t>
         </is>
       </c>
       <c r="D38" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>AV33 &amp; ~AV107</t>
+          <t>AV45 &amp; AV46 &amp; ~AV25</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>AV33</t>
+          <t>AV45</t>
         </is>
       </c>
       <c r="G38" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2708, não houve declaração afirmativa quanto à prática avaliada: possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
+          <t>A organização informou modelo de operação de TIC com execução predominantemente terceirizada, o que levou à análise de sua capacidade interna de coordenação e fiscalização</t>
         </is>
       </c>
       <c r="H38" s="9" t="b">
@@ -6451,7 +6341,7 @@
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>MR050</t>
+          <t>MR063</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
@@ -6461,25 +6351,25 @@
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>Ausência de cargos ou funções formalmente atribuídos à TIC ou à segurança da informação.</t>
+          <t>Operação de TIC predominantemente terceirizada sem profissionais internos de TIC.</t>
         </is>
       </c>
       <c r="D39" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>AV107</t>
+          <t>AV45 &amp; AV46 &amp; ~AV25</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>AV107</t>
+          <t>AV46</t>
         </is>
       </c>
       <c r="G39" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2708, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
+          <t>Não foram identificados profissionais internos de TIC para coordenar e fiscalizar a execução das atividades de tecnologia da informação</t>
         </is>
       </c>
       <c r="H39" s="9" t="b">
@@ -6489,17 +6379,17 @@
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>MR062</t>
+          <t>MR065</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA05</t>
         </is>
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>Operação de TIC predominantemente terceirizada sem profissionais internos de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D40" s="9" t="n">
@@ -6507,17 +6397,17 @@
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>AV45 &amp; AV46</t>
+          <t>AV54 &amp; ~AV124</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>AV45</t>
+          <t>AV54</t>
         </is>
       </c>
       <c r="G40" s="9" t="inlineStr">
         <is>
-          <t>A organização informou modelo de operação de TIC com execução predominantemente terceirizada, o que levou à análise de sua capacidade interna de coordenação e fiscalização</t>
+          <t>No subitem a) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
         </is>
       </c>
       <c r="H40" s="9" t="b">
@@ -6527,35 +6417,35 @@
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>MR063</t>
+          <t>MR066</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
         <is>
-          <t>PA04</t>
+          <t>PA05</t>
         </is>
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>Operação de TIC predominantemente terceirizada sem profissionais internos de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D41" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>AV45 &amp; AV46</t>
+          <t>AV124</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>AV46</t>
+          <t>AV124</t>
         </is>
       </c>
       <c r="G41" s="9" t="inlineStr">
         <is>
-          <t>Não foram identificados profissionais internos de TIC para coordenar e fiscalizar a execução das atividades de tecnologia da informação</t>
+          <t>No subitem a) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
         </is>
       </c>
       <c r="H41" s="9" t="b">
@@ -6565,7 +6455,7 @@
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>MR065</t>
+          <t>MR067</t>
         </is>
       </c>
       <c r="B42" s="9" t="inlineStr">
@@ -6575,7 +6465,7 @@
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="D42" s="9" t="n">
@@ -6583,17 +6473,17 @@
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>AV54 &amp; ~AV124</t>
+          <t>AV55 &amp; ~AV125</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>AV54</t>
+          <t>AV55</t>
         </is>
       </c>
       <c r="G42" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
+          <t>No subitem b) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
         </is>
       </c>
       <c r="H42" s="9" t="b">
@@ -6603,7 +6493,7 @@
     <row r="43" ht="45" customHeight="1">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>MR066</t>
+          <t>MR068</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
@@ -6613,25 +6503,25 @@
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
         </is>
       </c>
       <c r="D43" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>AV124</t>
+          <t>AV125</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>AV124</t>
+          <t>AV125</t>
         </is>
       </c>
       <c r="G43" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
+          <t>No subitem b) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
         </is>
       </c>
       <c r="H43" s="9" t="b">
@@ -6641,7 +6531,7 @@
     <row r="44" ht="45" customHeight="1">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>MR067</t>
+          <t>MR069</t>
         </is>
       </c>
       <c r="B44" s="9" t="inlineStr">
@@ -6655,21 +6545,21 @@
         </is>
       </c>
       <c r="D44" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>AV55 &amp; ~AV125</t>
+          <t>AV56 &amp; ~AV126</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>AV55</t>
+          <t>AV56</t>
         </is>
       </c>
       <c r="G44" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
+          <t>No subitem c) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
         </is>
       </c>
       <c r="H44" s="9" t="b">
@@ -6679,7 +6569,7 @@
     <row r="45" ht="45" customHeight="1">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>MR068</t>
+          <t>MR070</t>
         </is>
       </c>
       <c r="B45" s="9" t="inlineStr">
@@ -6693,21 +6583,21 @@
         </is>
       </c>
       <c r="D45" s="9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>AV125</t>
+          <t>AV126</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>AV125</t>
+          <t>AV126</t>
         </is>
       </c>
       <c r="G45" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo está atualizado e as informações que nele constam são compatíveis com os Acordos de Níveis de Serviço (ANS) estabelecidos pela área de tecnologia da informação e as áreas de negócio da organização</t>
+          <t>No subitem c) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
         </is>
       </c>
       <c r="H45" s="9" t="b">
@@ -6717,7 +6607,7 @@
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>MR069</t>
+          <t>MR071</t>
         </is>
       </c>
       <c r="B46" s="9" t="inlineStr">
@@ -6727,25 +6617,25 @@
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D46" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>AV56 &amp; ~AV126</t>
+          <t>AV57 &amp; ~AV127</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>AV56</t>
+          <t>AV57</t>
         </is>
       </c>
       <c r="G46" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2201, não houve declaração afirmativa quanto à prática avaliada: o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
+          <t>No subitem d) do item 2201, não houve declaração afirmativa quanto à prática avaliada: são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
         </is>
       </c>
       <c r="H46" s="9" t="b">
@@ -6755,7 +6645,7 @@
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>MR070</t>
+          <t>MR072</t>
         </is>
       </c>
       <c r="B47" s="9" t="inlineStr">
@@ -6765,7 +6655,7 @@
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou insuficiência do catálogo de serviços de TIC.</t>
+          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
         </is>
       </c>
       <c r="D47" s="9" t="n">
@@ -6773,17 +6663,17 @@
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>AV126</t>
+          <t>AV127</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>AV126</t>
+          <t>AV127</t>
         </is>
       </c>
       <c r="G47" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o catálogo é de fácil acesso e está amplamente disponível a seus usuários e às equipes de suporte</t>
+          <t>No subitem d) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
         </is>
       </c>
       <c r="H47" s="9" t="b">
@@ -6793,7 +6683,7 @@
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>MR071</t>
+          <t>MR073</t>
         </is>
       </c>
       <c r="B48" s="9" t="inlineStr">
@@ -6807,21 +6697,21 @@
         </is>
       </c>
       <c r="D48" s="9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>AV57 &amp; ~AV127</t>
+          <t>AV58 &amp; ~AV128</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>AV57</t>
+          <t>AV58</t>
         </is>
       </c>
       <c r="G48" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2201, não houve declaração afirmativa quanto à prática avaliada: são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
+          <t>No subitem e) do item 2201, não houve declaração afirmativa quanto à prática avaliada: a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
         </is>
       </c>
       <c r="H48" s="9" t="b">
@@ -6831,7 +6721,7 @@
     <row r="49" ht="45" customHeight="1">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>MR072</t>
+          <t>MR074</t>
         </is>
       </c>
       <c r="B49" s="9" t="inlineStr">
@@ -6845,21 +6735,21 @@
         </is>
       </c>
       <c r="D49" s="9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>AV127</t>
+          <t>AV128</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>AV127</t>
+          <t>AV128</t>
         </is>
       </c>
       <c r="G49" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que são formalizados ANS contendo metas de nível de serviço acordadas com representantes das áreas de negócio clientes</t>
+          <t>No subitem e) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
         </is>
       </c>
       <c r="H49" s="9" t="b">
@@ -6869,7 +6759,7 @@
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>MR073</t>
+          <t>MR075</t>
         </is>
       </c>
       <c r="B50" s="9" t="inlineStr">
@@ -6879,25 +6769,25 @@
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="D50" s="9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>AV58 &amp; ~AV128</t>
+          <t>AV59 &amp; ~AV134</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>AV58</t>
+          <t>AV59</t>
         </is>
       </c>
       <c r="G50" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2201, não houve declaração afirmativa quanto à prática avaliada: a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
+          <t>No subitem a) do item 2203, não houve declaração afirmativa quanto à prática avaliada: mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
         </is>
       </c>
       <c r="H50" s="9" t="b">
@@ -6907,7 +6797,7 @@
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>MR074</t>
+          <t>MR077</t>
         </is>
       </c>
       <c r="B51" s="9" t="inlineStr">
@@ -6917,25 +6807,25 @@
       </c>
       <c r="C51" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade na definição e no monitoramento de níveis mínimos de serviço de TIC.</t>
+          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
         </is>
       </c>
       <c r="D51" s="9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>AV128</t>
+          <t>AV62 &amp; ~AV132</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>AV128</t>
+          <t>AV62</t>
         </is>
       </c>
       <c r="G51" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2201, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que a área de gestão de tecnologia da informação monitora continuamente o alcance dos níveis de serviço estabelecidos nos ANS</t>
+          <t>No subitem a) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H51" s="9" t="b">
@@ -6945,7 +6835,7 @@
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="9" t="inlineStr">
         <is>
-          <t>MR075</t>
+          <t>MR078</t>
         </is>
       </c>
       <c r="B52" s="9" t="inlineStr">
@@ -6955,25 +6845,25 @@
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
         </is>
       </c>
       <c r="D52" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>AV59 &amp; ~AV134</t>
+          <t>AV132</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>AV59</t>
+          <t>AV132</t>
         </is>
       </c>
       <c r="G52" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2203, não houve declaração afirmativa quanto à prática avaliada: mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
+          <t>No subitem a) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H52" s="9" t="b">
@@ -6983,7 +6873,7 @@
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>MR077</t>
+          <t>MR079</t>
         </is>
       </c>
       <c r="B53" s="9" t="inlineStr">
@@ -6997,21 +6887,21 @@
         </is>
       </c>
       <c r="D53" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>AV62 &amp; ~AV132</t>
+          <t>AV63 &amp; ~AV133</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>AV62</t>
+          <t>AV63</t>
         </is>
       </c>
       <c r="G53" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
+          <t>No subitem b) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H53" s="9" t="b">
@@ -7021,7 +6911,7 @@
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t>MR078</t>
+          <t>MR080</t>
         </is>
       </c>
       <c r="B54" s="9" t="inlineStr">
@@ -7035,21 +6925,21 @@
         </is>
       </c>
       <c r="D54" s="9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>AV132</t>
+          <t>AV133</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>AV132</t>
+          <t>AV133</t>
         </is>
       </c>
       <c r="G54" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
+          <t>No subitem b) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
         </is>
       </c>
       <c r="H54" s="9" t="b">
@@ -7059,7 +6949,7 @@
     <row r="55" ht="45" customHeight="1">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>MR079</t>
+          <t>MR082</t>
         </is>
       </c>
       <c r="B55" s="9" t="inlineStr">
@@ -7069,25 +6959,25 @@
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="D55" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>AV63 &amp; ~AV133</t>
+          <t>AV134</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>AV63</t>
+          <t>AV134</t>
         </is>
       </c>
       <c r="G55" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2504, não houve declaração afirmativa quanto à prática avaliada: gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
+          <t>No subitem a) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
         </is>
       </c>
       <c r="H55" s="9" t="b">
@@ -7097,7 +6987,7 @@
     <row r="56" ht="45" customHeight="1">
       <c r="A56" s="9" t="inlineStr">
         <is>
-          <t>MR080</t>
+          <t>MR083</t>
         </is>
       </c>
       <c r="B56" s="9" t="inlineStr">
@@ -7107,25 +6997,25 @@
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>Inventário e controle de dispositivos e softwares de TIC inexistente ou insuficiente.</t>
+          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
         </is>
       </c>
       <c r="D56" s="9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>AV133</t>
+          <t>AV66 &amp; ~AV136</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>AV133</t>
+          <t>AV66</t>
         </is>
       </c>
       <c r="G56" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2504, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que gerencia (inventaria e controla) os softwares instalados nos dispositivos conectados em sua rede</t>
+          <t>No subitem c) do item 2203, não houve declaração afirmativa quanto à prática avaliada: o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H56" s="9" t="b">
@@ -7135,7 +7025,7 @@
     <row r="57" ht="45" customHeight="1">
       <c r="A57" s="9" t="inlineStr">
         <is>
-          <t>MR082</t>
+          <t>MR084</t>
         </is>
       </c>
       <c r="B57" s="9" t="inlineStr">
@@ -7149,21 +7039,21 @@
         </is>
       </c>
       <c r="D57" s="9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>AV134</t>
+          <t>AV136</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>AV134</t>
+          <t>AV136</t>
         </is>
       </c>
       <c r="G57" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que mantém uma base de dados consolidada e atualizada com as configurações dos serviços e ativos de TI e o relacionamento entre eles</t>
+          <t>No subitem c) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H57" s="9" t="b">
@@ -7173,7 +7063,7 @@
     <row r="58" ht="45" customHeight="1">
       <c r="A58" s="9" t="inlineStr">
         <is>
-          <t>MR083</t>
+          <t>MR085</t>
         </is>
       </c>
       <c r="B58" s="9" t="inlineStr">
@@ -7183,25 +7073,25 @@
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="D58" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>AV66 &amp; ~AV136</t>
+          <t>AV67 &amp; ~AV137</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>AV66</t>
+          <t>AV67</t>
         </is>
       </c>
       <c r="G58" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2203, não houve declaração afirmativa quanto à prática avaliada: o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem a) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu regras para a priorização e o escalamento de incidentes</t>
         </is>
       </c>
       <c r="H58" s="9" t="b">
@@ -7211,7 +7101,7 @@
     <row r="59" ht="45" customHeight="1">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>MR084</t>
+          <t>MR086</t>
         </is>
       </c>
       <c r="B59" s="9" t="inlineStr">
@@ -7221,25 +7111,25 @@
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>Ausência ou fragilidade do processo de gestão de configuração.</t>
+          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
         </is>
       </c>
       <c r="D59" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>AV136</t>
+          <t>AV137</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>AV136</t>
+          <t>AV137</t>
         </is>
       </c>
       <c r="G59" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2203, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem a) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu regras para a priorização e o escalamento de incidentes</t>
         </is>
       </c>
       <c r="H59" s="9" t="b">
@@ -7249,7 +7139,7 @@
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="9" t="inlineStr">
         <is>
-          <t>MR085</t>
+          <t>MR087</t>
         </is>
       </c>
       <c r="B60" s="9" t="inlineStr">
@@ -7263,21 +7153,21 @@
         </is>
       </c>
       <c r="D60" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>AV67 &amp; ~AV137</t>
+          <t>AV70 &amp; ~AV140</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>AV67</t>
+          <t>AV70</t>
         </is>
       </c>
       <c r="G60" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu regras para a priorização e o escalamento de incidentes</t>
+          <t>No subitem d) do item 2204, não houve declaração afirmativa quanto à prática avaliada: o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H60" s="9" t="b">
@@ -7287,7 +7177,7 @@
     <row r="61" ht="45" customHeight="1">
       <c r="A61" s="9" t="inlineStr">
         <is>
-          <t>MR086</t>
+          <t>MR088</t>
         </is>
       </c>
       <c r="B61" s="9" t="inlineStr">
@@ -7301,21 +7191,21 @@
         </is>
       </c>
       <c r="D61" s="9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>AV137</t>
+          <t>AV140</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>AV137</t>
+          <t>AV140</t>
         </is>
       </c>
       <c r="G61" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu regras para a priorização e o escalamento de incidentes</t>
+          <t>No subitem d) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
       <c r="H61" s="9" t="b">
@@ -7325,7 +7215,7 @@
     <row r="62" ht="45" customHeight="1">
       <c r="A62" s="9" t="inlineStr">
         <is>
-          <t>MR087</t>
+          <t>MR089</t>
         </is>
       </c>
       <c r="B62" s="9" t="inlineStr">
@@ -7339,21 +7229,21 @@
         </is>
       </c>
       <c r="D62" s="9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>AV70 &amp; ~AV140</t>
+          <t>AV71 &amp; ~AV141</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>AV70</t>
+          <t>AV71</t>
         </is>
       </c>
       <c r="G62" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2204, não houve declaração afirmativa quanto à prática avaliada: o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem e) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
         </is>
       </c>
       <c r="H62" s="9" t="b">
@@ -7363,7 +7253,7 @@
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>MR088</t>
+          <t>MR090</t>
         </is>
       </c>
       <c r="B63" s="9" t="inlineStr">
@@ -7377,21 +7267,21 @@
         </is>
       </c>
       <c r="D63" s="9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>AV140</t>
+          <t>AV141</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>AV140</t>
+          <t>AV141</t>
         </is>
       </c>
       <c r="G63" s="9" t="inlineStr">
         <is>
-          <t>No subitem d) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o(s) processo(s) de gestão de incidentes está(ão) formalizado(s) (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
+          <t>No subitem e) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
         </is>
       </c>
       <c r="H63" s="9" t="b">
@@ -7401,35 +7291,35 @@
     <row r="64" ht="45" customHeight="1">
       <c r="A64" s="9" t="inlineStr">
         <is>
-          <t>MR089</t>
+          <t>MR091</t>
         </is>
       </c>
       <c r="B64" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D64" s="9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>AV71 &amp; ~AV141</t>
+          <t>AV73 &amp; ~AV143</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>AV71</t>
+          <t>AV73</t>
         </is>
       </c>
       <c r="G64" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2204, não houve declaração afirmativa quanto à prática avaliada: definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
+          <t>No subitem a) do item 2801, não houve declaração afirmativa quanto à prática avaliada: o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
         </is>
       </c>
       <c r="H64" s="9" t="b">
@@ -7439,35 +7329,35 @@
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="9" t="inlineStr">
         <is>
-          <t>MR090</t>
+          <t>MR092</t>
         </is>
       </c>
       <c r="B65" s="9" t="inlineStr">
         <is>
-          <t>PA05</t>
+          <t>PA06</t>
         </is>
       </c>
       <c r="C65" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade do processo de gestão de incidentes de TIC.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D65" s="9" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>AV141</t>
+          <t>AV143</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>AV141</t>
+          <t>AV143</t>
         </is>
       </c>
       <c r="G65" s="9" t="inlineStr">
         <is>
-          <t>No subitem e) do item 2204, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que definiu procedimentos e responsabilidades quanto à notificação e ao tratamento das notificações de incidentes de segurança da informação, bem como quanto à adoção de ações emergenciais, diretrizes para escalamento e comunicação interna e externa</t>
+          <t>No subitem a) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
         </is>
       </c>
       <c r="H65" s="9" t="b">
@@ -7477,7 +7367,7 @@
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="9" t="inlineStr">
         <is>
-          <t>MR091</t>
+          <t>MR101</t>
         </is>
       </c>
       <c r="B66" s="9" t="inlineStr">
@@ -7487,7 +7377,7 @@
       </c>
       <c r="C66" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
         </is>
       </c>
       <c r="D66" s="9" t="n">
@@ -7495,17 +7385,17 @@
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>AV73 &amp; ~AV143</t>
+          <t>AV78 &amp; ~AV148</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>AV73</t>
+          <t>AV78</t>
         </is>
       </c>
       <c r="G66" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2801, não houve declaração afirmativa quanto à prática avaliada: o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
+          <t>No subitem a) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
         </is>
       </c>
       <c r="H66" s="9" t="b">
@@ -7515,7 +7405,7 @@
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="9" t="inlineStr">
         <is>
-          <t>MR092</t>
+          <t>MR102</t>
         </is>
       </c>
       <c r="B67" s="9" t="inlineStr">
@@ -7525,25 +7415,25 @@
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
+          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
         </is>
       </c>
       <c r="D67" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>AV143</t>
+          <t>AV148</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>AV143</t>
+          <t>AV148</t>
         </is>
       </c>
       <c r="G67" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2801, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que o processo de trabalho para o planejamento das contratações de TI contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
+          <t>No subitem a) do item 2804, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
         </is>
       </c>
       <c r="H67" s="9" t="b">
@@ -7553,7 +7443,7 @@
     <row r="68" ht="45" customHeight="1">
       <c r="A68" s="9" t="inlineStr">
         <is>
-          <t>MR101</t>
+          <t>MR109</t>
         </is>
       </c>
       <c r="B68" s="9" t="inlineStr">
@@ -7563,7 +7453,7 @@
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
+          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
         </is>
       </c>
       <c r="D68" s="9" t="n">
@@ -7571,17 +7461,17 @@
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>AV78 &amp; ~AV148</t>
+          <t>AV82</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>AV78</t>
+          <t>AV82</t>
         </is>
       </c>
       <c r="G68" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
+          <t>No subitem b) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de TI executadas no exercício encontram-se previamente estabelecidas nos instrumentos de planejamento vigentes (PDTI/PEDTIC e PCA)</t>
         </is>
       </c>
       <c r="H68" s="9" t="b">
@@ -7591,7 +7481,7 @@
     <row r="69" ht="60" customHeight="1">
       <c r="A69" s="9" t="inlineStr">
         <is>
-          <t>MR102</t>
+          <t>MR110</t>
         </is>
       </c>
       <c r="B69" s="9" t="inlineStr">
@@ -7601,25 +7491,25 @@
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem análise prévia e aprovação técnica da área de TIC.</t>
+          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
         </is>
       </c>
       <c r="D69" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>AV148</t>
+          <t>AV83</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>AV148</t>
+          <t>AV83</t>
         </is>
       </c>
       <c r="G69" s="9" t="inlineStr">
         <is>
-          <t>No subitem a) do item 2804, a organização declarou a prática avaliada, mas a evidência foi insuficiente para comprovar que as contratações de soluções de TI, independentemente de qual seja a área demandante, são obrigatoriamente submetidas à análise prévia e aprovação técnica da área de gestão de TI</t>
+          <t>No subitem c) do item 2804, não houve declaração afirmativa quanto à prática avaliada: a fase de planejamento de cada contratação de TI é conduzida por uma Equipe de Planejamento da Contratação formalmente designada (composta, minimamente, por integrante requisitante e integrante técnico da área de TI)</t>
         </is>
       </c>
       <c r="H69" s="9" t="b">
@@ -7629,7 +7519,7 @@
     <row r="70" ht="45" customHeight="1">
       <c r="A70" s="9" t="inlineStr">
         <is>
-          <t>MR109</t>
+          <t>MR111</t>
         </is>
       </c>
       <c r="B70" s="9" t="inlineStr">
@@ -7639,25 +7529,25 @@
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem alinhamento ao planejamento de TIC e ao Plano de Contratações Anual.</t>
+          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
         </is>
       </c>
       <c r="D70" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>AV82</t>
+          <t>AV152 &amp; ~AV153</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>AV82</t>
+          <t>AV152</t>
         </is>
       </c>
       <c r="G70" s="9" t="inlineStr">
         <is>
-          <t>No subitem b) do item 2804, não houve declaração afirmativa quanto à prática avaliada: as contratações de TI executadas no exercício encontram-se previamente estabelecidas nos instrumentos de planejamento vigentes (PDTI/PEDTIC e PCA)</t>
+          <t>No subitem b) do item 2801, não houve declaração afirmativa quanto à prática avaliada: são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
         </is>
       </c>
       <c r="H70" s="9" t="b">
@@ -7667,117 +7557,43 @@
     <row r="71" ht="45" customHeight="1">
       <c r="A71" s="9" t="inlineStr">
         <is>
-          <t>MR110</t>
+          <t>MR113</t>
         </is>
       </c>
       <c r="B71" s="9" t="inlineStr">
         <is>
-          <t>PA06</t>
+          <t>PA03</t>
         </is>
       </c>
       <c r="C71" s="9" t="inlineStr">
         <is>
-          <t>Contratações de TIC sem designação de equipe de planejamento com integrante técnico da área de TIC.</t>
+          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
         </is>
       </c>
       <c r="D71" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>AV83</t>
+          <t>AV154</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>AV83</t>
+          <t>AV154</t>
         </is>
       </c>
       <c r="G71" s="9" t="inlineStr">
         <is>
-          <t>No subitem c) do item 2804, não houve declaração afirmativa quanto à prática avaliada: a fase de planejamento de cada contratação de TI é conduzida por uma Equipe de Planejamento da Contratação formalmente designada (composta, minimamente, por integrante requisitante e integrante técnico da área de TI)</t>
+          <t>No item 2102, a organização não declarou possuir plano de tecnologia da informação vigente, ainda que parcialmente adotado</t>
         </is>
       </c>
       <c r="H71" s="9" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="72" ht="30" customHeight="1">
-      <c r="A72" s="9" t="inlineStr">
-        <is>
-          <t>MR111</t>
-        </is>
-      </c>
-      <c r="B72" s="9" t="inlineStr">
-        <is>
-          <t>PA06</t>
-        </is>
-      </c>
-      <c r="C72" s="9" t="inlineStr">
-        <is>
-          <t>Inexistência ou fragilidade de processo formal e padronizado para o planejamento das contratações de TIC.</t>
-        </is>
-      </c>
-      <c r="D72" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E72" s="9" t="inlineStr">
-        <is>
-          <t>AV152 &amp; ~AV153</t>
-        </is>
-      </c>
-      <c r="F72" s="9" t="inlineStr">
-        <is>
-          <t>AV152</t>
-        </is>
-      </c>
-      <c r="G72" s="9" t="inlineStr">
-        <is>
-          <t>No subitem b) do item 2801, não houve declaração afirmativa quanto à prática avaliada: são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI, como Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR), Matriz de Riscos ou documentos equivalentes</t>
-        </is>
-      </c>
-      <c r="H72" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="73" ht="30" customHeight="1">
-      <c r="A73" s="9" t="inlineStr">
-        <is>
-          <t>MR113</t>
-        </is>
-      </c>
-      <c r="B73" s="9" t="inlineStr">
-        <is>
-          <t>PA03</t>
-        </is>
-      </c>
-      <c r="C73" s="9" t="inlineStr">
-        <is>
-          <t>Inexistência ou insuficiência do processo de planejamento de TIC para produzir e manter plano de TIC adequado.</t>
-        </is>
-      </c>
-      <c r="D73" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E73" s="9" t="inlineStr">
-        <is>
-          <t>AV154</t>
-        </is>
-      </c>
-      <c r="F73" s="9" t="inlineStr">
-        <is>
-          <t>AV154</t>
-        </is>
-      </c>
-      <c r="G73" s="9" t="inlineStr">
-        <is>
-          <t>No item 2102, a organização não declarou possuir plano de tecnologia da informação vigente, ainda que parcialmente adotado</t>
-        </is>
-      </c>
-      <c r="H73" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
+    <row r="72" ht="30" customHeight="1"/>
+    <row r="73" ht="30" customHeight="1"/>
     <row r="74" ht="30" customHeight="1"/>
     <row r="75" ht="45" customHeight="1"/>
     <row r="76" ht="30" customHeight="1"/>

</xml_diff>

<commit_message>
Integra critérios específicos aos relatórios finais
</commit_message>
<xml_diff>
--- a/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
+++ b/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
@@ -21,7 +21,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Motivos do Relatório'!$A$3:$H$74</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Variáveis Temporárias'!$A$3:$E$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Critérios de Auditoria'!$A$3:$L$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Variantes de Encaminhamento'!$A$3:$L$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Variantes de Encaminhamento'!$A$3:$M$3</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
@@ -8475,7 +8475,7 @@
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>Decreto Estadual nº 47.278/2020, art. 6º — o nível setorial do SETIC deve ser representado por assessoria de informática ou setor equivalente em cada órgão ou entidade da Administração Direta e Indireta do Poder Executivo Estadual e exercer as competências de TIC previstas no dispositivo.</t>
+          <t>Decreto Estadual nº 48.997/2024, art. 4º — o nível setorial do SETIC deve ser representado por assessoria de informática ou setor equivalente em cada órgão ou entidade da Administração Direta e Indireta do Poder Executivo Estadual e exercer as competências de TIC previstas no dispositivo.</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
@@ -10415,7 +10415,7 @@
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>Decreto Estadual nº 47.278/2020, art. 6º, inciso V — os níveis setoriais de TIC devem manter e informar inventário permanente de equipamentos, licenças e softwares utilizados.</t>
+          <t>Decreto Estadual nº 48.997/2024, art. 4º, inciso V — o nível setorial deve alimentar as bases de dados do nível de Direção Geral com o inventário permanente de equipamentos, licenças e softwares utilizados.</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
@@ -11311,7 +11311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L74"/>
+  <dimension ref="A1:M74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -11326,6 +11326,7 @@
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
     <col width="60" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11393,6 +11394,11 @@
         </is>
       </c>
       <c r="L3" s="11" t="inlineStr">
+        <is>
+          <t>fundamentacao_encaminhamento</t>
+        </is>
+      </c>
+      <c r="M3" s="11" t="inlineStr">
         <is>
           <t>encaminhamento</t>
         </is>
@@ -11434,6 +11440,11 @@
       </c>
       <c r="L4" s="1" t="inlineStr">
         <is>
+          <t>alinhando-se à prática APO01.04 (Definir e implementar as estruturas organizacionais) do COBIT 2019 e ao princípio da eficiência previsto no art. 37, caput, da Constituição Federal</t>
+        </is>
+      </c>
+      <c r="M4" s="1" t="inlineStr">
+        <is>
           <t>formalize a área, unidade, setor ou função de TIC em instrumento compatível com a organização, definindo vinculação e responsabilidades essenciais de modo compatível com o porte, a complexidade e a dependência tecnológica da organização</t>
         </is>
       </c>
@@ -11478,6 +11489,11 @@
       </c>
       <c r="L5" s="1" t="inlineStr">
         <is>
+          <t>alinhando-se à prática APO01.04 (Definir e implementar as estruturas organizacionais) do COBIT 2019 e em observância ao art. 4º do Decreto Estadual nº 48.997/2024</t>
+        </is>
+      </c>
+      <c r="M5" s="1" t="inlineStr">
+        <is>
           <t>formalize a área, unidade, setor ou função de TIC em instrumento compatível com a organização, definindo vinculação e responsabilidades essenciais de modo compatível com o porte, a complexidade e a dependência tecnológica da organização</t>
         </is>
       </c>
@@ -11522,6 +11538,11 @@
       </c>
       <c r="L6" s="1" t="inlineStr">
         <is>
+          <t>alinhando-se à prática APO01.04 (Definir e implementar as estruturas organizacionais) do COBIT 2019 e em observância ao art. 21 da Resolução CNJ nº 370/2021</t>
+        </is>
+      </c>
+      <c r="M6" s="1" t="inlineStr">
+        <is>
           <t>formalize a área, unidade, setor ou função de TIC em instrumento compatível com a organização, definindo vinculação e responsabilidades essenciais de modo compatível com o porte, a complexidade e a dependência tecnológica da organização</t>
         </is>
       </c>
@@ -11565,6 +11586,11 @@
         </is>
       </c>
       <c r="L7" s="1" t="inlineStr">
+        <is>
+          <t>alinhando-se à prática APO01.04 (Definir e implementar as estruturas organizacionais) do COBIT 2019 e em observância ao art. 16 da Resolução CNMP nº 171/2017</t>
+        </is>
+      </c>
+      <c r="M7" s="1" t="inlineStr">
         <is>
           <t>formalize a área, unidade, setor ou função de TIC em instrumento compatível com a organização, definindo vinculação e responsabilidades essenciais de modo compatível com o porte, a complexidade e a dependência tecnológica da organização</t>
         </is>
@@ -11606,6 +11632,11 @@
       </c>
       <c r="L8" s="1" t="inlineStr">
         <is>
+          <t>alinhando-se à prática APO01.05 (Estabelecer papéis e responsabilidades) do COBIT 2019 e ao princípio da eficiência previsto no art. 37, caput, da Constituição Federal</t>
+        </is>
+      </c>
+      <c r="M8" s="1" t="inlineStr">
+        <is>
           <t>defina formalmente as atribuições da área de TIC, atentando-se, minimamente, em abranger as atividades de planejamento, coordenação, gestão e controle da TIC</t>
         </is>
       </c>
@@ -11650,6 +11681,11 @@
       </c>
       <c r="L9" s="1" t="inlineStr">
         <is>
+          <t>alinhando-se à prática APO01.05 (Estabelecer papéis e responsabilidades) do COBIT 2019 e em observância ao art. 4º do Decreto Estadual nº 48.997/2024</t>
+        </is>
+      </c>
+      <c r="M9" s="1" t="inlineStr">
+        <is>
           <t>defina formalmente as atribuições da área de TIC, atentando-se, minimamente, em abranger as atividades de planejamento, coordenação, gestão e controle da TIC</t>
         </is>
       </c>
@@ -11694,6 +11730,11 @@
       </c>
       <c r="L10" s="1" t="inlineStr">
         <is>
+          <t>alinhando-se à prática APO01.05 (Estabelecer papéis e responsabilidades) do COBIT 2019 e em observância ao art. 21 da Resolução CNJ nº 370/2021</t>
+        </is>
+      </c>
+      <c r="M10" s="1" t="inlineStr">
+        <is>
           <t>defina formalmente as atribuições da área de TIC, atentando-se, minimamente, em abranger as atividades de planejamento, coordenação, gestão e controle da TIC</t>
         </is>
       </c>
@@ -11737,6 +11778,11 @@
         </is>
       </c>
       <c r="L11" s="1" t="inlineStr">
+        <is>
+          <t>alinhando-se à prática APO01.05 (Estabelecer papéis e responsabilidades) do COBIT 2019 e em observância ao art. 16 da Resolução CNMP nº 171/2017</t>
+        </is>
+      </c>
+      <c r="M11" s="1" t="inlineStr">
         <is>
           <t>defina formalmente as atribuições da área de TIC, atentando-se, minimamente, em abranger as atividades de planejamento, coordenação, gestão e controle da TIC</t>
         </is>
@@ -11778,6 +11824,11 @@
       </c>
       <c r="L12" s="1" t="inlineStr">
         <is>
+          <t>alinhando-se à prática APO01.06 (Aprimorar o posicionamento da função de TI) do COBIT 2019 e à referência de posicionamento prevista no art. 4º, § 1º, da Portaria SGD/ME nº 778/2019</t>
+        </is>
+      </c>
+      <c r="M12" s="1" t="inlineStr">
+        <is>
           <t>avalie o posicionamento organizacional da área de TIC e adote, quando necessário, medidas para assegurar interlocução adequada com a alta administração e participação nas decisões estratégicas, orçamentárias, contratuais e de gestão de riscos relacionadas à tecnologia da informação.</t>
         </is>
       </c>
@@ -11821,6 +11872,11 @@
         </is>
       </c>
       <c r="L13" s="1" t="inlineStr">
+        <is>
+          <t>alinhando-se à prática APO01.06 (Aprimorar o posicionamento da função de TI) do COBIT 2019 e em observância ao art. 1º da Resolução GPGJ nº 2.675/2025</t>
+        </is>
+      </c>
+      <c r="M13" s="1" t="inlineStr">
         <is>
           <t>avalie o posicionamento organizacional da área de TIC e adote, quando necessário, medidas para assegurar interlocução adequada com a alta administração e participação nas decisões estratégicas, orçamentárias, contratuais e de gestão de riscos relacionadas à tecnologia da informação.</t>
         </is>
@@ -11862,6 +11918,11 @@
       </c>
       <c r="L14" s="1" t="inlineStr">
         <is>
+          <t>alinhando-se à prática MEA01.04 (Avaliar o desempenho) do COBIT 2019</t>
+        </is>
+      </c>
+      <c r="M14" s="1" t="inlineStr">
+        <is>
           <t>estabeleça objetivos, indicadores e metas para a gestão de TIC, de modo a possibilitar o acompanhamento periódico do desempenho da TIC pela alta administração</t>
         </is>
       </c>
@@ -11906,6 +11967,11 @@
       </c>
       <c r="L15" s="1" t="inlineStr">
         <is>
+          <t>alinhando-se à prática MEA01.04 (Avaliar o desempenho) do COBIT 2019 e em observância ao art. 7º, inciso I, da Resolução CNJ nº 370/2021</t>
+        </is>
+      </c>
+      <c r="M15" s="1" t="inlineStr">
+        <is>
           <t>estabeleça objetivos, indicadores e metas para a gestão de TIC, de modo a possibilitar o acompanhamento periódico do desempenho da TIC pela alta administração</t>
         </is>
       </c>
@@ -11949,6 +12015,11 @@
         </is>
       </c>
       <c r="L16" s="1" t="inlineStr">
+        <is>
+          <t>alinhando-se à prática MEA01.04 (Avaliar o desempenho) do COBIT 2019 e em observância ao art. 11, § 1º, da Resolução CNMP nº 171/2017</t>
+        </is>
+      </c>
+      <c r="M16" s="1" t="inlineStr">
         <is>
           <t>estabeleça objetivos, indicadores e metas para a gestão de TIC, de modo a possibilitar o acompanhamento periódico do desempenho da TIC pela alta administração</t>
         </is>
@@ -11990,6 +12061,11 @@
       </c>
       <c r="L17" s="1" t="inlineStr">
         <is>
+          <t>em consonância com o item II.1 do Acórdão TCE-RJ nº 44.490/2024-PLEN e com a referência do art. 6º, § 2º, do Decreto nº 12.198/2024</t>
+        </is>
+      </c>
+      <c r="M17" s="1" t="inlineStr">
+        <is>
           <t>institua formalmente Comitê de TIC ou instância colegiada equivalente, compatível com o porte e a estrutura decisória da organização, definindo em seu ato constitutivo, minimamente, a participação de representantes de áreas relevantes da organização, suas competências, a periodicidade de reuniões, a forma de registro das deliberações e os mecanismos de acompanhamento dos encaminhamentos</t>
         </is>
       </c>
@@ -12034,6 +12110,11 @@
       </c>
       <c r="L18" s="1" t="inlineStr">
         <is>
+          <t>em consonância com o item II.1 do Acórdão TCE-RJ nº 44.490/2024-PLEN e em observância ao art. 5º do Anexo C da Portaria PRODERJ/PRE nº 825/2021</t>
+        </is>
+      </c>
+      <c r="M18" s="1" t="inlineStr">
+        <is>
           <t>institua formalmente Comitê de TIC ou instância colegiada equivalente, compatível com o porte e a estrutura decisória da organização, definindo em seu ato constitutivo, minimamente, a participação de representantes de áreas relevantes da organização, suas competências, a periodicidade de reuniões, a forma de registro das deliberações e os mecanismos de acompanhamento dos encaminhamentos</t>
         </is>
       </c>
@@ -12078,6 +12159,11 @@
       </c>
       <c r="L19" s="1" t="inlineStr">
         <is>
+          <t>em consonância com o item II.1 do Acórdão TCE-RJ nº 44.490/2024-PLEN e em observância ao art. 7º da Resolução CNJ nº 370/2021</t>
+        </is>
+      </c>
+      <c r="M19" s="1" t="inlineStr">
+        <is>
           <t>institua formalmente Comitê de TIC ou instância colegiada equivalente, compatível com o porte e a estrutura decisória da organização, definindo em seu ato constitutivo, minimamente, a participação de representantes de áreas relevantes da organização, suas competências, a periodicidade de reuniões, a forma de registro das deliberações e os mecanismos de acompanhamento dos encaminhamentos</t>
         </is>
       </c>
@@ -12121,6 +12207,11 @@
         </is>
       </c>
       <c r="L20" s="1" t="inlineStr">
+        <is>
+          <t>em consonância com o item II.1 do Acórdão TCE-RJ nº 44.490/2024-PLEN e em observância ao art. 13 da Resolução CNMP nº 171/2017</t>
+        </is>
+      </c>
+      <c r="M20" s="1" t="inlineStr">
         <is>
           <t>institua formalmente Comitê de TIC ou instância colegiada equivalente, compatível com o porte e a estrutura decisória da organização, definindo em seu ato constitutivo, minimamente, a participação de representantes de áreas relevantes da organização, suas competências, a periodicidade de reuniões, a forma de registro das deliberações e os mecanismos de acompanhamento dos encaminhamentos</t>
         </is>
@@ -12162,6 +12253,11 @@
       </c>
       <c r="L21" s="1" t="inlineStr">
         <is>
+          <t>em consonância com o item II.1 do Acórdão TCE-RJ nº 44.490/2024-PLEN e com a referência do art. 6º, § 2º, do Decreto nº 12.198/2024</t>
+        </is>
+      </c>
+      <c r="M21" s="1" t="inlineStr">
+        <is>
           <t>assegure o funcionamento efetivo do Comitê de TIC ou instância colegiada equivalente, mediante o exercício das competências previstas em seu ato constitutivo, com registro das deliberações e acompanhamento dos respectivos encaminhamentos</t>
         </is>
       </c>
@@ -12206,6 +12302,11 @@
       </c>
       <c r="L22" s="1" t="inlineStr">
         <is>
+          <t>em consonância com o item II.1 do Acórdão TCE-RJ nº 44.490/2024-PLEN e em observância ao art. 7º da Resolução CNJ nº 370/2021</t>
+        </is>
+      </c>
+      <c r="M22" s="1" t="inlineStr">
+        <is>
           <t>assegure o funcionamento efetivo do Comitê de TIC ou instância colegiada equivalente, mediante o exercício das competências previstas em seu ato constitutivo, com registro das deliberações e acompanhamento dos respectivos encaminhamentos</t>
         </is>
       </c>
@@ -12249,6 +12350,11 @@
         </is>
       </c>
       <c r="L23" s="1" t="inlineStr">
+        <is>
+          <t>em consonância com o item II.1 do Acórdão TCE-RJ nº 44.490/2024-PLEN e em observância ao art. 14 da Resolução CNMP nº 171/2017</t>
+        </is>
+      </c>
+      <c r="M23" s="1" t="inlineStr">
         <is>
           <t>assegure o funcionamento efetivo do Comitê de TIC ou instância colegiada equivalente, mediante o exercício das competências previstas em seu ato constitutivo, com registro das deliberações e acompanhamento dos respectivos encaminhamentos</t>
         </is>
@@ -12290,6 +12396,11 @@
       </c>
       <c r="L24" s="1" t="inlineStr">
         <is>
+          <t>em consonância com o item II.3 do Acórdão TCE-RJ nº 44.490/2024-PLEN e com o item 9.1.6 do Acórdão nº 1.411/2014-TCU-Plenário</t>
+        </is>
+      </c>
+      <c r="M24" s="1" t="inlineStr">
+        <is>
           <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades e participação das áreas demandantes</t>
         </is>
       </c>
@@ -12334,6 +12445,11 @@
       </c>
       <c r="L25" s="1" t="inlineStr">
         <is>
+          <t>em consonância com o item II.3 do Acórdão TCE-RJ nº 44.490/2024-PLEN e em observância ao art. 2º da Portaria PRODERJ/PRE nº 825/2021</t>
+        </is>
+      </c>
+      <c r="M25" s="1" t="inlineStr">
+        <is>
           <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades e participação das áreas demandantes</t>
         </is>
       </c>
@@ -12378,6 +12494,11 @@
       </c>
       <c r="L26" s="1" t="inlineStr">
         <is>
+          <t>em consonância com o item II.3 do Acórdão TCE-RJ nº 44.490/2024-PLEN e em observância ao art. 6º da Resolução CNJ nº 370/2021</t>
+        </is>
+      </c>
+      <c r="M26" s="1" t="inlineStr">
+        <is>
           <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades e participação das áreas demandantes</t>
         </is>
       </c>
@@ -12421,6 +12542,11 @@
         </is>
       </c>
       <c r="L27" s="1" t="inlineStr">
+        <is>
+          <t>em consonância com o item II.3 do Acórdão TCE-RJ nº 44.490/2024-PLEN e em observância ao art. 12 da Resolução CNMP nº 171/2017</t>
+        </is>
+      </c>
+      <c r="M27" s="1" t="inlineStr">
         <is>
           <t>institua processo formal de planejamento de TIC, compatível com o porte e a complexidade da organização, que assegure a elaboração e manutenção de plano de TIC, atentando-se, minimamente, em definir etapas, responsabilidades e participação das áreas demandantes</t>
         </is>
@@ -12462,6 +12588,11 @@
       </c>
       <c r="L28" s="1" t="inlineStr">
         <is>
+          <t>em consonância com o item II.3 do Acórdão TCE-RJ nº 44.490/2024-PLEN e com o item 9.1.6 do Acórdão nº 1.411/2014-TCU-Plenário</t>
+        </is>
+      </c>
+      <c r="M28" s="1" t="inlineStr">
+        <is>
           <t>submeta o plano de TIC à aprovação formal do dirigente máximo ou de instância competente da alta administração, mantendo registro do respectivo ato de aprovação</t>
         </is>
       </c>
@@ -12506,6 +12637,11 @@
       </c>
       <c r="L29" s="1" t="inlineStr">
         <is>
+          <t>em consonância com o item II.3 do Acórdão TCE-RJ nº 44.490/2024-PLEN e em observância ao art. 11, parágrafo único, do Anexo C da Portaria PRODERJ/PRE nº 825/2021</t>
+        </is>
+      </c>
+      <c r="M29" s="1" t="inlineStr">
+        <is>
           <t>submeta o plano de TIC à aprovação formal do dirigente máximo ou de instância competente da alta administração, mantendo registro do respectivo ato de aprovação</t>
         </is>
       </c>
@@ -12550,6 +12686,11 @@
       </c>
       <c r="L30" s="1" t="inlineStr">
         <is>
+          <t>em consonância com o item II.3 do Acórdão TCE-RJ nº 44.490/2024-PLEN e em observância ao art. 7º, inciso II, da Resolução CNJ nº 370/2021</t>
+        </is>
+      </c>
+      <c r="M30" s="1" t="inlineStr">
+        <is>
           <t>submeta o plano de TIC à aprovação formal do dirigente máximo ou de instância competente da alta administração, mantendo registro do respectivo ato de aprovação</t>
         </is>
       </c>
@@ -12593,6 +12734,11 @@
         </is>
       </c>
       <c r="L31" s="1" t="inlineStr">
+        <is>
+          <t>em consonância com o item II.3 do Acórdão TCE-RJ nº 44.490/2024-PLEN e em observância ao art. 12 da Resolução CNMP nº 171/2017</t>
+        </is>
+      </c>
+      <c r="M31" s="1" t="inlineStr">
         <is>
           <t>submeta o plano de TIC à aprovação formal do dirigente máximo ou de instância competente da alta administração, mantendo registro do respectivo ato de aprovação</t>
         </is>
@@ -12634,6 +12780,11 @@
       </c>
       <c r="L32" s="1" t="inlineStr">
         <is>
+          <t>em consonância com o item II.3 do Acórdão TCE-RJ nº 44.490/2024-PLEN e com o item 9.1.6 do Acórdão nº 1.411/2014-TCU-Plenário</t>
+        </is>
+      </c>
+      <c r="M32" s="1" t="inlineStr">
+        <is>
           <t>revise o plano de TIC para explicitar seu alinhamento ao planejamento institucional, às diretrizes superiores e às necessidades das áreas finalísticas e administrativas, relacionando objetivos, iniciativas, indicadores e metas de TIC aos resultados institucionais pretendidos</t>
         </is>
       </c>
@@ -12678,6 +12829,11 @@
       </c>
       <c r="L33" s="1" t="inlineStr">
         <is>
+          <t>em consonância com o item II.3 do Acórdão TCE-RJ nº 44.490/2024-PLEN e em observância ao art. 3º da Portaria PRODERJ/PRE nº 825/2021</t>
+        </is>
+      </c>
+      <c r="M33" s="1" t="inlineStr">
+        <is>
           <t>revise o plano de TIC para explicitar seu alinhamento ao planejamento institucional, às diretrizes superiores e às necessidades das áreas finalísticas e administrativas, relacionando objetivos, iniciativas, indicadores e metas de TIC aos resultados institucionais pretendidos</t>
         </is>
       </c>
@@ -12722,6 +12878,11 @@
       </c>
       <c r="L34" s="1" t="inlineStr">
         <is>
+          <t>em consonância com o item II.3 do Acórdão TCE-RJ nº 44.490/2024-PLEN e em observância ao art. 6º da Resolução CNJ nº 370/2021</t>
+        </is>
+      </c>
+      <c r="M34" s="1" t="inlineStr">
+        <is>
           <t>revise o plano de TIC para explicitar seu alinhamento ao planejamento institucional, às diretrizes superiores e às necessidades das áreas finalísticas e administrativas, relacionando objetivos, iniciativas, indicadores e metas de TIC aos resultados institucionais pretendidos</t>
         </is>
       </c>
@@ -12765,6 +12926,11 @@
         </is>
       </c>
       <c r="L35" s="1" t="inlineStr">
+        <is>
+          <t>em consonância com o item II.3 do Acórdão TCE-RJ nº 44.490/2024-PLEN e em observância ao art. 11 da Resolução CNMP nº 171/2017</t>
+        </is>
+      </c>
+      <c r="M35" s="1" t="inlineStr">
         <is>
           <t>revise o plano de TIC para explicitar seu alinhamento ao planejamento institucional, às diretrizes superiores e às necessidades das áreas finalísticas e administrativas, relacionando objetivos, iniciativas, indicadores e metas de TIC aos resultados institucionais pretendidos</t>
         </is>
@@ -12806,6 +12972,11 @@
       </c>
       <c r="L36" s="1" t="inlineStr">
         <is>
+          <t>alinhando-se à prática APO06.03 (Criar e manter orçamentos) do COBIT 2019 e em consonância com o item II.3 do Acórdão TCE-RJ nº 44.490/2024-PLEN</t>
+        </is>
+      </c>
+      <c r="M36" s="1" t="inlineStr">
+        <is>
           <t>integre o plano de TIC à elaboração da proposta orçamentária e do plano de contratações, de maneira proporcional ao porte, à estrutura e à capacidade de planejamento da organização</t>
         </is>
       </c>
@@ -12850,6 +13021,11 @@
       </c>
       <c r="L37" s="1" t="inlineStr">
         <is>
+          <t>em consonância com o item II.3 do Acórdão TCE-RJ nº 44.490/2024-PLEN e em observância ao art. 5º da IN PRODERJ/PRE nº 5/2024</t>
+        </is>
+      </c>
+      <c r="M37" s="1" t="inlineStr">
+        <is>
           <t>integre o plano de TIC à elaboração da proposta orçamentária e do plano de contratações, de maneira proporcional ao porte, à estrutura e à capacidade de planejamento da organização</t>
         </is>
       </c>
@@ -12894,6 +13070,11 @@
       </c>
       <c r="L38" s="1" t="inlineStr">
         <is>
+          <t>em consonância com o item II.3 do Acórdão TCE-RJ nº 44.490/2024-PLEN e em observância ao art. 6º da Resolução CNJ nº 370/2021</t>
+        </is>
+      </c>
+      <c r="M38" s="1" t="inlineStr">
+        <is>
           <t>integre o plano de TIC à elaboração da proposta orçamentária e do plano de contratações, de maneira proporcional ao porte, à estrutura e à capacidade de planejamento da organização</t>
         </is>
       </c>
@@ -12937,6 +13118,11 @@
         </is>
       </c>
       <c r="L39" s="1" t="inlineStr">
+        <is>
+          <t>em consonância com o item II.3 do Acórdão TCE-RJ nº 44.490/2024-PLEN e em observância ao art. 5º da Resolução CNMP nº 283/2024</t>
+        </is>
+      </c>
+      <c r="M39" s="1" t="inlineStr">
         <is>
           <t>integre o plano de TIC à elaboração da proposta orçamentária e do plano de contratações, de maneira proporcional ao porte, à estrutura e à capacidade de planejamento da organização</t>
         </is>
@@ -12978,6 +13164,11 @@
       </c>
       <c r="L40" s="1" t="inlineStr">
         <is>
+          <t>em consonância com o item II.3 do Acórdão TCE-RJ nº 44.490/2024-PLEN</t>
+        </is>
+      </c>
+      <c r="M40" s="1" t="inlineStr">
+        <is>
           <t>estabeleça e execute rotina periódica de acompanhamento da execução do plano de TIC, promovendo sua revisão periódica e os ajustes ou atualizações necessários, com registro das principais decisões e reprogramações</t>
         </is>
       </c>
@@ -13022,6 +13213,11 @@
       </c>
       <c r="L41" s="1" t="inlineStr">
         <is>
+          <t>em consonância com o item II.3 do Acórdão TCE-RJ nº 44.490/2024-PLEN e em observância ao art. 13 do Anexo C da Portaria PRODERJ/PRE nº 825/2021</t>
+        </is>
+      </c>
+      <c r="M41" s="1" t="inlineStr">
+        <is>
           <t>estabeleça e execute rotina periódica de acompanhamento da execução do plano de TIC, promovendo sua revisão periódica e os ajustes ou atualizações necessários, com registro das principais decisões e reprogramações</t>
         </is>
       </c>
@@ -13065,6 +13261,11 @@
         </is>
       </c>
       <c r="L42" s="1" t="inlineStr">
+        <is>
+          <t>em consonância com o item II.3 do Acórdão TCE-RJ nº 44.490/2024-PLEN e em observância ao art. 12 da Resolução CNMP nº 171/2017</t>
+        </is>
+      </c>
+      <c r="M42" s="1" t="inlineStr">
         <is>
           <t>estabeleça e execute rotina periódica de acompanhamento da execução do plano de TIC, promovendo sua revisão periódica e os ajustes ou atualizações necessários, com registro das principais decisões e reprogramações</t>
         </is>
@@ -13106,6 +13307,11 @@
       </c>
       <c r="L43" s="1" t="inlineStr">
         <is>
+          <t>alinhando-se à prática APO07.01 (Adquirir e manter pessoal adequado e apropriado) do COBIT 2019 e ao item 9.1.7 do Acórdão nº 1.411/2014-TCU-Plenário</t>
+        </is>
+      </c>
+      <c r="M43" s="1" t="inlineStr">
+        <is>
           <t>avalie a força de trabalho dedicada à TIC e adote medidas proporcionais para assegurar capacidade mínima de planejamento, gestão, proteção, contratação, fiscalização e sustentação dos serviços e ativos de TIC</t>
         </is>
       </c>
@@ -13149,6 +13355,11 @@
         </is>
       </c>
       <c r="L44" s="1" t="inlineStr">
+        <is>
+          <t>em observância ao art. 24 da Resolução CNJ nº 370/2021 e alinhando-se à prática APO07.01 (Adquirir e manter pessoal adequado e apropriado) do COBIT 2019</t>
+        </is>
+      </c>
+      <c r="M44" s="1" t="inlineStr">
         <is>
           <t>avalie a força de trabalho dedicada à TIC e adote medidas proporcionais para assegurar capacidade mínima de planejamento, gestão, proteção, contratação, fiscalização e sustentação dos serviços e ativos de TIC</t>
         </is>
@@ -13190,6 +13401,11 @@
       </c>
       <c r="L45" s="1" t="inlineStr">
         <is>
+          <t>alinhando-se à prática APO07.05 (Planejar e monitorar o uso de recursos humanos de TI e de negócio) do COBIT 2019 e ao item 9.1.6.5 do Acórdão nº 1.411/2014-TCU-Plenário</t>
+        </is>
+      </c>
+      <c r="M45" s="1" t="inlineStr">
+        <is>
           <t>estime e mantenha atualizado o quantitativo necessário de pessoal de TIC e segurança da informação, considerando o porte e a complexidade da organização, os serviços críticos, os sistemas mantidos, as contratações vigentes e os riscos relevantes</t>
         </is>
       </c>
@@ -13233,6 +13449,11 @@
         </is>
       </c>
       <c r="L46" s="1" t="inlineStr">
+        <is>
+          <t>em observância ao art. 24 da Resolução CNJ nº 370/2021 e alinhando-se à prática APO07.05 (Planejar e monitorar o uso de recursos humanos de TI e de negócio) do COBIT 2019</t>
+        </is>
+      </c>
+      <c r="M46" s="1" t="inlineStr">
         <is>
           <t>estime e mantenha atualizado o quantitativo necessário de pessoal de TIC e segurança da informação, considerando o porte e a complexidade da organização, os serviços críticos, os sistemas mantidos, as contratações vigentes e os riscos relevantes</t>
         </is>
@@ -13274,6 +13495,11 @@
       </c>
       <c r="L47" s="1" t="inlineStr">
         <is>
+          <t>alinhando-se às práticas APO01.05 (Estabelecer papéis e responsabilidades) e APO07.01 (Adquirir e manter pessoal adequado e apropriado) do COBIT 2019</t>
+        </is>
+      </c>
+      <c r="M47" s="1" t="inlineStr">
+        <is>
           <t>avalie a necessidade de formalizar a atribuição de cargos ou funções à TIC e à segurança da informação e adote solução compatível com as necessidades institucionais e a capacidade administrativa da organização</t>
         </is>
       </c>
@@ -13314,6 +13540,11 @@
       </c>
       <c r="L48" s="1" t="inlineStr">
         <is>
+          <t>alinhando-se à prática APO07.06 (Gerenciar pessoal contratado) do COBIT 2019 e ao item I.10.11 do Acórdão TCE-RJ nº 44.490/2024-PLEN</t>
+        </is>
+      </c>
+      <c r="M48" s="1" t="inlineStr">
+        <is>
           <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente para coordenar, supervisionar e fiscalizar as atividades e os contratos de TIC executados predominantemente por terceiros, preservando responsabilização e retenção de conhecimento</t>
         </is>
       </c>
@@ -13357,6 +13588,11 @@
         </is>
       </c>
       <c r="L49" s="1" t="inlineStr">
+        <is>
+          <t>em observância ao art. 8º, § 1º, da Resolução CNJ nº 468/2022, em consonância com o item I.10.11 do Acórdão TCE-RJ nº 44.490/2024-PLEN e alinhando-se à prática APO07.06 (Gerenciar pessoal contratado) do COBIT 2019</t>
+        </is>
+      </c>
+      <c r="M49" s="1" t="inlineStr">
         <is>
           <t>avalie o modelo de operação de TIC e adote medidas proporcionais para assegurar capacidade interna suficiente para coordenar, supervisionar e fiscalizar as atividades e os contratos de TIC executados predominantemente por terceiros, preservando responsabilização e retenção de conhecimento</t>
         </is>
@@ -13398,6 +13634,11 @@
       </c>
       <c r="L50" s="1" t="inlineStr">
         <is>
+          <t>alinhando-se à prática APO09.02 (Catalogar serviços facilitados por TI) do COBIT 2019, ao item 8.2.4 da ABNT NBR ISO/IEC 20000-2:2021 e ao item II.7.4 do Acórdão TCE-RJ nº 44.490/2024-PLEN</t>
+        </is>
+      </c>
+      <c r="M50" s="1" t="inlineStr">
+        <is>
           <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
         </is>
       </c>
@@ -13442,6 +13683,11 @@
       </c>
       <c r="L51" s="1" t="inlineStr">
         <is>
+          <t>em observância ao art. 21, inciso IV, alínea "d", da Resolução CNJ nº 370/2021 e alinhando-se à prática APO09.02 (Catalogar serviços facilitados por TI) do COBIT 2019 e ao item 8.2.4 da ABNT NBR ISO/IEC 20000-2:2021</t>
+        </is>
+      </c>
+      <c r="M51" s="1" t="inlineStr">
+        <is>
           <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
         </is>
       </c>
@@ -13485,6 +13731,11 @@
         </is>
       </c>
       <c r="L52" s="1" t="inlineStr">
+        <is>
+          <t>em observância ao art. 23 da Resolução CNMP nº 171/2017 e alinhando-se à prática APO09.02 (Catalogar serviços facilitados por TI) do COBIT 2019 e ao item 8.2.4 da ABNT NBR ISO/IEC 20000-2:2021</t>
+        </is>
+      </c>
+      <c r="M52" s="1" t="inlineStr">
         <is>
           <t>institua e mantenha atualizado catálogo de serviços de TIC, atentando-se, minimamente, em identificar os serviços efetivamente prestados, seus responsáveis, usuários, condições de acesso e informações necessárias ao atendimento das áreas demandantes</t>
         </is>
@@ -13526,6 +13777,11 @@
       </c>
       <c r="L53" s="1" t="inlineStr">
         <is>
+          <t>alinhando-se à prática de gerenciamento de nível de serviço do ITIL 4 e ao item II.7.7 do Acórdão TCE-RJ nº 44.490/2024-PLEN</t>
+        </is>
+      </c>
+      <c r="M53" s="1" t="inlineStr">
+        <is>
           <t>defina, acorde e monitore níveis de serviço para os serviços de TIC relevantes, estabelecendo metas e mecanismos de acompanhamento de seu cumprimento</t>
         </is>
       </c>
@@ -13569,6 +13825,11 @@
         </is>
       </c>
       <c r="L54" s="1" t="inlineStr">
+        <is>
+          <t>em observância ao art. 23 da Resolução CNMP nº 171/2017 e alinhando-se à prática de gerenciamento de nível de serviço do ITIL 4</t>
+        </is>
+      </c>
+      <c r="M54" s="1" t="inlineStr">
         <is>
           <t>defina, acorde e monitore níveis de serviço para os serviços de TIC relevantes, estabelecendo metas e mecanismos de acompanhamento de seu cumprimento</t>
         </is>
@@ -13610,6 +13871,11 @@
       </c>
       <c r="L55" s="1" t="inlineStr">
         <is>
+          <t>alinhando-se à prática de gerenciamento de ativos de TI do ITIL 4 e ao item II.7.5 do Acórdão TCE-RJ nº 44.490/2024-PLEN</t>
+        </is>
+      </c>
+      <c r="M55" s="1" t="inlineStr">
+        <is>
           <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos sob gestão da organização, contemplando, minimamente, os dispositivos e softwares utilizados, com informações suficientes para sua identificação e controle</t>
         </is>
       </c>
@@ -13654,6 +13920,11 @@
       </c>
       <c r="L56" s="1" t="inlineStr">
         <is>
+          <t>em observância ao art. 4º, inciso V, do Decreto Estadual nº 48.997/2024 e alinhando-se à prática de gerenciamento de ativos de TI do ITIL 4</t>
+        </is>
+      </c>
+      <c r="M56" s="1" t="inlineStr">
+        <is>
           <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos sob gestão da organização, contemplando, minimamente, os dispositivos e softwares utilizados, com informações suficientes para sua identificação e controle</t>
         </is>
       </c>
@@ -13698,6 +13969,11 @@
       </c>
       <c r="L57" s="1" t="inlineStr">
         <is>
+          <t>em observância ao art. 34, § 2º, da Resolução CNJ nº 370/2021 e alinhando-se à prática de gerenciamento de ativos de TI do ITIL 4</t>
+        </is>
+      </c>
+      <c r="M57" s="1" t="inlineStr">
+        <is>
           <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos sob gestão da organização, contemplando, minimamente, os dispositivos e softwares utilizados, com informações suficientes para sua identificação e controle</t>
         </is>
       </c>
@@ -13741,6 +14017,11 @@
         </is>
       </c>
       <c r="L58" s="1" t="inlineStr">
+        <is>
+          <t>em observância ao art. 26, inciso II, da Resolução CNMP nº 171/2017 e alinhando-se à prática de gerenciamento de ativos de TI do ITIL 4</t>
+        </is>
+      </c>
+      <c r="M58" s="1" t="inlineStr">
         <is>
           <t>estabeleça e mantenha inventário atualizado dos ativos tecnológicos sob gestão da organização, contemplando, minimamente, os dispositivos e softwares utilizados, com informações suficientes para sua identificação e controle</t>
         </is>
@@ -13782,6 +14063,11 @@
       </c>
       <c r="L59" s="1" t="inlineStr">
         <is>
+          <t>alinhando-se à prática BAI10.01 (Estabelecer e manter um modelo de configuração) do COBIT 2019, ao item 8.2.6 da ABNT NBR ISO/IEC 20000-2:2021 e ao item II.7.5 do Acórdão TCE-RJ nº 44.490/2024-PLEN</t>
+        </is>
+      </c>
+      <c r="M59" s="1" t="inlineStr">
+        <is>
           <t>formalize e execute processo de gestão de configuração, atentando-se, minimamente, em manter base, ferramenta ou registro equivalente com os itens de configuração relevantes, seus responsáveis e os relacionamentos entre ativos</t>
         </is>
       </c>
@@ -13822,6 +14108,11 @@
       </c>
       <c r="L60" s="1" t="inlineStr">
         <is>
+          <t>alinhando-se à prática DSS02.02 (Classificar solicitações e incidentes) do COBIT 2019, ao item 8.6.1 da ABNT NBR ISO/IEC 20000-2:2021 e ao item II.7.6 do Acórdão TCE-RJ nº 44.490/2024-PLEN</t>
+        </is>
+      </c>
+      <c r="M60" s="1" t="inlineStr">
+        <is>
           <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
@@ -13866,6 +14157,11 @@
       </c>
       <c r="L61" s="1" t="inlineStr">
         <is>
+          <t>em observância ao art. 21, inciso IV, alínea "f", da Resolução CNJ nº 370/2021 e alinhando-se à prática DSS02.02 (Classificar solicitações e incidentes) do COBIT 2019 e ao item 8.6.1 da ABNT NBR ISO/IEC 20000-2:2021</t>
+        </is>
+      </c>
+      <c r="M61" s="1" t="inlineStr">
+        <is>
           <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
       </c>
@@ -13909,6 +14205,11 @@
         </is>
       </c>
       <c r="L62" s="1" t="inlineStr">
+        <is>
+          <t>em observância ao art. 23 da Resolução CNMP nº 171/2017 e alinhando-se à prática DSS02.02 (Classificar solicitações e incidentes) do COBIT 2019 e ao item 8.6.1 da ABNT NBR ISO/IEC 20000-2:2021</t>
+        </is>
+      </c>
+      <c r="M62" s="1" t="inlineStr">
         <is>
           <t>formalize e execute processo de gestão de incidentes de TIC, atentando-se, minimamente, em definir papéis, critérios de priorização e escalamento, tratamento de incidentes de serviços e de segurança da informação e registro sistemático e rastreável das ocorrências</t>
         </is>
@@ -13950,6 +14251,11 @@
       </c>
       <c r="L63" s="1" t="inlineStr">
         <is>
+          <t>em observância aos arts. 11, parágrafo único, e 19, inciso IV, da Lei nº 14.133/2021 e ao item 9.1.7 do Acórdão nº 2.342/2016-TCU-Plenário</t>
+        </is>
+      </c>
+      <c r="M63" s="1" t="inlineStr">
+        <is>
           <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
         </is>
       </c>
@@ -13994,6 +14300,11 @@
       </c>
       <c r="L64" s="1" t="inlineStr">
         <is>
+          <t>em observância aos arts. 11, parágrafo único, e 19, inciso IV, da Lei nº 14.133/2021 e em observância ao art. 4º da IN PRODERJ/PRE nº 5/2024</t>
+        </is>
+      </c>
+      <c r="M64" s="1" t="inlineStr">
+        <is>
           <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
         </is>
       </c>
@@ -14038,6 +14349,11 @@
       </c>
       <c r="L65" s="1" t="inlineStr">
         <is>
+          <t>em observância aos arts. 11, parágrafo único, e 19, inciso IV, da Lei nº 14.133/2021 e em observância ao art. 10 da Resolução CNJ nº 468/2022</t>
+        </is>
+      </c>
+      <c r="M65" s="1" t="inlineStr">
+        <is>
           <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
         </is>
       </c>
@@ -14081,6 +14397,11 @@
         </is>
       </c>
       <c r="L66" s="1" t="inlineStr">
+        <is>
+          <t>em observância aos arts. 11, parágrafo único, e 19, inciso IV, da Lei nº 14.133/2021 e em observância ao art. 8º da Resolução CNMP nº 283/2024</t>
+        </is>
+      </c>
+      <c r="M66" s="1" t="inlineStr">
         <is>
           <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
         </is>
@@ -14122,6 +14443,11 @@
       </c>
       <c r="L67" s="1" t="inlineStr">
         <is>
+          <t>em observância ao art. 11, parágrafo único, da Lei nº 14.133/2021 e alinhando-se à prática BAI02.04 (Obter aprovação dos requisitos da solução) do COBIT 2019 e à referência do art. 12, § 6º, da Instrução Normativa SGD/ME nº 94/2022</t>
+        </is>
+      </c>
+      <c r="M67" s="1" t="inlineStr">
+        <is>
           <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo procedimentos simplificados e proporcionais à natureza, ao risco e ao valor da contratação, preservada análise técnica compatível</t>
         </is>
       </c>
@@ -14162,6 +14488,11 @@
       </c>
       <c r="L68" s="1" t="inlineStr">
         <is>
+          <t>em observância aos arts. 11, parágrafo único, e 12, inciso VII, da Lei nº 14.133/2021 e em consonância com o item III.7 do Acórdão TCE-RJ nº 44.490/2024-PLEN</t>
+        </is>
+      </c>
+      <c r="M68" s="1" t="inlineStr">
+        <is>
           <t>assegure que as contratações de TIC sejam compatíveis com os instrumentos de planejamento de TIC e, quando elaborado, com o Plano de Contratações Anual, promovendo os ajustes ou justificativas cabíveis nos casos excepcionais</t>
         </is>
       </c>
@@ -14206,6 +14537,11 @@
       </c>
       <c r="L69" s="1" t="inlineStr">
         <is>
+          <t>em observância aos arts. 11, parágrafo único, e 12, inciso VII, da Lei nº 14.133/2021 e em observância ao art. 5º da IN PRODERJ/PRE nº 5/2024</t>
+        </is>
+      </c>
+      <c r="M69" s="1" t="inlineStr">
+        <is>
           <t>assegure que as contratações de TIC sejam compatíveis com os instrumentos de planejamento de TIC e, quando elaborado, com o Plano de Contratações Anual, promovendo os ajustes ou justificativas cabíveis nos casos excepcionais</t>
         </is>
       </c>
@@ -14250,6 +14586,11 @@
       </c>
       <c r="L70" s="1" t="inlineStr">
         <is>
+          <t>em observância aos arts. 11, parágrafo único, e 12, inciso VII, da Lei nº 14.133/2021 e em observância ao art. 4º da Resolução CNJ nº 468/2022</t>
+        </is>
+      </c>
+      <c r="M70" s="1" t="inlineStr">
+        <is>
           <t>assegure que as contratações de TIC sejam compatíveis com os instrumentos de planejamento de TIC e, quando elaborado, com o Plano de Contratações Anual, promovendo os ajustes ou justificativas cabíveis nos casos excepcionais</t>
         </is>
       </c>
@@ -14293,6 +14634,11 @@
         </is>
       </c>
       <c r="L71" s="1" t="inlineStr">
+        <is>
+          <t>em observância aos arts. 11, parágrafo único, e 12, inciso VII, da Lei nº 14.133/2021 e em observância ao art. 5º da Resolução CNMP nº 283/2024</t>
+        </is>
+      </c>
+      <c r="M71" s="1" t="inlineStr">
         <is>
           <t>assegure que as contratações de TIC sejam compatíveis com os instrumentos de planejamento de TIC e, quando elaborado, com o Plano de Contratações Anual, promovendo os ajustes ou justificativas cabíveis nos casos excepcionais</t>
         </is>
@@ -14334,6 +14680,11 @@
       </c>
       <c r="L72" s="1" t="inlineStr">
         <is>
+          <t>em observância aos arts. 11, parágrafo único, e 7º, caput, da Lei nº 14.133/2021 e alinhando-se à referência do art. 12, § 6º, da Instrução Normativa SGD/ME nº 94/2022</t>
+        </is>
+      </c>
+      <c r="M72" s="1" t="inlineStr">
+        <is>
           <t>designe formalmente equipe de planejamento para as contratações de TIC, atentando-se, minimamente, em assegurar a participação de integrante da área requisitante e da área técnica de TIC, com definição das responsabilidades de seus integrantes</t>
         </is>
       </c>
@@ -14378,6 +14729,11 @@
       </c>
       <c r="L73" s="1" t="inlineStr">
         <is>
+          <t>em observância aos arts. 11, parágrafo único, e 7º, caput, da Lei nº 14.133/2021 e em observância ao art. 7º da Resolução CNJ nº 468/2022</t>
+        </is>
+      </c>
+      <c r="M73" s="1" t="inlineStr">
+        <is>
           <t>designe formalmente equipe de planejamento para as contratações de TIC, atentando-se, minimamente, em assegurar a participação de integrante da área requisitante e da área técnica de TIC, com definição das responsabilidades de seus integrantes</t>
         </is>
       </c>
@@ -14422,14 +14778,19 @@
       </c>
       <c r="L74" s="1" t="inlineStr">
         <is>
+          <t>em observância aos arts. 11, parágrafo único, e 7º, caput, da Lei nº 14.133/2021 e em observância ao art. 9º da Resolução CNMP nº 283/2024</t>
+        </is>
+      </c>
+      <c r="M74" s="1" t="inlineStr">
+        <is>
           <t>designe formalmente equipe de planejamento para as contratações de TIC, atentando-se, minimamente, em assegurar a participação de integrante da área requisitante e da área técnica de TIC, com definição das responsabilidades de seus integrantes</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:L3"/>
+  <autoFilter ref="A3:M3"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(auditoria): adequar contratações de TIC ao regime das estatais
Declara recomendações nas quatro situações do Achado 6 para empresas estatais, utilizando os critérios existentes como referências orientativas da Lei nº 14.133/2021.

Restringe as variantes de determinação do Executivo estadual aos públicos abrangidos, esclarece as condições do Plano de Contratações Anual e sincroniza o mapa de verificação. Ajusta a narrativa dos critérios no fragmento individual para as estatais.
</commit_message>
<xml_diff>
--- a/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
+++ b/02-Execucao/03-Execucao_Procedimentos/01-Insumos/mapa-verificacao-achados-pos-comentarios-gestor.xlsx
@@ -8193,7 +8193,7 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="29" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="31" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
     <col width="33" customWidth="1" min="7" max="7"/>
     <col width="29" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
@@ -10680,7 +10680,7 @@
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>norma_legal_vinculante</t>
+          <t>norma_legal_com_aplicacao_condicionada</t>
         </is>
       </c>
       <c r="G64" s="1" t="b">
@@ -10711,12 +10711,12 @@
       <c r="D65" s="1" t="inlineStr"/>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>Lei nº 14.133/2021, art. 12, inciso VII — as contratações devem observar o plano de contratações anual, quando elaborado, nos termos do dispositivo.</t>
+          <t>Lei nº 14.133/2021, art. 12, inciso VII e § 1º, e art. 18, caput: previsão de elaboração do Plano de Contratações Anual e compatibilização das contratações com esse plano, quando elaborado, e com as leis orçamentárias.</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>norma_legal_vinculante</t>
+          <t>norma_legal_com_aplicacao_condicionada</t>
         </is>
       </c>
       <c r="G65" s="1" t="b">
@@ -10752,7 +10752,7 @@
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>norma_legal_vinculante</t>
+          <t>norma_legal_com_aplicacao_condicionada</t>
         </is>
       </c>
       <c r="G66" s="1" t="b">
@@ -10788,7 +10788,7 @@
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>norma_legal_vinculante</t>
+          <t>norma_legal_com_aplicacao_condicionada</t>
         </is>
       </c>
       <c r="G67" s="1" t="b">
@@ -11311,7 +11311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M74"/>
+  <dimension ref="A1:M78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -11319,7 +11319,7 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="29" customWidth="1" min="4" max="4"/>
     <col width="29" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="41" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
@@ -14263,7 +14263,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>S6.1.EXECUTIVO_ESTADUAL</t>
+          <t>S6.1.EMPRESAS_ESTATAIS</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -14276,15 +14276,15 @@
       </c>
       <c r="D64" s="1" t="inlineStr">
         <is>
-          <t>Poder Executivo Estadual</t>
-        </is>
-      </c>
-      <c r="E64" s="1" t="inlineStr">
-        <is>
-          <t>EXECUTIVO_ESTADUAL</t>
-        </is>
-      </c>
-      <c r="F64" s="1" t="inlineStr"/>
+          <t>Empresas estatais</t>
+        </is>
+      </c>
+      <c r="E64" s="1" t="inlineStr"/>
+      <c r="F64" s="1" t="inlineStr">
+        <is>
+          <t>EMPRESA_ESTATAL</t>
+        </is>
+      </c>
       <c r="G64" s="1" t="inlineStr"/>
       <c r="H64" s="1" t="inlineStr"/>
       <c r="I64" s="1" t="inlineStr"/>
@@ -14295,12 +14295,12 @@
       </c>
       <c r="K64" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="L64" s="1" t="inlineStr">
         <is>
-          <t>em observância aos arts. 11, parágrafo único, e 19, inciso IV, da Lei nº 14.133/2021 e em observância ao art. 4º da IN PRODERJ/PRE nº 5/2024</t>
+          <t>alinhando-se aos arts. 11, parágrafo único, e 19, inciso IV, da Lei nº 14.133/2021 e em observância ao art. 4º da IN PRODERJ/PRE nº 5/2024</t>
         </is>
       </c>
       <c r="M64" s="1" t="inlineStr">
@@ -14312,7 +14312,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>S6.1.JUDICIARIO_ESTADUAL</t>
+          <t>S6.1.EXECUTIVO_ESTADUAL</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -14325,21 +14325,25 @@
       </c>
       <c r="D65" s="1" t="inlineStr">
         <is>
-          <t>Poder Judiciário Estadual</t>
+          <t>Poder Executivo Estadual</t>
         </is>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>JUDICIARIO_ESTADUAL</t>
-        </is>
-      </c>
-      <c r="F65" s="1" t="inlineStr"/>
+          <t>EXECUTIVO_ESTADUAL</t>
+        </is>
+      </c>
+      <c r="F65" s="1" t="inlineStr">
+        <is>
+          <t>ADMINISTRACAO_DIRETA;AUTARQUIA;FUNDACAO</t>
+        </is>
+      </c>
       <c r="G65" s="1" t="inlineStr"/>
       <c r="H65" s="1" t="inlineStr"/>
       <c r="I65" s="1" t="inlineStr"/>
       <c r="J65" s="1" t="inlineStr">
         <is>
-          <t>Q6.C1;Q6.C3;Q6.C13</t>
+          <t>Q6.C1;Q6.C3;Q6.C11</t>
         </is>
       </c>
       <c r="K65" s="1" t="inlineStr">
@@ -14349,7 +14353,7 @@
       </c>
       <c r="L65" s="1" t="inlineStr">
         <is>
-          <t>em observância aos arts. 11, parágrafo único, e 19, inciso IV, da Lei nº 14.133/2021 e em observância ao art. 10 da Resolução CNJ nº 468/2022</t>
+          <t>em observância aos arts. 11, parágrafo único, e 19, inciso IV, da Lei nº 14.133/2021 e em observância ao art. 4º da IN PRODERJ/PRE nº 5/2024</t>
         </is>
       </c>
       <c r="M65" s="1" t="inlineStr">
@@ -14361,7 +14365,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>S6.1.MINISTERIO_PUBLICO_ESTADUAL</t>
+          <t>S6.1.JUDICIARIO_ESTADUAL</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -14374,12 +14378,12 @@
       </c>
       <c r="D66" s="1" t="inlineStr">
         <is>
-          <t>Ministério Público Estadual</t>
+          <t>Poder Judiciário Estadual</t>
         </is>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>MINISTERIO_PUBLICO_ESTADUAL</t>
+          <t>JUDICIARIO_ESTADUAL</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr"/>
@@ -14388,7 +14392,7 @@
       <c r="I66" s="1" t="inlineStr"/>
       <c r="J66" s="1" t="inlineStr">
         <is>
-          <t>Q6.C1;Q6.C3;Q6.C16</t>
+          <t>Q6.C1;Q6.C3;Q6.C13</t>
         </is>
       </c>
       <c r="K66" s="1" t="inlineStr">
@@ -14398,7 +14402,7 @@
       </c>
       <c r="L66" s="1" t="inlineStr">
         <is>
-          <t>em observância aos arts. 11, parágrafo único, e 19, inciso IV, da Lei nº 14.133/2021 e em observância ao art. 8º da Resolução CNMP nº 283/2024</t>
+          <t>em observância aos arts. 11, parágrafo único, e 19, inciso IV, da Lei nº 14.133/2021 e em observância ao art. 10 da Resolução CNJ nº 468/2022</t>
         </is>
       </c>
       <c r="M66" s="1" t="inlineStr">
@@ -14410,57 +14414,61 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>S6.2.GERAL</t>
+          <t>S6.1.MINISTERIO_PUBLICO_ESTADUAL</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
-          <t>S6.2</t>
+          <t>S6.1</t>
         </is>
       </c>
       <c r="C67" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D67" s="1" t="inlineStr">
         <is>
-          <t>Geral</t>
-        </is>
-      </c>
-      <c r="E67" s="1" t="inlineStr"/>
+          <t>Ministério Público Estadual</t>
+        </is>
+      </c>
+      <c r="E67" s="1" t="inlineStr">
+        <is>
+          <t>MINISTERIO_PUBLICO_ESTADUAL</t>
+        </is>
+      </c>
       <c r="F67" s="1" t="inlineStr"/>
       <c r="G67" s="1" t="inlineStr"/>
       <c r="H67" s="1" t="inlineStr"/>
       <c r="I67" s="1" t="inlineStr"/>
       <c r="J67" s="1" t="inlineStr">
         <is>
-          <t>Q6.C1;Q6.C5;Q6.C8</t>
+          <t>Q6.C1;Q6.C3;Q6.C16</t>
         </is>
       </c>
       <c r="K67" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="L67" s="1" t="inlineStr">
         <is>
-          <t>em observância ao art. 11, parágrafo único, da Lei nº 14.133/2021 e alinhando-se à prática BAI02.04 (Obter aprovação dos requisitos da solução) do COBIT 2019 e à referência do art. 12, § 6º, da Instrução Normativa SGD/ME nº 94/2022</t>
+          <t>em observância aos arts. 11, parágrafo único, e 19, inciso IV, da Lei nº 14.133/2021 e em observância ao art. 8º da Resolução CNMP nº 283/2024</t>
         </is>
       </c>
       <c r="M67" s="1" t="inlineStr">
         <is>
-          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo procedimentos simplificados e proporcionais à natureza, ao risco e ao valor da contratação, preservada análise técnica compatível</t>
+          <t>formalize e padronize o processo de planejamento das contratações de TIC, definindo etapas, responsabilidades e artefatos aplicáveis, podendo adotar modelos institucionais ou centralizados já existentes e prevendo fluxos proporcionais à natureza, complexidade e risco da contratação</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>S6.3.GERAL</t>
+          <t>S6.2.GERAL</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
-          <t>S6.3</t>
+          <t>S6.2</t>
         </is>
       </c>
       <c r="C68" s="1" t="b">
@@ -14478,34 +14486,34 @@
       <c r="I68" s="1" t="inlineStr"/>
       <c r="J68" s="1" t="inlineStr">
         <is>
-          <t>Q6.C1;Q6.C2;Q6.C9</t>
+          <t>Q6.C1;Q6.C5;Q6.C8</t>
         </is>
       </c>
       <c r="K68" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="L68" s="1" t="inlineStr">
         <is>
-          <t>em observância aos arts. 11, parágrafo único, e 12, inciso VII, da Lei nº 14.133/2021 e em consonância com o item III.7 do Acórdão TCE-RJ nº 44.490/2024-PLEN</t>
+          <t>em observância ao art. 11, parágrafo único, da Lei nº 14.133/2021 e alinhando-se à prática BAI02.04 (Obter aprovação dos requisitos da solução) do COBIT 2019 e à referência do art. 12, § 6º, da Instrução Normativa SGD/ME nº 94/2022</t>
         </is>
       </c>
       <c r="M68" s="1" t="inlineStr">
         <is>
-          <t>assegure que as contratações de TIC sejam compatíveis com os instrumentos de planejamento de TIC e, quando elaborado, com o Plano de Contratações Anual, promovendo os ajustes ou justificativas cabíveis nos casos excepcionais</t>
+          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo procedimentos simplificados e proporcionais à natureza, ao risco e ao valor da contratação, preservada análise técnica compatível</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>S6.3.EXECUTIVO_ESTADUAL</t>
+          <t>S6.2.EMPRESAS_ESTATAIS</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
         <is>
-          <t>S6.3</t>
+          <t>S6.2</t>
         </is>
       </c>
       <c r="C69" s="1" t="b">
@@ -14513,43 +14521,43 @@
       </c>
       <c r="D69" s="1" t="inlineStr">
         <is>
-          <t>Poder Executivo Estadual</t>
-        </is>
-      </c>
-      <c r="E69" s="1" t="inlineStr">
-        <is>
-          <t>EXECUTIVO_ESTADUAL</t>
-        </is>
-      </c>
-      <c r="F69" s="1" t="inlineStr"/>
+          <t>Empresas estatais</t>
+        </is>
+      </c>
+      <c r="E69" s="1" t="inlineStr"/>
+      <c r="F69" s="1" t="inlineStr">
+        <is>
+          <t>EMPRESA_ESTATAL</t>
+        </is>
+      </c>
       <c r="G69" s="1" t="inlineStr"/>
       <c r="H69" s="1" t="inlineStr"/>
       <c r="I69" s="1" t="inlineStr"/>
       <c r="J69" s="1" t="inlineStr">
         <is>
-          <t>Q6.C1;Q6.C2;Q6.C12</t>
+          <t>Q6.C1;Q6.C5;Q6.C8</t>
         </is>
       </c>
       <c r="K69" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="L69" s="1" t="inlineStr">
         <is>
-          <t>em observância aos arts. 11, parágrafo único, e 12, inciso VII, da Lei nº 14.133/2021 e em observância ao art. 5º da IN PRODERJ/PRE nº 5/2024</t>
+          <t>alinhando-se ao art. 11, parágrafo único, da Lei nº 14.133/2021 e à prática BAI02.04 (Obter aprovação dos requisitos da solução) do COBIT 2019 e à referência do art. 12, § 6º, da Instrução Normativa SGD/ME nº 94/2022</t>
         </is>
       </c>
       <c r="M69" s="1" t="inlineStr">
         <is>
-          <t>assegure que as contratações de TIC sejam compatíveis com os instrumentos de planejamento de TIC e, quando elaborado, com o Plano de Contratações Anual, promovendo os ajustes ou justificativas cabíveis nos casos excepcionais</t>
+          <t>estabeleça a submissão das contratações de TIC à análise prévia da área de TIC, de modo a verificar a compatibilidade da solução com os padrões tecnológicos, os requisitos institucionais e a arquitetura existente, admitindo procedimentos simplificados e proporcionais à natureza, ao risco e ao valor da contratação, preservada análise técnica compatível</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>S6.3.JUDICIARIO_ESTADUAL</t>
+          <t>S6.3.GERAL</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -14558,25 +14566,21 @@
         </is>
       </c>
       <c r="C70" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D70" s="1" t="inlineStr">
         <is>
-          <t>Poder Judiciário Estadual</t>
-        </is>
-      </c>
-      <c r="E70" s="1" t="inlineStr">
-        <is>
-          <t>JUDICIARIO_ESTADUAL</t>
-        </is>
-      </c>
+          <t>Geral</t>
+        </is>
+      </c>
+      <c r="E70" s="1" t="inlineStr"/>
       <c r="F70" s="1" t="inlineStr"/>
       <c r="G70" s="1" t="inlineStr"/>
       <c r="H70" s="1" t="inlineStr"/>
       <c r="I70" s="1" t="inlineStr"/>
       <c r="J70" s="1" t="inlineStr">
         <is>
-          <t>Q6.C1;Q6.C2;Q6.C14</t>
+          <t>Q6.C1;Q6.C2;Q6.C9</t>
         </is>
       </c>
       <c r="K70" s="1" t="inlineStr">
@@ -14586,7 +14590,7 @@
       </c>
       <c r="L70" s="1" t="inlineStr">
         <is>
-          <t>em observância aos arts. 11, parágrafo único, e 12, inciso VII, da Lei nº 14.133/2021 e em observância ao art. 4º da Resolução CNJ nº 468/2022</t>
+          <t>em observância aos arts. 11, parágrafo único, e 12, inciso VII, da Lei nº 14.133/2021 e em consonância com o item III.7 do Acórdão TCE-RJ nº 44.490/2024-PLEN</t>
         </is>
       </c>
       <c r="M70" s="1" t="inlineStr">
@@ -14598,7 +14602,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>S6.3.MINISTERIO_PUBLICO_ESTADUAL</t>
+          <t>S6.3.EMPRESAS_ESTATAIS</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -14611,31 +14615,31 @@
       </c>
       <c r="D71" s="1" t="inlineStr">
         <is>
-          <t>Ministério Público Estadual</t>
-        </is>
-      </c>
-      <c r="E71" s="1" t="inlineStr">
-        <is>
-          <t>MINISTERIO_PUBLICO_ESTADUAL</t>
-        </is>
-      </c>
-      <c r="F71" s="1" t="inlineStr"/>
+          <t>Empresas estatais</t>
+        </is>
+      </c>
+      <c r="E71" s="1" t="inlineStr"/>
+      <c r="F71" s="1" t="inlineStr">
+        <is>
+          <t>EMPRESA_ESTATAL</t>
+        </is>
+      </c>
       <c r="G71" s="1" t="inlineStr"/>
       <c r="H71" s="1" t="inlineStr"/>
       <c r="I71" s="1" t="inlineStr"/>
       <c r="J71" s="1" t="inlineStr">
         <is>
-          <t>Q6.C1;Q6.C2;Q6.C17</t>
+          <t>Q6.C1;Q6.C2;Q6.C12</t>
         </is>
       </c>
       <c r="K71" s="1" t="inlineStr">
         <is>
-          <t>Determinação</t>
+          <t>Recomendação</t>
         </is>
       </c>
       <c r="L71" s="1" t="inlineStr">
         <is>
-          <t>em observância aos arts. 11, parágrafo único, e 12, inciso VII, da Lei nº 14.133/2021 e em observância ao art. 5º da Resolução CNMP nº 283/2024</t>
+          <t>alinhando-se aos arts. 11, parágrafo único, e 12, inciso VII, da Lei nº 14.133/2021 e em observância ao art. 5º da IN PRODERJ/PRE nº 5/2024</t>
         </is>
       </c>
       <c r="M71" s="1" t="inlineStr">
@@ -14647,57 +14651,65 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>S6.4.GERAL</t>
+          <t>S6.3.EXECUTIVO_ESTADUAL</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
         <is>
-          <t>S6.4</t>
+          <t>S6.3</t>
         </is>
       </c>
       <c r="C72" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D72" s="1" t="inlineStr">
         <is>
-          <t>Geral</t>
-        </is>
-      </c>
-      <c r="E72" s="1" t="inlineStr"/>
-      <c r="F72" s="1" t="inlineStr"/>
+          <t>Poder Executivo Estadual</t>
+        </is>
+      </c>
+      <c r="E72" s="1" t="inlineStr">
+        <is>
+          <t>EXECUTIVO_ESTADUAL</t>
+        </is>
+      </c>
+      <c r="F72" s="1" t="inlineStr">
+        <is>
+          <t>ADMINISTRACAO_DIRETA;AUTARQUIA;FUNDACAO</t>
+        </is>
+      </c>
       <c r="G72" s="1" t="inlineStr"/>
       <c r="H72" s="1" t="inlineStr"/>
       <c r="I72" s="1" t="inlineStr"/>
       <c r="J72" s="1" t="inlineStr">
         <is>
-          <t>Q6.C1;Q6.C4;Q6.C8</t>
+          <t>Q6.C1;Q6.C2;Q6.C12</t>
         </is>
       </c>
       <c r="K72" s="1" t="inlineStr">
         <is>
-          <t>Recomendação</t>
+          <t>Determinação</t>
         </is>
       </c>
       <c r="L72" s="1" t="inlineStr">
         <is>
-          <t>em observância aos arts. 11, parágrafo único, e 7º, caput, da Lei nº 14.133/2021 e alinhando-se à referência do art. 12, § 6º, da Instrução Normativa SGD/ME nº 94/2022</t>
+          <t>em observância aos arts. 11, parágrafo único, e 12, inciso VII, da Lei nº 14.133/2021 e em observância ao art. 5º da IN PRODERJ/PRE nº 5/2024</t>
         </is>
       </c>
       <c r="M72" s="1" t="inlineStr">
         <is>
-          <t>designe formalmente equipe de planejamento para as contratações de TIC, atentando-se, minimamente, em assegurar a participação de integrante da área requisitante e da área técnica de TIC, com definição das responsabilidades de seus integrantes</t>
+          <t>assegure que as contratações de TIC sejam compatíveis com os instrumentos de planejamento de TIC e, quando elaborado, com o Plano de Contratações Anual, promovendo os ajustes ou justificativas cabíveis nos casos excepcionais</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>S6.4.JUDICIARIO_ESTADUAL</t>
+          <t>S6.3.JUDICIARIO_ESTADUAL</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
         <is>
-          <t>S6.4</t>
+          <t>S6.3</t>
         </is>
       </c>
       <c r="C73" s="1" t="b">
@@ -14719,7 +14731,7 @@
       <c r="I73" s="1" t="inlineStr"/>
       <c r="J73" s="1" t="inlineStr">
         <is>
-          <t>Q6.C1;Q6.C4;Q6.C15</t>
+          <t>Q6.C1;Q6.C2;Q6.C14</t>
         </is>
       </c>
       <c r="K73" s="1" t="inlineStr">
@@ -14729,24 +14741,24 @@
       </c>
       <c r="L73" s="1" t="inlineStr">
         <is>
-          <t>em observância aos arts. 11, parágrafo único, e 7º, caput, da Lei nº 14.133/2021 e em observância ao art. 7º da Resolução CNJ nº 468/2022</t>
+          <t>em observância aos arts. 11, parágrafo único, e 12, inciso VII, da Lei nº 14.133/2021 e em observância ao art. 4º da Resolução CNJ nº 468/2022</t>
         </is>
       </c>
       <c r="M73" s="1" t="inlineStr">
         <is>
-          <t>designe formalmente equipe de planejamento para as contratações de TIC, atentando-se, minimamente, em assegurar a participação de integrante da área requisitante e da área técnica de TIC, com definição das responsabilidades de seus integrantes</t>
+          <t>assegure que as contratações de TIC sejam compatíveis com os instrumentos de planejamento de TIC e, quando elaborado, com o Plano de Contratações Anual, promovendo os ajustes ou justificativas cabíveis nos casos excepcionais</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>S6.4.MINISTERIO_PUBLICO_ESTADUAL</t>
+          <t>S6.3.MINISTERIO_PUBLICO_ESTADUAL</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
         <is>
-          <t>S6.4</t>
+          <t>S6.3</t>
         </is>
       </c>
       <c r="C74" s="1" t="b">
@@ -14768,20 +14780,212 @@
       <c r="I74" s="1" t="inlineStr"/>
       <c r="J74" s="1" t="inlineStr">
         <is>
+          <t>Q6.C1;Q6.C2;Q6.C17</t>
+        </is>
+      </c>
+      <c r="K74" s="1" t="inlineStr">
+        <is>
+          <t>Determinação</t>
+        </is>
+      </c>
+      <c r="L74" s="1" t="inlineStr">
+        <is>
+          <t>em observância aos arts. 11, parágrafo único, e 12, inciso VII, da Lei nº 14.133/2021 e em observância ao art. 5º da Resolução CNMP nº 283/2024</t>
+        </is>
+      </c>
+      <c r="M74" s="1" t="inlineStr">
+        <is>
+          <t>assegure que as contratações de TIC sejam compatíveis com os instrumentos de planejamento de TIC e, quando elaborado, com o Plano de Contratações Anual, promovendo os ajustes ou justificativas cabíveis nos casos excepcionais</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="inlineStr">
+        <is>
+          <t>S6.4.GERAL</t>
+        </is>
+      </c>
+      <c r="B75" s="1" t="inlineStr">
+        <is>
+          <t>S6.4</t>
+        </is>
+      </c>
+      <c r="C75" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D75" s="1" t="inlineStr">
+        <is>
+          <t>Geral</t>
+        </is>
+      </c>
+      <c r="E75" s="1" t="inlineStr"/>
+      <c r="F75" s="1" t="inlineStr"/>
+      <c r="G75" s="1" t="inlineStr"/>
+      <c r="H75" s="1" t="inlineStr"/>
+      <c r="I75" s="1" t="inlineStr"/>
+      <c r="J75" s="1" t="inlineStr">
+        <is>
+          <t>Q6.C1;Q6.C4;Q6.C8</t>
+        </is>
+      </c>
+      <c r="K75" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="L75" s="1" t="inlineStr">
+        <is>
+          <t>em observância aos arts. 11, parágrafo único, e 7º, caput, da Lei nº 14.133/2021 e alinhando-se à referência do art. 12, § 6º, da Instrução Normativa SGD/ME nº 94/2022</t>
+        </is>
+      </c>
+      <c r="M75" s="1" t="inlineStr">
+        <is>
+          <t>designe formalmente equipe de planejamento para as contratações de TIC, atentando-se, minimamente, em assegurar a participação de integrante da área requisitante e da área técnica de TIC, com definição das responsabilidades de seus integrantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="inlineStr">
+        <is>
+          <t>S6.4.EMPRESAS_ESTATAIS</t>
+        </is>
+      </c>
+      <c r="B76" s="1" t="inlineStr">
+        <is>
+          <t>S6.4</t>
+        </is>
+      </c>
+      <c r="C76" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D76" s="1" t="inlineStr">
+        <is>
+          <t>Empresas estatais</t>
+        </is>
+      </c>
+      <c r="E76" s="1" t="inlineStr"/>
+      <c r="F76" s="1" t="inlineStr">
+        <is>
+          <t>EMPRESA_ESTATAL</t>
+        </is>
+      </c>
+      <c r="G76" s="1" t="inlineStr"/>
+      <c r="H76" s="1" t="inlineStr"/>
+      <c r="I76" s="1" t="inlineStr"/>
+      <c r="J76" s="1" t="inlineStr">
+        <is>
+          <t>Q6.C1;Q6.C4;Q6.C8</t>
+        </is>
+      </c>
+      <c r="K76" s="1" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="L76" s="1" t="inlineStr">
+        <is>
+          <t>alinhando-se aos arts. 11, parágrafo único, e 7º, caput, da Lei nº 14.133/2021 e à referência do art. 12, § 6º, da Instrução Normativa SGD/ME nº 94/2022</t>
+        </is>
+      </c>
+      <c r="M76" s="1" t="inlineStr">
+        <is>
+          <t>designe formalmente equipe de planejamento para as contratações de TIC, atentando-se, minimamente, em assegurar a participação de integrante da área requisitante e da área técnica de TIC, com definição das responsabilidades de seus integrantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="inlineStr">
+        <is>
+          <t>S6.4.JUDICIARIO_ESTADUAL</t>
+        </is>
+      </c>
+      <c r="B77" s="1" t="inlineStr">
+        <is>
+          <t>S6.4</t>
+        </is>
+      </c>
+      <c r="C77" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D77" s="1" t="inlineStr">
+        <is>
+          <t>Poder Judiciário Estadual</t>
+        </is>
+      </c>
+      <c r="E77" s="1" t="inlineStr">
+        <is>
+          <t>JUDICIARIO_ESTADUAL</t>
+        </is>
+      </c>
+      <c r="F77" s="1" t="inlineStr"/>
+      <c r="G77" s="1" t="inlineStr"/>
+      <c r="H77" s="1" t="inlineStr"/>
+      <c r="I77" s="1" t="inlineStr"/>
+      <c r="J77" s="1" t="inlineStr">
+        <is>
+          <t>Q6.C1;Q6.C4;Q6.C15</t>
+        </is>
+      </c>
+      <c r="K77" s="1" t="inlineStr">
+        <is>
+          <t>Determinação</t>
+        </is>
+      </c>
+      <c r="L77" s="1" t="inlineStr">
+        <is>
+          <t>em observância aos arts. 11, parágrafo único, e 7º, caput, da Lei nº 14.133/2021 e em observância ao art. 7º da Resolução CNJ nº 468/2022</t>
+        </is>
+      </c>
+      <c r="M77" s="1" t="inlineStr">
+        <is>
+          <t>designe formalmente equipe de planejamento para as contratações de TIC, atentando-se, minimamente, em assegurar a participação de integrante da área requisitante e da área técnica de TIC, com definição das responsabilidades de seus integrantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="inlineStr">
+        <is>
+          <t>S6.4.MINISTERIO_PUBLICO_ESTADUAL</t>
+        </is>
+      </c>
+      <c r="B78" s="1" t="inlineStr">
+        <is>
+          <t>S6.4</t>
+        </is>
+      </c>
+      <c r="C78" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D78" s="1" t="inlineStr">
+        <is>
+          <t>Ministério Público Estadual</t>
+        </is>
+      </c>
+      <c r="E78" s="1" t="inlineStr">
+        <is>
+          <t>MINISTERIO_PUBLICO_ESTADUAL</t>
+        </is>
+      </c>
+      <c r="F78" s="1" t="inlineStr"/>
+      <c r="G78" s="1" t="inlineStr"/>
+      <c r="H78" s="1" t="inlineStr"/>
+      <c r="I78" s="1" t="inlineStr"/>
+      <c r="J78" s="1" t="inlineStr">
+        <is>
           <t>Q6.C1;Q6.C4;Q6.C18</t>
         </is>
       </c>
-      <c r="K74" s="1" t="inlineStr">
+      <c r="K78" s="1" t="inlineStr">
         <is>
           <t>Determinação</t>
         </is>
       </c>
-      <c r="L74" s="1" t="inlineStr">
+      <c r="L78" s="1" t="inlineStr">
         <is>
           <t>em observância aos arts. 11, parágrafo único, e 7º, caput, da Lei nº 14.133/2021 e em observância ao art. 9º da Resolução CNMP nº 283/2024</t>
         </is>
       </c>
-      <c r="M74" s="1" t="inlineStr">
+      <c r="M78" s="1" t="inlineStr">
         <is>
           <t>designe formalmente equipe de planejamento para as contratações de TIC, atentando-se, minimamente, em assegurar a participação de integrante da área requisitante e da área técnica de TIC, com definição das responsabilidades de seus integrantes</t>
         </is>

</xml_diff>